<commit_message>
Nivå 2 og lavere: slett tittelrad og tom rad, kolonneoverskrifter starter nå på rad 1
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -26,15 +26,15 @@
     <sheet name="Scoringstidspunkt" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="Heatmap" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="Klubber" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Nivå 2 og lavere" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Aldersfordeling" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Spillere etter klubbland" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Alder" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Spillere etter klubbland" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Nivå 2 og lavere" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Klubber'!$A$2:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Nivå 2 og lavere'!$A$3:$F$3</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Spillere etter klubbland'!$A$3:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Spillere etter klubbland'!$A$3:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Nivå 2 og lavere'!$A$1:$F$1</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -46,7 +46,7 @@
     <numFmt numFmtId="164" formatCode="dd\.mm\.yyyy"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="52">
+  <fonts count="53">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -338,8 +338,14 @@
       <color rgb="006B7A99"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="50">
+  <fills count="56">
     <fill>
       <patternFill/>
     </fill>
@@ -586,8 +592,38 @@
         <fgColor rgb="00F0F5FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF5EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF9E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8E0F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2DCE8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -763,11 +799,25 @@
         <color rgb="00E2E8F0"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00CCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="173">
+  <cellXfs count="187">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1255,6 +1305,38 @@
     <xf numFmtId="0" fontId="47" fillId="49" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="52" fillId="50" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="51" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="51" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="52" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="52" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="53" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="53" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="54" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="54" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="51" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="52" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="53" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="55" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="54" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -47028,1943 +47110,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F71"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
-  <cols>
-    <col width="8" customWidth="1" style="143" min="1" max="1"/>
-    <col width="26" customWidth="1" style="143" min="2" max="2"/>
-    <col width="16" customWidth="1" style="143" min="3" max="3"/>
-    <col width="22" customWidth="1" style="143" min="4" max="4"/>
-    <col width="30" customWidth="1" style="143" min="5" max="5"/>
-    <col width="22" customWidth="1" style="143" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="18" customHeight="1" s="143">
-      <c r="A1" s="149" t="inlineStr">
-        <is>
-          <t>FIFA World Cup 2026 — Spillere på nivå 2 og lavere</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="128" t="inlineStr">
-        <is>
-          <t>Nivå</t>
-        </is>
-      </c>
-      <c r="B3" s="128" t="inlineStr">
-        <is>
-          <t>Klubb</t>
-        </is>
-      </c>
-      <c r="C3" s="128" t="inlineStr">
-        <is>
-          <t>Land</t>
-        </is>
-      </c>
-      <c r="D3" s="128" t="inlineStr">
-        <is>
-          <t>Liga</t>
-        </is>
-      </c>
-      <c r="E3" s="128" t="inlineStr">
-        <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="F3" s="128" t="inlineStr">
-        <is>
-          <t>Nasjonallag</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="130" t="inlineStr">
-        <is>
-          <t>Charlton Athletic</t>
-        </is>
-      </c>
-      <c r="C4" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D4" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E4" s="130" t="inlineStr">
-        <is>
-          <t>Lyndon Dykes</t>
-        </is>
-      </c>
-      <c r="F4" s="130" t="inlineStr">
-        <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="130" t="inlineStr">
-        <is>
-          <t>Coventry City</t>
-        </is>
-      </c>
-      <c r="C5" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D5" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E5" s="130" t="inlineStr">
-        <is>
-          <t>Brandon Thomas-Asante</t>
-        </is>
-      </c>
-      <c r="F5" s="130" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="130" t="inlineStr">
-        <is>
-          <t>Coventry City</t>
-        </is>
-      </c>
-      <c r="C6" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D6" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E6" s="130" t="inlineStr">
-        <is>
-          <t>Haji Wright</t>
-        </is>
-      </c>
-      <c r="F6" s="130" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="130" t="inlineStr">
-        <is>
-          <t>Derby County</t>
-        </is>
-      </c>
-      <c r="C7" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D7" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E7" s="130" t="inlineStr">
-        <is>
-          <t>Jacob Widell Zetterström</t>
-        </is>
-      </c>
-      <c r="F7" s="130" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="130" t="inlineStr">
-        <is>
-          <t>Derby County</t>
-        </is>
-      </c>
-      <c r="C8" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D8" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E8" s="130" t="inlineStr">
-        <is>
-          <t>Sondre Langås</t>
-        </is>
-      </c>
-      <c r="F8" s="130" t="inlineStr">
-        <is>
-          <t>Norge</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="130" t="inlineStr">
-        <is>
-          <t>Hull City</t>
-        </is>
-      </c>
-      <c r="C9" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D9" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E9" s="130" t="inlineStr">
-        <is>
-          <t>Amir Hadžiahmetović</t>
-        </is>
-      </c>
-      <c r="F9" s="130" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="130" t="inlineStr">
-        <is>
-          <t>Hull City</t>
-        </is>
-      </c>
-      <c r="C10" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D10" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E10" s="130" t="inlineStr">
-        <is>
-          <t>Ivor Pandur</t>
-        </is>
-      </c>
-      <c r="F10" s="130" t="inlineStr">
-        <is>
-          <t>Kroatia</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="130" t="inlineStr">
-        <is>
-          <t>Hull City</t>
-        </is>
-      </c>
-      <c r="C11" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D11" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E11" s="130" t="inlineStr">
-        <is>
-          <t>Liam Miller</t>
-        </is>
-      </c>
-      <c r="F11" s="130" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="130" t="inlineStr">
-        <is>
-          <t>Middlesbrough</t>
-        </is>
-      </c>
-      <c r="C12" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D12" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E12" s="130" t="inlineStr">
-        <is>
-          <t>Alfie Jones</t>
-        </is>
-      </c>
-      <c r="F12" s="130" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B13" s="130" t="inlineStr">
-        <is>
-          <t>Middlesbrough</t>
-        </is>
-      </c>
-      <c r="C13" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D13" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E13" s="130" t="inlineStr">
-        <is>
-          <t>Sontje Hansen</t>
-        </is>
-      </c>
-      <c r="F13" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B14" s="130" t="inlineStr">
-        <is>
-          <t>Millwall FC</t>
-        </is>
-      </c>
-      <c r="C14" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D14" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E14" s="130" t="inlineStr">
-        <is>
-          <t>Max Crocombe</t>
-        </is>
-      </c>
-      <c r="F14" s="130" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B15" s="130" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C15" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D15" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E15" s="130" t="inlineStr">
-        <is>
-          <t>Ali Ahmed</t>
-        </is>
-      </c>
-      <c r="F15" s="130" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="130" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C16" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D16" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E16" s="130" t="inlineStr">
-        <is>
-          <t>José Córdoba</t>
-        </is>
-      </c>
-      <c r="F16" s="130" t="inlineStr">
-        <is>
-          <t>Panama</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="130" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C17" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D17" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E17" s="130" t="inlineStr">
-        <is>
-          <t>Kenny McLean</t>
-        </is>
-      </c>
-      <c r="F17" s="130" t="inlineStr">
-        <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" s="130" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C18" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D18" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E18" s="130" t="inlineStr">
-        <is>
-          <t>Toure</t>
-        </is>
-      </c>
-      <c r="F18" s="130" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B19" s="130" t="inlineStr">
-        <is>
-          <t>Portsmouth</t>
-        </is>
-      </c>
-      <c r="C19" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D19" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E19" s="130" t="inlineStr">
-        <is>
-          <t>Gustavo Caballero</t>
-        </is>
-      </c>
-      <c r="F19" s="130" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="130" t="inlineStr">
-        <is>
-          <t>Sheffield United</t>
-        </is>
-      </c>
-      <c r="C20" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D20" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E20" s="130" t="inlineStr">
-        <is>
-          <t>Tahith Chong</t>
-        </is>
-      </c>
-      <c r="F20" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B21" s="130" t="inlineStr">
-        <is>
-          <t>Stoke City</t>
-        </is>
-      </c>
-      <c r="C21" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D21" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E21" s="130" t="inlineStr">
-        <is>
-          <t>Viktor Johansson</t>
-        </is>
-      </c>
-      <c r="F21" s="130" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="130" t="inlineStr">
-        <is>
-          <t>Swansea</t>
-        </is>
-      </c>
-      <c r="C22" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D22" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E22" s="130" t="inlineStr">
-        <is>
-          <t>Eom Jisung</t>
-        </is>
-      </c>
-      <c r="F22" s="130" t="inlineStr">
-        <is>
-          <t>Sør-Korea</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="130" t="inlineStr">
-        <is>
-          <t>Swansea City</t>
-        </is>
-      </c>
-      <c r="C23" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D23" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E23" s="130" t="inlineStr">
-        <is>
-          <t>Burgess</t>
-        </is>
-      </c>
-      <c r="F23" s="130" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B24" s="130" t="inlineStr">
-        <is>
-          <t>Swansea City</t>
-        </is>
-      </c>
-      <c r="C24" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D24" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E24" s="130" t="inlineStr">
-        <is>
-          <t>Marko Stamenić</t>
-        </is>
-      </c>
-      <c r="F24" s="130" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="130" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="C25" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D25" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E25" s="130" t="inlineStr">
-        <is>
-          <t>Edo Kayembe</t>
-        </is>
-      </c>
-      <c r="F25" s="130" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B26" s="130" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="C26" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D26" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E26" s="130" t="inlineStr">
-        <is>
-          <t>Egil Selvik</t>
-        </is>
-      </c>
-      <c r="F26" s="130" t="inlineStr">
-        <is>
-          <t>Norge</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" s="130" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="C27" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D27" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E27" s="130" t="inlineStr">
-        <is>
-          <t>Irankunda</t>
-        </is>
-      </c>
-      <c r="F27" s="130" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="130" t="inlineStr">
-        <is>
-          <t>Wrexham</t>
-        </is>
-      </c>
-      <c r="C28" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D28" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E28" s="130" t="inlineStr">
-        <is>
-          <t>Dom Hyam</t>
-        </is>
-      </c>
-      <c r="F28" s="130" t="inlineStr">
-        <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" s="130" t="inlineStr">
-        <is>
-          <t>Wrexham AFC</t>
-        </is>
-      </c>
-      <c r="C29" s="130" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D29" s="130" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E29" s="130" t="inlineStr">
-        <is>
-          <t>Liberato Cacace</t>
-        </is>
-      </c>
-      <c r="F29" s="130" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B30" s="130" t="inlineStr">
-        <is>
-          <t>AS Nancy-Lorraine</t>
-        </is>
-      </c>
-      <c r="C30" s="130" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="D30" s="130" t="inlineStr">
-        <is>
-          <t>Ligue 2</t>
-        </is>
-      </c>
-      <c r="E30" s="130" t="inlineStr">
-        <is>
-          <t>Martin Experience</t>
-        </is>
-      </c>
-      <c r="F30" s="130" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B31" s="130" t="inlineStr">
-        <is>
-          <t>SC Bastia</t>
-        </is>
-      </c>
-      <c r="C31" s="130" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="D31" s="130" t="inlineStr">
-        <is>
-          <t>Ligue 2</t>
-        </is>
-      </c>
-      <c r="E31" s="130" t="inlineStr">
-        <is>
-          <t>Johnny Placide</t>
-        </is>
-      </c>
-      <c r="F31" s="130" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B32" s="130" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="C32" s="130" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D32" s="130" t="inlineStr">
-        <is>
-          <t>Serie B</t>
-        </is>
-      </c>
-      <c r="E32" s="130" t="inlineStr">
-        <is>
-          <t>Farès Ghedjemis</t>
-        </is>
-      </c>
-      <c r="F32" s="130" t="inlineStr">
-        <is>
-          <t>Algerie</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="130" t="inlineStr">
-        <is>
-          <t>UC Sampdoria</t>
-        </is>
-      </c>
-      <c r="C33" s="130" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D33" s="130" t="inlineStr">
-        <is>
-          <t>Serie B</t>
-        </is>
-      </c>
-      <c r="E33" s="130" t="inlineStr">
-        <is>
-          <t>Dennis Hadžikadunić</t>
-        </is>
-      </c>
-      <c r="F33" s="130" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B34" s="130" t="inlineStr">
-        <is>
-          <t>Albirex Niigata</t>
-        </is>
-      </c>
-      <c r="C34" s="130" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D34" s="130" t="inlineStr">
-        <is>
-          <t>J2 League</t>
-        </is>
-      </c>
-      <c r="E34" s="130" t="inlineStr">
-        <is>
-          <t>Geria</t>
-        </is>
-      </c>
-      <c r="F34" s="130" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B35" s="130" t="inlineStr">
-        <is>
-          <t>FC Den Bosch</t>
-        </is>
-      </c>
-      <c r="C35" s="130" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D35" s="130" t="inlineStr">
-        <is>
-          <t>Eerste Divisie</t>
-        </is>
-      </c>
-      <c r="E35" s="130" t="inlineStr">
-        <is>
-          <t>Kevin Felida</t>
-        </is>
-      </c>
-      <c r="F35" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B36" s="130" t="inlineStr">
-        <is>
-          <t>VVV-Venlo</t>
-        </is>
-      </c>
-      <c r="C36" s="130" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D36" s="130" t="inlineStr">
-        <is>
-          <t>Eerste Divisie</t>
-        </is>
-      </c>
-      <c r="E36" s="130" t="inlineStr">
-        <is>
-          <t>Trevor Doornbusch</t>
-        </is>
-      </c>
-      <c r="F36" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B37" s="130" t="inlineStr">
-        <is>
-          <t>Chaves</t>
-        </is>
-      </c>
-      <c r="C37" s="130" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D37" s="130" t="inlineStr">
-        <is>
-          <t>Liga Portugal 2</t>
-        </is>
-      </c>
-      <c r="E37" s="130" t="inlineStr">
-        <is>
-          <t>Josimar Dias "Vozinha"</t>
-        </is>
-      </c>
-      <c r="F37" s="130" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B38" s="130" t="inlineStr">
-        <is>
-          <t>Torreense</t>
-        </is>
-      </c>
-      <c r="C38" s="130" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D38" s="130" t="inlineStr">
-        <is>
-          <t>Liga Portugal 2</t>
-        </is>
-      </c>
-      <c r="E38" s="130" t="inlineStr">
-        <is>
-          <t>Ianique Tavares "Stopira"</t>
-        </is>
-      </c>
-      <c r="F38" s="130" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B39" s="130" t="inlineStr">
-        <is>
-          <t>Castellón</t>
-        </is>
-      </c>
-      <c r="C39" s="130" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D39" s="130" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E39" s="130" t="inlineStr">
-        <is>
-          <t>Brian Cipenga</t>
-        </is>
-      </c>
-      <c r="F39" s="130" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B40" s="130" t="inlineStr">
-        <is>
-          <t>Castellón</t>
-        </is>
-      </c>
-      <c r="C40" s="130" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D40" s="130" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E40" s="130" t="inlineStr">
-        <is>
-          <t>Mabil</t>
-        </is>
-      </c>
-      <c r="F40" s="130" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="130" t="inlineStr">
-        <is>
-          <t>Cultural Leonesa</t>
-        </is>
-      </c>
-      <c r="C41" s="130" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D41" s="130" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E41" s="130" t="inlineStr">
-        <is>
-          <t>Homam Al-Amin</t>
-        </is>
-      </c>
-      <c r="F41" s="130" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B42" s="130" t="inlineStr">
-        <is>
-          <t>Real Oviedo</t>
-        </is>
-      </c>
-      <c r="C42" s="130" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D42" s="130" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E42" s="130" t="inlineStr">
-        <is>
-          <t>Federico Viñas</t>
-        </is>
-      </c>
-      <c r="F42" s="130" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B43" s="130" t="inlineStr">
-        <is>
-          <t>Real Oviedo</t>
-        </is>
-      </c>
-      <c r="C43" s="130" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D43" s="130" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E43" s="130" t="inlineStr">
-        <is>
-          <t>Haissem Hassan</t>
-        </is>
-      </c>
-      <c r="F43" s="130" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B44" s="130" t="inlineStr">
-        <is>
-          <t>Real Oviedo</t>
-        </is>
-      </c>
-      <c r="C44" s="130" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D44" s="130" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E44" s="130" t="inlineStr">
-        <is>
-          <t>Kwasi Sibo</t>
-        </is>
-      </c>
-      <c r="F44" s="130" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B45" s="130" t="inlineStr">
-        <is>
-          <t>Stade Nyonnais</t>
-        </is>
-      </c>
-      <c r="C45" s="130" t="inlineStr">
-        <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-      <c r="D45" s="130" t="inlineStr">
-        <is>
-          <t>Challenge League</t>
-        </is>
-      </c>
-      <c r="E45" s="130" t="inlineStr">
-        <is>
-          <t>Melvin Mastil</t>
-        </is>
-      </c>
-      <c r="F45" s="130" t="inlineStr">
-        <is>
-          <t>Algerie</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B46" s="130" t="inlineStr">
-        <is>
-          <t>IFK Norrköping</t>
-        </is>
-      </c>
-      <c r="C46" s="130" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-      <c r="D46" s="130" t="inlineStr">
-        <is>
-          <t>Superettan</t>
-        </is>
-      </c>
-      <c r="E46" s="130" t="inlineStr">
-        <is>
-          <t>Moutaz Neffati</t>
-        </is>
-      </c>
-      <c r="F46" s="130" t="inlineStr">
-        <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B47" s="130" t="inlineStr">
-        <is>
-          <t>Siwelele FC</t>
-        </is>
-      </c>
-      <c r="C47" s="130" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-      <c r="D47" s="130" t="inlineStr">
-        <is>
-          <t>National First Division</t>
-        </is>
-      </c>
-      <c r="E47" s="130" t="inlineStr">
-        <is>
-          <t>Ricardo Goss</t>
-        </is>
-      </c>
-      <c r="F47" s="130" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B48" s="130" t="inlineStr">
-        <is>
-          <t>Iğdır</t>
-        </is>
-      </c>
-      <c r="C48" s="130" t="inlineStr">
-        <is>
-          <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="D48" s="130" t="inlineStr">
-        <is>
-          <t>TFF 1. Lig</t>
-        </is>
-      </c>
-      <c r="E48" s="130" t="inlineStr">
-        <is>
-          <t>Leandro Bacuna</t>
-        </is>
-      </c>
-      <c r="F48" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B49" s="130" t="inlineStr">
-        <is>
-          <t>Iğdır</t>
-        </is>
-      </c>
-      <c r="C49" s="130" t="inlineStr">
-        <is>
-          <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="D49" s="130" t="inlineStr">
-        <is>
-          <t>TFF 1. Lig</t>
-        </is>
-      </c>
-      <c r="E49" s="130" t="inlineStr">
-        <is>
-          <t>Ryan Mendes</t>
-        </is>
-      </c>
-      <c r="F49" s="130" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B50" s="130" t="inlineStr">
-        <is>
-          <t>Fortuna Düsseldorf</t>
-        </is>
-      </c>
-      <c r="C50" s="130" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D50" s="130" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E50" s="130" t="inlineStr">
-        <is>
-          <t>Cedric Itten</t>
-        </is>
-      </c>
-      <c r="F50" s="130" t="inlineStr">
-        <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B51" s="130" t="inlineStr">
-        <is>
-          <t>Hannover 96</t>
-        </is>
-      </c>
-      <c r="C51" s="130" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D51" s="130" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E51" s="130" t="inlineStr">
-        <is>
-          <t>Ime Okon</t>
-        </is>
-      </c>
-      <c r="F51" s="130" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B52" s="130" t="inlineStr">
-        <is>
-          <t>Hannover 96</t>
-        </is>
-      </c>
-      <c r="C52" s="130" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D52" s="130" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E52" s="130" t="inlineStr">
-        <is>
-          <t>​Elias Saad</t>
-        </is>
-      </c>
-      <c r="F52" s="130" t="inlineStr">
-        <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="130" t="inlineStr">
-        <is>
-          <t>Karlsruher SC</t>
-        </is>
-      </c>
-      <c r="C53" s="130" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D53" s="130" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E53" s="130" t="inlineStr">
-        <is>
-          <t>Dženis Burnić</t>
-        </is>
-      </c>
-      <c r="F53" s="130" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B54" s="130" t="inlineStr">
-        <is>
-          <t>Schalke 04</t>
-        </is>
-      </c>
-      <c r="C54" s="130" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D54" s="130" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E54" s="130" t="inlineStr">
-        <is>
-          <t>Edin Džeko</t>
-        </is>
-      </c>
-      <c r="F54" s="130" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B55" s="130" t="inlineStr">
-        <is>
-          <t>Schalke 04</t>
-        </is>
-      </c>
-      <c r="C55" s="130" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D55" s="130" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E55" s="130" t="inlineStr">
-        <is>
-          <t>Nikola Katić</t>
-        </is>
-      </c>
-      <c r="F55" s="130" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B56" s="130" t="inlineStr">
-        <is>
-          <t>El Paso Locomotive FC</t>
-        </is>
-      </c>
-      <c r="C56" s="130" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D56" s="130" t="inlineStr">
-        <is>
-          <t>USL Championship</t>
-        </is>
-      </c>
-      <c r="E56" s="130" t="inlineStr">
-        <is>
-          <t>Carl-Fred Sainthe</t>
-        </is>
-      </c>
-      <c r="F56" s="130" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B57" s="130" t="inlineStr">
-        <is>
-          <t>Miami FC</t>
-        </is>
-      </c>
-      <c r="C57" s="130" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D57" s="130" t="inlineStr">
-        <is>
-          <t>USL Championship</t>
-        </is>
-      </c>
-      <c r="E57" s="130" t="inlineStr">
-        <is>
-          <t>Eloy Room</t>
-        </is>
-      </c>
-      <c r="F57" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="129" t="n">
-        <v>2</v>
-      </c>
-      <c r="B58" s="130" t="inlineStr">
-        <is>
-          <t>Miami FC</t>
-        </is>
-      </c>
-      <c r="C58" s="130" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D58" s="130" t="inlineStr">
-        <is>
-          <t>USL Championship</t>
-        </is>
-      </c>
-      <c r="E58" s="130" t="inlineStr">
-        <is>
-          <t>Jürgen Locadia</t>
-        </is>
-      </c>
-      <c r="F58" s="130" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="131" t="n">
-        <v>3</v>
-      </c>
-      <c r="B59" s="132" t="inlineStr">
-        <is>
-          <t>Port Vale</t>
-        </is>
-      </c>
-      <c r="C59" s="132" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D59" s="132" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="E59" s="132" t="inlineStr">
-        <is>
-          <t>Ben Waine</t>
-        </is>
-      </c>
-      <c r="F59" s="132" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="131" t="n">
-        <v>3</v>
-      </c>
-      <c r="B60" s="132" t="inlineStr">
-        <is>
-          <t>Rotherham United</t>
-        </is>
-      </c>
-      <c r="C60" s="132" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D60" s="132" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="E60" s="132" t="inlineStr">
-        <is>
-          <t>Ar’Jany Martha</t>
-        </is>
-      </c>
-      <c r="F60" s="132" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="131" t="n">
-        <v>3</v>
-      </c>
-      <c r="B61" s="132" t="inlineStr">
-        <is>
-          <t>FC Sochaux</t>
-        </is>
-      </c>
-      <c r="C61" s="132" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="D61" s="132" t="inlineStr">
-        <is>
-          <t>National</t>
-        </is>
-      </c>
-      <c r="E61" s="132" t="inlineStr">
-        <is>
-          <t>Alexandre Pierre</t>
-        </is>
-      </c>
-      <c r="F61" s="132" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="131" t="n">
-        <v>3</v>
-      </c>
-      <c r="B62" s="132" t="inlineStr">
-        <is>
-          <t>BSC Young Boys II</t>
-        </is>
-      </c>
-      <c r="C62" s="132" t="inlineStr">
-        <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-      <c r="D62" s="132" t="inlineStr">
-        <is>
-          <t>Promotion League</t>
-        </is>
-      </c>
-      <c r="E62" s="132" t="inlineStr">
-        <is>
-          <t>Keeto Thermoncy</t>
-        </is>
-      </c>
-      <c r="F62" s="132" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="133" t="n">
-        <v>4</v>
-      </c>
-      <c r="B63" s="134" t="inlineStr">
-        <is>
-          <t>FC Cosmos Koblenz</t>
-        </is>
-      </c>
-      <c r="C63" s="134" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D63" s="134" t="inlineStr">
-        <is>
-          <t>Regionalliga</t>
-        </is>
-      </c>
-      <c r="E63" s="134" t="inlineStr">
-        <is>
-          <t>Josué Duverger</t>
-        </is>
-      </c>
-      <c r="F63" s="134" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="135" t="n">
-        <v>6</v>
-      </c>
-      <c r="B64" s="136" t="inlineStr">
-        <is>
-          <t>Braintree Town</t>
-        </is>
-      </c>
-      <c r="C64" s="136" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D64" s="136" t="inlineStr">
-        <is>
-          <t>National League South</t>
-        </is>
-      </c>
-      <c r="E64" s="136" t="inlineStr">
-        <is>
-          <t>Tommy Smith</t>
-        </is>
-      </c>
-      <c r="F64" s="136" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="32" t="inlineStr">
-        <is>
-          <t>Fargeforklaring:</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="137" t="inlineStr">
-        <is>
-          <t>Nivå 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="138" t="inlineStr">
-        <is>
-          <t>Nivå 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="139" t="inlineStr">
-        <is>
-          <t>Nivå 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="140" t="inlineStr">
-        <is>
-          <t>Nivå 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="141" t="inlineStr">
-        <is>
-          <t>Nivå 6</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A3:F3"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5"/>
   <cols>
@@ -51201,7 +49346,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -51911,7 +50056,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -53461,6 +51606,1933 @@
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
   </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F69"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="143" min="1" max="1"/>
+    <col width="26" customWidth="1" style="143" min="2" max="2"/>
+    <col width="16" customWidth="1" style="143" min="3" max="3"/>
+    <col width="22" customWidth="1" style="143" min="4" max="4"/>
+    <col width="30" customWidth="1" style="143" min="5" max="5"/>
+    <col width="22" customWidth="1" style="143" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="173" t="inlineStr">
+        <is>
+          <t>Nivå</t>
+        </is>
+      </c>
+      <c r="B1" s="173" t="inlineStr">
+        <is>
+          <t>Klubb</t>
+        </is>
+      </c>
+      <c r="C1" s="173" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="D1" s="173" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+      <c r="E1" s="173" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="F1" s="173" t="inlineStr">
+        <is>
+          <t>Nasjonallag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" s="175" t="inlineStr">
+        <is>
+          <t>Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="C2" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D2" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E2" s="175" t="inlineStr">
+        <is>
+          <t>Lyndon Dykes</t>
+        </is>
+      </c>
+      <c r="F2" s="175" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="175" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="C3" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D3" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E3" s="175" t="inlineStr">
+        <is>
+          <t>Brandon Thomas-Asante</t>
+        </is>
+      </c>
+      <c r="F3" s="175" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="175" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="C4" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D4" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E4" s="175" t="inlineStr">
+        <is>
+          <t>Haji Wright</t>
+        </is>
+      </c>
+      <c r="F4" s="175" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="175" t="inlineStr">
+        <is>
+          <t>Derby County</t>
+        </is>
+      </c>
+      <c r="C5" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D5" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E5" s="175" t="inlineStr">
+        <is>
+          <t>Jacob Widell Zetterström</t>
+        </is>
+      </c>
+      <c r="F5" s="175" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="175" t="inlineStr">
+        <is>
+          <t>Derby County</t>
+        </is>
+      </c>
+      <c r="C6" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D6" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E6" s="175" t="inlineStr">
+        <is>
+          <t>Sondre Langås</t>
+        </is>
+      </c>
+      <c r="F6" s="175" t="inlineStr">
+        <is>
+          <t>Norge</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="175" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="C7" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D7" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E7" s="175" t="inlineStr">
+        <is>
+          <t>Amir Hadžiahmetović</t>
+        </is>
+      </c>
+      <c r="F7" s="175" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="175" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="C8" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D8" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E8" s="175" t="inlineStr">
+        <is>
+          <t>Ivor Pandur</t>
+        </is>
+      </c>
+      <c r="F8" s="175" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="175" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="C9" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D9" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E9" s="175" t="inlineStr">
+        <is>
+          <t>Liam Miller</t>
+        </is>
+      </c>
+      <c r="F9" s="175" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="175" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C10" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D10" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E10" s="175" t="inlineStr">
+        <is>
+          <t>Alfie Jones</t>
+        </is>
+      </c>
+      <c r="F10" s="175" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="175" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C11" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D11" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E11" s="175" t="inlineStr">
+        <is>
+          <t>Sontje Hansen</t>
+        </is>
+      </c>
+      <c r="F11" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="175" t="inlineStr">
+        <is>
+          <t>Millwall FC</t>
+        </is>
+      </c>
+      <c r="C12" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D12" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E12" s="175" t="inlineStr">
+        <is>
+          <t>Max Crocombe</t>
+        </is>
+      </c>
+      <c r="F12" s="175" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="175" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C13" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D13" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E13" s="175" t="inlineStr">
+        <is>
+          <t>Ali Ahmed</t>
+        </is>
+      </c>
+      <c r="F13" s="175" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="175" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C14" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D14" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E14" s="175" t="inlineStr">
+        <is>
+          <t>José Córdoba</t>
+        </is>
+      </c>
+      <c r="F14" s="175" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="175" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C15" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D15" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E15" s="175" t="inlineStr">
+        <is>
+          <t>Kenny McLean</t>
+        </is>
+      </c>
+      <c r="F15" s="175" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="175" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C16" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D16" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E16" s="175" t="inlineStr">
+        <is>
+          <t>Toure</t>
+        </is>
+      </c>
+      <c r="F16" s="175" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="175" t="inlineStr">
+        <is>
+          <t>Portsmouth</t>
+        </is>
+      </c>
+      <c r="C17" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D17" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E17" s="175" t="inlineStr">
+        <is>
+          <t>Gustavo Caballero</t>
+        </is>
+      </c>
+      <c r="F17" s="175" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="175" t="inlineStr">
+        <is>
+          <t>Sheffield United</t>
+        </is>
+      </c>
+      <c r="C18" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D18" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E18" s="175" t="inlineStr">
+        <is>
+          <t>Tahith Chong</t>
+        </is>
+      </c>
+      <c r="F18" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="175" t="inlineStr">
+        <is>
+          <t>Stoke City</t>
+        </is>
+      </c>
+      <c r="C19" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D19" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E19" s="175" t="inlineStr">
+        <is>
+          <t>Viktor Johansson</t>
+        </is>
+      </c>
+      <c r="F19" s="175" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="175" t="inlineStr">
+        <is>
+          <t>Swansea</t>
+        </is>
+      </c>
+      <c r="C20" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D20" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E20" s="175" t="inlineStr">
+        <is>
+          <t>Eom Jisung</t>
+        </is>
+      </c>
+      <c r="F20" s="175" t="inlineStr">
+        <is>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="175" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="C21" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D21" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E21" s="175" t="inlineStr">
+        <is>
+          <t>Burgess</t>
+        </is>
+      </c>
+      <c r="F21" s="175" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="175" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="C22" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D22" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E22" s="175" t="inlineStr">
+        <is>
+          <t>Marko Stamenić</t>
+        </is>
+      </c>
+      <c r="F22" s="175" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="175" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="C23" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D23" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E23" s="175" t="inlineStr">
+        <is>
+          <t>Edo Kayembe</t>
+        </is>
+      </c>
+      <c r="F23" s="175" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="175" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="C24" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D24" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E24" s="175" t="inlineStr">
+        <is>
+          <t>Egil Selvik</t>
+        </is>
+      </c>
+      <c r="F24" s="175" t="inlineStr">
+        <is>
+          <t>Norge</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="175" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="C25" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D25" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E25" s="175" t="inlineStr">
+        <is>
+          <t>Irankunda</t>
+        </is>
+      </c>
+      <c r="F25" s="175" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="175" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="C26" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D26" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E26" s="175" t="inlineStr">
+        <is>
+          <t>Dom Hyam</t>
+        </is>
+      </c>
+      <c r="F26" s="175" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="175" t="inlineStr">
+        <is>
+          <t>Wrexham AFC</t>
+        </is>
+      </c>
+      <c r="C27" s="175" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D27" s="175" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E27" s="175" t="inlineStr">
+        <is>
+          <t>Liberato Cacace</t>
+        </is>
+      </c>
+      <c r="F27" s="175" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="175" t="inlineStr">
+        <is>
+          <t>AS Nancy-Lorraine</t>
+        </is>
+      </c>
+      <c r="C28" s="175" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D28" s="175" t="inlineStr">
+        <is>
+          <t>Ligue 2</t>
+        </is>
+      </c>
+      <c r="E28" s="175" t="inlineStr">
+        <is>
+          <t>Martin Experience</t>
+        </is>
+      </c>
+      <c r="F28" s="175" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="175" t="inlineStr">
+        <is>
+          <t>SC Bastia</t>
+        </is>
+      </c>
+      <c r="C29" s="175" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D29" s="175" t="inlineStr">
+        <is>
+          <t>Ligue 2</t>
+        </is>
+      </c>
+      <c r="E29" s="175" t="inlineStr">
+        <is>
+          <t>Johnny Placide</t>
+        </is>
+      </c>
+      <c r="F29" s="175" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="175" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="C30" s="175" t="inlineStr">
+        <is>
+          <t>Italia</t>
+        </is>
+      </c>
+      <c r="D30" s="175" t="inlineStr">
+        <is>
+          <t>Serie B</t>
+        </is>
+      </c>
+      <c r="E30" s="175" t="inlineStr">
+        <is>
+          <t>Farès Ghedjemis</t>
+        </is>
+      </c>
+      <c r="F30" s="175" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="175" t="inlineStr">
+        <is>
+          <t>UC Sampdoria</t>
+        </is>
+      </c>
+      <c r="C31" s="175" t="inlineStr">
+        <is>
+          <t>Italia</t>
+        </is>
+      </c>
+      <c r="D31" s="175" t="inlineStr">
+        <is>
+          <t>Serie B</t>
+        </is>
+      </c>
+      <c r="E31" s="175" t="inlineStr">
+        <is>
+          <t>Dennis Hadžikadunić</t>
+        </is>
+      </c>
+      <c r="F31" s="175" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="175" t="inlineStr">
+        <is>
+          <t>Albirex Niigata</t>
+        </is>
+      </c>
+      <c r="C32" s="175" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D32" s="175" t="inlineStr">
+        <is>
+          <t>J2 League</t>
+        </is>
+      </c>
+      <c r="E32" s="175" t="inlineStr">
+        <is>
+          <t>Geria</t>
+        </is>
+      </c>
+      <c r="F32" s="175" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="175" t="inlineStr">
+        <is>
+          <t>FC Den Bosch</t>
+        </is>
+      </c>
+      <c r="C33" s="175" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D33" s="175" t="inlineStr">
+        <is>
+          <t>Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="E33" s="175" t="inlineStr">
+        <is>
+          <t>Kevin Felida</t>
+        </is>
+      </c>
+      <c r="F33" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="175" t="inlineStr">
+        <is>
+          <t>VVV-Venlo</t>
+        </is>
+      </c>
+      <c r="C34" s="175" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D34" s="175" t="inlineStr">
+        <is>
+          <t>Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="E34" s="175" t="inlineStr">
+        <is>
+          <t>Trevor Doornbusch</t>
+        </is>
+      </c>
+      <c r="F34" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="175" t="inlineStr">
+        <is>
+          <t>Chaves</t>
+        </is>
+      </c>
+      <c r="C35" s="175" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D35" s="175" t="inlineStr">
+        <is>
+          <t>Liga Portugal 2</t>
+        </is>
+      </c>
+      <c r="E35" s="175" t="inlineStr">
+        <is>
+          <t>Josimar Dias "Vozinha"</t>
+        </is>
+      </c>
+      <c r="F35" s="175" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="175" t="inlineStr">
+        <is>
+          <t>Torreense</t>
+        </is>
+      </c>
+      <c r="C36" s="175" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D36" s="175" t="inlineStr">
+        <is>
+          <t>Liga Portugal 2</t>
+        </is>
+      </c>
+      <c r="E36" s="175" t="inlineStr">
+        <is>
+          <t>Ianique Tavares "Stopira"</t>
+        </is>
+      </c>
+      <c r="F36" s="175" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="175" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="C37" s="175" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D37" s="175" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E37" s="175" t="inlineStr">
+        <is>
+          <t>Brian Cipenga</t>
+        </is>
+      </c>
+      <c r="F37" s="175" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="175" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="C38" s="175" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D38" s="175" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E38" s="175" t="inlineStr">
+        <is>
+          <t>Mabil</t>
+        </is>
+      </c>
+      <c r="F38" s="175" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="175" t="inlineStr">
+        <is>
+          <t>Cultural Leonesa</t>
+        </is>
+      </c>
+      <c r="C39" s="175" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D39" s="175" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E39" s="175" t="inlineStr">
+        <is>
+          <t>Homam Al-Amin</t>
+        </is>
+      </c>
+      <c r="F39" s="175" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="175" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C40" s="175" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D40" s="175" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E40" s="175" t="inlineStr">
+        <is>
+          <t>Federico Viñas</t>
+        </is>
+      </c>
+      <c r="F40" s="175" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="175" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C41" s="175" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D41" s="175" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E41" s="175" t="inlineStr">
+        <is>
+          <t>Haissem Hassan</t>
+        </is>
+      </c>
+      <c r="F41" s="175" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="175" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C42" s="175" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D42" s="175" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E42" s="175" t="inlineStr">
+        <is>
+          <t>Kwasi Sibo</t>
+        </is>
+      </c>
+      <c r="F42" s="175" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="175" t="inlineStr">
+        <is>
+          <t>Stade Nyonnais</t>
+        </is>
+      </c>
+      <c r="C43" s="175" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="D43" s="175" t="inlineStr">
+        <is>
+          <t>Challenge League</t>
+        </is>
+      </c>
+      <c r="E43" s="175" t="inlineStr">
+        <is>
+          <t>Melvin Mastil</t>
+        </is>
+      </c>
+      <c r="F43" s="175" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="175" t="inlineStr">
+        <is>
+          <t>IFK Norrköping</t>
+        </is>
+      </c>
+      <c r="C44" s="175" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+      <c r="D44" s="175" t="inlineStr">
+        <is>
+          <t>Superettan</t>
+        </is>
+      </c>
+      <c r="E44" s="175" t="inlineStr">
+        <is>
+          <t>Moutaz Neffati</t>
+        </is>
+      </c>
+      <c r="F44" s="175" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="175" t="inlineStr">
+        <is>
+          <t>Siwelele FC</t>
+        </is>
+      </c>
+      <c r="C45" s="175" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="D45" s="175" t="inlineStr">
+        <is>
+          <t>National First Division</t>
+        </is>
+      </c>
+      <c r="E45" s="175" t="inlineStr">
+        <is>
+          <t>Ricardo Goss</t>
+        </is>
+      </c>
+      <c r="F45" s="175" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" s="175" t="inlineStr">
+        <is>
+          <t>Iğdır</t>
+        </is>
+      </c>
+      <c r="C46" s="175" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="D46" s="175" t="inlineStr">
+        <is>
+          <t>TFF 1. Lig</t>
+        </is>
+      </c>
+      <c r="E46" s="175" t="inlineStr">
+        <is>
+          <t>Leandro Bacuna</t>
+        </is>
+      </c>
+      <c r="F46" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="175" t="inlineStr">
+        <is>
+          <t>Iğdır</t>
+        </is>
+      </c>
+      <c r="C47" s="175" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="D47" s="175" t="inlineStr">
+        <is>
+          <t>TFF 1. Lig</t>
+        </is>
+      </c>
+      <c r="E47" s="175" t="inlineStr">
+        <is>
+          <t>Ryan Mendes</t>
+        </is>
+      </c>
+      <c r="F47" s="175" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="175" t="inlineStr">
+        <is>
+          <t>Fortuna Düsseldorf</t>
+        </is>
+      </c>
+      <c r="C48" s="175" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D48" s="175" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E48" s="175" t="inlineStr">
+        <is>
+          <t>Cedric Itten</t>
+        </is>
+      </c>
+      <c r="F48" s="175" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="175" t="inlineStr">
+        <is>
+          <t>Hannover 96</t>
+        </is>
+      </c>
+      <c r="C49" s="175" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D49" s="175" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E49" s="175" t="inlineStr">
+        <is>
+          <t>Ime Okon</t>
+        </is>
+      </c>
+      <c r="F49" s="175" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="175" t="inlineStr">
+        <is>
+          <t>Hannover 96</t>
+        </is>
+      </c>
+      <c r="C50" s="175" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D50" s="175" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E50" s="175" t="inlineStr">
+        <is>
+          <t>​Elias Saad</t>
+        </is>
+      </c>
+      <c r="F50" s="175" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="175" t="inlineStr">
+        <is>
+          <t>Karlsruher SC</t>
+        </is>
+      </c>
+      <c r="C51" s="175" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D51" s="175" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E51" s="175" t="inlineStr">
+        <is>
+          <t>Dženis Burnić</t>
+        </is>
+      </c>
+      <c r="F51" s="175" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="175" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="C52" s="175" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D52" s="175" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E52" s="175" t="inlineStr">
+        <is>
+          <t>Edin Džeko</t>
+        </is>
+      </c>
+      <c r="F52" s="175" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="175" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="C53" s="175" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D53" s="175" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E53" s="175" t="inlineStr">
+        <is>
+          <t>Nikola Katić</t>
+        </is>
+      </c>
+      <c r="F53" s="175" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="175" t="inlineStr">
+        <is>
+          <t>El Paso Locomotive FC</t>
+        </is>
+      </c>
+      <c r="C54" s="175" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D54" s="175" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E54" s="175" t="inlineStr">
+        <is>
+          <t>Carl-Fred Sainthe</t>
+        </is>
+      </c>
+      <c r="F54" s="175" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="175" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="C55" s="175" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D55" s="175" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E55" s="175" t="inlineStr">
+        <is>
+          <t>Eloy Room</t>
+        </is>
+      </c>
+      <c r="F55" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="175" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="C56" s="175" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D56" s="175" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E56" s="175" t="inlineStr">
+        <is>
+          <t>Jürgen Locadia</t>
+        </is>
+      </c>
+      <c r="F56" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="B57" s="177" t="inlineStr">
+        <is>
+          <t>Port Vale</t>
+        </is>
+      </c>
+      <c r="C57" s="177" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D57" s="177" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="E57" s="177" t="inlineStr">
+        <is>
+          <t>Ben Waine</t>
+        </is>
+      </c>
+      <c r="F57" s="177" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="B58" s="177" t="inlineStr">
+        <is>
+          <t>Rotherham United</t>
+        </is>
+      </c>
+      <c r="C58" s="177" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D58" s="177" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="E58" s="177" t="inlineStr">
+        <is>
+          <t>Ar’Jany Martha</t>
+        </is>
+      </c>
+      <c r="F58" s="177" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" s="177" t="inlineStr">
+        <is>
+          <t>FC Sochaux</t>
+        </is>
+      </c>
+      <c r="C59" s="177" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D59" s="177" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="E59" s="177" t="inlineStr">
+        <is>
+          <t>Alexandre Pierre</t>
+        </is>
+      </c>
+      <c r="F59" s="177" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="B60" s="177" t="inlineStr">
+        <is>
+          <t>BSC Young Boys II</t>
+        </is>
+      </c>
+      <c r="C60" s="177" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="D60" s="177" t="inlineStr">
+        <is>
+          <t>Promotion League</t>
+        </is>
+      </c>
+      <c r="E60" s="177" t="inlineStr">
+        <is>
+          <t>Keeto Thermoncy</t>
+        </is>
+      </c>
+      <c r="F60" s="177" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="178" t="n">
+        <v>4</v>
+      </c>
+      <c r="B61" s="179" t="inlineStr">
+        <is>
+          <t>FC Cosmos Koblenz</t>
+        </is>
+      </c>
+      <c r="C61" s="179" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D61" s="179" t="inlineStr">
+        <is>
+          <t>Regionalliga</t>
+        </is>
+      </c>
+      <c r="E61" s="179" t="inlineStr">
+        <is>
+          <t>Josué Duverger</t>
+        </is>
+      </c>
+      <c r="F61" s="179" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="180" t="n">
+        <v>6</v>
+      </c>
+      <c r="B62" s="181" t="inlineStr">
+        <is>
+          <t>Braintree Town</t>
+        </is>
+      </c>
+      <c r="C62" s="181" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D62" s="181" t="inlineStr">
+        <is>
+          <t>National League South</t>
+        </is>
+      </c>
+      <c r="E62" s="181" t="inlineStr">
+        <is>
+          <t>Tommy Smith</t>
+        </is>
+      </c>
+      <c r="F62" s="181" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="32" t="inlineStr">
+        <is>
+          <t>Fargeforklaring:</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="182" t="inlineStr">
+        <is>
+          <t>Nivå 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="183" t="inlineStr">
+        <is>
+          <t>Nivå 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="184" t="inlineStr">
+        <is>
+          <t>Nivå 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="185" t="inlineStr">
+        <is>
+          <t>Nivå 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="186" t="inlineStr">
+        <is>
+          <t>Nivå 6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:F1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Legg til navy tittelrad på Nivå 2 og lavere + Spillere etter klubbland
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -33,8 +33,8 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Klubber'!$A$2:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Nivå 2 og lavere'!$A$1:$F$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Spillere etter klubbland'!$A$1:$I$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Nivå 2 og lavere'!$A$2:$F$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -817,7 +817,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="187">
+  <cellXfs count="188">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1337,6 +1337,9 @@
     <xf numFmtId="0" fontId="16" fillId="53" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="55" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="54" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="45" fillId="44" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -50062,7 +50065,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F69"/>
+  <dimension ref="A1:F70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="143" min="1" max="1"/>
@@ -50073,65 +50076,42 @@
     <col width="22" customWidth="1" style="143" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="173" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="143">
+      <c r="A1" s="150" t="inlineStr">
+        <is>
+          <t>VM 2026 — Spillere på nivå 2 og lavere   61 spillere</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="143">
+      <c r="A2" s="187" t="inlineStr">
         <is>
           <t>Nivå</t>
         </is>
       </c>
-      <c r="B1" s="173" t="inlineStr">
+      <c r="B2" s="187" t="inlineStr">
         <is>
           <t>Klubb</t>
         </is>
       </c>
-      <c r="C1" s="173" t="inlineStr">
+      <c r="C2" s="187" t="inlineStr">
         <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="D1" s="173" t="inlineStr">
+      <c r="D2" s="187" t="inlineStr">
         <is>
           <t>Liga</t>
         </is>
       </c>
-      <c r="E1" s="173" t="inlineStr">
+      <c r="E2" s="187" t="inlineStr">
         <is>
           <t>Spiller</t>
         </is>
       </c>
-      <c r="F1" s="173" t="inlineStr">
+      <c r="F2" s="187" t="inlineStr">
         <is>
           <t>Nasjonallag</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" s="175" t="inlineStr">
-        <is>
-          <t>Charlton Athletic</t>
-        </is>
-      </c>
-      <c r="C2" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D2" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E2" s="175" t="inlineStr">
-        <is>
-          <t>Lyndon Dykes</t>
-        </is>
-      </c>
-      <c r="F2" s="175" t="inlineStr">
-        <is>
-          <t>Skottland</t>
         </is>
       </c>
     </row>
@@ -50141,7 +50121,7 @@
       </c>
       <c r="B3" s="175" t="inlineStr">
         <is>
-          <t>Coventry City</t>
+          <t>Charlton Athletic</t>
         </is>
       </c>
       <c r="C3" s="175" t="inlineStr">
@@ -50156,12 +50136,12 @@
       </c>
       <c r="E3" s="175" t="inlineStr">
         <is>
-          <t>Brandon Thomas-Asante</t>
+          <t>Lyndon Dykes</t>
         </is>
       </c>
       <c r="F3" s="175" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Skottland</t>
         </is>
       </c>
     </row>
@@ -50186,12 +50166,12 @@
       </c>
       <c r="E4" s="175" t="inlineStr">
         <is>
-          <t>Haji Wright</t>
+          <t>Brandon Thomas-Asante</t>
         </is>
       </c>
       <c r="F4" s="175" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Ghana</t>
         </is>
       </c>
     </row>
@@ -50201,7 +50181,7 @@
       </c>
       <c r="B5" s="175" t="inlineStr">
         <is>
-          <t>Derby County</t>
+          <t>Coventry City</t>
         </is>
       </c>
       <c r="C5" s="175" t="inlineStr">
@@ -50216,12 +50196,12 @@
       </c>
       <c r="E5" s="175" t="inlineStr">
         <is>
-          <t>Jacob Widell Zetterström</t>
+          <t>Haji Wright</t>
         </is>
       </c>
       <c r="F5" s="175" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>USA</t>
         </is>
       </c>
     </row>
@@ -50246,12 +50226,12 @@
       </c>
       <c r="E6" s="175" t="inlineStr">
         <is>
-          <t>Sondre Langås</t>
+          <t>Jacob Widell Zetterström</t>
         </is>
       </c>
       <c r="F6" s="175" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Sverige</t>
         </is>
       </c>
     </row>
@@ -50261,7 +50241,7 @@
       </c>
       <c r="B7" s="175" t="inlineStr">
         <is>
-          <t>Hull City</t>
+          <t>Derby County</t>
         </is>
       </c>
       <c r="C7" s="175" t="inlineStr">
@@ -50276,12 +50256,12 @@
       </c>
       <c r="E7" s="175" t="inlineStr">
         <is>
-          <t>Amir Hadžiahmetović</t>
+          <t>Sondre Langås</t>
         </is>
       </c>
       <c r="F7" s="175" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Norge</t>
         </is>
       </c>
     </row>
@@ -50306,12 +50286,12 @@
       </c>
       <c r="E8" s="175" t="inlineStr">
         <is>
-          <t>Ivor Pandur</t>
+          <t>Amir Hadžiahmetović</t>
         </is>
       </c>
       <c r="F8" s="175" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
     </row>
@@ -50336,12 +50316,12 @@
       </c>
       <c r="E9" s="175" t="inlineStr">
         <is>
-          <t>Liam Miller</t>
+          <t>Ivor Pandur</t>
         </is>
       </c>
       <c r="F9" s="175" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Kroatia</t>
         </is>
       </c>
     </row>
@@ -50351,7 +50331,7 @@
       </c>
       <c r="B10" s="175" t="inlineStr">
         <is>
-          <t>Middlesbrough</t>
+          <t>Hull City</t>
         </is>
       </c>
       <c r="C10" s="175" t="inlineStr">
@@ -50366,7 +50346,7 @@
       </c>
       <c r="E10" s="175" t="inlineStr">
         <is>
-          <t>Alfie Jones</t>
+          <t>Liam Miller</t>
         </is>
       </c>
       <c r="F10" s="175" t="inlineStr">
@@ -50396,12 +50376,12 @@
       </c>
       <c r="E11" s="175" t="inlineStr">
         <is>
-          <t>Sontje Hansen</t>
+          <t>Alfie Jones</t>
         </is>
       </c>
       <c r="F11" s="175" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Canada</t>
         </is>
       </c>
     </row>
@@ -50411,7 +50391,7 @@
       </c>
       <c r="B12" s="175" t="inlineStr">
         <is>
-          <t>Millwall FC</t>
+          <t>Middlesbrough</t>
         </is>
       </c>
       <c r="C12" s="175" t="inlineStr">
@@ -50426,12 +50406,12 @@
       </c>
       <c r="E12" s="175" t="inlineStr">
         <is>
-          <t>Max Crocombe</t>
+          <t>Sontje Hansen</t>
         </is>
       </c>
       <c r="F12" s="175" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -50441,7 +50421,7 @@
       </c>
       <c r="B13" s="175" t="inlineStr">
         <is>
-          <t>Norwich City</t>
+          <t>Millwall FC</t>
         </is>
       </c>
       <c r="C13" s="175" t="inlineStr">
@@ -50456,12 +50436,12 @@
       </c>
       <c r="E13" s="175" t="inlineStr">
         <is>
-          <t>Ali Ahmed</t>
+          <t>Max Crocombe</t>
         </is>
       </c>
       <c r="F13" s="175" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -50486,12 +50466,12 @@
       </c>
       <c r="E14" s="175" t="inlineStr">
         <is>
-          <t>José Córdoba</t>
+          <t>Ali Ahmed</t>
         </is>
       </c>
       <c r="F14" s="175" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Canada</t>
         </is>
       </c>
     </row>
@@ -50516,12 +50496,12 @@
       </c>
       <c r="E15" s="175" t="inlineStr">
         <is>
-          <t>Kenny McLean</t>
+          <t>José Córdoba</t>
         </is>
       </c>
       <c r="F15" s="175" t="inlineStr">
         <is>
-          <t>Skottland</t>
+          <t>Panama</t>
         </is>
       </c>
     </row>
@@ -50546,12 +50526,12 @@
       </c>
       <c r="E16" s="175" t="inlineStr">
         <is>
-          <t>Toure</t>
+          <t>Kenny McLean</t>
         </is>
       </c>
       <c r="F16" s="175" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Skottland</t>
         </is>
       </c>
     </row>
@@ -50561,7 +50541,7 @@
       </c>
       <c r="B17" s="175" t="inlineStr">
         <is>
-          <t>Portsmouth</t>
+          <t>Norwich City</t>
         </is>
       </c>
       <c r="C17" s="175" t="inlineStr">
@@ -50576,12 +50556,12 @@
       </c>
       <c r="E17" s="175" t="inlineStr">
         <is>
-          <t>Gustavo Caballero</t>
+          <t>Toure</t>
         </is>
       </c>
       <c r="F17" s="175" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Australia</t>
         </is>
       </c>
     </row>
@@ -50591,7 +50571,7 @@
       </c>
       <c r="B18" s="175" t="inlineStr">
         <is>
-          <t>Sheffield United</t>
+          <t>Portsmouth</t>
         </is>
       </c>
       <c r="C18" s="175" t="inlineStr">
@@ -50606,12 +50586,12 @@
       </c>
       <c r="E18" s="175" t="inlineStr">
         <is>
-          <t>Tahith Chong</t>
+          <t>Gustavo Caballero</t>
         </is>
       </c>
       <c r="F18" s="175" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -50621,7 +50601,7 @@
       </c>
       <c r="B19" s="175" t="inlineStr">
         <is>
-          <t>Stoke City</t>
+          <t>Sheffield United</t>
         </is>
       </c>
       <c r="C19" s="175" t="inlineStr">
@@ -50636,12 +50616,12 @@
       </c>
       <c r="E19" s="175" t="inlineStr">
         <is>
-          <t>Viktor Johansson</t>
+          <t>Tahith Chong</t>
         </is>
       </c>
       <c r="F19" s="175" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -50651,7 +50631,7 @@
       </c>
       <c r="B20" s="175" t="inlineStr">
         <is>
-          <t>Swansea</t>
+          <t>Stoke City</t>
         </is>
       </c>
       <c r="C20" s="175" t="inlineStr">
@@ -50666,12 +50646,12 @@
       </c>
       <c r="E20" s="175" t="inlineStr">
         <is>
-          <t>Eom Jisung</t>
+          <t>Viktor Johansson</t>
         </is>
       </c>
       <c r="F20" s="175" t="inlineStr">
         <is>
-          <t>Sør-Korea</t>
+          <t>Sverige</t>
         </is>
       </c>
     </row>
@@ -50681,7 +50661,7 @@
       </c>
       <c r="B21" s="175" t="inlineStr">
         <is>
-          <t>Swansea City</t>
+          <t>Swansea</t>
         </is>
       </c>
       <c r="C21" s="175" t="inlineStr">
@@ -50696,12 +50676,12 @@
       </c>
       <c r="E21" s="175" t="inlineStr">
         <is>
-          <t>Burgess</t>
+          <t>Eom Jisung</t>
         </is>
       </c>
       <c r="F21" s="175" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Sør-Korea</t>
         </is>
       </c>
     </row>
@@ -50726,12 +50706,12 @@
       </c>
       <c r="E22" s="175" t="inlineStr">
         <is>
-          <t>Marko Stamenić</t>
+          <t>Burgess</t>
         </is>
       </c>
       <c r="F22" s="175" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Australia</t>
         </is>
       </c>
     </row>
@@ -50741,7 +50721,7 @@
       </c>
       <c r="B23" s="175" t="inlineStr">
         <is>
-          <t>Watford</t>
+          <t>Swansea City</t>
         </is>
       </c>
       <c r="C23" s="175" t="inlineStr">
@@ -50756,12 +50736,12 @@
       </c>
       <c r="E23" s="175" t="inlineStr">
         <is>
-          <t>Edo Kayembe</t>
+          <t>Marko Stamenić</t>
         </is>
       </c>
       <c r="F23" s="175" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -50786,12 +50766,12 @@
       </c>
       <c r="E24" s="175" t="inlineStr">
         <is>
-          <t>Egil Selvik</t>
+          <t>Edo Kayembe</t>
         </is>
       </c>
       <c r="F24" s="175" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -50816,12 +50796,12 @@
       </c>
       <c r="E25" s="175" t="inlineStr">
         <is>
-          <t>Irankunda</t>
+          <t>Egil Selvik</t>
         </is>
       </c>
       <c r="F25" s="175" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Norge</t>
         </is>
       </c>
     </row>
@@ -50831,7 +50811,7 @@
       </c>
       <c r="B26" s="175" t="inlineStr">
         <is>
-          <t>Wrexham</t>
+          <t>Watford</t>
         </is>
       </c>
       <c r="C26" s="175" t="inlineStr">
@@ -50846,12 +50826,12 @@
       </c>
       <c r="E26" s="175" t="inlineStr">
         <is>
-          <t>Dom Hyam</t>
+          <t>Irankunda</t>
         </is>
       </c>
       <c r="F26" s="175" t="inlineStr">
         <is>
-          <t>Skottland</t>
+          <t>Australia</t>
         </is>
       </c>
     </row>
@@ -50861,7 +50841,7 @@
       </c>
       <c r="B27" s="175" t="inlineStr">
         <is>
-          <t>Wrexham AFC</t>
+          <t>Wrexham</t>
         </is>
       </c>
       <c r="C27" s="175" t="inlineStr">
@@ -50876,12 +50856,12 @@
       </c>
       <c r="E27" s="175" t="inlineStr">
         <is>
-          <t>Liberato Cacace</t>
+          <t>Dom Hyam</t>
         </is>
       </c>
       <c r="F27" s="175" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Skottland</t>
         </is>
       </c>
     </row>
@@ -50891,27 +50871,27 @@
       </c>
       <c r="B28" s="175" t="inlineStr">
         <is>
-          <t>AS Nancy-Lorraine</t>
+          <t>Wrexham AFC</t>
         </is>
       </c>
       <c r="C28" s="175" t="inlineStr">
         <is>
-          <t>Frankrike</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D28" s="175" t="inlineStr">
         <is>
-          <t>Ligue 2</t>
+          <t>Championship</t>
         </is>
       </c>
       <c r="E28" s="175" t="inlineStr">
         <is>
-          <t>Martin Experience</t>
+          <t>Liberato Cacace</t>
         </is>
       </c>
       <c r="F28" s="175" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -50921,7 +50901,7 @@
       </c>
       <c r="B29" s="175" t="inlineStr">
         <is>
-          <t>SC Bastia</t>
+          <t>AS Nancy-Lorraine</t>
         </is>
       </c>
       <c r="C29" s="175" t="inlineStr">
@@ -50936,7 +50916,7 @@
       </c>
       <c r="E29" s="175" t="inlineStr">
         <is>
-          <t>Johnny Placide</t>
+          <t>Martin Experience</t>
         </is>
       </c>
       <c r="F29" s="175" t="inlineStr">
@@ -50951,27 +50931,27 @@
       </c>
       <c r="B30" s="175" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>SC Bastia</t>
         </is>
       </c>
       <c r="C30" s="175" t="inlineStr">
         <is>
-          <t>Italia</t>
+          <t>Frankrike</t>
         </is>
       </c>
       <c r="D30" s="175" t="inlineStr">
         <is>
-          <t>Serie B</t>
+          <t>Ligue 2</t>
         </is>
       </c>
       <c r="E30" s="175" t="inlineStr">
         <is>
-          <t>Farès Ghedjemis</t>
+          <t>Johnny Placide</t>
         </is>
       </c>
       <c r="F30" s="175" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Haiti</t>
         </is>
       </c>
     </row>
@@ -50981,7 +50961,7 @@
       </c>
       <c r="B31" s="175" t="inlineStr">
         <is>
-          <t>UC Sampdoria</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="C31" s="175" t="inlineStr">
@@ -50996,12 +50976,12 @@
       </c>
       <c r="E31" s="175" t="inlineStr">
         <is>
-          <t>Dennis Hadžikadunić</t>
+          <t>Farès Ghedjemis</t>
         </is>
       </c>
       <c r="F31" s="175" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -51011,27 +50991,27 @@
       </c>
       <c r="B32" s="175" t="inlineStr">
         <is>
-          <t>Albirex Niigata</t>
+          <t>UC Sampdoria</t>
         </is>
       </c>
       <c r="C32" s="175" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Italia</t>
         </is>
       </c>
       <c r="D32" s="175" t="inlineStr">
         <is>
-          <t>J2 League</t>
+          <t>Serie B</t>
         </is>
       </c>
       <c r="E32" s="175" t="inlineStr">
         <is>
-          <t>Geria</t>
+          <t>Dennis Hadžikadunić</t>
         </is>
       </c>
       <c r="F32" s="175" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
     </row>
@@ -51041,27 +51021,27 @@
       </c>
       <c r="B33" s="175" t="inlineStr">
         <is>
-          <t>FC Den Bosch</t>
+          <t>Albirex Niigata</t>
         </is>
       </c>
       <c r="C33" s="175" t="inlineStr">
         <is>
-          <t>Nederland</t>
+          <t>Japan</t>
         </is>
       </c>
       <c r="D33" s="175" t="inlineStr">
         <is>
-          <t>Eerste Divisie</t>
+          <t>J2 League</t>
         </is>
       </c>
       <c r="E33" s="175" t="inlineStr">
         <is>
-          <t>Kevin Felida</t>
+          <t>Geria</t>
         </is>
       </c>
       <c r="F33" s="175" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Australia</t>
         </is>
       </c>
     </row>
@@ -51071,7 +51051,7 @@
       </c>
       <c r="B34" s="175" t="inlineStr">
         <is>
-          <t>VVV-Venlo</t>
+          <t>FC Den Bosch</t>
         </is>
       </c>
       <c r="C34" s="175" t="inlineStr">
@@ -51086,7 +51066,7 @@
       </c>
       <c r="E34" s="175" t="inlineStr">
         <is>
-          <t>Trevor Doornbusch</t>
+          <t>Kevin Felida</t>
         </is>
       </c>
       <c r="F34" s="175" t="inlineStr">
@@ -51101,27 +51081,27 @@
       </c>
       <c r="B35" s="175" t="inlineStr">
         <is>
-          <t>Chaves</t>
+          <t>VVV-Venlo</t>
         </is>
       </c>
       <c r="C35" s="175" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Nederland</t>
         </is>
       </c>
       <c r="D35" s="175" t="inlineStr">
         <is>
-          <t>Liga Portugal 2</t>
+          <t>Eerste Divisie</t>
         </is>
       </c>
       <c r="E35" s="175" t="inlineStr">
         <is>
-          <t>Josimar Dias "Vozinha"</t>
+          <t>Trevor Doornbusch</t>
         </is>
       </c>
       <c r="F35" s="175" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -51131,7 +51111,7 @@
       </c>
       <c r="B36" s="175" t="inlineStr">
         <is>
-          <t>Torreense</t>
+          <t>Chaves</t>
         </is>
       </c>
       <c r="C36" s="175" t="inlineStr">
@@ -51146,7 +51126,7 @@
       </c>
       <c r="E36" s="175" t="inlineStr">
         <is>
-          <t>Ianique Tavares "Stopira"</t>
+          <t>Josimar Dias "Vozinha"</t>
         </is>
       </c>
       <c r="F36" s="175" t="inlineStr">
@@ -51161,27 +51141,27 @@
       </c>
       <c r="B37" s="175" t="inlineStr">
         <is>
-          <t>Castellón</t>
+          <t>Torreense</t>
         </is>
       </c>
       <c r="C37" s="175" t="inlineStr">
         <is>
-          <t>Spania</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="D37" s="175" t="inlineStr">
         <is>
-          <t>Segunda División</t>
+          <t>Liga Portugal 2</t>
         </is>
       </c>
       <c r="E37" s="175" t="inlineStr">
         <is>
-          <t>Brian Cipenga</t>
+          <t>Ianique Tavares "Stopira"</t>
         </is>
       </c>
       <c r="F37" s="175" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
@@ -51206,12 +51186,12 @@
       </c>
       <c r="E38" s="175" t="inlineStr">
         <is>
-          <t>Mabil</t>
+          <t>Brian Cipenga</t>
         </is>
       </c>
       <c r="F38" s="175" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -51221,7 +51201,7 @@
       </c>
       <c r="B39" s="175" t="inlineStr">
         <is>
-          <t>Cultural Leonesa</t>
+          <t>Castellón</t>
         </is>
       </c>
       <c r="C39" s="175" t="inlineStr">
@@ -51236,12 +51216,12 @@
       </c>
       <c r="E39" s="175" t="inlineStr">
         <is>
-          <t>Homam Al-Amin</t>
+          <t>Mabil</t>
         </is>
       </c>
       <c r="F39" s="175" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Australia</t>
         </is>
       </c>
     </row>
@@ -51251,7 +51231,7 @@
       </c>
       <c r="B40" s="175" t="inlineStr">
         <is>
-          <t>Real Oviedo</t>
+          <t>Cultural Leonesa</t>
         </is>
       </c>
       <c r="C40" s="175" t="inlineStr">
@@ -51266,12 +51246,12 @@
       </c>
       <c r="E40" s="175" t="inlineStr">
         <is>
-          <t>Federico Viñas</t>
+          <t>Homam Al-Amin</t>
         </is>
       </c>
       <c r="F40" s="175" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>Qatar</t>
         </is>
       </c>
     </row>
@@ -51296,12 +51276,12 @@
       </c>
       <c r="E41" s="175" t="inlineStr">
         <is>
-          <t>Haissem Hassan</t>
+          <t>Federico Viñas</t>
         </is>
       </c>
       <c r="F41" s="175" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Uruguay</t>
         </is>
       </c>
     </row>
@@ -51326,12 +51306,12 @@
       </c>
       <c r="E42" s="175" t="inlineStr">
         <is>
-          <t>Kwasi Sibo</t>
+          <t>Haissem Hassan</t>
         </is>
       </c>
       <c r="F42" s="175" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Egypt</t>
         </is>
       </c>
     </row>
@@ -51341,27 +51321,27 @@
       </c>
       <c r="B43" s="175" t="inlineStr">
         <is>
-          <t>Stade Nyonnais</t>
+          <t>Real Oviedo</t>
         </is>
       </c>
       <c r="C43" s="175" t="inlineStr">
         <is>
-          <t>Sveits</t>
+          <t>Spania</t>
         </is>
       </c>
       <c r="D43" s="175" t="inlineStr">
         <is>
-          <t>Challenge League</t>
+          <t>Segunda División</t>
         </is>
       </c>
       <c r="E43" s="175" t="inlineStr">
         <is>
-          <t>Melvin Mastil</t>
+          <t>Kwasi Sibo</t>
         </is>
       </c>
       <c r="F43" s="175" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Ghana</t>
         </is>
       </c>
     </row>
@@ -51371,27 +51351,27 @@
       </c>
       <c r="B44" s="175" t="inlineStr">
         <is>
-          <t>IFK Norrköping</t>
+          <t>Stade Nyonnais</t>
         </is>
       </c>
       <c r="C44" s="175" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>Sveits</t>
         </is>
       </c>
       <c r="D44" s="175" t="inlineStr">
         <is>
-          <t>Superettan</t>
+          <t>Challenge League</t>
         </is>
       </c>
       <c r="E44" s="175" t="inlineStr">
         <is>
-          <t>Moutaz Neffati</t>
+          <t>Melvin Mastil</t>
         </is>
       </c>
       <c r="F44" s="175" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -51401,27 +51381,27 @@
       </c>
       <c r="B45" s="175" t="inlineStr">
         <is>
-          <t>Siwelele FC</t>
+          <t>IFK Norrköping</t>
         </is>
       </c>
       <c r="C45" s="175" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
+          <t>Sverige</t>
         </is>
       </c>
       <c r="D45" s="175" t="inlineStr">
         <is>
-          <t>National First Division</t>
+          <t>Superettan</t>
         </is>
       </c>
       <c r="E45" s="175" t="inlineStr">
         <is>
-          <t>Ricardo Goss</t>
+          <t>Moutaz Neffati</t>
         </is>
       </c>
       <c r="F45" s="175" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
+          <t>Tunisia</t>
         </is>
       </c>
     </row>
@@ -51431,27 +51411,27 @@
       </c>
       <c r="B46" s="175" t="inlineStr">
         <is>
-          <t>Iğdır</t>
+          <t>Siwelele FC</t>
         </is>
       </c>
       <c r="C46" s="175" t="inlineStr">
         <is>
-          <t>Tyrkia</t>
+          <t>Sør-Afrika</t>
         </is>
       </c>
       <c r="D46" s="175" t="inlineStr">
         <is>
-          <t>TFF 1. Lig</t>
+          <t>National First Division</t>
         </is>
       </c>
       <c r="E46" s="175" t="inlineStr">
         <is>
-          <t>Leandro Bacuna</t>
+          <t>Ricardo Goss</t>
         </is>
       </c>
       <c r="F46" s="175" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Sør-Afrika</t>
         </is>
       </c>
     </row>
@@ -51476,12 +51456,12 @@
       </c>
       <c r="E47" s="175" t="inlineStr">
         <is>
-          <t>Ryan Mendes</t>
+          <t>Leandro Bacuna</t>
         </is>
       </c>
       <c r="F47" s="175" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -51491,27 +51471,27 @@
       </c>
       <c r="B48" s="175" t="inlineStr">
         <is>
-          <t>Fortuna Düsseldorf</t>
+          <t>Iğdır</t>
         </is>
       </c>
       <c r="C48" s="175" t="inlineStr">
         <is>
-          <t>Tyskland</t>
+          <t>Tyrkia</t>
         </is>
       </c>
       <c r="D48" s="175" t="inlineStr">
         <is>
-          <t>2. Bundesliga</t>
+          <t>TFF 1. Lig</t>
         </is>
       </c>
       <c r="E48" s="175" t="inlineStr">
         <is>
-          <t>Cedric Itten</t>
+          <t>Ryan Mendes</t>
         </is>
       </c>
       <c r="F48" s="175" t="inlineStr">
         <is>
-          <t>Sveits</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
@@ -51521,7 +51501,7 @@
       </c>
       <c r="B49" s="175" t="inlineStr">
         <is>
-          <t>Hannover 96</t>
+          <t>Fortuna Düsseldorf</t>
         </is>
       </c>
       <c r="C49" s="175" t="inlineStr">
@@ -51536,12 +51516,12 @@
       </c>
       <c r="E49" s="175" t="inlineStr">
         <is>
-          <t>Ime Okon</t>
+          <t>Cedric Itten</t>
         </is>
       </c>
       <c r="F49" s="175" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
+          <t>Sveits</t>
         </is>
       </c>
     </row>
@@ -51566,12 +51546,12 @@
       </c>
       <c r="E50" s="175" t="inlineStr">
         <is>
-          <t>​Elias Saad</t>
+          <t>Ime Okon</t>
         </is>
       </c>
       <c r="F50" s="175" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Sør-Afrika</t>
         </is>
       </c>
     </row>
@@ -51581,7 +51561,7 @@
       </c>
       <c r="B51" s="175" t="inlineStr">
         <is>
-          <t>Karlsruher SC</t>
+          <t>Hannover 96</t>
         </is>
       </c>
       <c r="C51" s="175" t="inlineStr">
@@ -51596,12 +51576,12 @@
       </c>
       <c r="E51" s="175" t="inlineStr">
         <is>
-          <t>Dženis Burnić</t>
+          <t>​Elias Saad</t>
         </is>
       </c>
       <c r="F51" s="175" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Tunisia</t>
         </is>
       </c>
     </row>
@@ -51611,7 +51591,7 @@
       </c>
       <c r="B52" s="175" t="inlineStr">
         <is>
-          <t>Schalke 04</t>
+          <t>Karlsruher SC</t>
         </is>
       </c>
       <c r="C52" s="175" t="inlineStr">
@@ -51626,7 +51606,7 @@
       </c>
       <c r="E52" s="175" t="inlineStr">
         <is>
-          <t>Edin Džeko</t>
+          <t>Dženis Burnić</t>
         </is>
       </c>
       <c r="F52" s="175" t="inlineStr">
@@ -51656,7 +51636,7 @@
       </c>
       <c r="E53" s="175" t="inlineStr">
         <is>
-          <t>Nikola Katić</t>
+          <t>Edin Džeko</t>
         </is>
       </c>
       <c r="F53" s="175" t="inlineStr">
@@ -51671,27 +51651,27 @@
       </c>
       <c r="B54" s="175" t="inlineStr">
         <is>
-          <t>El Paso Locomotive FC</t>
+          <t>Schalke 04</t>
         </is>
       </c>
       <c r="C54" s="175" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Tyskland</t>
         </is>
       </c>
       <c r="D54" s="175" t="inlineStr">
         <is>
-          <t>USL Championship</t>
+          <t>2. Bundesliga</t>
         </is>
       </c>
       <c r="E54" s="175" t="inlineStr">
         <is>
-          <t>Carl-Fred Sainthe</t>
+          <t>Nikola Katić</t>
         </is>
       </c>
       <c r="F54" s="175" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
     </row>
@@ -51701,7 +51681,7 @@
       </c>
       <c r="B55" s="175" t="inlineStr">
         <is>
-          <t>Miami FC</t>
+          <t>El Paso Locomotive FC</t>
         </is>
       </c>
       <c r="C55" s="175" t="inlineStr">
@@ -51716,12 +51696,12 @@
       </c>
       <c r="E55" s="175" t="inlineStr">
         <is>
-          <t>Eloy Room</t>
+          <t>Carl-Fred Sainthe</t>
         </is>
       </c>
       <c r="F55" s="175" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Haiti</t>
         </is>
       </c>
     </row>
@@ -51746,42 +51726,42 @@
       </c>
       <c r="E56" s="175" t="inlineStr">
         <is>
+          <t>Eloy Room</t>
+        </is>
+      </c>
+      <c r="F56" s="175" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="B57" s="175" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="C57" s="175" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D57" s="175" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E57" s="175" t="inlineStr">
+        <is>
           <t>Jürgen Locadia</t>
         </is>
       </c>
-      <c r="F56" s="175" t="inlineStr">
+      <c r="F57" s="175" t="inlineStr">
         <is>
           <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="176" t="n">
-        <v>3</v>
-      </c>
-      <c r="B57" s="177" t="inlineStr">
-        <is>
-          <t>Port Vale</t>
-        </is>
-      </c>
-      <c r="C57" s="177" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D57" s="177" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="E57" s="177" t="inlineStr">
-        <is>
-          <t>Ben Waine</t>
-        </is>
-      </c>
-      <c r="F57" s="177" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -51791,7 +51771,7 @@
       </c>
       <c r="B58" s="177" t="inlineStr">
         <is>
-          <t>Rotherham United</t>
+          <t>Port Vale</t>
         </is>
       </c>
       <c r="C58" s="177" t="inlineStr">
@@ -51806,12 +51786,12 @@
       </c>
       <c r="E58" s="177" t="inlineStr">
         <is>
-          <t>Ar’Jany Martha</t>
+          <t>Ben Waine</t>
         </is>
       </c>
       <c r="F58" s="177" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -51821,27 +51801,27 @@
       </c>
       <c r="B59" s="177" t="inlineStr">
         <is>
-          <t>FC Sochaux</t>
+          <t>Rotherham United</t>
         </is>
       </c>
       <c r="C59" s="177" t="inlineStr">
         <is>
-          <t>Frankrike</t>
+          <t>England</t>
         </is>
       </c>
       <c r="D59" s="177" t="inlineStr">
         <is>
-          <t>National</t>
+          <t>League One</t>
         </is>
       </c>
       <c r="E59" s="177" t="inlineStr">
         <is>
-          <t>Alexandre Pierre</t>
+          <t>Ar’Jany Martha</t>
         </is>
       </c>
       <c r="F59" s="177" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -51851,134 +51831,167 @@
       </c>
       <c r="B60" s="177" t="inlineStr">
         <is>
+          <t>FC Sochaux</t>
+        </is>
+      </c>
+      <c r="C60" s="177" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D60" s="177" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="E60" s="177" t="inlineStr">
+        <is>
+          <t>Alexandre Pierre</t>
+        </is>
+      </c>
+      <c r="F60" s="177" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="B61" s="177" t="inlineStr">
+        <is>
           <t>BSC Young Boys II</t>
         </is>
       </c>
-      <c r="C60" s="177" t="inlineStr">
+      <c r="C61" s="177" t="inlineStr">
         <is>
           <t>Sveits</t>
         </is>
       </c>
-      <c r="D60" s="177" t="inlineStr">
+      <c r="D61" s="177" t="inlineStr">
         <is>
           <t>Promotion League</t>
         </is>
       </c>
-      <c r="E60" s="177" t="inlineStr">
+      <c r="E61" s="177" t="inlineStr">
         <is>
           <t>Keeto Thermoncy</t>
         </is>
       </c>
-      <c r="F60" s="177" t="inlineStr">
+      <c r="F61" s="177" t="inlineStr">
         <is>
           <t>Haiti</t>
         </is>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="178" t="n">
+    <row r="62">
+      <c r="A62" s="178" t="n">
         <v>4</v>
       </c>
-      <c r="B61" s="179" t="inlineStr">
+      <c r="B62" s="179" t="inlineStr">
         <is>
           <t>FC Cosmos Koblenz</t>
         </is>
       </c>
-      <c r="C61" s="179" t="inlineStr">
+      <c r="C62" s="179" t="inlineStr">
         <is>
           <t>Tyskland</t>
         </is>
       </c>
-      <c r="D61" s="179" t="inlineStr">
+      <c r="D62" s="179" t="inlineStr">
         <is>
           <t>Regionalliga</t>
         </is>
       </c>
-      <c r="E61" s="179" t="inlineStr">
+      <c r="E62" s="179" t="inlineStr">
         <is>
           <t>Josué Duverger</t>
         </is>
       </c>
-      <c r="F61" s="179" t="inlineStr">
+      <c r="F62" s="179" t="inlineStr">
         <is>
           <t>Haiti</t>
         </is>
       </c>
     </row>
-    <row r="62">
-      <c r="A62" s="180" t="n">
+    <row r="63">
+      <c r="A63" s="180" t="n">
         <v>6</v>
       </c>
-      <c r="B62" s="181" t="inlineStr">
+      <c r="B63" s="181" t="inlineStr">
         <is>
           <t>Braintree Town</t>
         </is>
       </c>
-      <c r="C62" s="181" t="inlineStr">
+      <c r="C63" s="181" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="D62" s="181" t="inlineStr">
+      <c r="D63" s="181" t="inlineStr">
         <is>
           <t>National League South</t>
         </is>
       </c>
-      <c r="E62" s="181" t="inlineStr">
+      <c r="E63" s="181" t="inlineStr">
         <is>
           <t>Tommy Smith</t>
         </is>
       </c>
-      <c r="F62" s="181" t="inlineStr">
+      <c r="F63" s="181" t="inlineStr">
         <is>
           <t>New Zealand</t>
         </is>
       </c>
     </row>
-    <row r="64">
-      <c r="A64" s="32" t="inlineStr">
+    <row r="65">
+      <c r="A65" s="32" t="inlineStr">
         <is>
           <t>Fargeforklaring:</t>
         </is>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="182" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="182" t="inlineStr">
         <is>
           <t>Nivå 2</t>
         </is>
       </c>
     </row>
-    <row r="66">
-      <c r="A66" s="183" t="inlineStr">
+    <row r="67">
+      <c r="A67" s="183" t="inlineStr">
         <is>
           <t>Nivå 3</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" s="184" t="inlineStr">
+    <row r="68">
+      <c r="A68" s="184" t="inlineStr">
         <is>
           <t>Nivå 4</t>
         </is>
       </c>
     </row>
-    <row r="68">
-      <c r="A68" s="185" t="inlineStr">
+    <row r="69">
+      <c r="A69" s="185" t="inlineStr">
         <is>
           <t>Nivå 5</t>
         </is>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="186" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="186" t="inlineStr">
         <is>
           <t>Nivå 6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F1"/>
+  <autoFilter ref="A2:F2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -51989,7 +52002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I69"/>
+  <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="143" min="1" max="1"/>
@@ -52003,1525 +52016,1535 @@
     <col width="8" customWidth="1" style="143" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" s="143">
-      <c r="A1" s="151" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="143">
+      <c r="A1" s="150" t="inlineStr">
+        <is>
+          <t>VM 2026 — Spillere etter klubbland   68 land, 1248 spillere</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="143">
+      <c r="A2" s="151" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B1" s="152" t="inlineStr">
+      <c r="B2" s="152" t="inlineStr">
         <is>
           <t>Land</t>
         </is>
       </c>
-      <c r="C1" s="151" t="inlineStr">
+      <c r="C2" s="151" t="inlineStr">
         <is>
           <t>Spillere</t>
         </is>
       </c>
-      <c r="D1" s="151" t="inlineStr">
+      <c r="D2" s="151" t="inlineStr">
         <is>
           <t>Nivå 1</t>
         </is>
       </c>
-      <c r="E1" s="151" t="inlineStr">
+      <c r="E2" s="151" t="inlineStr">
         <is>
           <t>Nivå 2</t>
         </is>
       </c>
-      <c r="F1" s="151" t="inlineStr">
+      <c r="F2" s="151" t="inlineStr">
         <is>
           <t>Nivå 3</t>
         </is>
       </c>
-      <c r="G1" s="151" t="inlineStr">
+      <c r="G2" s="151" t="inlineStr">
         <is>
           <t>Nivå 4</t>
         </is>
       </c>
-      <c r="H1" s="151" t="inlineStr">
+      <c r="H2" s="151" t="inlineStr">
         <is>
           <t>Nivå 5</t>
         </is>
       </c>
-      <c r="I1" s="151" t="inlineStr">
+      <c r="I2" s="151" t="inlineStr">
         <is>
           <t>Nivå 6</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="17" customHeight="1" s="143">
-      <c r="A2" s="153" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="154" t="inlineStr">
+    <row r="3" ht="17" customHeight="1" s="143">
+      <c r="A3" s="153" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="154" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="C2" s="155" t="n">
+      <c r="C3" s="155" t="n">
         <v>205</v>
       </c>
-      <c r="D2" s="156" t="n">
+      <c r="D3" s="156" t="n">
         <v>168</v>
       </c>
-      <c r="E2" s="156" t="n">
+      <c r="E3" s="156" t="n">
         <v>34</v>
       </c>
-      <c r="F2" s="156" t="n">
+      <c r="F3" s="156" t="n">
         <v>2</v>
       </c>
-      <c r="G2" s="156" t="inlineStr"/>
-      <c r="H2" s="156" t="inlineStr"/>
-      <c r="I2" s="156" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" ht="17" customHeight="1" s="143">
-      <c r="A3" s="157" t="n">
+      <c r="G3" s="156" t="inlineStr"/>
+      <c r="H3" s="156" t="inlineStr"/>
+      <c r="I3" s="156" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1" s="143">
+      <c r="A4" s="157" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="158" t="inlineStr">
+      <c r="B4" s="158" t="inlineStr">
         <is>
           <t>Tyskland</t>
         </is>
       </c>
-      <c r="C3" s="159" t="n">
+      <c r="C4" s="159" t="n">
         <v>111</v>
       </c>
-      <c r="D3" s="160" t="n">
+      <c r="D4" s="160" t="n">
         <v>101</v>
       </c>
-      <c r="E3" s="160" t="n">
+      <c r="E4" s="160" t="n">
         <v>9</v>
       </c>
-      <c r="F3" s="160" t="inlineStr"/>
-      <c r="G3" s="160" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" s="160" t="inlineStr"/>
-      <c r="I3" s="160" t="inlineStr"/>
-    </row>
-    <row r="4" ht="17" customHeight="1" s="143">
-      <c r="A4" s="161" t="n">
+      <c r="F4" s="160" t="inlineStr"/>
+      <c r="G4" s="160" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" s="160" t="inlineStr"/>
+      <c r="I4" s="160" t="inlineStr"/>
+    </row>
+    <row r="5" ht="17" customHeight="1" s="143">
+      <c r="A5" s="161" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="162" t="inlineStr">
+      <c r="B5" s="162" t="inlineStr">
         <is>
           <t>Frankrike</t>
         </is>
       </c>
-      <c r="C4" s="163" t="n">
+      <c r="C5" s="163" t="n">
         <v>86</v>
       </c>
-      <c r="D4" s="164" t="n">
+      <c r="D5" s="164" t="n">
         <v>78</v>
       </c>
-      <c r="E4" s="164" t="n">
+      <c r="E5" s="164" t="n">
         <v>6</v>
       </c>
-      <c r="F4" s="164" t="n">
+      <c r="F5" s="164" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="164" t="inlineStr"/>
-      <c r="H4" s="164" t="inlineStr"/>
-      <c r="I4" s="164" t="inlineStr"/>
-    </row>
-    <row r="5" ht="17" customHeight="1" s="143">
-      <c r="A5" s="165" t="n">
+      <c r="G5" s="164" t="inlineStr"/>
+      <c r="H5" s="164" t="inlineStr"/>
+      <c r="I5" s="164" t="inlineStr"/>
+    </row>
+    <row r="6" ht="17" customHeight="1" s="143">
+      <c r="A6" s="165" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="166" t="inlineStr">
+      <c r="B6" s="166" t="inlineStr">
         <is>
           <t>Spania</t>
         </is>
       </c>
-      <c r="C5" s="167" t="n">
+      <c r="C6" s="167" t="n">
         <v>85</v>
       </c>
-      <c r="D5" s="168" t="n">
+      <c r="D6" s="168" t="n">
         <v>77</v>
       </c>
-      <c r="E5" s="168" t="n">
+      <c r="E6" s="168" t="n">
         <v>8</v>
       </c>
-      <c r="F5" s="168" t="inlineStr"/>
-      <c r="G5" s="168" t="inlineStr"/>
-      <c r="H5" s="168" t="inlineStr"/>
-      <c r="I5" s="168" t="inlineStr"/>
-    </row>
-    <row r="6" ht="17" customHeight="1" s="143">
-      <c r="A6" s="169" t="n">
+      <c r="F6" s="168" t="inlineStr"/>
+      <c r="G6" s="168" t="inlineStr"/>
+      <c r="H6" s="168" t="inlineStr"/>
+      <c r="I6" s="168" t="inlineStr"/>
+    </row>
+    <row r="7" ht="17" customHeight="1" s="143">
+      <c r="A7" s="169" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="170" t="inlineStr">
+      <c r="B7" s="170" t="inlineStr">
         <is>
           <t>Italia</t>
         </is>
       </c>
-      <c r="C6" s="171" t="n">
+      <c r="C7" s="171" t="n">
         <v>70</v>
       </c>
-      <c r="D6" s="172" t="n">
+      <c r="D7" s="172" t="n">
         <v>65</v>
       </c>
-      <c r="E6" s="172" t="n">
+      <c r="E7" s="172" t="n">
         <v>5</v>
       </c>
-      <c r="F6" s="172" t="inlineStr"/>
-      <c r="G6" s="172" t="inlineStr"/>
-      <c r="H6" s="172" t="inlineStr"/>
-      <c r="I6" s="172" t="inlineStr"/>
-    </row>
-    <row r="7" ht="17" customHeight="1" s="143">
-      <c r="A7" s="165" t="n">
+      <c r="F7" s="172" t="inlineStr"/>
+      <c r="G7" s="172" t="inlineStr"/>
+      <c r="H7" s="172" t="inlineStr"/>
+      <c r="I7" s="172" t="inlineStr"/>
+    </row>
+    <row r="8" ht="17" customHeight="1" s="143">
+      <c r="A8" s="165" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="166" t="inlineStr">
+      <c r="B8" s="166" t="inlineStr">
         <is>
           <t>Saudi-Arabia</t>
         </is>
       </c>
-      <c r="C7" s="167" t="n">
+      <c r="C8" s="167" t="n">
         <v>51</v>
       </c>
-      <c r="D7" s="168" t="n">
+      <c r="D8" s="168" t="n">
         <v>50</v>
       </c>
-      <c r="E7" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="168" t="inlineStr"/>
-      <c r="G7" s="168" t="inlineStr"/>
-      <c r="H7" s="168" t="inlineStr"/>
-      <c r="I7" s="168" t="inlineStr"/>
-    </row>
-    <row r="8" ht="17" customHeight="1" s="143">
-      <c r="A8" s="169" t="n">
+      <c r="E8" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="168" t="inlineStr"/>
+      <c r="G8" s="168" t="inlineStr"/>
+      <c r="H8" s="168" t="inlineStr"/>
+      <c r="I8" s="168" t="inlineStr"/>
+    </row>
+    <row r="9" ht="17" customHeight="1" s="143">
+      <c r="A9" s="169" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="170" t="inlineStr">
+      <c r="B9" s="170" t="inlineStr">
         <is>
           <t>Tyrkia</t>
         </is>
       </c>
-      <c r="C8" s="171" t="n">
+      <c r="C9" s="171" t="n">
         <v>45</v>
       </c>
-      <c r="D8" s="172" t="n">
+      <c r="D9" s="172" t="n">
         <v>43</v>
       </c>
-      <c r="E8" s="172" t="n">
+      <c r="E9" s="172" t="n">
         <v>2</v>
       </c>
-      <c r="F8" s="172" t="inlineStr"/>
-      <c r="G8" s="172" t="inlineStr"/>
-      <c r="H8" s="172" t="inlineStr"/>
-      <c r="I8" s="172" t="inlineStr"/>
-    </row>
-    <row r="9" ht="17" customHeight="1" s="143">
-      <c r="A9" s="165" t="n">
+      <c r="F9" s="172" t="inlineStr"/>
+      <c r="G9" s="172" t="inlineStr"/>
+      <c r="H9" s="172" t="inlineStr"/>
+      <c r="I9" s="172" t="inlineStr"/>
+    </row>
+    <row r="10" ht="17" customHeight="1" s="143">
+      <c r="A10" s="165" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="166" t="inlineStr">
+      <c r="B10" s="166" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="C9" s="167" t="n">
+      <c r="C10" s="167" t="n">
         <v>41</v>
       </c>
-      <c r="D9" s="168" t="n">
+      <c r="D10" s="168" t="n">
         <v>36</v>
       </c>
-      <c r="E9" s="168" t="n">
+      <c r="E10" s="168" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="168" t="inlineStr"/>
-      <c r="G9" s="168" t="inlineStr"/>
-      <c r="H9" s="168" t="inlineStr"/>
-      <c r="I9" s="168" t="inlineStr"/>
-    </row>
-    <row r="10" ht="17" customHeight="1" s="143">
-      <c r="A10" s="169" t="n">
+      <c r="F10" s="168" t="inlineStr"/>
+      <c r="G10" s="168" t="inlineStr"/>
+      <c r="H10" s="168" t="inlineStr"/>
+      <c r="I10" s="168" t="inlineStr"/>
+    </row>
+    <row r="11" ht="17" customHeight="1" s="143">
+      <c r="A11" s="169" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="170" t="inlineStr">
+      <c r="B11" s="170" t="inlineStr">
         <is>
           <t>Nederland</t>
         </is>
       </c>
-      <c r="C10" s="171" t="n">
+      <c r="C11" s="171" t="n">
         <v>38</v>
       </c>
-      <c r="D10" s="172" t="n">
+      <c r="D11" s="172" t="n">
         <v>33</v>
       </c>
-      <c r="E10" s="172" t="n">
+      <c r="E11" s="172" t="n">
         <v>5</v>
       </c>
-      <c r="F10" s="172" t="inlineStr"/>
-      <c r="G10" s="172" t="inlineStr"/>
-      <c r="H10" s="172" t="inlineStr"/>
-      <c r="I10" s="172" t="inlineStr"/>
-    </row>
-    <row r="11" ht="17" customHeight="1" s="143">
-      <c r="A11" s="165" t="n">
+      <c r="F11" s="172" t="inlineStr"/>
+      <c r="G11" s="172" t="inlineStr"/>
+      <c r="H11" s="172" t="inlineStr"/>
+      <c r="I11" s="172" t="inlineStr"/>
+    </row>
+    <row r="12" ht="17" customHeight="1" s="143">
+      <c r="A12" s="165" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="166" t="inlineStr">
+      <c r="B12" s="166" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="C11" s="167" t="n">
+      <c r="C12" s="167" t="n">
         <v>32</v>
       </c>
-      <c r="D11" s="168" t="n">
+      <c r="D12" s="168" t="n">
         <v>29</v>
       </c>
-      <c r="E11" s="168" t="n">
+      <c r="E12" s="168" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="168" t="inlineStr"/>
-      <c r="H11" s="168" t="inlineStr"/>
-      <c r="I11" s="168" t="inlineStr"/>
-    </row>
-    <row r="12" ht="17" customHeight="1" s="143">
-      <c r="A12" s="169" t="n">
+      <c r="F12" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="168" t="inlineStr"/>
+      <c r="H12" s="168" t="inlineStr"/>
+      <c r="I12" s="168" t="inlineStr"/>
+    </row>
+    <row r="13" ht="17" customHeight="1" s="143">
+      <c r="A13" s="169" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="170" t="inlineStr">
+      <c r="B13" s="170" t="inlineStr">
         <is>
           <t>Brasil</t>
         </is>
       </c>
-      <c r="C12" s="171" t="n">
+      <c r="C13" s="171" t="n">
         <v>31</v>
       </c>
-      <c r="D12" s="172" t="n">
+      <c r="D13" s="172" t="n">
         <v>31</v>
       </c>
-      <c r="E12" s="172" t="inlineStr"/>
-      <c r="F12" s="172" t="inlineStr"/>
-      <c r="G12" s="172" t="inlineStr"/>
-      <c r="H12" s="172" t="inlineStr"/>
-      <c r="I12" s="172" t="inlineStr"/>
-    </row>
-    <row r="13" ht="17" customHeight="1" s="143">
-      <c r="A13" s="165" t="n">
+      <c r="E13" s="172" t="inlineStr"/>
+      <c r="F13" s="172" t="inlineStr"/>
+      <c r="G13" s="172" t="inlineStr"/>
+      <c r="H13" s="172" t="inlineStr"/>
+      <c r="I13" s="172" t="inlineStr"/>
+    </row>
+    <row r="14" ht="17" customHeight="1" s="143">
+      <c r="A14" s="165" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="166" t="inlineStr">
+      <c r="B14" s="166" t="inlineStr">
         <is>
           <t>Belgia</t>
         </is>
       </c>
-      <c r="C13" s="167" t="n">
+      <c r="C14" s="167" t="n">
         <v>29</v>
       </c>
-      <c r="D13" s="168" t="n">
+      <c r="D14" s="168" t="n">
         <v>28</v>
       </c>
-      <c r="E13" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="F13" s="168" t="inlineStr"/>
-      <c r="G13" s="168" t="inlineStr"/>
-      <c r="H13" s="168" t="inlineStr"/>
-      <c r="I13" s="168" t="inlineStr"/>
-    </row>
-    <row r="14" ht="17" customHeight="1" s="143">
-      <c r="A14" s="169" t="n">
+      <c r="E14" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="168" t="inlineStr"/>
+      <c r="G14" s="168" t="inlineStr"/>
+      <c r="H14" s="168" t="inlineStr"/>
+      <c r="I14" s="168" t="inlineStr"/>
+    </row>
+    <row r="15" ht="17" customHeight="1" s="143">
+      <c r="A15" s="169" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="170" t="inlineStr">
+      <c r="B15" s="170" t="inlineStr">
         <is>
           <t>Qatar</t>
         </is>
       </c>
-      <c r="C14" s="171" t="n">
+      <c r="C15" s="171" t="n">
         <v>29</v>
       </c>
-      <c r="D14" s="172" t="n">
+      <c r="D15" s="172" t="n">
         <v>29</v>
       </c>
-      <c r="E14" s="172" t="inlineStr"/>
-      <c r="F14" s="172" t="inlineStr"/>
-      <c r="G14" s="172" t="inlineStr"/>
-      <c r="H14" s="172" t="inlineStr"/>
-      <c r="I14" s="172" t="inlineStr"/>
-    </row>
-    <row r="15" ht="17" customHeight="1" s="143">
-      <c r="A15" s="165" t="n">
+      <c r="E15" s="172" t="inlineStr"/>
+      <c r="F15" s="172" t="inlineStr"/>
+      <c r="G15" s="172" t="inlineStr"/>
+      <c r="H15" s="172" t="inlineStr"/>
+      <c r="I15" s="172" t="inlineStr"/>
+    </row>
+    <row r="16" ht="17" customHeight="1" s="143">
+      <c r="A16" s="165" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="166" t="inlineStr">
+      <c r="B16" s="166" t="inlineStr">
         <is>
           <t>Mexico</t>
         </is>
       </c>
-      <c r="C15" s="167" t="n">
+      <c r="C16" s="167" t="n">
         <v>27</v>
       </c>
-      <c r="D15" s="168" t="n">
+      <c r="D16" s="168" t="n">
         <v>27</v>
       </c>
-      <c r="E15" s="168" t="inlineStr"/>
-      <c r="F15" s="168" t="inlineStr"/>
-      <c r="G15" s="168" t="inlineStr"/>
-      <c r="H15" s="168" t="inlineStr"/>
-      <c r="I15" s="168" t="inlineStr"/>
-    </row>
-    <row r="16" ht="17" customHeight="1" s="143">
-      <c r="A16" s="169" t="n">
+      <c r="E16" s="168" t="inlineStr"/>
+      <c r="F16" s="168" t="inlineStr"/>
+      <c r="G16" s="168" t="inlineStr"/>
+      <c r="H16" s="168" t="inlineStr"/>
+      <c r="I16" s="168" t="inlineStr"/>
+    </row>
+    <row r="17" ht="17" customHeight="1" s="143">
+      <c r="A17" s="169" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="170" t="inlineStr">
+      <c r="B17" s="170" t="inlineStr">
         <is>
           <t>Tsjekkia</t>
         </is>
       </c>
-      <c r="C16" s="171" t="n">
+      <c r="C17" s="171" t="n">
         <v>22</v>
       </c>
-      <c r="D16" s="172" t="n">
+      <c r="D17" s="172" t="n">
         <v>22</v>
       </c>
-      <c r="E16" s="172" t="inlineStr"/>
-      <c r="F16" s="172" t="inlineStr"/>
-      <c r="G16" s="172" t="inlineStr"/>
-      <c r="H16" s="172" t="inlineStr"/>
-      <c r="I16" s="172" t="inlineStr"/>
-    </row>
-    <row r="17" ht="17" customHeight="1" s="143">
-      <c r="A17" s="165" t="n">
+      <c r="E17" s="172" t="inlineStr"/>
+      <c r="F17" s="172" t="inlineStr"/>
+      <c r="G17" s="172" t="inlineStr"/>
+      <c r="H17" s="172" t="inlineStr"/>
+      <c r="I17" s="172" t="inlineStr"/>
+    </row>
+    <row r="18" ht="17" customHeight="1" s="143">
+      <c r="A18" s="165" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="166" t="inlineStr">
+      <c r="B18" s="166" t="inlineStr">
         <is>
           <t>Iran</t>
         </is>
       </c>
-      <c r="C17" s="167" t="n">
+      <c r="C18" s="167" t="n">
         <v>22</v>
       </c>
-      <c r="D17" s="168" t="n">
+      <c r="D18" s="168" t="n">
         <v>22</v>
       </c>
-      <c r="E17" s="168" t="inlineStr"/>
-      <c r="F17" s="168" t="inlineStr"/>
-      <c r="G17" s="168" t="inlineStr"/>
-      <c r="H17" s="168" t="inlineStr"/>
-      <c r="I17" s="168" t="inlineStr"/>
-    </row>
-    <row r="18" ht="17" customHeight="1" s="143">
-      <c r="A18" s="169" t="n">
+      <c r="E18" s="168" t="inlineStr"/>
+      <c r="F18" s="168" t="inlineStr"/>
+      <c r="G18" s="168" t="inlineStr"/>
+      <c r="H18" s="168" t="inlineStr"/>
+      <c r="I18" s="168" t="inlineStr"/>
+    </row>
+    <row r="19" ht="17" customHeight="1" s="143">
+      <c r="A19" s="169" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="170" t="inlineStr">
+      <c r="B19" s="170" t="inlineStr">
         <is>
           <t>Egypt</t>
         </is>
       </c>
-      <c r="C18" s="171" t="n">
+      <c r="C19" s="171" t="n">
         <v>21</v>
       </c>
-      <c r="D18" s="172" t="n">
+      <c r="D19" s="172" t="n">
         <v>21</v>
       </c>
-      <c r="E18" s="172" t="inlineStr"/>
-      <c r="F18" s="172" t="inlineStr"/>
-      <c r="G18" s="172" t="inlineStr"/>
-      <c r="H18" s="172" t="inlineStr"/>
-      <c r="I18" s="172" t="inlineStr"/>
-    </row>
-    <row r="19" ht="17" customHeight="1" s="143">
-      <c r="A19" s="165" t="n">
+      <c r="E19" s="172" t="inlineStr"/>
+      <c r="F19" s="172" t="inlineStr"/>
+      <c r="G19" s="172" t="inlineStr"/>
+      <c r="H19" s="172" t="inlineStr"/>
+      <c r="I19" s="172" t="inlineStr"/>
+    </row>
+    <row r="20" ht="17" customHeight="1" s="143">
+      <c r="A20" s="165" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="166" t="inlineStr">
+      <c r="B20" s="166" t="inlineStr">
         <is>
           <t>Skottland</t>
         </is>
       </c>
-      <c r="C19" s="167" t="n">
+      <c r="C20" s="167" t="n">
         <v>20</v>
       </c>
-      <c r="D19" s="168" t="n">
+      <c r="D20" s="168" t="n">
         <v>20</v>
       </c>
-      <c r="E19" s="168" t="inlineStr"/>
-      <c r="F19" s="168" t="inlineStr"/>
-      <c r="G19" s="168" t="inlineStr"/>
-      <c r="H19" s="168" t="inlineStr"/>
-      <c r="I19" s="168" t="inlineStr"/>
-    </row>
-    <row r="20" ht="17" customHeight="1" s="143">
-      <c r="A20" s="169" t="n">
+      <c r="E20" s="168" t="inlineStr"/>
+      <c r="F20" s="168" t="inlineStr"/>
+      <c r="G20" s="168" t="inlineStr"/>
+      <c r="H20" s="168" t="inlineStr"/>
+      <c r="I20" s="168" t="inlineStr"/>
+    </row>
+    <row r="21" ht="17" customHeight="1" s="143">
+      <c r="A21" s="169" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="170" t="inlineStr">
+      <c r="B21" s="170" t="inlineStr">
         <is>
           <t>Sør-Afrika</t>
         </is>
       </c>
-      <c r="C20" s="171" t="n">
+      <c r="C21" s="171" t="n">
         <v>19</v>
       </c>
-      <c r="D20" s="172" t="n">
+      <c r="D21" s="172" t="n">
         <v>18</v>
       </c>
-      <c r="E20" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="172" t="inlineStr"/>
-      <c r="G20" s="172" t="inlineStr"/>
-      <c r="H20" s="172" t="inlineStr"/>
-      <c r="I20" s="172" t="inlineStr"/>
-    </row>
-    <row r="21" ht="17" customHeight="1" s="143">
-      <c r="A21" s="165" t="n">
+      <c r="E21" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="172" t="inlineStr"/>
+      <c r="G21" s="172" t="inlineStr"/>
+      <c r="H21" s="172" t="inlineStr"/>
+      <c r="I21" s="172" t="inlineStr"/>
+    </row>
+    <row r="22" ht="17" customHeight="1" s="143">
+      <c r="A22" s="165" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="166" t="inlineStr">
+      <c r="B22" s="166" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="C21" s="167" t="n">
+      <c r="C22" s="167" t="n">
         <v>16</v>
       </c>
-      <c r="D21" s="168" t="n">
+      <c r="D22" s="168" t="n">
         <v>16</v>
       </c>
-      <c r="E21" s="168" t="inlineStr"/>
-      <c r="F21" s="168" t="inlineStr"/>
-      <c r="G21" s="168" t="inlineStr"/>
-      <c r="H21" s="168" t="inlineStr"/>
-      <c r="I21" s="168" t="inlineStr"/>
-    </row>
-    <row r="22" ht="17" customHeight="1" s="143">
-      <c r="A22" s="169" t="n">
+      <c r="E22" s="168" t="inlineStr"/>
+      <c r="F22" s="168" t="inlineStr"/>
+      <c r="G22" s="168" t="inlineStr"/>
+      <c r="H22" s="168" t="inlineStr"/>
+      <c r="I22" s="168" t="inlineStr"/>
+    </row>
+    <row r="23" ht="17" customHeight="1" s="143">
+      <c r="A23" s="169" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="170" t="inlineStr">
+      <c r="B23" s="170" t="inlineStr">
         <is>
           <t>Russland</t>
         </is>
       </c>
-      <c r="C22" s="171" t="n">
+      <c r="C23" s="171" t="n">
         <v>15</v>
       </c>
-      <c r="D22" s="172" t="n">
+      <c r="D23" s="172" t="n">
         <v>15</v>
       </c>
-      <c r="E22" s="172" t="inlineStr"/>
-      <c r="F22" s="172" t="inlineStr"/>
-      <c r="G22" s="172" t="inlineStr"/>
-      <c r="H22" s="172" t="inlineStr"/>
-      <c r="I22" s="172" t="inlineStr"/>
-    </row>
-    <row r="23" ht="17" customHeight="1" s="143">
-      <c r="A23" s="165" t="n">
+      <c r="E23" s="172" t="inlineStr"/>
+      <c r="F23" s="172" t="inlineStr"/>
+      <c r="G23" s="172" t="inlineStr"/>
+      <c r="H23" s="172" t="inlineStr"/>
+      <c r="I23" s="172" t="inlineStr"/>
+    </row>
+    <row r="24" ht="17" customHeight="1" s="143">
+      <c r="A24" s="165" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="166" t="inlineStr">
+      <c r="B24" s="166" t="inlineStr">
         <is>
           <t>Irak</t>
         </is>
       </c>
-      <c r="C23" s="167" t="n">
+      <c r="C24" s="167" t="n">
         <v>14</v>
       </c>
-      <c r="D23" s="168" t="n">
+      <c r="D24" s="168" t="n">
         <v>14</v>
       </c>
-      <c r="E23" s="168" t="inlineStr"/>
-      <c r="F23" s="168" t="inlineStr"/>
-      <c r="G23" s="168" t="inlineStr"/>
-      <c r="H23" s="168" t="inlineStr"/>
-      <c r="I23" s="168" t="inlineStr"/>
-    </row>
-    <row r="24" ht="17" customHeight="1" s="143">
-      <c r="A24" s="169" t="n">
+      <c r="E24" s="168" t="inlineStr"/>
+      <c r="F24" s="168" t="inlineStr"/>
+      <c r="G24" s="168" t="inlineStr"/>
+      <c r="H24" s="168" t="inlineStr"/>
+      <c r="I24" s="168" t="inlineStr"/>
+    </row>
+    <row r="25" ht="17" customHeight="1" s="143">
+      <c r="A25" s="169" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="170" t="inlineStr">
+      <c r="B25" s="170" t="inlineStr">
         <is>
           <t>Usbekistan</t>
         </is>
       </c>
-      <c r="C24" s="171" t="n">
+      <c r="C25" s="171" t="n">
         <v>14</v>
       </c>
-      <c r="D24" s="172" t="n">
+      <c r="D25" s="172" t="n">
         <v>14</v>
       </c>
-      <c r="E24" s="172" t="inlineStr"/>
-      <c r="F24" s="172" t="inlineStr"/>
-      <c r="G24" s="172" t="inlineStr"/>
-      <c r="H24" s="172" t="inlineStr"/>
-      <c r="I24" s="172" t="inlineStr"/>
-    </row>
-    <row r="25" ht="17" customHeight="1" s="143">
-      <c r="A25" s="165" t="n">
+      <c r="E25" s="172" t="inlineStr"/>
+      <c r="F25" s="172" t="inlineStr"/>
+      <c r="G25" s="172" t="inlineStr"/>
+      <c r="H25" s="172" t="inlineStr"/>
+      <c r="I25" s="172" t="inlineStr"/>
+    </row>
+    <row r="26" ht="17" customHeight="1" s="143">
+      <c r="A26" s="165" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="166" t="inlineStr">
+      <c r="B26" s="166" t="inlineStr">
         <is>
           <t>UAE</t>
         </is>
       </c>
-      <c r="C25" s="167" t="n">
+      <c r="C26" s="167" t="n">
         <v>13</v>
       </c>
-      <c r="D25" s="168" t="n">
+      <c r="D26" s="168" t="n">
         <v>10</v>
       </c>
-      <c r="E25" s="168" t="n">
+      <c r="E26" s="168" t="n">
         <v>3</v>
       </c>
-      <c r="F25" s="168" t="inlineStr"/>
-      <c r="G25" s="168" t="inlineStr"/>
-      <c r="H25" s="168" t="inlineStr"/>
-      <c r="I25" s="168" t="inlineStr"/>
-    </row>
-    <row r="26" ht="17" customHeight="1" s="143">
-      <c r="A26" s="169" t="n">
+      <c r="F26" s="168" t="inlineStr"/>
+      <c r="G26" s="168" t="inlineStr"/>
+      <c r="H26" s="168" t="inlineStr"/>
+      <c r="I26" s="168" t="inlineStr"/>
+    </row>
+    <row r="27" ht="17" customHeight="1" s="143">
+      <c r="A27" s="169" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="170" t="inlineStr">
+      <c r="B27" s="170" t="inlineStr">
         <is>
           <t>Hellas</t>
         </is>
       </c>
-      <c r="C26" s="171" t="n">
+      <c r="C27" s="171" t="n">
         <v>12</v>
       </c>
-      <c r="D26" s="172" t="n">
+      <c r="D27" s="172" t="n">
         <v>12</v>
       </c>
-      <c r="E26" s="172" t="inlineStr"/>
-      <c r="F26" s="172" t="inlineStr"/>
-      <c r="G26" s="172" t="inlineStr"/>
-      <c r="H26" s="172" t="inlineStr"/>
-      <c r="I26" s="172" t="inlineStr"/>
-    </row>
-    <row r="27" ht="17" customHeight="1" s="143">
-      <c r="A27" s="165" t="n">
+      <c r="E27" s="172" t="inlineStr"/>
+      <c r="F27" s="172" t="inlineStr"/>
+      <c r="G27" s="172" t="inlineStr"/>
+      <c r="H27" s="172" t="inlineStr"/>
+      <c r="I27" s="172" t="inlineStr"/>
+    </row>
+    <row r="28" ht="17" customHeight="1" s="143">
+      <c r="A28" s="165" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="166" t="inlineStr">
+      <c r="B28" s="166" t="inlineStr">
         <is>
           <t>Danmark</t>
         </is>
       </c>
-      <c r="C27" s="167" t="n">
+      <c r="C28" s="167" t="n">
         <v>12</v>
       </c>
-      <c r="D27" s="168" t="n">
+      <c r="D28" s="168" t="n">
         <v>12</v>
       </c>
-      <c r="E27" s="168" t="inlineStr"/>
-      <c r="F27" s="168" t="inlineStr"/>
-      <c r="G27" s="168" t="inlineStr"/>
-      <c r="H27" s="168" t="inlineStr"/>
-      <c r="I27" s="168" t="inlineStr"/>
-    </row>
-    <row r="28" ht="17" customHeight="1" s="143">
-      <c r="A28" s="169" t="n">
+      <c r="E28" s="168" t="inlineStr"/>
+      <c r="F28" s="168" t="inlineStr"/>
+      <c r="G28" s="168" t="inlineStr"/>
+      <c r="H28" s="168" t="inlineStr"/>
+      <c r="I28" s="168" t="inlineStr"/>
+    </row>
+    <row r="29" ht="17" customHeight="1" s="143">
+      <c r="A29" s="169" t="n">
         <v>25</v>
       </c>
-      <c r="B28" s="170" t="inlineStr">
+      <c r="B29" s="170" t="inlineStr">
         <is>
           <t>Sveits</t>
         </is>
       </c>
-      <c r="C28" s="171" t="n">
+      <c r="C29" s="171" t="n">
         <v>12</v>
       </c>
-      <c r="D28" s="172" t="n">
+      <c r="D29" s="172" t="n">
         <v>11</v>
       </c>
-      <c r="E28" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="F28" s="172" t="inlineStr"/>
-      <c r="G28" s="172" t="inlineStr"/>
-      <c r="H28" s="172" t="inlineStr"/>
-      <c r="I28" s="172" t="inlineStr"/>
-    </row>
-    <row r="29" ht="17" customHeight="1" s="143">
-      <c r="A29" s="165" t="n">
+      <c r="E29" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="172" t="inlineStr"/>
+      <c r="G29" s="172" t="inlineStr"/>
+      <c r="H29" s="172" t="inlineStr"/>
+      <c r="I29" s="172" t="inlineStr"/>
+    </row>
+    <row r="30" ht="17" customHeight="1" s="143">
+      <c r="A30" s="165" t="n">
         <v>25</v>
       </c>
-      <c r="B29" s="166" t="inlineStr">
+      <c r="B30" s="166" t="inlineStr">
         <is>
           <t>Jordan</t>
         </is>
       </c>
-      <c r="C29" s="167" t="n">
+      <c r="C30" s="167" t="n">
         <v>12</v>
       </c>
-      <c r="D29" s="168" t="n">
+      <c r="D30" s="168" t="n">
         <v>12</v>
       </c>
-      <c r="E29" s="168" t="inlineStr"/>
-      <c r="F29" s="168" t="inlineStr"/>
-      <c r="G29" s="168" t="inlineStr"/>
-      <c r="H29" s="168" t="inlineStr"/>
-      <c r="I29" s="168" t="inlineStr"/>
-    </row>
-    <row r="30" ht="17" customHeight="1" s="143">
-      <c r="A30" s="169" t="n">
+      <c r="E30" s="168" t="inlineStr"/>
+      <c r="F30" s="168" t="inlineStr"/>
+      <c r="G30" s="168" t="inlineStr"/>
+      <c r="H30" s="168" t="inlineStr"/>
+      <c r="I30" s="168" t="inlineStr"/>
+    </row>
+    <row r="31" ht="17" customHeight="1" s="143">
+      <c r="A31" s="169" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="170" t="inlineStr">
+      <c r="B31" s="170" t="inlineStr">
         <is>
           <t>Kypros</t>
         </is>
       </c>
-      <c r="C30" s="171" t="n">
+      <c r="C31" s="171" t="n">
         <v>10</v>
       </c>
-      <c r="D30" s="172" t="n">
+      <c r="D31" s="172" t="n">
         <v>10</v>
       </c>
-      <c r="E30" s="172" t="inlineStr"/>
-      <c r="F30" s="172" t="inlineStr"/>
-      <c r="G30" s="172" t="inlineStr"/>
-      <c r="H30" s="172" t="inlineStr"/>
-      <c r="I30" s="172" t="inlineStr"/>
-    </row>
-    <row r="31" ht="17" customHeight="1" s="143">
-      <c r="A31" s="165" t="n">
+      <c r="E31" s="172" t="inlineStr"/>
+      <c r="F31" s="172" t="inlineStr"/>
+      <c r="G31" s="172" t="inlineStr"/>
+      <c r="H31" s="172" t="inlineStr"/>
+      <c r="I31" s="172" t="inlineStr"/>
+    </row>
+    <row r="32" ht="17" customHeight="1" s="143">
+      <c r="A32" s="165" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="166" t="inlineStr">
+      <c r="B32" s="166" t="inlineStr">
         <is>
           <t>Sør-Korea</t>
         </is>
       </c>
-      <c r="C31" s="167" t="n">
+      <c r="C32" s="167" t="n">
         <v>9</v>
       </c>
-      <c r="D31" s="168" t="n">
+      <c r="D32" s="168" t="n">
         <v>9</v>
       </c>
-      <c r="E31" s="168" t="inlineStr"/>
-      <c r="F31" s="168" t="inlineStr"/>
-      <c r="G31" s="168" t="inlineStr"/>
-      <c r="H31" s="168" t="inlineStr"/>
-      <c r="I31" s="168" t="inlineStr"/>
-    </row>
-    <row r="32" ht="17" customHeight="1" s="143">
-      <c r="A32" s="169" t="n">
+      <c r="E32" s="168" t="inlineStr"/>
+      <c r="F32" s="168" t="inlineStr"/>
+      <c r="G32" s="168" t="inlineStr"/>
+      <c r="H32" s="168" t="inlineStr"/>
+      <c r="I32" s="168" t="inlineStr"/>
+    </row>
+    <row r="33" ht="17" customHeight="1" s="143">
+      <c r="A33" s="169" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="170" t="inlineStr">
+      <c r="B33" s="170" t="inlineStr">
         <is>
           <t>Ny-Zealand</t>
         </is>
       </c>
-      <c r="C32" s="171" t="n">
+      <c r="C33" s="171" t="n">
         <v>9</v>
       </c>
-      <c r="D32" s="172" t="n">
+      <c r="D33" s="172" t="n">
         <v>9</v>
       </c>
-      <c r="E32" s="172" t="inlineStr"/>
-      <c r="F32" s="172" t="inlineStr"/>
-      <c r="G32" s="172" t="inlineStr"/>
-      <c r="H32" s="172" t="inlineStr"/>
-      <c r="I32" s="172" t="inlineStr"/>
-    </row>
-    <row r="33" ht="17" customHeight="1" s="143">
-      <c r="A33" s="165" t="n">
+      <c r="E33" s="172" t="inlineStr"/>
+      <c r="F33" s="172" t="inlineStr"/>
+      <c r="G33" s="172" t="inlineStr"/>
+      <c r="H33" s="172" t="inlineStr"/>
+      <c r="I33" s="172" t="inlineStr"/>
+    </row>
+    <row r="34" ht="17" customHeight="1" s="143">
+      <c r="A34" s="165" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="166" t="inlineStr">
+      <c r="B34" s="166" t="inlineStr">
         <is>
           <t>Østerrike</t>
         </is>
       </c>
-      <c r="C33" s="167" t="n">
+      <c r="C34" s="167" t="n">
         <v>8</v>
       </c>
-      <c r="D33" s="168" t="n">
+      <c r="D34" s="168" t="n">
         <v>8</v>
       </c>
-      <c r="E33" s="168" t="inlineStr"/>
-      <c r="F33" s="168" t="inlineStr"/>
-      <c r="G33" s="168" t="inlineStr"/>
-      <c r="H33" s="168" t="inlineStr"/>
-      <c r="I33" s="168" t="inlineStr"/>
-    </row>
-    <row r="34" ht="17" customHeight="1" s="143">
-      <c r="A34" s="169" t="n">
+      <c r="E34" s="168" t="inlineStr"/>
+      <c r="F34" s="168" t="inlineStr"/>
+      <c r="G34" s="168" t="inlineStr"/>
+      <c r="H34" s="168" t="inlineStr"/>
+      <c r="I34" s="168" t="inlineStr"/>
+    </row>
+    <row r="35" ht="17" customHeight="1" s="143">
+      <c r="A35" s="169" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="170" t="inlineStr">
+      <c r="B35" s="170" t="inlineStr">
         <is>
           <t>Norge</t>
         </is>
       </c>
-      <c r="C34" s="171" t="n">
+      <c r="C35" s="171" t="n">
         <v>7</v>
       </c>
-      <c r="D34" s="172" t="n">
+      <c r="D35" s="172" t="n">
         <v>7</v>
       </c>
-      <c r="E34" s="172" t="inlineStr"/>
-      <c r="F34" s="172" t="inlineStr"/>
-      <c r="G34" s="172" t="inlineStr"/>
-      <c r="H34" s="172" t="inlineStr"/>
-      <c r="I34" s="172" t="inlineStr"/>
-    </row>
-    <row r="35" ht="17" customHeight="1" s="143">
-      <c r="A35" s="165" t="n">
+      <c r="E35" s="172" t="inlineStr"/>
+      <c r="F35" s="172" t="inlineStr"/>
+      <c r="G35" s="172" t="inlineStr"/>
+      <c r="H35" s="172" t="inlineStr"/>
+      <c r="I35" s="172" t="inlineStr"/>
+    </row>
+    <row r="36" ht="17" customHeight="1" s="143">
+      <c r="A36" s="165" t="n">
         <v>33</v>
       </c>
-      <c r="B35" s="166" t="inlineStr">
+      <c r="B36" s="166" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="C35" s="167" t="n">
+      <c r="C36" s="167" t="n">
         <v>7</v>
       </c>
-      <c r="D35" s="168" t="n">
+      <c r="D36" s="168" t="n">
         <v>6</v>
       </c>
-      <c r="E35" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="F35" s="168" t="inlineStr"/>
-      <c r="G35" s="168" t="inlineStr"/>
-      <c r="H35" s="168" t="inlineStr"/>
-      <c r="I35" s="168" t="inlineStr"/>
-    </row>
-    <row r="36" ht="17" customHeight="1" s="143">
-      <c r="A36" s="169" t="n">
+      <c r="E36" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="168" t="inlineStr"/>
+      <c r="G36" s="168" t="inlineStr"/>
+      <c r="H36" s="168" t="inlineStr"/>
+      <c r="I36" s="168" t="inlineStr"/>
+    </row>
+    <row r="37" ht="17" customHeight="1" s="143">
+      <c r="A37" s="169" t="n">
         <v>33</v>
       </c>
-      <c r="B36" s="170" t="inlineStr">
+      <c r="B37" s="170" t="inlineStr">
         <is>
           <t>Canada</t>
         </is>
       </c>
-      <c r="C36" s="171" t="n">
+      <c r="C37" s="171" t="n">
         <v>7</v>
       </c>
-      <c r="D36" s="172" t="n">
+      <c r="D37" s="172" t="n">
         <v>7</v>
       </c>
-      <c r="E36" s="172" t="inlineStr"/>
-      <c r="F36" s="172" t="inlineStr"/>
-      <c r="G36" s="172" t="inlineStr"/>
-      <c r="H36" s="172" t="inlineStr"/>
-      <c r="I36" s="172" t="inlineStr"/>
-    </row>
-    <row r="37" ht="17" customHeight="1" s="143">
-      <c r="A37" s="165" t="n">
+      <c r="E37" s="172" t="inlineStr"/>
+      <c r="F37" s="172" t="inlineStr"/>
+      <c r="G37" s="172" t="inlineStr"/>
+      <c r="H37" s="172" t="inlineStr"/>
+      <c r="I37" s="172" t="inlineStr"/>
+    </row>
+    <row r="38" ht="17" customHeight="1" s="143">
+      <c r="A38" s="165" t="n">
         <v>33</v>
       </c>
-      <c r="B37" s="166" t="inlineStr">
+      <c r="B38" s="166" t="inlineStr">
         <is>
           <t>Polen</t>
         </is>
       </c>
-      <c r="C37" s="167" t="n">
+      <c r="C38" s="167" t="n">
         <v>7</v>
       </c>
-      <c r="D37" s="168" t="n">
+      <c r="D38" s="168" t="n">
         <v>7</v>
       </c>
-      <c r="E37" s="168" t="inlineStr"/>
-      <c r="F37" s="168" t="inlineStr"/>
-      <c r="G37" s="168" t="inlineStr"/>
-      <c r="H37" s="168" t="inlineStr"/>
-      <c r="I37" s="168" t="inlineStr"/>
-    </row>
-    <row r="38" ht="17" customHeight="1" s="143">
-      <c r="A38" s="169" t="n">
+      <c r="E38" s="168" t="inlineStr"/>
+      <c r="F38" s="168" t="inlineStr"/>
+      <c r="G38" s="168" t="inlineStr"/>
+      <c r="H38" s="168" t="inlineStr"/>
+      <c r="I38" s="168" t="inlineStr"/>
+    </row>
+    <row r="39" ht="17" customHeight="1" s="143">
+      <c r="A39" s="169" t="n">
         <v>33</v>
       </c>
-      <c r="B38" s="170" t="inlineStr">
+      <c r="B39" s="170" t="inlineStr">
         <is>
           <t>Tunisia</t>
         </is>
       </c>
-      <c r="C38" s="171" t="n">
+      <c r="C39" s="171" t="n">
         <v>7</v>
       </c>
-      <c r="D38" s="172" t="n">
+      <c r="D39" s="172" t="n">
         <v>7</v>
       </c>
-      <c r="E38" s="172" t="inlineStr"/>
-      <c r="F38" s="172" t="inlineStr"/>
-      <c r="G38" s="172" t="inlineStr"/>
-      <c r="H38" s="172" t="inlineStr"/>
-      <c r="I38" s="172" t="inlineStr"/>
-    </row>
-    <row r="39" ht="17" customHeight="1" s="143">
-      <c r="A39" s="165" t="n">
+      <c r="E39" s="172" t="inlineStr"/>
+      <c r="F39" s="172" t="inlineStr"/>
+      <c r="G39" s="172" t="inlineStr"/>
+      <c r="H39" s="172" t="inlineStr"/>
+      <c r="I39" s="172" t="inlineStr"/>
+    </row>
+    <row r="40" ht="17" customHeight="1" s="143">
+      <c r="A40" s="165" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="166" t="inlineStr">
+      <c r="B40" s="166" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
-      <c r="C39" s="167" t="n">
+      <c r="C40" s="167" t="n">
         <v>6</v>
       </c>
-      <c r="D39" s="168" t="n">
+      <c r="D40" s="168" t="n">
         <v>6</v>
       </c>
-      <c r="E39" s="168" t="inlineStr"/>
-      <c r="F39" s="168" t="inlineStr"/>
-      <c r="G39" s="168" t="inlineStr"/>
-      <c r="H39" s="168" t="inlineStr"/>
-      <c r="I39" s="168" t="inlineStr"/>
-    </row>
-    <row r="40" ht="17" customHeight="1" s="143">
-      <c r="A40" s="169" t="n">
+      <c r="E40" s="168" t="inlineStr"/>
+      <c r="F40" s="168" t="inlineStr"/>
+      <c r="G40" s="168" t="inlineStr"/>
+      <c r="H40" s="168" t="inlineStr"/>
+      <c r="I40" s="168" t="inlineStr"/>
+    </row>
+    <row r="41" ht="17" customHeight="1" s="143">
+      <c r="A41" s="169" t="n">
         <v>38</v>
       </c>
-      <c r="B40" s="170" t="inlineStr">
+      <c r="B41" s="170" t="inlineStr">
         <is>
           <t>Australia</t>
         </is>
       </c>
-      <c r="C40" s="171" t="n">
+      <c r="C41" s="171" t="n">
         <v>6</v>
       </c>
-      <c r="D40" s="172" t="n">
+      <c r="D41" s="172" t="n">
         <v>6</v>
       </c>
-      <c r="E40" s="172" t="inlineStr"/>
-      <c r="F40" s="172" t="inlineStr"/>
-      <c r="G40" s="172" t="inlineStr"/>
-      <c r="H40" s="172" t="inlineStr"/>
-      <c r="I40" s="172" t="inlineStr"/>
-    </row>
-    <row r="41" ht="17" customHeight="1" s="143">
-      <c r="A41" s="165" t="n">
+      <c r="E41" s="172" t="inlineStr"/>
+      <c r="F41" s="172" t="inlineStr"/>
+      <c r="G41" s="172" t="inlineStr"/>
+      <c r="H41" s="172" t="inlineStr"/>
+      <c r="I41" s="172" t="inlineStr"/>
+    </row>
+    <row r="42" ht="17" customHeight="1" s="143">
+      <c r="A42" s="165" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="166" t="inlineStr">
+      <c r="B42" s="166" t="inlineStr">
         <is>
           <t>Israel</t>
         </is>
       </c>
-      <c r="C41" s="167" t="n">
+      <c r="C42" s="167" t="n">
         <v>4</v>
       </c>
-      <c r="D41" s="168" t="n">
+      <c r="D42" s="168" t="n">
         <v>4</v>
       </c>
-      <c r="E41" s="168" t="inlineStr"/>
-      <c r="F41" s="168" t="inlineStr"/>
-      <c r="G41" s="168" t="inlineStr"/>
-      <c r="H41" s="168" t="inlineStr"/>
-      <c r="I41" s="168" t="inlineStr"/>
-    </row>
-    <row r="42" ht="17" customHeight="1" s="143">
-      <c r="A42" s="169" t="n">
+      <c r="E42" s="168" t="inlineStr"/>
+      <c r="F42" s="168" t="inlineStr"/>
+      <c r="G42" s="168" t="inlineStr"/>
+      <c r="H42" s="168" t="inlineStr"/>
+      <c r="I42" s="168" t="inlineStr"/>
+    </row>
+    <row r="43" ht="17" customHeight="1" s="143">
+      <c r="A43" s="169" t="n">
         <v>40</v>
       </c>
-      <c r="B42" s="170" t="inlineStr">
+      <c r="B43" s="170" t="inlineStr">
         <is>
           <t>Malaysia</t>
         </is>
       </c>
-      <c r="C42" s="171" t="n">
+      <c r="C43" s="171" t="n">
         <v>4</v>
       </c>
-      <c r="D42" s="172" t="n">
+      <c r="D43" s="172" t="n">
         <v>4</v>
       </c>
-      <c r="E42" s="172" t="inlineStr"/>
-      <c r="F42" s="172" t="inlineStr"/>
-      <c r="G42" s="172" t="inlineStr"/>
-      <c r="H42" s="172" t="inlineStr"/>
-      <c r="I42" s="172" t="inlineStr"/>
-    </row>
-    <row r="43" ht="17" customHeight="1" s="143">
-      <c r="A43" s="165" t="n">
+      <c r="E43" s="172" t="inlineStr"/>
+      <c r="F43" s="172" t="inlineStr"/>
+      <c r="G43" s="172" t="inlineStr"/>
+      <c r="H43" s="172" t="inlineStr"/>
+      <c r="I43" s="172" t="inlineStr"/>
+    </row>
+    <row r="44" ht="17" customHeight="1" s="143">
+      <c r="A44" s="165" t="n">
         <v>40</v>
       </c>
-      <c r="B43" s="166" t="inlineStr">
+      <c r="B44" s="166" t="inlineStr">
         <is>
           <t>Sverige</t>
         </is>
       </c>
-      <c r="C43" s="167" t="n">
+      <c r="C44" s="167" t="n">
         <v>4</v>
       </c>
-      <c r="D43" s="168" t="n">
+      <c r="D44" s="168" t="n">
         <v>3</v>
       </c>
-      <c r="E43" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="168" t="inlineStr"/>
-      <c r="G43" s="168" t="inlineStr"/>
-      <c r="H43" s="168" t="inlineStr"/>
-      <c r="I43" s="168" t="inlineStr"/>
-    </row>
-    <row r="44" ht="17" customHeight="1" s="143">
-      <c r="A44" s="169" t="n">
+      <c r="E44" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="168" t="inlineStr"/>
+      <c r="G44" s="168" t="inlineStr"/>
+      <c r="H44" s="168" t="inlineStr"/>
+      <c r="I44" s="168" t="inlineStr"/>
+    </row>
+    <row r="45" ht="17" customHeight="1" s="143">
+      <c r="A45" s="169" t="n">
         <v>40</v>
       </c>
-      <c r="B44" s="170" t="inlineStr">
+      <c r="B45" s="170" t="inlineStr">
         <is>
           <t>Aserbajdsjan</t>
         </is>
       </c>
-      <c r="C44" s="171" t="n">
+      <c r="C45" s="171" t="n">
         <v>4</v>
       </c>
-      <c r="D44" s="172" t="n">
+      <c r="D45" s="172" t="n">
         <v>4</v>
       </c>
-      <c r="E44" s="172" t="inlineStr"/>
-      <c r="F44" s="172" t="inlineStr"/>
-      <c r="G44" s="172" t="inlineStr"/>
-      <c r="H44" s="172" t="inlineStr"/>
-      <c r="I44" s="172" t="inlineStr"/>
-    </row>
-    <row r="45" ht="17" customHeight="1" s="143">
-      <c r="A45" s="165" t="n">
+      <c r="E45" s="172" t="inlineStr"/>
+      <c r="F45" s="172" t="inlineStr"/>
+      <c r="G45" s="172" t="inlineStr"/>
+      <c r="H45" s="172" t="inlineStr"/>
+      <c r="I45" s="172" t="inlineStr"/>
+    </row>
+    <row r="46" ht="17" customHeight="1" s="143">
+      <c r="A46" s="165" t="n">
         <v>40</v>
       </c>
-      <c r="B45" s="166" t="inlineStr">
+      <c r="B46" s="166" t="inlineStr">
         <is>
           <t>Chile</t>
         </is>
       </c>
-      <c r="C45" s="167" t="n">
+      <c r="C46" s="167" t="n">
         <v>4</v>
       </c>
-      <c r="D45" s="168" t="n">
+      <c r="D46" s="168" t="n">
         <v>4</v>
       </c>
-      <c r="E45" s="168" t="inlineStr"/>
-      <c r="F45" s="168" t="inlineStr"/>
-      <c r="G45" s="168" t="inlineStr"/>
-      <c r="H45" s="168" t="inlineStr"/>
-      <c r="I45" s="168" t="inlineStr"/>
-    </row>
-    <row r="46" ht="17" customHeight="1" s="143">
-      <c r="A46" s="169" t="n">
+      <c r="E46" s="168" t="inlineStr"/>
+      <c r="F46" s="168" t="inlineStr"/>
+      <c r="G46" s="168" t="inlineStr"/>
+      <c r="H46" s="168" t="inlineStr"/>
+      <c r="I46" s="168" t="inlineStr"/>
+    </row>
+    <row r="47" ht="17" customHeight="1" s="143">
+      <c r="A47" s="169" t="n">
         <v>45</v>
       </c>
-      <c r="B46" s="170" t="inlineStr">
+      <c r="B47" s="170" t="inlineStr">
         <is>
           <t>Marokko</t>
         </is>
       </c>
-      <c r="C46" s="171" t="n">
+      <c r="C47" s="171" t="n">
         <v>3</v>
       </c>
-      <c r="D46" s="172" t="n">
+      <c r="D47" s="172" t="n">
         <v>3</v>
       </c>
-      <c r="E46" s="172" t="inlineStr"/>
-      <c r="F46" s="172" t="inlineStr"/>
-      <c r="G46" s="172" t="inlineStr"/>
-      <c r="H46" s="172" t="inlineStr"/>
-      <c r="I46" s="172" t="inlineStr"/>
-    </row>
-    <row r="47" ht="17" customHeight="1" s="143">
-      <c r="A47" s="165" t="n">
+      <c r="E47" s="172" t="inlineStr"/>
+      <c r="F47" s="172" t="inlineStr"/>
+      <c r="G47" s="172" t="inlineStr"/>
+      <c r="H47" s="172" t="inlineStr"/>
+      <c r="I47" s="172" t="inlineStr"/>
+    </row>
+    <row r="48" ht="17" customHeight="1" s="143">
+      <c r="A48" s="165" t="n">
         <v>45</v>
       </c>
-      <c r="B47" s="166" t="inlineStr">
+      <c r="B48" s="166" t="inlineStr">
         <is>
           <t>Ungarn</t>
         </is>
       </c>
-      <c r="C47" s="167" t="n">
+      <c r="C48" s="167" t="n">
         <v>3</v>
       </c>
-      <c r="D47" s="168" t="n">
+      <c r="D48" s="168" t="n">
         <v>3</v>
       </c>
-      <c r="E47" s="168" t="inlineStr"/>
-      <c r="F47" s="168" t="inlineStr"/>
-      <c r="G47" s="168" t="inlineStr"/>
-      <c r="H47" s="168" t="inlineStr"/>
-      <c r="I47" s="168" t="inlineStr"/>
-    </row>
-    <row r="48" ht="17" customHeight="1" s="143">
-      <c r="A48" s="169" t="n">
+      <c r="E48" s="168" t="inlineStr"/>
+      <c r="F48" s="168" t="inlineStr"/>
+      <c r="G48" s="168" t="inlineStr"/>
+      <c r="H48" s="168" t="inlineStr"/>
+      <c r="I48" s="168" t="inlineStr"/>
+    </row>
+    <row r="49" ht="17" customHeight="1" s="143">
+      <c r="A49" s="169" t="n">
         <v>45</v>
       </c>
-      <c r="B48" s="170" t="inlineStr">
+      <c r="B49" s="170" t="inlineStr">
         <is>
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="C48" s="171" t="n">
+      <c r="C49" s="171" t="n">
         <v>3</v>
       </c>
-      <c r="D48" s="172" t="n">
+      <c r="D49" s="172" t="n">
         <v>3</v>
       </c>
-      <c r="E48" s="172" t="inlineStr"/>
-      <c r="F48" s="172" t="inlineStr"/>
-      <c r="G48" s="172" t="inlineStr"/>
-      <c r="H48" s="172" t="inlineStr"/>
-      <c r="I48" s="172" t="inlineStr"/>
-    </row>
-    <row r="49" ht="17" customHeight="1" s="143">
-      <c r="A49" s="165" t="n">
+      <c r="E49" s="172" t="inlineStr"/>
+      <c r="F49" s="172" t="inlineStr"/>
+      <c r="G49" s="172" t="inlineStr"/>
+      <c r="H49" s="172" t="inlineStr"/>
+      <c r="I49" s="172" t="inlineStr"/>
+    </row>
+    <row r="50" ht="17" customHeight="1" s="143">
+      <c r="A50" s="165" t="n">
         <v>45</v>
       </c>
-      <c r="B49" s="166" t="inlineStr">
+      <c r="B50" s="166" t="inlineStr">
         <is>
           <t>Algerie</t>
         </is>
       </c>
-      <c r="C49" s="167" t="n">
+      <c r="C50" s="167" t="n">
         <v>3</v>
       </c>
-      <c r="D49" s="168" t="n">
+      <c r="D50" s="168" t="n">
         <v>3</v>
       </c>
-      <c r="E49" s="168" t="inlineStr"/>
-      <c r="F49" s="168" t="inlineStr"/>
-      <c r="G49" s="168" t="inlineStr"/>
-      <c r="H49" s="168" t="inlineStr"/>
-      <c r="I49" s="168" t="inlineStr"/>
-    </row>
-    <row r="50" ht="17" customHeight="1" s="143">
-      <c r="A50" s="169" t="n">
+      <c r="E50" s="168" t="inlineStr"/>
+      <c r="F50" s="168" t="inlineStr"/>
+      <c r="G50" s="168" t="inlineStr"/>
+      <c r="H50" s="168" t="inlineStr"/>
+      <c r="I50" s="168" t="inlineStr"/>
+    </row>
+    <row r="51" ht="17" customHeight="1" s="143">
+      <c r="A51" s="169" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="170" t="inlineStr">
+      <c r="B51" s="170" t="inlineStr">
         <is>
           <t>Romania</t>
         </is>
       </c>
-      <c r="C50" s="171" t="n">
+      <c r="C51" s="171" t="n">
         <v>2</v>
       </c>
-      <c r="D50" s="172" t="n">
+      <c r="D51" s="172" t="n">
         <v>2</v>
       </c>
-      <c r="E50" s="172" t="inlineStr"/>
-      <c r="F50" s="172" t="inlineStr"/>
-      <c r="G50" s="172" t="inlineStr"/>
-      <c r="H50" s="172" t="inlineStr"/>
-      <c r="I50" s="172" t="inlineStr"/>
-    </row>
-    <row r="51" ht="17" customHeight="1" s="143">
-      <c r="A51" s="165" t="n">
+      <c r="E51" s="172" t="inlineStr"/>
+      <c r="F51" s="172" t="inlineStr"/>
+      <c r="G51" s="172" t="inlineStr"/>
+      <c r="H51" s="172" t="inlineStr"/>
+      <c r="I51" s="172" t="inlineStr"/>
+    </row>
+    <row r="52" ht="17" customHeight="1" s="143">
+      <c r="A52" s="165" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="166" t="inlineStr">
+      <c r="B52" s="166" t="inlineStr">
         <is>
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="C51" s="167" t="n">
+      <c r="C52" s="167" t="n">
         <v>2</v>
       </c>
-      <c r="D51" s="168" t="n">
+      <c r="D52" s="168" t="n">
         <v>2</v>
       </c>
-      <c r="E51" s="168" t="inlineStr"/>
-      <c r="F51" s="168" t="inlineStr"/>
-      <c r="G51" s="168" t="inlineStr"/>
-      <c r="H51" s="168" t="inlineStr"/>
-      <c r="I51" s="168" t="inlineStr"/>
-    </row>
-    <row r="52" ht="17" customHeight="1" s="143">
-      <c r="A52" s="169" t="n">
+      <c r="E52" s="168" t="inlineStr"/>
+      <c r="F52" s="168" t="inlineStr"/>
+      <c r="G52" s="168" t="inlineStr"/>
+      <c r="H52" s="168" t="inlineStr"/>
+      <c r="I52" s="168" t="inlineStr"/>
+    </row>
+    <row r="53" ht="17" customHeight="1" s="143">
+      <c r="A53" s="169" t="n">
         <v>49</v>
       </c>
-      <c r="B52" s="170" t="inlineStr">
+      <c r="B53" s="170" t="inlineStr">
         <is>
           <t>Slovakia</t>
         </is>
       </c>
-      <c r="C52" s="171" t="n">
+      <c r="C53" s="171" t="n">
         <v>2</v>
       </c>
-      <c r="D52" s="172" t="n">
+      <c r="D53" s="172" t="n">
         <v>2</v>
       </c>
-      <c r="E52" s="172" t="inlineStr"/>
-      <c r="F52" s="172" t="inlineStr"/>
-      <c r="G52" s="172" t="inlineStr"/>
-      <c r="H52" s="172" t="inlineStr"/>
-      <c r="I52" s="172" t="inlineStr"/>
-    </row>
-    <row r="53" ht="17" customHeight="1" s="143">
-      <c r="A53" s="165" t="n">
+      <c r="E53" s="172" t="inlineStr"/>
+      <c r="F53" s="172" t="inlineStr"/>
+      <c r="G53" s="172" t="inlineStr"/>
+      <c r="H53" s="172" t="inlineStr"/>
+      <c r="I53" s="172" t="inlineStr"/>
+    </row>
+    <row r="54" ht="17" customHeight="1" s="143">
+      <c r="A54" s="165" t="n">
         <v>49</v>
       </c>
-      <c r="B53" s="166" t="inlineStr">
+      <c r="B54" s="166" t="inlineStr">
         <is>
           <t>Slovenia</t>
         </is>
       </c>
-      <c r="C53" s="167" t="n">
+      <c r="C54" s="167" t="n">
         <v>2</v>
       </c>
-      <c r="D53" s="168" t="n">
+      <c r="D54" s="168" t="n">
         <v>2</v>
       </c>
-      <c r="E53" s="168" t="inlineStr"/>
-      <c r="F53" s="168" t="inlineStr"/>
-      <c r="G53" s="168" t="inlineStr"/>
-      <c r="H53" s="168" t="inlineStr"/>
-      <c r="I53" s="168" t="inlineStr"/>
-    </row>
-    <row r="54" ht="17" customHeight="1" s="143">
-      <c r="A54" s="169" t="n">
+      <c r="E54" s="168" t="inlineStr"/>
+      <c r="F54" s="168" t="inlineStr"/>
+      <c r="G54" s="168" t="inlineStr"/>
+      <c r="H54" s="168" t="inlineStr"/>
+      <c r="I54" s="168" t="inlineStr"/>
+    </row>
+    <row r="55" ht="17" customHeight="1" s="143">
+      <c r="A55" s="169" t="n">
         <v>49</v>
       </c>
-      <c r="B54" s="170" t="inlineStr">
+      <c r="B55" s="170" t="inlineStr">
         <is>
           <t>Irland</t>
         </is>
       </c>
-      <c r="C54" s="171" t="n">
+      <c r="C55" s="171" t="n">
         <v>2</v>
       </c>
-      <c r="D54" s="172" t="n">
+      <c r="D55" s="172" t="n">
         <v>2</v>
       </c>
-      <c r="E54" s="172" t="inlineStr"/>
-      <c r="F54" s="172" t="inlineStr"/>
-      <c r="G54" s="172" t="inlineStr"/>
-      <c r="H54" s="172" t="inlineStr"/>
-      <c r="I54" s="172" t="inlineStr"/>
-    </row>
-    <row r="55" ht="17" customHeight="1" s="143">
-      <c r="A55" s="165" t="n">
+      <c r="E55" s="172" t="inlineStr"/>
+      <c r="F55" s="172" t="inlineStr"/>
+      <c r="G55" s="172" t="inlineStr"/>
+      <c r="H55" s="172" t="inlineStr"/>
+      <c r="I55" s="172" t="inlineStr"/>
+    </row>
+    <row r="56" ht="17" customHeight="1" s="143">
+      <c r="A56" s="165" t="n">
         <v>49</v>
       </c>
-      <c r="B55" s="166" t="inlineStr">
+      <c r="B56" s="166" t="inlineStr">
         <is>
           <t>Bulgaria</t>
         </is>
       </c>
-      <c r="C55" s="167" t="n">
+      <c r="C56" s="167" t="n">
         <v>2</v>
       </c>
-      <c r="D55" s="168" t="n">
+      <c r="D56" s="168" t="n">
         <v>2</v>
       </c>
-      <c r="E55" s="168" t="inlineStr"/>
-      <c r="F55" s="168" t="inlineStr"/>
-      <c r="G55" s="168" t="inlineStr"/>
-      <c r="H55" s="168" t="inlineStr"/>
-      <c r="I55" s="168" t="inlineStr"/>
-    </row>
-    <row r="56" ht="17" customHeight="1" s="143">
-      <c r="A56" s="169" t="n">
+      <c r="E56" s="168" t="inlineStr"/>
+      <c r="F56" s="168" t="inlineStr"/>
+      <c r="G56" s="168" t="inlineStr"/>
+      <c r="H56" s="168" t="inlineStr"/>
+      <c r="I56" s="168" t="inlineStr"/>
+    </row>
+    <row r="57" ht="17" customHeight="1" s="143">
+      <c r="A57" s="169" t="n">
         <v>49</v>
       </c>
-      <c r="B56" s="170" t="inlineStr">
+      <c r="B57" s="170" t="inlineStr">
         <is>
           <t>Costa Rica</t>
         </is>
       </c>
-      <c r="C56" s="171" t="n">
+      <c r="C57" s="171" t="n">
         <v>2</v>
       </c>
-      <c r="D56" s="172" t="n">
+      <c r="D57" s="172" t="n">
         <v>2</v>
       </c>
-      <c r="E56" s="172" t="inlineStr"/>
-      <c r="F56" s="172" t="inlineStr"/>
-      <c r="G56" s="172" t="inlineStr"/>
-      <c r="H56" s="172" t="inlineStr"/>
-      <c r="I56" s="172" t="inlineStr"/>
-    </row>
-    <row r="57" ht="17" customHeight="1" s="143">
-      <c r="A57" s="165" t="n">
+      <c r="E57" s="172" t="inlineStr"/>
+      <c r="F57" s="172" t="inlineStr"/>
+      <c r="G57" s="172" t="inlineStr"/>
+      <c r="H57" s="172" t="inlineStr"/>
+      <c r="I57" s="172" t="inlineStr"/>
+    </row>
+    <row r="58" ht="17" customHeight="1" s="143">
+      <c r="A58" s="165" t="n">
         <v>49</v>
       </c>
-      <c r="B57" s="166" t="inlineStr">
+      <c r="B58" s="166" t="inlineStr">
         <is>
           <t>Venezuela</t>
         </is>
       </c>
-      <c r="C57" s="167" t="n">
+      <c r="C58" s="167" t="n">
         <v>2</v>
       </c>
-      <c r="D57" s="168" t="n">
+      <c r="D58" s="168" t="n">
         <v>2</v>
       </c>
-      <c r="E57" s="168" t="inlineStr"/>
-      <c r="F57" s="168" t="inlineStr"/>
-      <c r="G57" s="168" t="inlineStr"/>
-      <c r="H57" s="168" t="inlineStr"/>
-      <c r="I57" s="168" t="inlineStr"/>
-    </row>
-    <row r="58" ht="17" customHeight="1" s="143">
-      <c r="A58" s="169" t="n">
+      <c r="E58" s="168" t="inlineStr"/>
+      <c r="F58" s="168" t="inlineStr"/>
+      <c r="G58" s="168" t="inlineStr"/>
+      <c r="H58" s="168" t="inlineStr"/>
+      <c r="I58" s="168" t="inlineStr"/>
+    </row>
+    <row r="59" ht="17" customHeight="1" s="143">
+      <c r="A59" s="169" t="n">
         <v>49</v>
       </c>
-      <c r="B58" s="170" t="inlineStr">
+      <c r="B59" s="170" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
-      <c r="C58" s="171" t="n">
+      <c r="C59" s="171" t="n">
         <v>2</v>
       </c>
-      <c r="D58" s="172" t="n">
+      <c r="D59" s="172" t="n">
         <v>2</v>
       </c>
-      <c r="E58" s="172" t="inlineStr"/>
-      <c r="F58" s="172" t="inlineStr"/>
-      <c r="G58" s="172" t="inlineStr"/>
-      <c r="H58" s="172" t="inlineStr"/>
-      <c r="I58" s="172" t="inlineStr"/>
-    </row>
-    <row r="59" ht="17" customHeight="1" s="143">
-      <c r="A59" s="165" t="n">
+      <c r="E59" s="172" t="inlineStr"/>
+      <c r="F59" s="172" t="inlineStr"/>
+      <c r="G59" s="172" t="inlineStr"/>
+      <c r="H59" s="172" t="inlineStr"/>
+      <c r="I59" s="172" t="inlineStr"/>
+    </row>
+    <row r="60" ht="17" customHeight="1" s="143">
+      <c r="A60" s="165" t="n">
         <v>58</v>
       </c>
-      <c r="B59" s="166" t="inlineStr">
+      <c r="B60" s="166" t="inlineStr">
         <is>
           <t>Bosnia og Hercegovina</t>
         </is>
       </c>
-      <c r="C59" s="167" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="E59" s="168" t="inlineStr"/>
-      <c r="F59" s="168" t="inlineStr"/>
-      <c r="G59" s="168" t="inlineStr"/>
-      <c r="H59" s="168" t="inlineStr"/>
-      <c r="I59" s="168" t="inlineStr"/>
-    </row>
-    <row r="60" ht="17" customHeight="1" s="143">
-      <c r="A60" s="169" t="n">
+      <c r="C60" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E60" s="168" t="inlineStr"/>
+      <c r="F60" s="168" t="inlineStr"/>
+      <c r="G60" s="168" t="inlineStr"/>
+      <c r="H60" s="168" t="inlineStr"/>
+      <c r="I60" s="168" t="inlineStr"/>
+    </row>
+    <row r="61" ht="17" customHeight="1" s="143">
+      <c r="A61" s="169" t="n">
         <v>58</v>
       </c>
-      <c r="B60" s="170" t="inlineStr">
+      <c r="B61" s="170" t="inlineStr">
         <is>
           <t>Kasakhstan</t>
         </is>
       </c>
-      <c r="C60" s="171" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="E60" s="172" t="inlineStr"/>
-      <c r="F60" s="172" t="inlineStr"/>
-      <c r="G60" s="172" t="inlineStr"/>
-      <c r="H60" s="172" t="inlineStr"/>
-      <c r="I60" s="172" t="inlineStr"/>
-    </row>
-    <row r="61" ht="17" customHeight="1" s="143">
-      <c r="A61" s="165" t="n">
+      <c r="C61" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D61" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E61" s="172" t="inlineStr"/>
+      <c r="F61" s="172" t="inlineStr"/>
+      <c r="G61" s="172" t="inlineStr"/>
+      <c r="H61" s="172" t="inlineStr"/>
+      <c r="I61" s="172" t="inlineStr"/>
+    </row>
+    <row r="62" ht="17" customHeight="1" s="143">
+      <c r="A62" s="165" t="n">
         <v>58</v>
       </c>
-      <c r="B61" s="166" t="inlineStr">
+      <c r="B62" s="166" t="inlineStr">
         <is>
           <t>Finland</t>
         </is>
       </c>
-      <c r="C61" s="167" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="E61" s="168" t="inlineStr"/>
-      <c r="F61" s="168" t="inlineStr"/>
-      <c r="G61" s="168" t="inlineStr"/>
-      <c r="H61" s="168" t="inlineStr"/>
-      <c r="I61" s="168" t="inlineStr"/>
-    </row>
-    <row r="62" ht="17" customHeight="1" s="143">
-      <c r="A62" s="169" t="n">
+      <c r="C62" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D62" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="168" t="inlineStr"/>
+      <c r="F62" s="168" t="inlineStr"/>
+      <c r="G62" s="168" t="inlineStr"/>
+      <c r="H62" s="168" t="inlineStr"/>
+      <c r="I62" s="168" t="inlineStr"/>
+    </row>
+    <row r="63" ht="17" customHeight="1" s="143">
+      <c r="A63" s="169" t="n">
         <v>58</v>
       </c>
-      <c r="B62" s="170" t="inlineStr">
+      <c r="B63" s="170" t="inlineStr">
         <is>
           <t>Thailand</t>
         </is>
       </c>
-      <c r="C62" s="171" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="E62" s="172" t="inlineStr"/>
-      <c r="F62" s="172" t="inlineStr"/>
-      <c r="G62" s="172" t="inlineStr"/>
-      <c r="H62" s="172" t="inlineStr"/>
-      <c r="I62" s="172" t="inlineStr"/>
-    </row>
-    <row r="63" ht="17" customHeight="1" s="143">
-      <c r="A63" s="165" t="n">
+      <c r="C63" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D63" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E63" s="172" t="inlineStr"/>
+      <c r="F63" s="172" t="inlineStr"/>
+      <c r="G63" s="172" t="inlineStr"/>
+      <c r="H63" s="172" t="inlineStr"/>
+      <c r="I63" s="172" t="inlineStr"/>
+    </row>
+    <row r="64" ht="17" customHeight="1" s="143">
+      <c r="A64" s="165" t="n">
         <v>58</v>
       </c>
-      <c r="B63" s="166" t="inlineStr">
+      <c r="B64" s="166" t="inlineStr">
         <is>
           <t>Indonesia</t>
         </is>
       </c>
-      <c r="C63" s="167" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="E63" s="168" t="inlineStr"/>
-      <c r="F63" s="168" t="inlineStr"/>
-      <c r="G63" s="168" t="inlineStr"/>
-      <c r="H63" s="168" t="inlineStr"/>
-      <c r="I63" s="168" t="inlineStr"/>
-    </row>
-    <row r="64" ht="17" customHeight="1" s="143">
-      <c r="A64" s="169" t="n">
+      <c r="C64" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D64" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E64" s="168" t="inlineStr"/>
+      <c r="F64" s="168" t="inlineStr"/>
+      <c r="G64" s="168" t="inlineStr"/>
+      <c r="H64" s="168" t="inlineStr"/>
+      <c r="I64" s="168" t="inlineStr"/>
+    </row>
+    <row r="65" ht="17" customHeight="1" s="143">
+      <c r="A65" s="169" t="n">
         <v>58</v>
       </c>
-      <c r="B64" s="170" t="inlineStr">
+      <c r="B65" s="170" t="inlineStr">
         <is>
           <t>Serbia</t>
         </is>
       </c>
-      <c r="C64" s="171" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="E64" s="172" t="inlineStr"/>
-      <c r="F64" s="172" t="inlineStr"/>
-      <c r="G64" s="172" t="inlineStr"/>
-      <c r="H64" s="172" t="inlineStr"/>
-      <c r="I64" s="172" t="inlineStr"/>
-    </row>
-    <row r="65" ht="17" customHeight="1" s="143">
-      <c r="A65" s="165" t="n">
+      <c r="C65" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D65" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E65" s="172" t="inlineStr"/>
+      <c r="F65" s="172" t="inlineStr"/>
+      <c r="G65" s="172" t="inlineStr"/>
+      <c r="H65" s="172" t="inlineStr"/>
+      <c r="I65" s="172" t="inlineStr"/>
+    </row>
+    <row r="66" ht="17" customHeight="1" s="143">
+      <c r="A66" s="165" t="n">
         <v>58</v>
       </c>
-      <c r="B65" s="166" t="inlineStr">
+      <c r="B66" s="166" t="inlineStr">
         <is>
           <t>Armenia</t>
         </is>
       </c>
-      <c r="C65" s="167" t="n">
-        <v>1</v>
-      </c>
-      <c r="D65" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="E65" s="168" t="inlineStr"/>
-      <c r="F65" s="168" t="inlineStr"/>
-      <c r="G65" s="168" t="inlineStr"/>
-      <c r="H65" s="168" t="inlineStr"/>
-      <c r="I65" s="168" t="inlineStr"/>
-    </row>
-    <row r="66" ht="17" customHeight="1" s="143">
-      <c r="A66" s="169" t="n">
+      <c r="C66" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D66" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E66" s="168" t="inlineStr"/>
+      <c r="F66" s="168" t="inlineStr"/>
+      <c r="G66" s="168" t="inlineStr"/>
+      <c r="H66" s="168" t="inlineStr"/>
+      <c r="I66" s="168" t="inlineStr"/>
+    </row>
+    <row r="67" ht="17" customHeight="1" s="143">
+      <c r="A67" s="169" t="n">
         <v>58</v>
       </c>
-      <c r="B66" s="170" t="inlineStr">
+      <c r="B67" s="170" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
-      <c r="C66" s="171" t="n">
-        <v>1</v>
-      </c>
-      <c r="D66" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="E66" s="172" t="inlineStr"/>
-      <c r="F66" s="172" t="inlineStr"/>
-      <c r="G66" s="172" t="inlineStr"/>
-      <c r="H66" s="172" t="inlineStr"/>
-      <c r="I66" s="172" t="inlineStr"/>
-    </row>
-    <row r="67" ht="17" customHeight="1" s="143">
-      <c r="A67" s="165" t="n">
+      <c r="C67" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D67" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E67" s="172" t="inlineStr"/>
+      <c r="F67" s="172" t="inlineStr"/>
+      <c r="G67" s="172" t="inlineStr"/>
+      <c r="H67" s="172" t="inlineStr"/>
+      <c r="I67" s="172" t="inlineStr"/>
+    </row>
+    <row r="68" ht="17" customHeight="1" s="143">
+      <c r="A68" s="165" t="n">
         <v>58</v>
       </c>
-      <c r="B67" s="166" t="inlineStr">
+      <c r="B68" s="166" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C67" s="167" t="n">
-        <v>1</v>
-      </c>
-      <c r="D67" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="E67" s="168" t="inlineStr"/>
-      <c r="F67" s="168" t="inlineStr"/>
-      <c r="G67" s="168" t="inlineStr"/>
-      <c r="H67" s="168" t="inlineStr"/>
-      <c r="I67" s="168" t="inlineStr"/>
-    </row>
-    <row r="68" ht="17" customHeight="1" s="143">
-      <c r="A68" s="169" t="n">
+      <c r="C68" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D68" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="168" t="inlineStr"/>
+      <c r="F68" s="168" t="inlineStr"/>
+      <c r="G68" s="168" t="inlineStr"/>
+      <c r="H68" s="168" t="inlineStr"/>
+      <c r="I68" s="168" t="inlineStr"/>
+    </row>
+    <row r="69" ht="17" customHeight="1" s="143">
+      <c r="A69" s="169" t="n">
         <v>58</v>
       </c>
-      <c r="B68" s="170" t="inlineStr">
+      <c r="B69" s="170" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="C68" s="171" t="n">
-        <v>1</v>
-      </c>
-      <c r="D68" s="172" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" s="172" t="inlineStr"/>
-      <c r="F68" s="172" t="inlineStr"/>
-      <c r="G68" s="172" t="inlineStr"/>
-      <c r="H68" s="172" t="inlineStr"/>
-      <c r="I68" s="172" t="inlineStr"/>
-    </row>
-    <row r="69" ht="17" customHeight="1" s="143">
-      <c r="A69" s="165" t="n">
+      <c r="C69" s="171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D69" s="172" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="172" t="inlineStr"/>
+      <c r="F69" s="172" t="inlineStr"/>
+      <c r="G69" s="172" t="inlineStr"/>
+      <c r="H69" s="172" t="inlineStr"/>
+      <c r="I69" s="172" t="inlineStr"/>
+    </row>
+    <row r="70" ht="17" customHeight="1" s="143">
+      <c r="A70" s="165" t="n">
         <v>58</v>
       </c>
-      <c r="B69" s="166" t="inlineStr">
+      <c r="B70" s="166" t="inlineStr">
         <is>
           <t>Honduras</t>
         </is>
       </c>
-      <c r="C69" s="167" t="n">
-        <v>1</v>
-      </c>
-      <c r="D69" s="168" t="n">
-        <v>1</v>
-      </c>
-      <c r="E69" s="168" t="inlineStr"/>
-      <c r="F69" s="168" t="inlineStr"/>
-      <c r="G69" s="168" t="inlineStr"/>
-      <c r="H69" s="168" t="inlineStr"/>
-      <c r="I69" s="168" t="inlineStr"/>
+      <c r="C70" s="167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D70" s="168" t="n">
+        <v>1</v>
+      </c>
+      <c r="E70" s="168" t="inlineStr"/>
+      <c r="F70" s="168" t="inlineStr"/>
+      <c r="G70" s="168" t="inlineStr"/>
+      <c r="H70" s="168" t="inlineStr"/>
+      <c r="I70" s="168" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I1"/>
+  <autoFilter ref="A2:I2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:I1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Nivå 2 og lavere: Calibri 10pt, bunnkant-only, konsistent med øvrige ark
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -28,13 +28,13 @@
     <sheet name="Klubber" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
     <sheet name="Alder" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Nivå 2 og lavere" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Spillere etter klubbland" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Spillere etter klubbland" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Nivå 2 og lavere" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Klubber'!$A$2:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Nivå 2 og lavere'!$A$2:$F$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'Nivå 2 og lavere'!$A$2:$F$2</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -817,7 +817,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="188">
+  <cellXfs count="202">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1340,6 +1340,36 @@
     <xf numFmtId="0" fontId="45" fillId="44" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="47" fillId="51" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="51" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="52" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="52" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="53" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="53" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="54" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="47" fillId="54" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="51" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="52" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="53" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="55" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="47" fillId="54" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -50065,1943 +50095,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F70"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="8" customWidth="1" style="143" min="1" max="1"/>
-    <col width="26" customWidth="1" style="143" min="2" max="2"/>
-    <col width="16" customWidth="1" style="143" min="3" max="3"/>
-    <col width="22" customWidth="1" style="143" min="4" max="4"/>
-    <col width="30" customWidth="1" style="143" min="5" max="5"/>
-    <col width="22" customWidth="1" style="143" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" s="143">
-      <c r="A1" s="150" t="inlineStr">
-        <is>
-          <t>VM 2026 — Spillere på nivå 2 og lavere   61 spillere</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" s="143">
-      <c r="A2" s="187" t="inlineStr">
-        <is>
-          <t>Nivå</t>
-        </is>
-      </c>
-      <c r="B2" s="187" t="inlineStr">
-        <is>
-          <t>Klubb</t>
-        </is>
-      </c>
-      <c r="C2" s="187" t="inlineStr">
-        <is>
-          <t>Land</t>
-        </is>
-      </c>
-      <c r="D2" s="187" t="inlineStr">
-        <is>
-          <t>Liga</t>
-        </is>
-      </c>
-      <c r="E2" s="187" t="inlineStr">
-        <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="F2" s="187" t="inlineStr">
-        <is>
-          <t>Nasjonallag</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="175" t="inlineStr">
-        <is>
-          <t>Charlton Athletic</t>
-        </is>
-      </c>
-      <c r="C3" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D3" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E3" s="175" t="inlineStr">
-        <is>
-          <t>Lyndon Dykes</t>
-        </is>
-      </c>
-      <c r="F3" s="175" t="inlineStr">
-        <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B4" s="175" t="inlineStr">
-        <is>
-          <t>Coventry City</t>
-        </is>
-      </c>
-      <c r="C4" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D4" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E4" s="175" t="inlineStr">
-        <is>
-          <t>Brandon Thomas-Asante</t>
-        </is>
-      </c>
-      <c r="F4" s="175" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B5" s="175" t="inlineStr">
-        <is>
-          <t>Coventry City</t>
-        </is>
-      </c>
-      <c r="C5" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D5" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E5" s="175" t="inlineStr">
-        <is>
-          <t>Haji Wright</t>
-        </is>
-      </c>
-      <c r="F5" s="175" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B6" s="175" t="inlineStr">
-        <is>
-          <t>Derby County</t>
-        </is>
-      </c>
-      <c r="C6" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D6" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E6" s="175" t="inlineStr">
-        <is>
-          <t>Jacob Widell Zetterström</t>
-        </is>
-      </c>
-      <c r="F6" s="175" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="175" t="inlineStr">
-        <is>
-          <t>Derby County</t>
-        </is>
-      </c>
-      <c r="C7" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D7" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E7" s="175" t="inlineStr">
-        <is>
-          <t>Sondre Langås</t>
-        </is>
-      </c>
-      <c r="F7" s="175" t="inlineStr">
-        <is>
-          <t>Norge</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B8" s="175" t="inlineStr">
-        <is>
-          <t>Hull City</t>
-        </is>
-      </c>
-      <c r="C8" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D8" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E8" s="175" t="inlineStr">
-        <is>
-          <t>Amir Hadžiahmetović</t>
-        </is>
-      </c>
-      <c r="F8" s="175" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B9" s="175" t="inlineStr">
-        <is>
-          <t>Hull City</t>
-        </is>
-      </c>
-      <c r="C9" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D9" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E9" s="175" t="inlineStr">
-        <is>
-          <t>Ivor Pandur</t>
-        </is>
-      </c>
-      <c r="F9" s="175" t="inlineStr">
-        <is>
-          <t>Kroatia</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B10" s="175" t="inlineStr">
-        <is>
-          <t>Hull City</t>
-        </is>
-      </c>
-      <c r="C10" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D10" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E10" s="175" t="inlineStr">
-        <is>
-          <t>Liam Miller</t>
-        </is>
-      </c>
-      <c r="F10" s="175" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B11" s="175" t="inlineStr">
-        <is>
-          <t>Middlesbrough</t>
-        </is>
-      </c>
-      <c r="C11" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D11" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E11" s="175" t="inlineStr">
-        <is>
-          <t>Alfie Jones</t>
-        </is>
-      </c>
-      <c r="F11" s="175" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B12" s="175" t="inlineStr">
-        <is>
-          <t>Middlesbrough</t>
-        </is>
-      </c>
-      <c r="C12" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D12" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E12" s="175" t="inlineStr">
-        <is>
-          <t>Sontje Hansen</t>
-        </is>
-      </c>
-      <c r="F12" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B13" s="175" t="inlineStr">
-        <is>
-          <t>Millwall FC</t>
-        </is>
-      </c>
-      <c r="C13" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D13" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E13" s="175" t="inlineStr">
-        <is>
-          <t>Max Crocombe</t>
-        </is>
-      </c>
-      <c r="F13" s="175" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B14" s="175" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C14" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D14" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E14" s="175" t="inlineStr">
-        <is>
-          <t>Ali Ahmed</t>
-        </is>
-      </c>
-      <c r="F14" s="175" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B15" s="175" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C15" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D15" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E15" s="175" t="inlineStr">
-        <is>
-          <t>José Córdoba</t>
-        </is>
-      </c>
-      <c r="F15" s="175" t="inlineStr">
-        <is>
-          <t>Panama</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B16" s="175" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C16" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D16" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E16" s="175" t="inlineStr">
-        <is>
-          <t>Kenny McLean</t>
-        </is>
-      </c>
-      <c r="F16" s="175" t="inlineStr">
-        <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="175" t="inlineStr">
-        <is>
-          <t>Norwich City</t>
-        </is>
-      </c>
-      <c r="C17" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D17" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E17" s="175" t="inlineStr">
-        <is>
-          <t>Toure</t>
-        </is>
-      </c>
-      <c r="F17" s="175" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B18" s="175" t="inlineStr">
-        <is>
-          <t>Portsmouth</t>
-        </is>
-      </c>
-      <c r="C18" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D18" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E18" s="175" t="inlineStr">
-        <is>
-          <t>Gustavo Caballero</t>
-        </is>
-      </c>
-      <c r="F18" s="175" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B19" s="175" t="inlineStr">
-        <is>
-          <t>Sheffield United</t>
-        </is>
-      </c>
-      <c r="C19" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D19" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E19" s="175" t="inlineStr">
-        <is>
-          <t>Tahith Chong</t>
-        </is>
-      </c>
-      <c r="F19" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B20" s="175" t="inlineStr">
-        <is>
-          <t>Stoke City</t>
-        </is>
-      </c>
-      <c r="C20" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D20" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E20" s="175" t="inlineStr">
-        <is>
-          <t>Viktor Johansson</t>
-        </is>
-      </c>
-      <c r="F20" s="175" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B21" s="175" t="inlineStr">
-        <is>
-          <t>Swansea</t>
-        </is>
-      </c>
-      <c r="C21" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D21" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E21" s="175" t="inlineStr">
-        <is>
-          <t>Eom Jisung</t>
-        </is>
-      </c>
-      <c r="F21" s="175" t="inlineStr">
-        <is>
-          <t>Sør-Korea</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B22" s="175" t="inlineStr">
-        <is>
-          <t>Swansea City</t>
-        </is>
-      </c>
-      <c r="C22" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D22" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E22" s="175" t="inlineStr">
-        <is>
-          <t>Burgess</t>
-        </is>
-      </c>
-      <c r="F22" s="175" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B23" s="175" t="inlineStr">
-        <is>
-          <t>Swansea City</t>
-        </is>
-      </c>
-      <c r="C23" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D23" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E23" s="175" t="inlineStr">
-        <is>
-          <t>Marko Stamenić</t>
-        </is>
-      </c>
-      <c r="F23" s="175" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B24" s="175" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="C24" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D24" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E24" s="175" t="inlineStr">
-        <is>
-          <t>Edo Kayembe</t>
-        </is>
-      </c>
-      <c r="F24" s="175" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="175" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="C25" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D25" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E25" s="175" t="inlineStr">
-        <is>
-          <t>Egil Selvik</t>
-        </is>
-      </c>
-      <c r="F25" s="175" t="inlineStr">
-        <is>
-          <t>Norge</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B26" s="175" t="inlineStr">
-        <is>
-          <t>Watford</t>
-        </is>
-      </c>
-      <c r="C26" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D26" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E26" s="175" t="inlineStr">
-        <is>
-          <t>Irankunda</t>
-        </is>
-      </c>
-      <c r="F26" s="175" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" s="175" t="inlineStr">
-        <is>
-          <t>Wrexham</t>
-        </is>
-      </c>
-      <c r="C27" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D27" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E27" s="175" t="inlineStr">
-        <is>
-          <t>Dom Hyam</t>
-        </is>
-      </c>
-      <c r="F27" s="175" t="inlineStr">
-        <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B28" s="175" t="inlineStr">
-        <is>
-          <t>Wrexham AFC</t>
-        </is>
-      </c>
-      <c r="C28" s="175" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D28" s="175" t="inlineStr">
-        <is>
-          <t>Championship</t>
-        </is>
-      </c>
-      <c r="E28" s="175" t="inlineStr">
-        <is>
-          <t>Liberato Cacace</t>
-        </is>
-      </c>
-      <c r="F28" s="175" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B29" s="175" t="inlineStr">
-        <is>
-          <t>AS Nancy-Lorraine</t>
-        </is>
-      </c>
-      <c r="C29" s="175" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="D29" s="175" t="inlineStr">
-        <is>
-          <t>Ligue 2</t>
-        </is>
-      </c>
-      <c r="E29" s="175" t="inlineStr">
-        <is>
-          <t>Martin Experience</t>
-        </is>
-      </c>
-      <c r="F29" s="175" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B30" s="175" t="inlineStr">
-        <is>
-          <t>SC Bastia</t>
-        </is>
-      </c>
-      <c r="C30" s="175" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="D30" s="175" t="inlineStr">
-        <is>
-          <t>Ligue 2</t>
-        </is>
-      </c>
-      <c r="E30" s="175" t="inlineStr">
-        <is>
-          <t>Johnny Placide</t>
-        </is>
-      </c>
-      <c r="F30" s="175" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B31" s="175" t="inlineStr">
-        <is>
-          <t>Frosinone</t>
-        </is>
-      </c>
-      <c r="C31" s="175" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D31" s="175" t="inlineStr">
-        <is>
-          <t>Serie B</t>
-        </is>
-      </c>
-      <c r="E31" s="175" t="inlineStr">
-        <is>
-          <t>Farès Ghedjemis</t>
-        </is>
-      </c>
-      <c r="F31" s="175" t="inlineStr">
-        <is>
-          <t>Algerie</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B32" s="175" t="inlineStr">
-        <is>
-          <t>UC Sampdoria</t>
-        </is>
-      </c>
-      <c r="C32" s="175" t="inlineStr">
-        <is>
-          <t>Italia</t>
-        </is>
-      </c>
-      <c r="D32" s="175" t="inlineStr">
-        <is>
-          <t>Serie B</t>
-        </is>
-      </c>
-      <c r="E32" s="175" t="inlineStr">
-        <is>
-          <t>Dennis Hadžikadunić</t>
-        </is>
-      </c>
-      <c r="F32" s="175" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B33" s="175" t="inlineStr">
-        <is>
-          <t>Albirex Niigata</t>
-        </is>
-      </c>
-      <c r="C33" s="175" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D33" s="175" t="inlineStr">
-        <is>
-          <t>J2 League</t>
-        </is>
-      </c>
-      <c r="E33" s="175" t="inlineStr">
-        <is>
-          <t>Geria</t>
-        </is>
-      </c>
-      <c r="F33" s="175" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B34" s="175" t="inlineStr">
-        <is>
-          <t>FC Den Bosch</t>
-        </is>
-      </c>
-      <c r="C34" s="175" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D34" s="175" t="inlineStr">
-        <is>
-          <t>Eerste Divisie</t>
-        </is>
-      </c>
-      <c r="E34" s="175" t="inlineStr">
-        <is>
-          <t>Kevin Felida</t>
-        </is>
-      </c>
-      <c r="F34" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B35" s="175" t="inlineStr">
-        <is>
-          <t>VVV-Venlo</t>
-        </is>
-      </c>
-      <c r="C35" s="175" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D35" s="175" t="inlineStr">
-        <is>
-          <t>Eerste Divisie</t>
-        </is>
-      </c>
-      <c r="E35" s="175" t="inlineStr">
-        <is>
-          <t>Trevor Doornbusch</t>
-        </is>
-      </c>
-      <c r="F35" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B36" s="175" t="inlineStr">
-        <is>
-          <t>Chaves</t>
-        </is>
-      </c>
-      <c r="C36" s="175" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D36" s="175" t="inlineStr">
-        <is>
-          <t>Liga Portugal 2</t>
-        </is>
-      </c>
-      <c r="E36" s="175" t="inlineStr">
-        <is>
-          <t>Josimar Dias "Vozinha"</t>
-        </is>
-      </c>
-      <c r="F36" s="175" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B37" s="175" t="inlineStr">
-        <is>
-          <t>Torreense</t>
-        </is>
-      </c>
-      <c r="C37" s="175" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="D37" s="175" t="inlineStr">
-        <is>
-          <t>Liga Portugal 2</t>
-        </is>
-      </c>
-      <c r="E37" s="175" t="inlineStr">
-        <is>
-          <t>Ianique Tavares "Stopira"</t>
-        </is>
-      </c>
-      <c r="F37" s="175" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B38" s="175" t="inlineStr">
-        <is>
-          <t>Castellón</t>
-        </is>
-      </c>
-      <c r="C38" s="175" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D38" s="175" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E38" s="175" t="inlineStr">
-        <is>
-          <t>Brian Cipenga</t>
-        </is>
-      </c>
-      <c r="F38" s="175" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B39" s="175" t="inlineStr">
-        <is>
-          <t>Castellón</t>
-        </is>
-      </c>
-      <c r="C39" s="175" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D39" s="175" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E39" s="175" t="inlineStr">
-        <is>
-          <t>Mabil</t>
-        </is>
-      </c>
-      <c r="F39" s="175" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B40" s="175" t="inlineStr">
-        <is>
-          <t>Cultural Leonesa</t>
-        </is>
-      </c>
-      <c r="C40" s="175" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D40" s="175" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E40" s="175" t="inlineStr">
-        <is>
-          <t>Homam Al-Amin</t>
-        </is>
-      </c>
-      <c r="F40" s="175" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B41" s="175" t="inlineStr">
-        <is>
-          <t>Real Oviedo</t>
-        </is>
-      </c>
-      <c r="C41" s="175" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D41" s="175" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E41" s="175" t="inlineStr">
-        <is>
-          <t>Federico Viñas</t>
-        </is>
-      </c>
-      <c r="F41" s="175" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B42" s="175" t="inlineStr">
-        <is>
-          <t>Real Oviedo</t>
-        </is>
-      </c>
-      <c r="C42" s="175" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D42" s="175" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E42" s="175" t="inlineStr">
-        <is>
-          <t>Haissem Hassan</t>
-        </is>
-      </c>
-      <c r="F42" s="175" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B43" s="175" t="inlineStr">
-        <is>
-          <t>Real Oviedo</t>
-        </is>
-      </c>
-      <c r="C43" s="175" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="D43" s="175" t="inlineStr">
-        <is>
-          <t>Segunda División</t>
-        </is>
-      </c>
-      <c r="E43" s="175" t="inlineStr">
-        <is>
-          <t>Kwasi Sibo</t>
-        </is>
-      </c>
-      <c r="F43" s="175" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B44" s="175" t="inlineStr">
-        <is>
-          <t>Stade Nyonnais</t>
-        </is>
-      </c>
-      <c r="C44" s="175" t="inlineStr">
-        <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-      <c r="D44" s="175" t="inlineStr">
-        <is>
-          <t>Challenge League</t>
-        </is>
-      </c>
-      <c r="E44" s="175" t="inlineStr">
-        <is>
-          <t>Melvin Mastil</t>
-        </is>
-      </c>
-      <c r="F44" s="175" t="inlineStr">
-        <is>
-          <t>Algerie</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B45" s="175" t="inlineStr">
-        <is>
-          <t>IFK Norrköping</t>
-        </is>
-      </c>
-      <c r="C45" s="175" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-      <c r="D45" s="175" t="inlineStr">
-        <is>
-          <t>Superettan</t>
-        </is>
-      </c>
-      <c r="E45" s="175" t="inlineStr">
-        <is>
-          <t>Moutaz Neffati</t>
-        </is>
-      </c>
-      <c r="F45" s="175" t="inlineStr">
-        <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-    </row>
-    <row r="46">
-      <c r="A46" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B46" s="175" t="inlineStr">
-        <is>
-          <t>Siwelele FC</t>
-        </is>
-      </c>
-      <c r="C46" s="175" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-      <c r="D46" s="175" t="inlineStr">
-        <is>
-          <t>National First Division</t>
-        </is>
-      </c>
-      <c r="E46" s="175" t="inlineStr">
-        <is>
-          <t>Ricardo Goss</t>
-        </is>
-      </c>
-      <c r="F46" s="175" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B47" s="175" t="inlineStr">
-        <is>
-          <t>Iğdır</t>
-        </is>
-      </c>
-      <c r="C47" s="175" t="inlineStr">
-        <is>
-          <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="D47" s="175" t="inlineStr">
-        <is>
-          <t>TFF 1. Lig</t>
-        </is>
-      </c>
-      <c r="E47" s="175" t="inlineStr">
-        <is>
-          <t>Leandro Bacuna</t>
-        </is>
-      </c>
-      <c r="F47" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B48" s="175" t="inlineStr">
-        <is>
-          <t>Iğdır</t>
-        </is>
-      </c>
-      <c r="C48" s="175" t="inlineStr">
-        <is>
-          <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="D48" s="175" t="inlineStr">
-        <is>
-          <t>TFF 1. Lig</t>
-        </is>
-      </c>
-      <c r="E48" s="175" t="inlineStr">
-        <is>
-          <t>Ryan Mendes</t>
-        </is>
-      </c>
-      <c r="F48" s="175" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B49" s="175" t="inlineStr">
-        <is>
-          <t>Fortuna Düsseldorf</t>
-        </is>
-      </c>
-      <c r="C49" s="175" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D49" s="175" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E49" s="175" t="inlineStr">
-        <is>
-          <t>Cedric Itten</t>
-        </is>
-      </c>
-      <c r="F49" s="175" t="inlineStr">
-        <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B50" s="175" t="inlineStr">
-        <is>
-          <t>Hannover 96</t>
-        </is>
-      </c>
-      <c r="C50" s="175" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D50" s="175" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E50" s="175" t="inlineStr">
-        <is>
-          <t>Ime Okon</t>
-        </is>
-      </c>
-      <c r="F50" s="175" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B51" s="175" t="inlineStr">
-        <is>
-          <t>Hannover 96</t>
-        </is>
-      </c>
-      <c r="C51" s="175" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D51" s="175" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E51" s="175" t="inlineStr">
-        <is>
-          <t>​Elias Saad</t>
-        </is>
-      </c>
-      <c r="F51" s="175" t="inlineStr">
-        <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B52" s="175" t="inlineStr">
-        <is>
-          <t>Karlsruher SC</t>
-        </is>
-      </c>
-      <c r="C52" s="175" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D52" s="175" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E52" s="175" t="inlineStr">
-        <is>
-          <t>Dženis Burnić</t>
-        </is>
-      </c>
-      <c r="F52" s="175" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="175" t="inlineStr">
-        <is>
-          <t>Schalke 04</t>
-        </is>
-      </c>
-      <c r="C53" s="175" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D53" s="175" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E53" s="175" t="inlineStr">
-        <is>
-          <t>Edin Džeko</t>
-        </is>
-      </c>
-      <c r="F53" s="175" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B54" s="175" t="inlineStr">
-        <is>
-          <t>Schalke 04</t>
-        </is>
-      </c>
-      <c r="C54" s="175" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D54" s="175" t="inlineStr">
-        <is>
-          <t>2. Bundesliga</t>
-        </is>
-      </c>
-      <c r="E54" s="175" t="inlineStr">
-        <is>
-          <t>Nikola Katić</t>
-        </is>
-      </c>
-      <c r="F54" s="175" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B55" s="175" t="inlineStr">
-        <is>
-          <t>El Paso Locomotive FC</t>
-        </is>
-      </c>
-      <c r="C55" s="175" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D55" s="175" t="inlineStr">
-        <is>
-          <t>USL Championship</t>
-        </is>
-      </c>
-      <c r="E55" s="175" t="inlineStr">
-        <is>
-          <t>Carl-Fred Sainthe</t>
-        </is>
-      </c>
-      <c r="F55" s="175" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B56" s="175" t="inlineStr">
-        <is>
-          <t>Miami FC</t>
-        </is>
-      </c>
-      <c r="C56" s="175" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D56" s="175" t="inlineStr">
-        <is>
-          <t>USL Championship</t>
-        </is>
-      </c>
-      <c r="E56" s="175" t="inlineStr">
-        <is>
-          <t>Eloy Room</t>
-        </is>
-      </c>
-      <c r="F56" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="B57" s="175" t="inlineStr">
-        <is>
-          <t>Miami FC</t>
-        </is>
-      </c>
-      <c r="C57" s="175" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="D57" s="175" t="inlineStr">
-        <is>
-          <t>USL Championship</t>
-        </is>
-      </c>
-      <c r="E57" s="175" t="inlineStr">
-        <is>
-          <t>Jürgen Locadia</t>
-        </is>
-      </c>
-      <c r="F57" s="175" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="176" t="n">
-        <v>3</v>
-      </c>
-      <c r="B58" s="177" t="inlineStr">
-        <is>
-          <t>Port Vale</t>
-        </is>
-      </c>
-      <c r="C58" s="177" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D58" s="177" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="E58" s="177" t="inlineStr">
-        <is>
-          <t>Ben Waine</t>
-        </is>
-      </c>
-      <c r="F58" s="177" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="176" t="n">
-        <v>3</v>
-      </c>
-      <c r="B59" s="177" t="inlineStr">
-        <is>
-          <t>Rotherham United</t>
-        </is>
-      </c>
-      <c r="C59" s="177" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D59" s="177" t="inlineStr">
-        <is>
-          <t>League One</t>
-        </is>
-      </c>
-      <c r="E59" s="177" t="inlineStr">
-        <is>
-          <t>Ar’Jany Martha</t>
-        </is>
-      </c>
-      <c r="F59" s="177" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="176" t="n">
-        <v>3</v>
-      </c>
-      <c r="B60" s="177" t="inlineStr">
-        <is>
-          <t>FC Sochaux</t>
-        </is>
-      </c>
-      <c r="C60" s="177" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="D60" s="177" t="inlineStr">
-        <is>
-          <t>National</t>
-        </is>
-      </c>
-      <c r="E60" s="177" t="inlineStr">
-        <is>
-          <t>Alexandre Pierre</t>
-        </is>
-      </c>
-      <c r="F60" s="177" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="176" t="n">
-        <v>3</v>
-      </c>
-      <c r="B61" s="177" t="inlineStr">
-        <is>
-          <t>BSC Young Boys II</t>
-        </is>
-      </c>
-      <c r="C61" s="177" t="inlineStr">
-        <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-      <c r="D61" s="177" t="inlineStr">
-        <is>
-          <t>Promotion League</t>
-        </is>
-      </c>
-      <c r="E61" s="177" t="inlineStr">
-        <is>
-          <t>Keeto Thermoncy</t>
-        </is>
-      </c>
-      <c r="F61" s="177" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="178" t="n">
-        <v>4</v>
-      </c>
-      <c r="B62" s="179" t="inlineStr">
-        <is>
-          <t>FC Cosmos Koblenz</t>
-        </is>
-      </c>
-      <c r="C62" s="179" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D62" s="179" t="inlineStr">
-        <is>
-          <t>Regionalliga</t>
-        </is>
-      </c>
-      <c r="E62" s="179" t="inlineStr">
-        <is>
-          <t>Josué Duverger</t>
-        </is>
-      </c>
-      <c r="F62" s="179" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="180" t="n">
-        <v>6</v>
-      </c>
-      <c r="B63" s="181" t="inlineStr">
-        <is>
-          <t>Braintree Town</t>
-        </is>
-      </c>
-      <c r="C63" s="181" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="D63" s="181" t="inlineStr">
-        <is>
-          <t>National League South</t>
-        </is>
-      </c>
-      <c r="E63" s="181" t="inlineStr">
-        <is>
-          <t>Tommy Smith</t>
-        </is>
-      </c>
-      <c r="F63" s="181" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="32" t="inlineStr">
-        <is>
-          <t>Fargeforklaring:</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="182" t="inlineStr">
-        <is>
-          <t>Nivå 2</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="183" t="inlineStr">
-        <is>
-          <t>Nivå 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="184" t="inlineStr">
-        <is>
-          <t>Nivå 4</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="185" t="inlineStr">
-        <is>
-          <t>Nivå 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="186" t="inlineStr">
-        <is>
-          <t>Nivå 6</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A2:F2"/>
-  <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:I70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -53544,6 +51637,1943 @@
   <autoFilter ref="A2:I2"/>
   <mergeCells count="1">
     <mergeCell ref="A1:I1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F70"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" style="143" min="1" max="1"/>
+    <col width="26" customWidth="1" style="143" min="2" max="2"/>
+    <col width="16" customWidth="1" style="143" min="3" max="3"/>
+    <col width="22" customWidth="1" style="143" min="4" max="4"/>
+    <col width="30" customWidth="1" style="143" min="5" max="5"/>
+    <col width="22" customWidth="1" style="143" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="143">
+      <c r="A1" s="150" t="inlineStr">
+        <is>
+          <t>VM 2026 — Spillere på nivå 2 og lavere   61 spillere</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="143">
+      <c r="A2" s="151" t="inlineStr">
+        <is>
+          <t>Nivå</t>
+        </is>
+      </c>
+      <c r="B2" s="151" t="inlineStr">
+        <is>
+          <t>Klubb</t>
+        </is>
+      </c>
+      <c r="C2" s="151" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="D2" s="151" t="inlineStr">
+        <is>
+          <t>Liga</t>
+        </is>
+      </c>
+      <c r="E2" s="151" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="F2" s="151" t="inlineStr">
+        <is>
+          <t>Nasjonallag</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1" s="143">
+      <c r="A3" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="189" t="inlineStr">
+        <is>
+          <t>Charlton Athletic</t>
+        </is>
+      </c>
+      <c r="C3" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D3" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E3" s="189" t="inlineStr">
+        <is>
+          <t>Lyndon Dykes</t>
+        </is>
+      </c>
+      <c r="F3" s="189" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="17" customHeight="1" s="143">
+      <c r="A4" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" s="189" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="C4" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D4" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E4" s="189" t="inlineStr">
+        <is>
+          <t>Brandon Thomas-Asante</t>
+        </is>
+      </c>
+      <c r="F4" s="189" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17" customHeight="1" s="143">
+      <c r="A5" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B5" s="189" t="inlineStr">
+        <is>
+          <t>Coventry City</t>
+        </is>
+      </c>
+      <c r="C5" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D5" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E5" s="189" t="inlineStr">
+        <is>
+          <t>Haji Wright</t>
+        </is>
+      </c>
+      <c r="F5" s="189" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="17" customHeight="1" s="143">
+      <c r="A6" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="189" t="inlineStr">
+        <is>
+          <t>Derby County</t>
+        </is>
+      </c>
+      <c r="C6" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D6" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E6" s="189" t="inlineStr">
+        <is>
+          <t>Jacob Widell Zetterström</t>
+        </is>
+      </c>
+      <c r="F6" s="189" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1" s="143">
+      <c r="A7" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="189" t="inlineStr">
+        <is>
+          <t>Derby County</t>
+        </is>
+      </c>
+      <c r="C7" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D7" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E7" s="189" t="inlineStr">
+        <is>
+          <t>Sondre Langås</t>
+        </is>
+      </c>
+      <c r="F7" s="189" t="inlineStr">
+        <is>
+          <t>Norge</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="17" customHeight="1" s="143">
+      <c r="A8" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B8" s="189" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="C8" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D8" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E8" s="189" t="inlineStr">
+        <is>
+          <t>Amir Hadžiahmetović</t>
+        </is>
+      </c>
+      <c r="F8" s="189" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="17" customHeight="1" s="143">
+      <c r="A9" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="189" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="C9" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D9" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E9" s="189" t="inlineStr">
+        <is>
+          <t>Ivor Pandur</t>
+        </is>
+      </c>
+      <c r="F9" s="189" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="17" customHeight="1" s="143">
+      <c r="A10" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B10" s="189" t="inlineStr">
+        <is>
+          <t>Hull City</t>
+        </is>
+      </c>
+      <c r="C10" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D10" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E10" s="189" t="inlineStr">
+        <is>
+          <t>Liam Miller</t>
+        </is>
+      </c>
+      <c r="F10" s="189" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="17" customHeight="1" s="143">
+      <c r="A11" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="189" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C11" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D11" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E11" s="189" t="inlineStr">
+        <is>
+          <t>Alfie Jones</t>
+        </is>
+      </c>
+      <c r="F11" s="189" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1" s="143">
+      <c r="A12" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="189" t="inlineStr">
+        <is>
+          <t>Middlesbrough</t>
+        </is>
+      </c>
+      <c r="C12" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D12" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E12" s="189" t="inlineStr">
+        <is>
+          <t>Sontje Hansen</t>
+        </is>
+      </c>
+      <c r="F12" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1" s="143">
+      <c r="A13" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B13" s="189" t="inlineStr">
+        <is>
+          <t>Millwall FC</t>
+        </is>
+      </c>
+      <c r="C13" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D13" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E13" s="189" t="inlineStr">
+        <is>
+          <t>Max Crocombe</t>
+        </is>
+      </c>
+      <c r="F13" s="189" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1" s="143">
+      <c r="A14" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="189" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C14" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D14" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E14" s="189" t="inlineStr">
+        <is>
+          <t>Ali Ahmed</t>
+        </is>
+      </c>
+      <c r="F14" s="189" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1" s="143">
+      <c r="A15" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B15" s="189" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C15" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D15" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E15" s="189" t="inlineStr">
+        <is>
+          <t>José Córdoba</t>
+        </is>
+      </c>
+      <c r="F15" s="189" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1" s="143">
+      <c r="A16" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="189" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C16" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D16" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E16" s="189" t="inlineStr">
+        <is>
+          <t>Kenny McLean</t>
+        </is>
+      </c>
+      <c r="F16" s="189" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="17" customHeight="1" s="143">
+      <c r="A17" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B17" s="189" t="inlineStr">
+        <is>
+          <t>Norwich City</t>
+        </is>
+      </c>
+      <c r="C17" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D17" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E17" s="189" t="inlineStr">
+        <is>
+          <t>Toure</t>
+        </is>
+      </c>
+      <c r="F17" s="189" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="17" customHeight="1" s="143">
+      <c r="A18" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="189" t="inlineStr">
+        <is>
+          <t>Portsmouth</t>
+        </is>
+      </c>
+      <c r="C18" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D18" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E18" s="189" t="inlineStr">
+        <is>
+          <t>Gustavo Caballero</t>
+        </is>
+      </c>
+      <c r="F18" s="189" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="17" customHeight="1" s="143">
+      <c r="A19" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="189" t="inlineStr">
+        <is>
+          <t>Sheffield United</t>
+        </is>
+      </c>
+      <c r="C19" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D19" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E19" s="189" t="inlineStr">
+        <is>
+          <t>Tahith Chong</t>
+        </is>
+      </c>
+      <c r="F19" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1" s="143">
+      <c r="A20" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B20" s="189" t="inlineStr">
+        <is>
+          <t>Stoke City</t>
+        </is>
+      </c>
+      <c r="C20" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D20" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E20" s="189" t="inlineStr">
+        <is>
+          <t>Viktor Johansson</t>
+        </is>
+      </c>
+      <c r="F20" s="189" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="17" customHeight="1" s="143">
+      <c r="A21" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B21" s="189" t="inlineStr">
+        <is>
+          <t>Swansea</t>
+        </is>
+      </c>
+      <c r="C21" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D21" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E21" s="189" t="inlineStr">
+        <is>
+          <t>Eom Jisung</t>
+        </is>
+      </c>
+      <c r="F21" s="189" t="inlineStr">
+        <is>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="17" customHeight="1" s="143">
+      <c r="A22" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B22" s="189" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="C22" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D22" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E22" s="189" t="inlineStr">
+        <is>
+          <t>Burgess</t>
+        </is>
+      </c>
+      <c r="F22" s="189" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="17" customHeight="1" s="143">
+      <c r="A23" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B23" s="189" t="inlineStr">
+        <is>
+          <t>Swansea City</t>
+        </is>
+      </c>
+      <c r="C23" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D23" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E23" s="189" t="inlineStr">
+        <is>
+          <t>Marko Stamenić</t>
+        </is>
+      </c>
+      <c r="F23" s="189" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="17" customHeight="1" s="143">
+      <c r="A24" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B24" s="189" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="C24" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D24" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E24" s="189" t="inlineStr">
+        <is>
+          <t>Edo Kayembe</t>
+        </is>
+      </c>
+      <c r="F24" s="189" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="17" customHeight="1" s="143">
+      <c r="A25" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B25" s="189" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="C25" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D25" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E25" s="189" t="inlineStr">
+        <is>
+          <t>Egil Selvik</t>
+        </is>
+      </c>
+      <c r="F25" s="189" t="inlineStr">
+        <is>
+          <t>Norge</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="17" customHeight="1" s="143">
+      <c r="A26" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B26" s="189" t="inlineStr">
+        <is>
+          <t>Watford</t>
+        </is>
+      </c>
+      <c r="C26" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D26" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E26" s="189" t="inlineStr">
+        <is>
+          <t>Irankunda</t>
+        </is>
+      </c>
+      <c r="F26" s="189" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="17" customHeight="1" s="143">
+      <c r="A27" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="189" t="inlineStr">
+        <is>
+          <t>Wrexham</t>
+        </is>
+      </c>
+      <c r="C27" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D27" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E27" s="189" t="inlineStr">
+        <is>
+          <t>Dom Hyam</t>
+        </is>
+      </c>
+      <c r="F27" s="189" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="17" customHeight="1" s="143">
+      <c r="A28" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B28" s="189" t="inlineStr">
+        <is>
+          <t>Wrexham AFC</t>
+        </is>
+      </c>
+      <c r="C28" s="189" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D28" s="189" t="inlineStr">
+        <is>
+          <t>Championship</t>
+        </is>
+      </c>
+      <c r="E28" s="189" t="inlineStr">
+        <is>
+          <t>Liberato Cacace</t>
+        </is>
+      </c>
+      <c r="F28" s="189" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="17" customHeight="1" s="143">
+      <c r="A29" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B29" s="189" t="inlineStr">
+        <is>
+          <t>AS Nancy-Lorraine</t>
+        </is>
+      </c>
+      <c r="C29" s="189" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D29" s="189" t="inlineStr">
+        <is>
+          <t>Ligue 2</t>
+        </is>
+      </c>
+      <c r="E29" s="189" t="inlineStr">
+        <is>
+          <t>Martin Experience</t>
+        </is>
+      </c>
+      <c r="F29" s="189" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="17" customHeight="1" s="143">
+      <c r="A30" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B30" s="189" t="inlineStr">
+        <is>
+          <t>SC Bastia</t>
+        </is>
+      </c>
+      <c r="C30" s="189" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D30" s="189" t="inlineStr">
+        <is>
+          <t>Ligue 2</t>
+        </is>
+      </c>
+      <c r="E30" s="189" t="inlineStr">
+        <is>
+          <t>Johnny Placide</t>
+        </is>
+      </c>
+      <c r="F30" s="189" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="17" customHeight="1" s="143">
+      <c r="A31" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B31" s="189" t="inlineStr">
+        <is>
+          <t>Frosinone</t>
+        </is>
+      </c>
+      <c r="C31" s="189" t="inlineStr">
+        <is>
+          <t>Italia</t>
+        </is>
+      </c>
+      <c r="D31" s="189" t="inlineStr">
+        <is>
+          <t>Serie B</t>
+        </is>
+      </c>
+      <c r="E31" s="189" t="inlineStr">
+        <is>
+          <t>Farès Ghedjemis</t>
+        </is>
+      </c>
+      <c r="F31" s="189" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="17" customHeight="1" s="143">
+      <c r="A32" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B32" s="189" t="inlineStr">
+        <is>
+          <t>UC Sampdoria</t>
+        </is>
+      </c>
+      <c r="C32" s="189" t="inlineStr">
+        <is>
+          <t>Italia</t>
+        </is>
+      </c>
+      <c r="D32" s="189" t="inlineStr">
+        <is>
+          <t>Serie B</t>
+        </is>
+      </c>
+      <c r="E32" s="189" t="inlineStr">
+        <is>
+          <t>Dennis Hadžikadunić</t>
+        </is>
+      </c>
+      <c r="F32" s="189" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="17" customHeight="1" s="143">
+      <c r="A33" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B33" s="189" t="inlineStr">
+        <is>
+          <t>Albirex Niigata</t>
+        </is>
+      </c>
+      <c r="C33" s="189" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D33" s="189" t="inlineStr">
+        <is>
+          <t>J2 League</t>
+        </is>
+      </c>
+      <c r="E33" s="189" t="inlineStr">
+        <is>
+          <t>Geria</t>
+        </is>
+      </c>
+      <c r="F33" s="189" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="17" customHeight="1" s="143">
+      <c r="A34" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B34" s="189" t="inlineStr">
+        <is>
+          <t>FC Den Bosch</t>
+        </is>
+      </c>
+      <c r="C34" s="189" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D34" s="189" t="inlineStr">
+        <is>
+          <t>Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="E34" s="189" t="inlineStr">
+        <is>
+          <t>Kevin Felida</t>
+        </is>
+      </c>
+      <c r="F34" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="17" customHeight="1" s="143">
+      <c r="A35" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B35" s="189" t="inlineStr">
+        <is>
+          <t>VVV-Venlo</t>
+        </is>
+      </c>
+      <c r="C35" s="189" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D35" s="189" t="inlineStr">
+        <is>
+          <t>Eerste Divisie</t>
+        </is>
+      </c>
+      <c r="E35" s="189" t="inlineStr">
+        <is>
+          <t>Trevor Doornbusch</t>
+        </is>
+      </c>
+      <c r="F35" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="17" customHeight="1" s="143">
+      <c r="A36" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B36" s="189" t="inlineStr">
+        <is>
+          <t>Chaves</t>
+        </is>
+      </c>
+      <c r="C36" s="189" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D36" s="189" t="inlineStr">
+        <is>
+          <t>Liga Portugal 2</t>
+        </is>
+      </c>
+      <c r="E36" s="189" t="inlineStr">
+        <is>
+          <t>Josimar Dias "Vozinha"</t>
+        </is>
+      </c>
+      <c r="F36" s="189" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="17" customHeight="1" s="143">
+      <c r="A37" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B37" s="189" t="inlineStr">
+        <is>
+          <t>Torreense</t>
+        </is>
+      </c>
+      <c r="C37" s="189" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D37" s="189" t="inlineStr">
+        <is>
+          <t>Liga Portugal 2</t>
+        </is>
+      </c>
+      <c r="E37" s="189" t="inlineStr">
+        <is>
+          <t>Ianique Tavares "Stopira"</t>
+        </is>
+      </c>
+      <c r="F37" s="189" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="17" customHeight="1" s="143">
+      <c r="A38" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B38" s="189" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="C38" s="189" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D38" s="189" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E38" s="189" t="inlineStr">
+        <is>
+          <t>Brian Cipenga</t>
+        </is>
+      </c>
+      <c r="F38" s="189" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="17" customHeight="1" s="143">
+      <c r="A39" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B39" s="189" t="inlineStr">
+        <is>
+          <t>Castellón</t>
+        </is>
+      </c>
+      <c r="C39" s="189" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D39" s="189" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E39" s="189" t="inlineStr">
+        <is>
+          <t>Mabil</t>
+        </is>
+      </c>
+      <c r="F39" s="189" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="17" customHeight="1" s="143">
+      <c r="A40" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" s="189" t="inlineStr">
+        <is>
+          <t>Cultural Leonesa</t>
+        </is>
+      </c>
+      <c r="C40" s="189" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D40" s="189" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E40" s="189" t="inlineStr">
+        <is>
+          <t>Homam Al-Amin</t>
+        </is>
+      </c>
+      <c r="F40" s="189" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="17" customHeight="1" s="143">
+      <c r="A41" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B41" s="189" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C41" s="189" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D41" s="189" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E41" s="189" t="inlineStr">
+        <is>
+          <t>Federico Viñas</t>
+        </is>
+      </c>
+      <c r="F41" s="189" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="17" customHeight="1" s="143">
+      <c r="A42" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B42" s="189" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C42" s="189" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D42" s="189" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E42" s="189" t="inlineStr">
+        <is>
+          <t>Haissem Hassan</t>
+        </is>
+      </c>
+      <c r="F42" s="189" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="17" customHeight="1" s="143">
+      <c r="A43" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B43" s="189" t="inlineStr">
+        <is>
+          <t>Real Oviedo</t>
+        </is>
+      </c>
+      <c r="C43" s="189" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D43" s="189" t="inlineStr">
+        <is>
+          <t>Segunda División</t>
+        </is>
+      </c>
+      <c r="E43" s="189" t="inlineStr">
+        <is>
+          <t>Kwasi Sibo</t>
+        </is>
+      </c>
+      <c r="F43" s="189" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="17" customHeight="1" s="143">
+      <c r="A44" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B44" s="189" t="inlineStr">
+        <is>
+          <t>Stade Nyonnais</t>
+        </is>
+      </c>
+      <c r="C44" s="189" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="D44" s="189" t="inlineStr">
+        <is>
+          <t>Challenge League</t>
+        </is>
+      </c>
+      <c r="E44" s="189" t="inlineStr">
+        <is>
+          <t>Melvin Mastil</t>
+        </is>
+      </c>
+      <c r="F44" s="189" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="17" customHeight="1" s="143">
+      <c r="A45" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B45" s="189" t="inlineStr">
+        <is>
+          <t>IFK Norrköping</t>
+        </is>
+      </c>
+      <c r="C45" s="189" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+      <c r="D45" s="189" t="inlineStr">
+        <is>
+          <t>Superettan</t>
+        </is>
+      </c>
+      <c r="E45" s="189" t="inlineStr">
+        <is>
+          <t>Moutaz Neffati</t>
+        </is>
+      </c>
+      <c r="F45" s="189" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="17" customHeight="1" s="143">
+      <c r="A46" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B46" s="189" t="inlineStr">
+        <is>
+          <t>Siwelele FC</t>
+        </is>
+      </c>
+      <c r="C46" s="189" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="D46" s="189" t="inlineStr">
+        <is>
+          <t>National First Division</t>
+        </is>
+      </c>
+      <c r="E46" s="189" t="inlineStr">
+        <is>
+          <t>Ricardo Goss</t>
+        </is>
+      </c>
+      <c r="F46" s="189" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="17" customHeight="1" s="143">
+      <c r="A47" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B47" s="189" t="inlineStr">
+        <is>
+          <t>Iğdır</t>
+        </is>
+      </c>
+      <c r="C47" s="189" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="D47" s="189" t="inlineStr">
+        <is>
+          <t>TFF 1. Lig</t>
+        </is>
+      </c>
+      <c r="E47" s="189" t="inlineStr">
+        <is>
+          <t>Leandro Bacuna</t>
+        </is>
+      </c>
+      <c r="F47" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="17" customHeight="1" s="143">
+      <c r="A48" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="189" t="inlineStr">
+        <is>
+          <t>Iğdır</t>
+        </is>
+      </c>
+      <c r="C48" s="189" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="D48" s="189" t="inlineStr">
+        <is>
+          <t>TFF 1. Lig</t>
+        </is>
+      </c>
+      <c r="E48" s="189" t="inlineStr">
+        <is>
+          <t>Ryan Mendes</t>
+        </is>
+      </c>
+      <c r="F48" s="189" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="17" customHeight="1" s="143">
+      <c r="A49" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B49" s="189" t="inlineStr">
+        <is>
+          <t>Fortuna Düsseldorf</t>
+        </is>
+      </c>
+      <c r="C49" s="189" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D49" s="189" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E49" s="189" t="inlineStr">
+        <is>
+          <t>Cedric Itten</t>
+        </is>
+      </c>
+      <c r="F49" s="189" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="17" customHeight="1" s="143">
+      <c r="A50" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B50" s="189" t="inlineStr">
+        <is>
+          <t>Hannover 96</t>
+        </is>
+      </c>
+      <c r="C50" s="189" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D50" s="189" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E50" s="189" t="inlineStr">
+        <is>
+          <t>Ime Okon</t>
+        </is>
+      </c>
+      <c r="F50" s="189" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="17" customHeight="1" s="143">
+      <c r="A51" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B51" s="189" t="inlineStr">
+        <is>
+          <t>Hannover 96</t>
+        </is>
+      </c>
+      <c r="C51" s="189" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D51" s="189" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E51" s="189" t="inlineStr">
+        <is>
+          <t>​Elias Saad</t>
+        </is>
+      </c>
+      <c r="F51" s="189" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="17" customHeight="1" s="143">
+      <c r="A52" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B52" s="189" t="inlineStr">
+        <is>
+          <t>Karlsruher SC</t>
+        </is>
+      </c>
+      <c r="C52" s="189" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D52" s="189" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E52" s="189" t="inlineStr">
+        <is>
+          <t>Dženis Burnić</t>
+        </is>
+      </c>
+      <c r="F52" s="189" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="17" customHeight="1" s="143">
+      <c r="A53" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="189" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="C53" s="189" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D53" s="189" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E53" s="189" t="inlineStr">
+        <is>
+          <t>Edin Džeko</t>
+        </is>
+      </c>
+      <c r="F53" s="189" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="17" customHeight="1" s="143">
+      <c r="A54" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B54" s="189" t="inlineStr">
+        <is>
+          <t>Schalke 04</t>
+        </is>
+      </c>
+      <c r="C54" s="189" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D54" s="189" t="inlineStr">
+        <is>
+          <t>2. Bundesliga</t>
+        </is>
+      </c>
+      <c r="E54" s="189" t="inlineStr">
+        <is>
+          <t>Nikola Katić</t>
+        </is>
+      </c>
+      <c r="F54" s="189" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="17" customHeight="1" s="143">
+      <c r="A55" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B55" s="189" t="inlineStr">
+        <is>
+          <t>El Paso Locomotive FC</t>
+        </is>
+      </c>
+      <c r="C55" s="189" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D55" s="189" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E55" s="189" t="inlineStr">
+        <is>
+          <t>Carl-Fred Sainthe</t>
+        </is>
+      </c>
+      <c r="F55" s="189" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="17" customHeight="1" s="143">
+      <c r="A56" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B56" s="189" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="C56" s="189" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D56" s="189" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E56" s="189" t="inlineStr">
+        <is>
+          <t>Eloy Room</t>
+        </is>
+      </c>
+      <c r="F56" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="17" customHeight="1" s="143">
+      <c r="A57" s="188" t="n">
+        <v>2</v>
+      </c>
+      <c r="B57" s="189" t="inlineStr">
+        <is>
+          <t>Miami FC</t>
+        </is>
+      </c>
+      <c r="C57" s="189" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D57" s="189" t="inlineStr">
+        <is>
+          <t>USL Championship</t>
+        </is>
+      </c>
+      <c r="E57" s="189" t="inlineStr">
+        <is>
+          <t>Jürgen Locadia</t>
+        </is>
+      </c>
+      <c r="F57" s="189" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="17" customHeight="1" s="143">
+      <c r="A58" s="190" t="n">
+        <v>3</v>
+      </c>
+      <c r="B58" s="191" t="inlineStr">
+        <is>
+          <t>Port Vale</t>
+        </is>
+      </c>
+      <c r="C58" s="191" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D58" s="191" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="E58" s="191" t="inlineStr">
+        <is>
+          <t>Ben Waine</t>
+        </is>
+      </c>
+      <c r="F58" s="191" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="17" customHeight="1" s="143">
+      <c r="A59" s="190" t="n">
+        <v>3</v>
+      </c>
+      <c r="B59" s="191" t="inlineStr">
+        <is>
+          <t>Rotherham United</t>
+        </is>
+      </c>
+      <c r="C59" s="191" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D59" s="191" t="inlineStr">
+        <is>
+          <t>League One</t>
+        </is>
+      </c>
+      <c r="E59" s="191" t="inlineStr">
+        <is>
+          <t>Ar’Jany Martha</t>
+        </is>
+      </c>
+      <c r="F59" s="191" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="17" customHeight="1" s="143">
+      <c r="A60" s="190" t="n">
+        <v>3</v>
+      </c>
+      <c r="B60" s="191" t="inlineStr">
+        <is>
+          <t>FC Sochaux</t>
+        </is>
+      </c>
+      <c r="C60" s="191" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D60" s="191" t="inlineStr">
+        <is>
+          <t>National</t>
+        </is>
+      </c>
+      <c r="E60" s="191" t="inlineStr">
+        <is>
+          <t>Alexandre Pierre</t>
+        </is>
+      </c>
+      <c r="F60" s="191" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="17" customHeight="1" s="143">
+      <c r="A61" s="190" t="n">
+        <v>3</v>
+      </c>
+      <c r="B61" s="191" t="inlineStr">
+        <is>
+          <t>BSC Young Boys II</t>
+        </is>
+      </c>
+      <c r="C61" s="191" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="D61" s="191" t="inlineStr">
+        <is>
+          <t>Promotion League</t>
+        </is>
+      </c>
+      <c r="E61" s="191" t="inlineStr">
+        <is>
+          <t>Keeto Thermoncy</t>
+        </is>
+      </c>
+      <c r="F61" s="191" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="17" customHeight="1" s="143">
+      <c r="A62" s="192" t="n">
+        <v>4</v>
+      </c>
+      <c r="B62" s="193" t="inlineStr">
+        <is>
+          <t>FC Cosmos Koblenz</t>
+        </is>
+      </c>
+      <c r="C62" s="193" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D62" s="193" t="inlineStr">
+        <is>
+          <t>Regionalliga</t>
+        </is>
+      </c>
+      <c r="E62" s="193" t="inlineStr">
+        <is>
+          <t>Josué Duverger</t>
+        </is>
+      </c>
+      <c r="F62" s="193" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="17" customHeight="1" s="143">
+      <c r="A63" s="194" t="n">
+        <v>6</v>
+      </c>
+      <c r="B63" s="195" t="inlineStr">
+        <is>
+          <t>Braintree Town</t>
+        </is>
+      </c>
+      <c r="C63" s="195" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D63" s="195" t="inlineStr">
+        <is>
+          <t>National League South</t>
+        </is>
+      </c>
+      <c r="E63" s="195" t="inlineStr">
+        <is>
+          <t>Tommy Smith</t>
+        </is>
+      </c>
+      <c r="F63" s="195" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="196" t="inlineStr">
+        <is>
+          <t>Fargeforklaring:</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="197" t="inlineStr">
+        <is>
+          <t>Nivå 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="198" t="inlineStr">
+        <is>
+          <t>Nivå 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="199" t="inlineStr">
+        <is>
+          <t>Nivå 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="200" t="inlineStr">
+        <is>
+          <t>Nivå 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="201" t="inlineStr">
+        <is>
+          <t>Nivå 6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A2:F2"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Oppdater Ballbesittelse-ark med nye kampdata (wc2026_stats.json)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -33863,7 +33863,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N34"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="143" min="1" max="1"/>
@@ -33986,44 +33986,44 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="C4" s="232" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="D4" s="233" t="n">
-        <v>16</v>
+      <c r="C4" s="238" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D4" s="234" t="n">
+        <v>8</v>
       </c>
       <c r="E4" s="233" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F4" s="234" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="G4" s="235" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H4" s="236" t="inlineStr">
         <is>
-          <t>2–0</t>
+          <t>1–0</t>
         </is>
       </c>
       <c r="I4" s="237" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J4" s="234" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K4" s="234" t="n">
         <v>2</v>
       </c>
       <c r="L4" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="M4" s="238" t="n">
-        <v>0.39</v>
+        <v>8</v>
+      </c>
+      <c r="M4" s="232" t="n">
+        <v>0.57</v>
       </c>
       <c r="N4" s="231" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
+          <t>Sør-Korea</t>
         </is>
       </c>
     </row>
@@ -34031,95 +34031,99 @@
       <c r="A5" s="239" t="inlineStr"/>
       <c r="B5" s="240" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Tsjekkia</t>
         </is>
       </c>
       <c r="C5" s="238" t="n">
-        <v>0.43</v>
+        <v>0.39</v>
       </c>
       <c r="D5" s="241" t="n">
+        <v>12</v>
+      </c>
+      <c r="E5" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="241" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="243" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" s="244" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I5" s="245" t="n">
         <v>8</v>
       </c>
-      <c r="E5" s="242" t="n">
+      <c r="J5" s="241" t="n">
         <v>4</v>
       </c>
-      <c r="F5" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="243" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="244" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I5" s="245" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="K5" s="241" t="n">
+      <c r="K5" s="242" t="n">
+        <v>5</v>
+      </c>
+      <c r="L5" s="242" t="n">
+        <v>17</v>
+      </c>
+      <c r="M5" s="232" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="N5" s="240" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="143">
+      <c r="A6" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe B</t>
+        </is>
+      </c>
+      <c r="B6" s="231" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C6" s="247" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D6" s="233" t="n">
+        <v>31</v>
+      </c>
+      <c r="E6" s="233" t="n">
+        <v>10</v>
+      </c>
+      <c r="F6" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="G6" s="235" t="n">
+        <v>13</v>
+      </c>
+      <c r="H6" s="236" t="inlineStr">
+        <is>
+          <t>6–0</t>
+        </is>
+      </c>
+      <c r="I6" s="237" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="234" t="n">
         <v>2</v>
       </c>
-      <c r="L5" s="241" t="n">
-        <v>8</v>
-      </c>
-      <c r="M5" s="232" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="N5" s="240" t="inlineStr">
-        <is>
-          <t>Sør-Korea</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" s="143">
-      <c r="A6" s="246" t="inlineStr"/>
-      <c r="B6" s="231" t="inlineStr">
-        <is>
-          <t>Sør-Korea</t>
-        </is>
-      </c>
-      <c r="C6" s="232" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D6" s="233" t="n">
-        <v>15</v>
-      </c>
-      <c r="E6" s="233" t="n">
-        <v>7</v>
-      </c>
-      <c r="F6" s="234" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" s="235" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="236" t="inlineStr">
-        <is>
-          <t>2–1</t>
-        </is>
-      </c>
-      <c r="I6" s="237" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="234" t="n">
-        <v>4</v>
-      </c>
-      <c r="L6" s="234" t="n">
-        <v>8</v>
-      </c>
       <c r="M6" s="238" t="n">
-        <v>0.38</v>
+        <v>0.22</v>
       </c>
       <c r="N6" s="231" t="inlineStr">
         <is>
-          <t>Tsjekkia</t>
+          <t>Qatar</t>
         </is>
       </c>
     </row>
@@ -34127,99 +34131,99 @@
       <c r="A7" s="239" t="inlineStr"/>
       <c r="B7" s="240" t="inlineStr">
         <is>
-          <t>Tsjekkia</t>
-        </is>
-      </c>
-      <c r="C7" s="238" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="D7" s="241" t="n">
-        <v>12</v>
-      </c>
-      <c r="E7" s="241" t="n">
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="C7" s="232" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D7" s="242" t="n">
+        <v>13</v>
+      </c>
+      <c r="E7" s="242" t="n">
+        <v>8</v>
+      </c>
+      <c r="F7" s="241" t="n">
         <v>3</v>
       </c>
-      <c r="F7" s="241" t="n">
-        <v>6</v>
-      </c>
       <c r="G7" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H7" s="244" t="inlineStr">
+        <is>
+          <t>4–1</t>
+        </is>
+      </c>
+      <c r="I7" s="245" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" s="241" t="n">
         <v>3</v>
       </c>
-      <c r="H7" s="244" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I7" s="245" t="n">
-        <v>8</v>
-      </c>
-      <c r="J7" s="241" t="n">
+      <c r="L7" s="241" t="n">
         <v>4</v>
       </c>
-      <c r="K7" s="242" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" s="242" t="n">
-        <v>17</v>
-      </c>
-      <c r="M7" s="232" t="n">
-        <v>0.61</v>
+      <c r="M7" s="238" t="n">
+        <v>0.38</v>
       </c>
       <c r="N7" s="240" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="143">
       <c r="A8" s="230" t="inlineStr">
         <is>
-          <t>Gruppe B</t>
+          <t>Gruppe C</t>
         </is>
       </c>
       <c r="B8" s="231" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="C8" s="232" t="n">
-        <v>0.6</v>
+        <v>0.57</v>
       </c>
       <c r="D8" s="233" t="n">
-        <v>13</v>
-      </c>
-      <c r="E8" s="234" t="n">
-        <v>3</v>
+        <v>9</v>
+      </c>
+      <c r="E8" s="233" t="n">
+        <v>5</v>
       </c>
       <c r="F8" s="234" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G8" s="235" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H8" s="236" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I8" s="237" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J8" s="234" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="233" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="234" t="n">
         <v>4</v>
       </c>
       <c r="L8" s="234" t="n">
         <v>8</v>
       </c>
       <c r="M8" s="238" t="n">
-        <v>0.4</v>
+        <v>0.43</v>
       </c>
       <c r="N8" s="231" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Haiti</t>
         </is>
       </c>
     </row>
@@ -34227,95 +34231,99 @@
       <c r="A9" s="239" t="inlineStr"/>
       <c r="B9" s="240" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C9" s="247" t="n">
+          <t>Skottland</t>
+        </is>
+      </c>
+      <c r="C9" s="238" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D9" s="241" t="n">
+        <v>6</v>
+      </c>
+      <c r="E9" s="241" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="G9" s="243" t="n">
+        <v>3</v>
+      </c>
+      <c r="H9" s="244" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I9" s="245" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="K9" s="242" t="n">
+        <v>3</v>
+      </c>
+      <c r="L9" s="242" t="n">
+        <v>12</v>
+      </c>
+      <c r="M9" s="232" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="N9" s="240" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="143">
+      <c r="A10" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe D</t>
+        </is>
+      </c>
+      <c r="B10" s="231" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="C10" s="247" t="n">
         <v>0.78</v>
       </c>
-      <c r="D9" s="242" t="n">
-        <v>31</v>
-      </c>
-      <c r="E9" s="242" t="n">
-        <v>10</v>
-      </c>
-      <c r="F9" s="241" t="n">
-        <v>8</v>
-      </c>
-      <c r="G9" s="243" t="n">
-        <v>13</v>
-      </c>
-      <c r="H9" s="244" t="inlineStr">
-        <is>
-          <t>6–0</t>
-        </is>
-      </c>
-      <c r="I9" s="245" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="241" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="241" t="n">
-        <v>0</v>
-      </c>
-      <c r="L9" s="241" t="n">
+      <c r="D10" s="233" t="n">
+        <v>33</v>
+      </c>
+      <c r="E10" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F10" s="234" t="n">
+        <v>15</v>
+      </c>
+      <c r="G10" s="235" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" s="236" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I10" s="237" t="n">
         <v>2</v>
       </c>
-      <c r="M9" s="238" t="n">
+      <c r="J10" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="L10" s="234" t="n">
+        <v>6</v>
+      </c>
+      <c r="M10" s="238" t="n">
         <v>0.22</v>
       </c>
-      <c r="N9" s="240" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="143">
-      <c r="A10" s="246" t="inlineStr"/>
-      <c r="B10" s="231" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="C10" s="238" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D10" s="234" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="235" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="236" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I10" s="237" t="n">
-        <v>9</v>
-      </c>
-      <c r="J10" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="K10" s="233" t="n">
-        <v>10</v>
-      </c>
-      <c r="L10" s="233" t="n">
-        <v>27</v>
-      </c>
-      <c r="M10" s="247" t="n">
-        <v>0.7</v>
-      </c>
       <c r="N10" s="231" t="inlineStr">
         <is>
-          <t>Sveits</t>
+          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -34323,199 +34331,199 @@
       <c r="A11" s="239" t="inlineStr"/>
       <c r="B11" s="240" t="inlineStr">
         <is>
-          <t>Sveits</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C11" s="232" t="n">
-        <v>0.62</v>
+        <v>0.57</v>
       </c>
       <c r="D11" s="242" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="E11" s="242" t="n">
+        <v>7</v>
+      </c>
+      <c r="F11" s="241" t="n">
+        <v>7</v>
+      </c>
+      <c r="G11" s="243" t="n">
+        <v>3</v>
+      </c>
+      <c r="H11" s="244" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="I11" s="245" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="K11" s="241" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="241" t="n">
+        <v>6</v>
+      </c>
+      <c r="M11" s="238" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="N11" s="240" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="143">
+      <c r="A12" s="246" t="inlineStr"/>
+      <c r="B12" s="231" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C12" s="232" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D12" s="233" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="243" t="n">
+      <c r="E12" s="234" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="244" t="inlineStr">
-        <is>
-          <t>4–1</t>
-        </is>
-      </c>
-      <c r="I11" s="245" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="241" t="n">
+      <c r="F12" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="235" t="n">
+        <v>5</v>
+      </c>
+      <c r="H12" s="236" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I12" s="237" t="n">
         <v>0</v>
-      </c>
-      <c r="K11" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" s="238" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N11" s="240" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="143">
-      <c r="A12" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe C</t>
-        </is>
-      </c>
-      <c r="B12" s="231" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C12" s="248" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D12" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" s="233" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" s="234" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="235" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="236" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I12" s="237" t="n">
-        <v>6</v>
       </c>
       <c r="J12" s="234" t="n">
         <v>3</v>
       </c>
       <c r="K12" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="L12" s="234" t="n">
+        <v>5</v>
+      </c>
+      <c r="M12" s="238" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="N12" s="231" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="143">
+      <c r="A13" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="B13" s="240" t="inlineStr">
+        <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="C13" s="248" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D13" s="242" t="n">
+        <v>12</v>
+      </c>
+      <c r="E13" s="242" t="n">
+        <v>5</v>
+      </c>
+      <c r="F13" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="G13" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H13" s="244" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="I13" s="245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J13" s="241" t="n">
         <v>4</v>
       </c>
-      <c r="L12" s="233" t="n">
-        <v>13</v>
-      </c>
-      <c r="M12" s="248" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="N12" s="231" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="143">
-      <c r="A13" s="239" t="inlineStr"/>
-      <c r="B13" s="240" t="inlineStr">
-        <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-      <c r="C13" s="248" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D13" s="242" t="n">
-        <v>13</v>
-      </c>
-      <c r="E13" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="F13" s="241" t="n">
-        <v>7</v>
-      </c>
-      <c r="G13" s="243" t="n">
-        <v>3</v>
-      </c>
-      <c r="H13" s="244" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="I13" s="245" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="241" t="n">
-        <v>3</v>
-      </c>
       <c r="K13" s="241" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L13" s="241" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="M13" s="248" t="n">
-        <v>0.5</v>
+        <v>0.51</v>
       </c>
       <c r="N13" s="240" t="inlineStr">
         <is>
-          <t>Skottland</t>
+          <t>Ecuador</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" s="143">
       <c r="A14" s="230" t="inlineStr">
         <is>
-          <t>Gruppe D</t>
+          <t>Gruppe G</t>
         </is>
       </c>
       <c r="B14" s="231" t="inlineStr">
         <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C14" s="238" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D14" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="E14" s="234" t="n">
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="C14" s="232" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D14" s="233" t="n">
+        <v>14</v>
+      </c>
+      <c r="E14" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F14" s="234" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="235" t="n">
+        <v>3</v>
+      </c>
+      <c r="H14" s="236" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I14" s="237" t="n">
+        <v>2</v>
+      </c>
+      <c r="J14" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="234" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" s="235" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="236" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I14" s="237" t="n">
-        <v>11</v>
-      </c>
-      <c r="J14" s="234" t="n">
-        <v>10</v>
-      </c>
-      <c r="K14" s="233" t="n">
-        <v>7</v>
-      </c>
-      <c r="L14" s="233" t="n">
-        <v>28</v>
-      </c>
-      <c r="M14" s="232" t="n">
-        <v>0.63</v>
+      <c r="L14" s="234" t="n">
+        <v>9</v>
+      </c>
+      <c r="M14" s="238" t="n">
+        <v>0.44</v>
       </c>
       <c r="N14" s="231" t="inlineStr">
         <is>
-          <t>Tyrkia</t>
+          <t>Egypt</t>
         </is>
       </c>
     </row>
@@ -34523,199 +34531,203 @@
       <c r="A15" s="239" t="inlineStr"/>
       <c r="B15" s="240" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C15" s="232" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="D15" s="242" t="n">
-        <v>17</v>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C15" s="248" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D15" s="241" t="n">
+        <v>10</v>
       </c>
       <c r="E15" s="242" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F15" s="241" t="n">
+        <v>4</v>
+      </c>
+      <c r="G15" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="244" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I15" s="245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J15" s="241" t="n">
         <v>5</v>
       </c>
-      <c r="G15" s="243" t="n">
-        <v>6</v>
-      </c>
-      <c r="H15" s="244" t="inlineStr">
-        <is>
-          <t>4–1</t>
-        </is>
-      </c>
-      <c r="I15" s="245" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="241" t="n">
-        <v>2</v>
-      </c>
       <c r="K15" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="L15" s="241" t="n">
-        <v>8</v>
-      </c>
-      <c r="M15" s="238" t="n">
-        <v>0.37</v>
+        <v>3</v>
+      </c>
+      <c r="L15" s="242" t="n">
+        <v>11</v>
+      </c>
+      <c r="M15" s="248" t="n">
+        <v>0.52</v>
       </c>
       <c r="N15" s="240" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="143">
       <c r="A16" s="230" t="inlineStr">
         <is>
-          <t>Gruppe E</t>
+          <t>Gruppe H</t>
         </is>
       </c>
       <c r="B16" s="231" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-      <c r="C16" s="248" t="n">
-        <v>0.49</v>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C16" s="247" t="n">
+        <v>0.74</v>
       </c>
       <c r="D16" s="233" t="n">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="E16" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="234" t="n">
+        <v>12</v>
+      </c>
+      <c r="G16" s="235" t="n">
+        <v>6</v>
+      </c>
+      <c r="H16" s="236" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I16" s="237" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="K16" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" s="234" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="234" t="n">
-        <v>9</v>
-      </c>
-      <c r="G16" s="235" t="n">
+      <c r="M16" s="238" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="N16" s="231" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="143">
+      <c r="A17" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
+      <c r="B17" s="240" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C17" s="238" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D17" s="241" t="n">
+        <v>7</v>
+      </c>
+      <c r="E17" s="241" t="n">
         <v>3</v>
       </c>
-      <c r="H16" s="236" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I16" s="237" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="K16" s="234" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" s="234" t="n">
-        <v>10</v>
-      </c>
-      <c r="M16" s="248" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="N16" s="231" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="143">
-      <c r="A17" s="239" t="inlineStr"/>
-      <c r="B17" s="240" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="C17" s="247" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D17" s="242" t="n">
-        <v>26</v>
-      </c>
-      <c r="E17" s="242" t="n">
-        <v>11</v>
-      </c>
       <c r="F17" s="241" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G17" s="243" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H17" s="244" t="inlineStr">
         <is>
-          <t>7–1</t>
+          <t>1–3</t>
         </is>
       </c>
       <c r="I17" s="245" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J17" s="241" t="n">
         <v>5</v>
       </c>
-      <c r="K17" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="L17" s="241" t="n">
-        <v>7</v>
-      </c>
-      <c r="M17" s="238" t="n">
-        <v>0.35</v>
+      <c r="K17" s="242" t="n">
+        <v>6</v>
+      </c>
+      <c r="L17" s="242" t="n">
+        <v>15</v>
+      </c>
+      <c r="M17" s="247" t="n">
+        <v>0.67</v>
       </c>
       <c r="N17" s="240" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Colombia</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="143">
       <c r="A18" s="230" t="inlineStr">
         <is>
-          <t>Gruppe F</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="B18" s="231" t="inlineStr">
         <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="C18" s="232" t="n">
-        <v>0.6</v>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C18" s="247" t="n">
+        <v>0.65</v>
       </c>
       <c r="D18" s="233" t="n">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="E18" s="233" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" s="234" t="n">
+        <v>9</v>
+      </c>
+      <c r="G18" s="235" t="n">
+        <v>5</v>
+      </c>
+      <c r="H18" s="236" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I18" s="237" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" s="234" t="n">
+        <v>4</v>
+      </c>
+      <c r="K18" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="L18" s="234" t="n">
         <v>7</v>
       </c>
-      <c r="F18" s="234" t="n">
-        <v>4</v>
-      </c>
-      <c r="G18" s="235" t="n">
-        <v>0</v>
-      </c>
-      <c r="H18" s="236" t="inlineStr">
-        <is>
-          <t>2–2</t>
-        </is>
-      </c>
-      <c r="I18" s="237" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="234" t="n">
-        <v>5</v>
-      </c>
-      <c r="K18" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="L18" s="234" t="n">
-        <v>8</v>
-      </c>
       <c r="M18" s="238" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="N18" s="231" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Kroatia</t>
         </is>
       </c>
     </row>
@@ -34723,679 +34735,79 @@
       <c r="A19" s="239" t="inlineStr"/>
       <c r="B19" s="240" t="inlineStr">
         <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-      <c r="C19" s="248" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="D19" s="242" t="n">
-        <v>13</v>
-      </c>
-      <c r="E19" s="242" t="n">
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C19" s="238" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D19" s="241" t="n">
         <v>8</v>
       </c>
+      <c r="E19" s="241" t="n">
+        <v>3</v>
+      </c>
       <c r="F19" s="241" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G19" s="243" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="244" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I19" s="245" t="n">
         <v>2</v>
       </c>
-      <c r="H19" s="244" t="inlineStr">
-        <is>
-          <t>5–1</t>
-        </is>
-      </c>
-      <c r="I19" s="245" t="n">
-        <v>1</v>
-      </c>
       <c r="J19" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="K19" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="241" t="n">
         <v>5</v>
       </c>
-      <c r="M19" s="248" t="n">
-        <v>0.51</v>
+      <c r="K19" s="242" t="n">
+        <v>4</v>
+      </c>
+      <c r="L19" s="242" t="n">
+        <v>11</v>
+      </c>
+      <c r="M19" s="232" t="n">
+        <v>0.63</v>
       </c>
       <c r="N19" s="240" t="inlineStr">
         <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="143">
-      <c r="A20" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe G</t>
-        </is>
-      </c>
-      <c r="B20" s="231" t="inlineStr">
-        <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C20" s="248" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="D20" s="233" t="n">
-        <v>15</v>
-      </c>
-      <c r="E20" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="F20" s="234" t="n">
-        <v>7</v>
-      </c>
-      <c r="G20" s="235" t="n">
-        <v>5</v>
-      </c>
-      <c r="H20" s="236" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I20" s="237" t="n">
-        <v>8</v>
-      </c>
-      <c r="J20" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="233" t="n">
-        <v>4</v>
-      </c>
-      <c r="L20" s="234" t="n">
-        <v>14</v>
-      </c>
-      <c r="M20" s="248" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="N20" s="231" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1" s="143">
-      <c r="A21" s="239" t="inlineStr"/>
-      <c r="B21" s="240" t="inlineStr">
-        <is>
-          <t>Iran</t>
-        </is>
-      </c>
-      <c r="C21" s="248" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D21" s="242" t="n">
-        <v>17</v>
-      </c>
-      <c r="E21" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="F21" s="241" t="n">
-        <v>8</v>
-      </c>
-      <c r="G21" s="243" t="n">
-        <v>5</v>
-      </c>
-      <c r="H21" s="244" t="inlineStr">
-        <is>
-          <t>2–2</t>
-        </is>
-      </c>
-      <c r="I21" s="245" t="n">
-        <v>3</v>
-      </c>
-      <c r="J21" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" s="242" t="n">
-        <v>8</v>
-      </c>
-      <c r="L21" s="241" t="n">
-        <v>13</v>
-      </c>
-      <c r="M21" s="248" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N21" s="240" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
+          <t>Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="14" customHeight="1" s="143">
+      <c r="A21" s="227" t="inlineStr">
+        <is>
+          <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
     <row r="22" ht="18" customHeight="1" s="143">
-      <c r="A22" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe H</t>
-        </is>
-      </c>
-      <c r="B22" s="231" t="inlineStr">
-        <is>
-          <t>Saudi-Arabia</t>
-        </is>
-      </c>
-      <c r="C22" s="238" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D22" s="234" t="n">
-        <v>7</v>
-      </c>
-      <c r="E22" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="G22" s="235" t="n">
-        <v>1</v>
-      </c>
-      <c r="H22" s="236" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I22" s="237" t="n">
-        <v>9</v>
-      </c>
-      <c r="J22" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="K22" s="233" t="n">
-        <v>10</v>
-      </c>
-      <c r="L22" s="233" t="n">
-        <v>27</v>
-      </c>
-      <c r="M22" s="247" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="N22" s="231" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="18" customHeight="1" s="143">
-      <c r="A23" s="239" t="inlineStr"/>
-      <c r="B23" s="240" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C23" s="247" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="D23" s="242" t="n">
-        <v>23</v>
-      </c>
-      <c r="E23" s="242" t="n">
-        <v>8</v>
-      </c>
-      <c r="F23" s="241" t="n">
-        <v>9</v>
-      </c>
-      <c r="G23" s="243" t="n">
-        <v>6</v>
-      </c>
-      <c r="H23" s="244" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I23" s="245" t="n">
-        <v>2</v>
-      </c>
-      <c r="J23" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="K23" s="241" t="n">
-        <v>1</v>
-      </c>
-      <c r="L23" s="241" t="n">
-        <v>6</v>
-      </c>
-      <c r="M23" s="238" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="N23" s="240" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1" s="143">
-      <c r="A24" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe I</t>
-        </is>
-      </c>
-      <c r="B24" s="231" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C24" s="248" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D24" s="233" t="n">
-        <v>11</v>
-      </c>
-      <c r="E24" s="233" t="n">
-        <v>8</v>
-      </c>
-      <c r="F24" s="234" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="235" t="n">
-        <v>2</v>
-      </c>
-      <c r="H24" s="236" t="inlineStr">
-        <is>
-          <t>3–1</t>
-        </is>
-      </c>
-      <c r="I24" s="237" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="K24" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" s="234" t="n">
-        <v>6</v>
-      </c>
-      <c r="M24" s="248" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="N24" s="231" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1" s="143">
-      <c r="A25" s="239" t="inlineStr"/>
-      <c r="B25" s="240" t="inlineStr">
-        <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="C25" s="238" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D25" s="241" t="n">
-        <v>11</v>
-      </c>
-      <c r="E25" s="241" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="241" t="n">
-        <v>8</v>
-      </c>
-      <c r="G25" s="243" t="n">
-        <v>2</v>
-      </c>
-      <c r="H25" s="244" t="inlineStr">
-        <is>
-          <t>1–4</t>
-        </is>
-      </c>
-      <c r="I25" s="245" t="n">
-        <v>2</v>
-      </c>
-      <c r="J25" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="K25" s="242" t="n">
-        <v>6</v>
-      </c>
-      <c r="L25" s="242" t="n">
-        <v>12</v>
-      </c>
-      <c r="M25" s="232" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="N25" s="240" t="inlineStr">
-        <is>
-          <t>Norge</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1" s="143">
-      <c r="A26" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe J</t>
-        </is>
-      </c>
-      <c r="B26" s="231" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C26" s="248" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D26" s="233" t="n">
-        <v>9</v>
-      </c>
-      <c r="E26" s="233" t="n">
-        <v>6</v>
-      </c>
-      <c r="F26" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="G26" s="235" t="n">
-        <v>0</v>
-      </c>
-      <c r="H26" s="236" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I26" s="237" t="n">
-        <v>3</v>
-      </c>
-      <c r="J26" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="K26" s="234" t="n">
-        <v>0</v>
-      </c>
-      <c r="L26" s="234" t="n">
-        <v>6</v>
-      </c>
-      <c r="M26" s="248" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N26" s="231" t="inlineStr">
-        <is>
-          <t>Algerie</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="18" customHeight="1" s="143">
-      <c r="A27" s="239" t="inlineStr"/>
-      <c r="B27" s="240" t="inlineStr">
-        <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C27" s="232" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D27" s="241" t="n">
-        <v>9</v>
-      </c>
-      <c r="E27" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="F27" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="G27" s="243" t="n">
-        <v>2</v>
-      </c>
-      <c r="H27" s="244" t="inlineStr">
-        <is>
-          <t>3–1</t>
-        </is>
-      </c>
-      <c r="I27" s="245" t="n">
-        <v>3</v>
-      </c>
-      <c r="J27" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="K27" s="242" t="n">
-        <v>4</v>
-      </c>
-      <c r="L27" s="242" t="n">
-        <v>11</v>
-      </c>
-      <c r="M27" s="238" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N27" s="240" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1" s="143">
-      <c r="A28" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe K</t>
-        </is>
-      </c>
-      <c r="B28" s="231" t="inlineStr">
-        <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C28" s="247" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D28" s="233" t="n">
-        <v>9</v>
-      </c>
-      <c r="E28" s="233" t="n">
-        <v>3</v>
-      </c>
-      <c r="F28" s="234" t="n">
-        <v>4</v>
-      </c>
-      <c r="G28" s="235" t="n">
-        <v>2</v>
-      </c>
-      <c r="H28" s="236" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I28" s="237" t="n">
-        <v>3</v>
-      </c>
-      <c r="J28" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="L28" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="M28" s="238" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N28" s="231" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="18" customHeight="1" s="143">
-      <c r="A29" s="239" t="inlineStr"/>
-      <c r="B29" s="240" t="inlineStr">
-        <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C29" s="238" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D29" s="241" t="n">
-        <v>7</v>
-      </c>
-      <c r="E29" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="F29" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="G29" s="243" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="244" t="inlineStr">
-        <is>
-          <t>1–3</t>
-        </is>
-      </c>
-      <c r="I29" s="245" t="n">
-        <v>4</v>
-      </c>
-      <c r="J29" s="241" t="n">
-        <v>5</v>
-      </c>
-      <c r="K29" s="242" t="n">
-        <v>6</v>
-      </c>
-      <c r="L29" s="242" t="n">
-        <v>15</v>
-      </c>
-      <c r="M29" s="247" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="N29" s="240" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1" s="143">
-      <c r="A30" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe L</t>
-        </is>
-      </c>
-      <c r="B30" s="231" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C30" s="248" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D30" s="233" t="n">
-        <v>20</v>
-      </c>
-      <c r="E30" s="233" t="n">
-        <v>12</v>
-      </c>
-      <c r="F30" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="G30" s="235" t="n">
-        <v>5</v>
-      </c>
-      <c r="H30" s="236" t="inlineStr">
-        <is>
-          <t>4–2</t>
-        </is>
-      </c>
-      <c r="I30" s="237" t="n">
-        <v>3</v>
-      </c>
-      <c r="J30" s="234" t="n">
-        <v>3</v>
-      </c>
-      <c r="K30" s="234" t="n">
-        <v>5</v>
-      </c>
-      <c r="L30" s="234" t="n">
-        <v>11</v>
-      </c>
-      <c r="M30" s="248" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="N30" s="231" t="inlineStr">
-        <is>
-          <t>Kroatia</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1" s="143">
-      <c r="A31" s="239" t="inlineStr"/>
-      <c r="B31" s="240" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="C31" s="238" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D31" s="241" t="n">
-        <v>8</v>
-      </c>
-      <c r="E31" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="F31" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="G31" s="243" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" s="244" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I31" s="245" t="n">
-        <v>2</v>
-      </c>
-      <c r="J31" s="241" t="n">
-        <v>5</v>
-      </c>
-      <c r="K31" s="242" t="n">
-        <v>4</v>
-      </c>
-      <c r="L31" s="242" t="n">
-        <v>11</v>
-      </c>
-      <c r="M31" s="232" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="N31" s="240" t="inlineStr">
-        <is>
-          <t>Panama</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="14" customHeight="1" s="143">
-      <c r="A33" s="227" t="inlineStr">
-        <is>
-          <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1" s="143">
-      <c r="A34" s="219" t="inlineStr">
+      <c r="A22" s="219" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B34" s="226" t="inlineStr">
+      <c r="B22" s="226" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C34" s="225" t="inlineStr">
+      <c r="C22" s="225" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D34" s="222" t="inlineStr">
+      <c r="D22" s="222" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E34" s="249" t="inlineStr">
+      <c r="E22" s="249" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -35404,7 +34816,7 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A33:N33"/>
+    <mergeCell ref="A21:N21"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Oppdater Ballbesittelse-ark med verifiserte kampdata (wc2026_stats3.json)
- Bytter kilde til wc2026_stats3.json: 32 kamper fra runde 1 og 2,
  alle verifisert via SportRadar Soccer API v4
- Fikser home/away-reversert matching i bygg_data()
- Fjerner feil kampdata fra wc2026_stats.json (gamle SportRadar-IDer
  returnerte feil lag)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -39096,7 +39096,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N22"/>
+  <dimension ref="A1:N38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="143" min="1" max="1"/>
@@ -39219,44 +39219,44 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="C4" s="238" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="D4" s="234" t="n">
-        <v>8</v>
+      <c r="C4" s="232" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="D4" s="233" t="n">
+        <v>16</v>
       </c>
       <c r="E4" s="233" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" s="234" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G4" s="235" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H4" s="236" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I4" s="237" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J4" s="234" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K4" s="234" t="n">
         <v>2</v>
       </c>
       <c r="L4" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="M4" s="232" t="n">
-        <v>0.57</v>
+        <v>3</v>
+      </c>
+      <c r="M4" s="238" t="n">
+        <v>0.39</v>
       </c>
       <c r="N4" s="231" t="inlineStr">
         <is>
-          <t>Sør-Korea</t>
+          <t>Sør-Afrika</t>
         </is>
       </c>
     </row>
@@ -39264,99 +39264,95 @@
       <c r="A5" s="239" t="inlineStr"/>
       <c r="B5" s="240" t="inlineStr">
         <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C5" s="238" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D5" s="241" t="n">
+        <v>8</v>
+      </c>
+      <c r="E5" s="242" t="n">
+        <v>4</v>
+      </c>
+      <c r="F5" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" s="243" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" s="244" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I5" s="245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L5" s="241" t="n">
+        <v>8</v>
+      </c>
+      <c r="M5" s="232" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="N5" s="240" t="inlineStr">
+        <is>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="143">
+      <c r="A6" s="246" t="inlineStr"/>
+      <c r="B6" s="231" t="inlineStr">
+        <is>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+      <c r="C6" s="232" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D6" s="233" t="n">
+        <v>15</v>
+      </c>
+      <c r="E6" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F6" s="234" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="235" t="n">
+        <v>3</v>
+      </c>
+      <c r="H6" s="236" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="I6" s="237" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="234" t="n">
+        <v>4</v>
+      </c>
+      <c r="L6" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="M6" s="238" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N6" s="231" t="inlineStr">
+        <is>
           <t>Tsjekkia</t>
-        </is>
-      </c>
-      <c r="C5" s="238" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="D5" s="241" t="n">
-        <v>12</v>
-      </c>
-      <c r="E5" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="F5" s="241" t="n">
-        <v>6</v>
-      </c>
-      <c r="G5" s="243" t="n">
-        <v>3</v>
-      </c>
-      <c r="H5" s="244" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I5" s="245" t="n">
-        <v>8</v>
-      </c>
-      <c r="J5" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="K5" s="242" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" s="242" t="n">
-        <v>17</v>
-      </c>
-      <c r="M5" s="232" t="n">
-        <v>0.61</v>
-      </c>
-      <c r="N5" s="240" t="inlineStr">
-        <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="18" customHeight="1" s="143">
-      <c r="A6" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe B</t>
-        </is>
-      </c>
-      <c r="B6" s="231" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C6" s="247" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="D6" s="233" t="n">
-        <v>31</v>
-      </c>
-      <c r="E6" s="233" t="n">
-        <v>10</v>
-      </c>
-      <c r="F6" s="234" t="n">
-        <v>8</v>
-      </c>
-      <c r="G6" s="235" t="n">
-        <v>13</v>
-      </c>
-      <c r="H6" s="236" t="inlineStr">
-        <is>
-          <t>6–0</t>
-        </is>
-      </c>
-      <c r="I6" s="237" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="234" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="234" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="M6" s="238" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="N6" s="231" t="inlineStr">
-        <is>
-          <t>Qatar</t>
         </is>
       </c>
     </row>
@@ -39364,99 +39360,99 @@
       <c r="A7" s="239" t="inlineStr"/>
       <c r="B7" s="240" t="inlineStr">
         <is>
-          <t>Sveits</t>
-        </is>
-      </c>
-      <c r="C7" s="232" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D7" s="242" t="n">
-        <v>13</v>
-      </c>
-      <c r="E7" s="242" t="n">
+          <t>Tsjekkia</t>
+        </is>
+      </c>
+      <c r="C7" s="238" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="D7" s="241" t="n">
+        <v>12</v>
+      </c>
+      <c r="E7" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="F7" s="241" t="n">
+        <v>6</v>
+      </c>
+      <c r="G7" s="243" t="n">
+        <v>3</v>
+      </c>
+      <c r="H7" s="244" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I7" s="245" t="n">
         <v>8</v>
       </c>
-      <c r="F7" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="G7" s="243" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" s="244" t="inlineStr">
-        <is>
-          <t>4–1</t>
-        </is>
-      </c>
-      <c r="I7" s="245" t="n">
-        <v>1</v>
-      </c>
       <c r="J7" s="241" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" s="241" t="n">
         <v>4</v>
       </c>
-      <c r="M7" s="238" t="n">
-        <v>0.38</v>
+      <c r="K7" s="242" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="242" t="n">
+        <v>17</v>
+      </c>
+      <c r="M7" s="232" t="n">
+        <v>0.61</v>
       </c>
       <c r="N7" s="240" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Sør-Afrika</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="143">
       <c r="A8" s="230" t="inlineStr">
         <is>
-          <t>Gruppe C</t>
+          <t>Gruppe B</t>
         </is>
       </c>
       <c r="B8" s="231" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C8" s="232" t="n">
-        <v>0.57</v>
+        <v>0.6</v>
       </c>
       <c r="D8" s="233" t="n">
-        <v>9</v>
-      </c>
-      <c r="E8" s="233" t="n">
+        <v>13</v>
+      </c>
+      <c r="E8" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="F8" s="234" t="n">
         <v>5</v>
       </c>
-      <c r="F8" s="234" t="n">
-        <v>2</v>
-      </c>
       <c r="G8" s="235" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H8" s="236" t="inlineStr">
         <is>
-          <t>3–0</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I8" s="237" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J8" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="234" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="233" t="n">
         <v>4</v>
       </c>
       <c r="L8" s="234" t="n">
         <v>8</v>
       </c>
       <c r="M8" s="238" t="n">
-        <v>0.43</v>
+        <v>0.4</v>
       </c>
       <c r="N8" s="231" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
     </row>
@@ -39464,99 +39460,95 @@
       <c r="A9" s="239" t="inlineStr"/>
       <c r="B9" s="240" t="inlineStr">
         <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-      <c r="C9" s="238" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D9" s="241" t="n">
-        <v>6</v>
-      </c>
-      <c r="E9" s="241" t="n">
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C9" s="247" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D9" s="242" t="n">
+        <v>31</v>
+      </c>
+      <c r="E9" s="242" t="n">
+        <v>10</v>
+      </c>
+      <c r="F9" s="241" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="243" t="n">
+        <v>13</v>
+      </c>
+      <c r="H9" s="244" t="inlineStr">
+        <is>
+          <t>6–0</t>
+        </is>
+      </c>
+      <c r="I9" s="245" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" s="241" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="241" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="241" t="n">
+      <c r="L9" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="M9" s="238" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N9" s="240" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="143">
+      <c r="A10" s="246" t="inlineStr"/>
+      <c r="B10" s="231" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="C10" s="238" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D10" s="234" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="234" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="243" t="n">
-        <v>3</v>
-      </c>
-      <c r="H9" s="244" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="I9" s="245" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" s="241" t="n">
-        <v>5</v>
-      </c>
-      <c r="K9" s="242" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" s="242" t="n">
-        <v>12</v>
-      </c>
-      <c r="M9" s="232" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="N9" s="240" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="143">
-      <c r="A10" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe D</t>
-        </is>
-      </c>
-      <c r="B10" s="231" t="inlineStr">
-        <is>
-          <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="C10" s="247" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="D10" s="233" t="n">
-        <v>33</v>
-      </c>
-      <c r="E10" s="233" t="n">
-        <v>6</v>
-      </c>
       <c r="F10" s="234" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G10" s="235" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="H10" s="236" t="inlineStr">
         <is>
-          <t>0–1</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I10" s="237" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J10" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="K10" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="L10" s="234" t="n">
-        <v>6</v>
-      </c>
-      <c r="M10" s="238" t="n">
-        <v>0.22</v>
+        <v>8</v>
+      </c>
+      <c r="K10" s="233" t="n">
+        <v>10</v>
+      </c>
+      <c r="L10" s="233" t="n">
+        <v>27</v>
+      </c>
+      <c r="M10" s="247" t="n">
+        <v>0.7</v>
       </c>
       <c r="N10" s="231" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Sveits</t>
         </is>
       </c>
     </row>
@@ -39564,179 +39556,175 @@
       <c r="A11" s="239" t="inlineStr"/>
       <c r="B11" s="240" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Sveits</t>
         </is>
       </c>
       <c r="C11" s="232" t="n">
-        <v>0.57</v>
+        <v>0.62</v>
       </c>
       <c r="D11" s="242" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E11" s="242" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F11" s="241" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G11" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H11" s="244" t="inlineStr">
+        <is>
+          <t>4–1</t>
+        </is>
+      </c>
+      <c r="I11" s="245" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="241" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="241" t="n">
         <v>3</v>
       </c>
-      <c r="H11" s="244" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I11" s="245" t="n">
+      <c r="L11" s="241" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" s="238" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N11" s="240" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="143">
+      <c r="A12" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe C</t>
+        </is>
+      </c>
+      <c r="B12" s="231" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C12" s="248" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D12" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="E12" s="233" t="n">
+        <v>5</v>
+      </c>
+      <c r="F12" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="235" t="n">
         <v>2</v>
       </c>
-      <c r="J11" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="K11" s="241" t="n">
-        <v>1</v>
-      </c>
-      <c r="L11" s="241" t="n">
+      <c r="H12" s="236" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I12" s="237" t="n">
         <v>6</v>
-      </c>
-      <c r="M11" s="238" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="N11" s="240" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="143">
-      <c r="A12" s="246" t="inlineStr"/>
-      <c r="B12" s="231" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C12" s="232" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="D12" s="233" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" s="234" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="235" t="n">
-        <v>5</v>
-      </c>
-      <c r="H12" s="236" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I12" s="237" t="n">
-        <v>0</v>
       </c>
       <c r="J12" s="234" t="n">
         <v>3</v>
       </c>
       <c r="K12" s="234" t="n">
-        <v>2</v>
-      </c>
-      <c r="L12" s="234" t="n">
-        <v>5</v>
-      </c>
-      <c r="M12" s="238" t="n">
-        <v>0.37</v>
+        <v>4</v>
+      </c>
+      <c r="L12" s="233" t="n">
+        <v>13</v>
+      </c>
+      <c r="M12" s="248" t="n">
+        <v>0.46</v>
       </c>
       <c r="N12" s="231" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1" s="143">
-      <c r="A13" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe E</t>
-        </is>
-      </c>
+      <c r="A13" s="239" t="inlineStr"/>
       <c r="B13" s="240" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-      <c r="C13" s="248" t="n">
-        <v>0.49</v>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C13" s="232" t="n">
+        <v>0.57</v>
       </c>
       <c r="D13" s="242" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="E13" s="242" t="n">
         <v>5</v>
       </c>
       <c r="F13" s="241" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="G13" s="243" t="n">
         <v>2</v>
       </c>
       <c r="H13" s="244" t="inlineStr">
         <is>
-          <t>2–1</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I13" s="245" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J13" s="241" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K13" s="241" t="n">
         <v>4</v>
       </c>
       <c r="L13" s="241" t="n">
-        <v>11</v>
-      </c>
-      <c r="M13" s="248" t="n">
-        <v>0.51</v>
+        <v>8</v>
+      </c>
+      <c r="M13" s="238" t="n">
+        <v>0.43</v>
       </c>
       <c r="N13" s="240" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Haiti</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1" s="143">
-      <c r="A14" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe G</t>
-        </is>
-      </c>
+      <c r="A14" s="246" t="inlineStr"/>
       <c r="B14" s="231" t="inlineStr">
         <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C14" s="232" t="n">
-        <v>0.5600000000000001</v>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="C14" s="248" t="n">
+        <v>0.5</v>
       </c>
       <c r="D14" s="233" t="n">
-        <v>14</v>
-      </c>
-      <c r="E14" s="233" t="n">
-        <v>5</v>
+        <v>13</v>
+      </c>
+      <c r="E14" s="234" t="n">
+        <v>3</v>
       </c>
       <c r="F14" s="234" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G14" s="235" t="n">
         <v>3</v>
       </c>
       <c r="H14" s="236" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>0–1</t>
         </is>
       </c>
       <c r="I14" s="237" t="n">
@@ -39746,17 +39734,17 @@
         <v>3</v>
       </c>
       <c r="K14" s="234" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L14" s="234" t="n">
-        <v>9</v>
-      </c>
-      <c r="M14" s="238" t="n">
-        <v>0.44</v>
+        <v>8</v>
+      </c>
+      <c r="M14" s="248" t="n">
+        <v>0.5</v>
       </c>
       <c r="N14" s="231" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Skottland</t>
         </is>
       </c>
     </row>
@@ -39764,203 +39752,195 @@
       <c r="A15" s="239" t="inlineStr"/>
       <c r="B15" s="240" t="inlineStr">
         <is>
-          <t>Iran</t>
-        </is>
-      </c>
-      <c r="C15" s="248" t="n">
-        <v>0.48</v>
+          <t>Skottland</t>
+        </is>
+      </c>
+      <c r="C15" s="238" t="n">
+        <v>0.4</v>
       </c>
       <c r="D15" s="241" t="n">
-        <v>10</v>
-      </c>
-      <c r="E15" s="242" t="n">
+        <v>6</v>
+      </c>
+      <c r="E15" s="241" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="243" t="n">
+        <v>3</v>
+      </c>
+      <c r="H15" s="244" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I15" s="245" t="n">
         <v>4</v>
-      </c>
-      <c r="F15" s="241" t="n">
-        <v>4</v>
-      </c>
-      <c r="G15" s="243" t="n">
-        <v>2</v>
-      </c>
-      <c r="H15" s="244" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I15" s="245" t="n">
-        <v>3</v>
       </c>
       <c r="J15" s="241" t="n">
         <v>5</v>
       </c>
-      <c r="K15" s="241" t="n">
+      <c r="K15" s="242" t="n">
         <v>3</v>
       </c>
       <c r="L15" s="242" t="n">
-        <v>11</v>
-      </c>
-      <c r="M15" s="248" t="n">
-        <v>0.52</v>
+        <v>12</v>
+      </c>
+      <c r="M15" s="232" t="n">
+        <v>0.6</v>
       </c>
       <c r="N15" s="240" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="143">
       <c r="A16" s="230" t="inlineStr">
         <is>
-          <t>Gruppe H</t>
+          <t>Gruppe D</t>
         </is>
       </c>
       <c r="B16" s="231" t="inlineStr">
         <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C16" s="247" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="D16" s="233" t="n">
-        <v>24</v>
-      </c>
-      <c r="E16" s="233" t="n">
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C16" s="238" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D16" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="E16" s="234" t="n">
+        <v>4</v>
+      </c>
+      <c r="F16" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="235" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="236" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I16" s="237" t="n">
+        <v>11</v>
+      </c>
+      <c r="J16" s="234" t="n">
+        <v>10</v>
+      </c>
+      <c r="K16" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="L16" s="233" t="n">
+        <v>28</v>
+      </c>
+      <c r="M16" s="232" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N16" s="231" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="143">
+      <c r="A17" s="239" t="inlineStr"/>
+      <c r="B17" s="240" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="C17" s="247" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D17" s="242" t="n">
+        <v>33</v>
+      </c>
+      <c r="E17" s="242" t="n">
         <v>6</v>
       </c>
-      <c r="F16" s="234" t="n">
+      <c r="F17" s="241" t="n">
+        <v>15</v>
+      </c>
+      <c r="G17" s="243" t="n">
         <v>12</v>
       </c>
-      <c r="G16" s="235" t="n">
+      <c r="H17" s="244" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I17" s="245" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="K17" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" s="241" t="n">
         <v>6</v>
       </c>
-      <c r="H16" s="236" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I16" s="237" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="234" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="234" t="n">
+      <c r="M17" s="238" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N17" s="240" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="143">
+      <c r="A18" s="246" t="inlineStr"/>
+      <c r="B18" s="231" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C18" s="232" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D18" s="233" t="n">
+        <v>17</v>
+      </c>
+      <c r="E18" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F18" s="234" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" s="235" t="n">
+        <v>6</v>
+      </c>
+      <c r="H18" s="236" t="inlineStr">
+        <is>
+          <t>4–1</t>
+        </is>
+      </c>
+      <c r="I18" s="237" t="n">
+        <v>4</v>
+      </c>
+      <c r="J18" s="234" t="n">
         <v>2</v>
-      </c>
-      <c r="L16" s="234" t="n">
-        <v>4</v>
-      </c>
-      <c r="M16" s="238" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="N16" s="231" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="143">
-      <c r="A17" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe K</t>
-        </is>
-      </c>
-      <c r="B17" s="240" t="inlineStr">
-        <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C17" s="238" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D17" s="241" t="n">
-        <v>7</v>
-      </c>
-      <c r="E17" s="241" t="n">
-        <v>3</v>
-      </c>
-      <c r="F17" s="241" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="243" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="244" t="inlineStr">
-        <is>
-          <t>1–3</t>
-        </is>
-      </c>
-      <c r="I17" s="245" t="n">
-        <v>4</v>
-      </c>
-      <c r="J17" s="241" t="n">
-        <v>5</v>
-      </c>
-      <c r="K17" s="242" t="n">
-        <v>6</v>
-      </c>
-      <c r="L17" s="242" t="n">
-        <v>15</v>
-      </c>
-      <c r="M17" s="247" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="N17" s="240" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="143">
-      <c r="A18" s="230" t="inlineStr">
-        <is>
-          <t>Gruppe L</t>
-        </is>
-      </c>
-      <c r="B18" s="231" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C18" s="247" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D18" s="233" t="n">
-        <v>22</v>
-      </c>
-      <c r="E18" s="233" t="n">
-        <v>8</v>
-      </c>
-      <c r="F18" s="234" t="n">
-        <v>9</v>
-      </c>
-      <c r="G18" s="235" t="n">
-        <v>5</v>
-      </c>
-      <c r="H18" s="236" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I18" s="237" t="n">
-        <v>1</v>
-      </c>
-      <c r="J18" s="234" t="n">
-        <v>4</v>
       </c>
       <c r="K18" s="234" t="n">
         <v>2</v>
       </c>
       <c r="L18" s="234" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M18" s="238" t="n">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
       <c r="N18" s="231" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -39968,79 +39948,879 @@
       <c r="A19" s="239" t="inlineStr"/>
       <c r="B19" s="240" t="inlineStr">
         <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C19" s="232" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D19" s="242" t="n">
+        <v>8</v>
+      </c>
+      <c r="E19" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="241" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="243" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="244" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I19" s="245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="K19" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="238" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="N19" s="240" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="143">
+      <c r="A20" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="B20" s="231" t="inlineStr">
+        <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="C20" s="248" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D20" s="233" t="n">
+        <v>16</v>
+      </c>
+      <c r="E20" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="234" t="n">
+        <v>9</v>
+      </c>
+      <c r="G20" s="235" t="n">
+        <v>3</v>
+      </c>
+      <c r="H20" s="236" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I20" s="237" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="K20" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="L20" s="234" t="n">
+        <v>10</v>
+      </c>
+      <c r="M20" s="248" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="N20" s="231" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="143">
+      <c r="A21" s="239" t="inlineStr"/>
+      <c r="B21" s="240" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C21" s="247" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D21" s="242" t="n">
+        <v>26</v>
+      </c>
+      <c r="E21" s="242" t="n">
+        <v>11</v>
+      </c>
+      <c r="F21" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="G21" s="243" t="n">
+        <v>10</v>
+      </c>
+      <c r="H21" s="244" t="inlineStr">
+        <is>
+          <t>7–1</t>
+        </is>
+      </c>
+      <c r="I21" s="245" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="K21" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L21" s="241" t="n">
+        <v>7</v>
+      </c>
+      <c r="M21" s="238" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="N21" s="240" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="143">
+      <c r="A22" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="B22" s="231" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="C22" s="232" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D22" s="233" t="n">
+        <v>11</v>
+      </c>
+      <c r="E22" s="233" t="n">
+        <v>7</v>
+      </c>
+      <c r="F22" s="234" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="236" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I22" s="237" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="234" t="n">
+        <v>5</v>
+      </c>
+      <c r="K22" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="L22" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="M22" s="238" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N22" s="231" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="143">
+      <c r="A23" s="239" t="inlineStr"/>
+      <c r="B23" s="240" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+      <c r="C23" s="248" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D23" s="242" t="n">
+        <v>13</v>
+      </c>
+      <c r="E23" s="242" t="n">
+        <v>8</v>
+      </c>
+      <c r="F23" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" s="244" t="inlineStr">
+        <is>
+          <t>5–1</t>
+        </is>
+      </c>
+      <c r="I23" s="245" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="M23" s="248" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="N23" s="240" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="143">
+      <c r="A24" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
+      <c r="B24" s="231" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="C24" s="248" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D24" s="233" t="n">
+        <v>15</v>
+      </c>
+      <c r="E24" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="F24" s="234" t="n">
+        <v>7</v>
+      </c>
+      <c r="G24" s="235" t="n">
+        <v>5</v>
+      </c>
+      <c r="H24" s="236" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I24" s="237" t="n">
+        <v>8</v>
+      </c>
+      <c r="J24" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="K24" s="233" t="n">
+        <v>4</v>
+      </c>
+      <c r="L24" s="234" t="n">
+        <v>14</v>
+      </c>
+      <c r="M24" s="248" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="N24" s="231" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="143">
+      <c r="A25" s="239" t="inlineStr"/>
+      <c r="B25" s="240" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C25" s="248" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D25" s="242" t="n">
+        <v>17</v>
+      </c>
+      <c r="E25" s="241" t="n">
+        <v>4</v>
+      </c>
+      <c r="F25" s="241" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" s="243" t="n">
+        <v>5</v>
+      </c>
+      <c r="H25" s="244" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I25" s="245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J25" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="K25" s="242" t="n">
+        <v>8</v>
+      </c>
+      <c r="L25" s="241" t="n">
+        <v>13</v>
+      </c>
+      <c r="M25" s="248" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N25" s="240" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="143">
+      <c r="A26" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="B26" s="231" t="inlineStr">
+        <is>
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="C26" s="238" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D26" s="234" t="n">
+        <v>7</v>
+      </c>
+      <c r="E26" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="G26" s="235" t="n">
+        <v>1</v>
+      </c>
+      <c r="H26" s="236" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I26" s="237" t="n">
+        <v>9</v>
+      </c>
+      <c r="J26" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="K26" s="233" t="n">
+        <v>10</v>
+      </c>
+      <c r="L26" s="233" t="n">
+        <v>27</v>
+      </c>
+      <c r="M26" s="247" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="N26" s="231" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="143">
+      <c r="A27" s="239" t="inlineStr"/>
+      <c r="B27" s="240" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C27" s="247" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D27" s="242" t="n">
+        <v>23</v>
+      </c>
+      <c r="E27" s="242" t="n">
+        <v>8</v>
+      </c>
+      <c r="F27" s="241" t="n">
+        <v>9</v>
+      </c>
+      <c r="G27" s="243" t="n">
+        <v>6</v>
+      </c>
+      <c r="H27" s="244" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I27" s="245" t="n">
+        <v>2</v>
+      </c>
+      <c r="J27" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="K27" s="241" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="241" t="n">
+        <v>6</v>
+      </c>
+      <c r="M27" s="238" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="N27" s="240" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="143">
+      <c r="A28" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe I</t>
+        </is>
+      </c>
+      <c r="B28" s="231" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C28" s="248" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D28" s="233" t="n">
+        <v>12</v>
+      </c>
+      <c r="E28" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="F28" s="234" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="235" t="n">
+        <v>2</v>
+      </c>
+      <c r="H28" s="236" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="I28" s="237" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="K28" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="L28" s="234" t="n">
+        <v>6</v>
+      </c>
+      <c r="M28" s="248" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N28" s="231" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="143">
+      <c r="A29" s="239" t="inlineStr"/>
+      <c r="B29" s="240" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="C29" s="238" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D29" s="241" t="n">
+        <v>11</v>
+      </c>
+      <c r="E29" s="241" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="241" t="n">
+        <v>8</v>
+      </c>
+      <c r="G29" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="244" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="I29" s="245" t="n">
+        <v>2</v>
+      </c>
+      <c r="J29" s="241" t="n">
+        <v>4</v>
+      </c>
+      <c r="K29" s="242" t="n">
+        <v>6</v>
+      </c>
+      <c r="L29" s="242" t="n">
+        <v>12</v>
+      </c>
+      <c r="M29" s="232" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N29" s="240" t="inlineStr">
+        <is>
+          <t>Norge</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="143">
+      <c r="A30" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe J</t>
+        </is>
+      </c>
+      <c r="B30" s="231" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C30" s="248" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D30" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E30" s="233" t="n">
+        <v>6</v>
+      </c>
+      <c r="F30" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="G30" s="235" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="236" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="I30" s="237" t="n">
+        <v>3</v>
+      </c>
+      <c r="J30" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" s="234" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="234" t="n">
+        <v>6</v>
+      </c>
+      <c r="M30" s="248" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N30" s="231" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="143">
+      <c r="A31" s="239" t="inlineStr"/>
+      <c r="B31" s="240" t="inlineStr">
+        <is>
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C31" s="232" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D31" s="241" t="n">
+        <v>9</v>
+      </c>
+      <c r="E31" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="F31" s="241" t="n">
+        <v>4</v>
+      </c>
+      <c r="G31" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="244" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="I31" s="245" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" s="241" t="n">
+        <v>4</v>
+      </c>
+      <c r="K31" s="242" t="n">
+        <v>4</v>
+      </c>
+      <c r="L31" s="242" t="n">
+        <v>11</v>
+      </c>
+      <c r="M31" s="238" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N31" s="240" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="143">
+      <c r="A32" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
+      <c r="B32" s="231" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C32" s="247" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D32" s="233" t="n">
+        <v>9</v>
+      </c>
+      <c r="E32" s="233" t="n">
+        <v>3</v>
+      </c>
+      <c r="F32" s="234" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="235" t="n">
+        <v>2</v>
+      </c>
+      <c r="H32" s="236" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I32" s="237" t="n">
+        <v>3</v>
+      </c>
+      <c r="J32" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="K32" s="234" t="n">
+        <v>2</v>
+      </c>
+      <c r="L32" s="234" t="n">
+        <v>8</v>
+      </c>
+      <c r="M32" s="238" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N32" s="231" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="143">
+      <c r="A33" s="239" t="inlineStr"/>
+      <c r="B33" s="240" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C33" s="238" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D33" s="241" t="n">
+        <v>7</v>
+      </c>
+      <c r="E33" s="241" t="n">
+        <v>3</v>
+      </c>
+      <c r="F33" s="241" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="243" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="244" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I33" s="245" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" s="241" t="n">
+        <v>5</v>
+      </c>
+      <c r="K33" s="242" t="n">
+        <v>6</v>
+      </c>
+      <c r="L33" s="242" t="n">
+        <v>15</v>
+      </c>
+      <c r="M33" s="247" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N33" s="240" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="143">
+      <c r="A34" s="230" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="B34" s="231" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C34" s="248" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D34" s="233" t="n">
+        <v>20</v>
+      </c>
+      <c r="E34" s="233" t="n">
+        <v>12</v>
+      </c>
+      <c r="F34" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="235" t="n">
+        <v>5</v>
+      </c>
+      <c r="H34" s="236" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="I34" s="237" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" s="234" t="n">
+        <v>3</v>
+      </c>
+      <c r="K34" s="234" t="n">
+        <v>5</v>
+      </c>
+      <c r="L34" s="234" t="n">
+        <v>11</v>
+      </c>
+      <c r="M34" s="248" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N34" s="231" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="143">
+      <c r="A35" s="239" t="inlineStr"/>
+      <c r="B35" s="240" t="inlineStr">
+        <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C19" s="238" t="n">
+      <c r="C35" s="238" t="n">
         <v>0.37</v>
       </c>
-      <c r="D19" s="241" t="n">
+      <c r="D35" s="241" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="241" t="n">
+      <c r="E35" s="241" t="n">
         <v>3</v>
       </c>
-      <c r="F19" s="241" t="n">
+      <c r="F35" s="241" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="243" t="n">
-        <v>1</v>
-      </c>
-      <c r="H19" s="244" t="inlineStr">
+      <c r="G35" s="243" t="n">
+        <v>1</v>
+      </c>
+      <c r="H35" s="244" t="inlineStr">
         <is>
           <t>1–0</t>
         </is>
       </c>
-      <c r="I19" s="245" t="n">
+      <c r="I35" s="245" t="n">
         <v>2</v>
       </c>
-      <c r="J19" s="241" t="n">
+      <c r="J35" s="241" t="n">
         <v>5</v>
       </c>
-      <c r="K19" s="242" t="n">
+      <c r="K35" s="242" t="n">
         <v>4</v>
       </c>
-      <c r="L19" s="242" t="n">
+      <c r="L35" s="242" t="n">
         <v>11</v>
       </c>
-      <c r="M19" s="232" t="n">
+      <c r="M35" s="232" t="n">
         <v>0.63</v>
       </c>
-      <c r="N19" s="240" t="inlineStr">
+      <c r="N35" s="240" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="14" customHeight="1" s="143">
-      <c r="A21" s="227" t="inlineStr">
+    <row r="37" ht="14" customHeight="1" s="143">
+      <c r="A37" s="227" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" s="143">
-      <c r="A22" s="219" t="inlineStr">
+    <row r="38" ht="18" customHeight="1" s="143">
+      <c r="A38" s="219" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B22" s="226" t="inlineStr">
+      <c r="B38" s="226" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C22" s="225" t="inlineStr">
+      <c r="C38" s="225" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D22" s="222" t="inlineStr">
+      <c r="D38" s="222" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E22" s="249" t="inlineStr">
+      <c r="E38" s="249" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -40049,7 +40829,7 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A21:N21"/>
+    <mergeCell ref="A37:N37"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fiks bred #-kolonne i Alder-arket: merge fotnote over alle kolonner
Fotnoteraden ble skrevet kun til kolonne A utan colspan, noe som med
white-space:nowrap tvang #-kolonnen til å bli like bred som den lange
fotnote-teksten. Løst ved å merge fotnoteraden over alle 6 kolonner i
add_alder_sheet.py — HTML-generatoren plukker opp colspan automatisk.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1039,7 +1039,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="256">
+  <cellXfs count="257">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1744,6 +1744,9 @@
     <xf numFmtId="0" fontId="67" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="45" fillId="61" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -38620,7 +38623,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L19"/>
+  <dimension ref="A1:L22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="143" min="1" max="1"/>
@@ -38810,12 +38813,10 @@
       <c r="H7" s="211" t="n">
         <v>2</v>
       </c>
-      <c r="I7" s="211" t="n">
-        <v>2</v>
-      </c>
+      <c r="I7" s="210" t="n"/>
       <c r="J7" s="210" t="n"/>
-      <c r="K7" s="216" t="n">
-        <v>7</v>
+      <c r="K7" s="212" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" s="143">
@@ -38944,7 +38945,7 @@
     <row r="13" ht="16" customHeight="1" s="143">
       <c r="A13" s="209" t="inlineStr">
         <is>
-          <t>ET</t>
+          <t>45+</t>
         </is>
       </c>
       <c r="B13" s="218" t="inlineStr">
@@ -39001,82 +39002,173 @@
     <row r="14" ht="20" customHeight="1" s="143">
       <c r="A14" s="209" t="inlineStr">
         <is>
+          <t>HT</t>
+        </is>
+      </c>
+      <c r="B14" s="210" t="n"/>
+      <c r="C14" s="210" t="n"/>
+      <c r="D14" s="211" t="n">
+        <v>2</v>
+      </c>
+      <c r="E14" s="210" t="n"/>
+      <c r="F14" s="256" t="n">
+        <v>4</v>
+      </c>
+      <c r="G14" s="210" t="n"/>
+      <c r="H14" s="210" t="n"/>
+      <c r="I14" s="210" t="n"/>
+      <c r="J14" s="210" t="n"/>
+      <c r="K14" s="210" t="n"/>
+    </row>
+    <row r="15" ht="8" customHeight="1" s="143">
+      <c r="A15" s="217" t="n"/>
+      <c r="B15" s="217" t="n"/>
+      <c r="C15" s="217" t="n"/>
+      <c r="D15" s="217" t="n"/>
+      <c r="E15" s="217" t="n"/>
+      <c r="F15" s="217" t="n"/>
+      <c r="G15" s="217" t="n"/>
+      <c r="H15" s="217" t="n"/>
+      <c r="I15" s="217" t="n"/>
+      <c r="J15" s="217" t="n"/>
+      <c r="K15" s="217" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1" s="143">
+      <c r="A16" s="209" t="inlineStr">
+        <is>
+          <t>ET</t>
+        </is>
+      </c>
+      <c r="B16" s="218" t="inlineStr">
+        <is>
+          <t>+1</t>
+        </is>
+      </c>
+      <c r="C16" s="218" t="inlineStr">
+        <is>
+          <t>+2</t>
+        </is>
+      </c>
+      <c r="D16" s="218" t="inlineStr">
+        <is>
+          <t>+3</t>
+        </is>
+      </c>
+      <c r="E16" s="218" t="inlineStr">
+        <is>
+          <t>+4</t>
+        </is>
+      </c>
+      <c r="F16" s="218" t="inlineStr">
+        <is>
+          <t>+5</t>
+        </is>
+      </c>
+      <c r="G16" s="218" t="inlineStr">
+        <is>
+          <t>+6</t>
+        </is>
+      </c>
+      <c r="H16" s="218" t="inlineStr">
+        <is>
+          <t>+7</t>
+        </is>
+      </c>
+      <c r="I16" s="218" t="inlineStr">
+        <is>
+          <t>+8</t>
+        </is>
+      </c>
+      <c r="J16" s="218" t="inlineStr">
+        <is>
+          <t>+9</t>
+        </is>
+      </c>
+      <c r="K16" s="218" t="inlineStr">
+        <is>
+          <t>+10</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1" s="143">
+      <c r="A17" s="209" t="inlineStr">
+        <is>
           <t>90+</t>
         </is>
       </c>
-      <c r="B14" s="210" t="n"/>
-      <c r="C14" s="213" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" s="213" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="213" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="211" t="n">
+      <c r="B17" s="210" t="n"/>
+      <c r="C17" s="213" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="213" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="213" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="211" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="212" t="n">
+      <c r="G17" s="212" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="213" t="n">
-        <v>1</v>
-      </c>
-      <c r="I14" s="213" t="n">
-        <v>1</v>
-      </c>
-      <c r="J14" s="213" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="210" t="n"/>
-    </row>
-    <row r="16" ht="14" customHeight="1" s="143">
-      <c r="A16" s="219" t="inlineStr">
+      <c r="H17" s="213" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="213" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" s="213" t="n">
+        <v>1</v>
+      </c>
+      <c r="K17" s="210" t="n"/>
+    </row>
+    <row r="19" ht="14" customHeight="1" s="143">
+      <c r="A19" s="219" t="inlineStr">
         <is>
           <t>Fargeskala:</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" s="143">
-      <c r="B17" s="220" t="inlineStr">
+    <row r="20" ht="18" customHeight="1" s="143">
+      <c r="B20" s="220" t="inlineStr">
         <is>
           <t>0 mål</t>
         </is>
       </c>
-      <c r="C17" s="221" t="inlineStr">
+      <c r="C20" s="221" t="inlineStr">
         <is>
           <t>1 mål</t>
         </is>
       </c>
-      <c r="D17" s="222" t="inlineStr">
+      <c r="D20" s="222" t="inlineStr">
         <is>
           <t>2 mål</t>
         </is>
       </c>
-      <c r="E17" s="223" t="inlineStr">
+      <c r="E20" s="223" t="inlineStr">
         <is>
           <t>3 mål</t>
         </is>
       </c>
-      <c r="F17" s="224" t="inlineStr">
+      <c r="F20" s="224" t="inlineStr">
         <is>
           <t>4 mål</t>
         </is>
       </c>
-      <c r="G17" s="225" t="inlineStr">
+      <c r="G20" s="225" t="inlineStr">
         <is>
           <t>5 mål</t>
         </is>
       </c>
-      <c r="H17" s="226" t="inlineStr">
+      <c r="H20" s="226" t="inlineStr">
         <is>
           <t>6+ mål</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="14" customHeight="1" s="143">
-      <c r="A19" s="227" t="inlineStr">
+    <row r="22" ht="14" customHeight="1" s="143">
+      <c r="A22" s="227" t="inlineStr">
         <is>
           <t>| Tykk strek markerer halvtidspausen (mellom minutt 45 og 46)</t>
         </is>
@@ -58982,9 +59074,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A14:F14"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A27:F27"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-21 08:11 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Alder" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -809,13 +809,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -834,7 +834,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -858,12 +858,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -877,7 +877,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -890,8 +889,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -905,7 +904,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -915,7 +913,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -930,9 +928,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Runde 2 stats: Germany-Ivory Coast 2-1, Ecuador-Curacao 0-0 (2026-06-20)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Alder" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -809,13 +809,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -834,7 +834,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -858,12 +858,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -877,6 +877,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -889,8 +890,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -904,6 +905,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -913,7 +915,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -928,9 +930,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -57278,7 +57280,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N39"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58182,47 +58184,47 @@
       </c>
       <c r="B20" s="66" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-      <c r="C20" s="83" t="n">
-        <v>0.49</v>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="C20" s="82" t="n">
+        <v>0.75</v>
       </c>
       <c r="D20" s="68" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="E20" s="68" t="n">
+        <v>15</v>
+      </c>
+      <c r="F20" s="69" t="n">
+        <v>7</v>
+      </c>
+      <c r="G20" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="G20" s="70" t="n">
-        <v>3</v>
-      </c>
       <c r="H20" s="71" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>0–0</t>
         </is>
       </c>
       <c r="I20" s="72" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J20" s="69" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K20" s="69" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L20" s="69" t="n">
         <v>10</v>
       </c>
-      <c r="M20" s="83" t="n">
-        <v>0.51</v>
+      <c r="M20" s="73" t="n">
+        <v>0.25</v>
       </c>
       <c r="N20" s="66" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -58230,79 +58232,75 @@
       <c r="A21" s="74" t="inlineStr"/>
       <c r="B21" s="75" t="inlineStr">
         <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="C21" s="83" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D21" s="77" t="n">
+        <v>16</v>
+      </c>
+      <c r="E21" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" s="76" t="n">
+        <v>9</v>
+      </c>
+      <c r="G21" s="78" t="n">
+        <v>3</v>
+      </c>
+      <c r="H21" s="79" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I21" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="76" t="n">
+        <v>8</v>
+      </c>
+      <c r="K21" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" s="76" t="n">
+        <v>10</v>
+      </c>
+      <c r="M21" s="83" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="N21" s="75" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="81" t="inlineStr"/>
+      <c r="B22" s="66" t="inlineStr">
+        <is>
           <t>Tyskland</t>
         </is>
       </c>
-      <c r="C21" s="82" t="n">
+      <c r="C22" s="82" t="n">
         <v>0.65</v>
       </c>
-      <c r="D21" s="77" t="n">
+      <c r="D22" s="68" t="n">
         <v>26</v>
       </c>
-      <c r="E21" s="77" t="n">
+      <c r="E22" s="68" t="n">
         <v>11</v>
       </c>
-      <c r="F21" s="76" t="n">
+      <c r="F22" s="69" t="n">
         <v>5</v>
       </c>
-      <c r="G21" s="78" t="n">
+      <c r="G22" s="70" t="n">
         <v>10</v>
       </c>
-      <c r="H21" s="79" t="inlineStr">
+      <c r="H22" s="71" t="inlineStr">
         <is>
           <t>7–1</t>
-        </is>
-      </c>
-      <c r="I21" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" s="76" t="n">
-        <v>5</v>
-      </c>
-      <c r="K21" s="76" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="76" t="n">
-        <v>7</v>
-      </c>
-      <c r="M21" s="73" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="N21" s="75" t="inlineStr">
-        <is>
-          <t>Curaçao</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="65" t="inlineStr">
-        <is>
-          <t>Gruppe F</t>
-        </is>
-      </c>
-      <c r="B22" s="66" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="C22" s="67" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D22" s="68" t="n">
-        <v>11</v>
-      </c>
-      <c r="E22" s="68" t="n">
-        <v>7</v>
-      </c>
-      <c r="F22" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="G22" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="H22" s="71" t="inlineStr">
-        <is>
-          <t>2–2</t>
         </is>
       </c>
       <c r="I22" s="72" t="n">
@@ -58312,17 +58310,17 @@
         <v>5</v>
       </c>
       <c r="K22" s="69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L22" s="69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M22" s="73" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="N22" s="66" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -58330,147 +58328,147 @@
       <c r="A23" s="74" t="inlineStr"/>
       <c r="B23" s="75" t="inlineStr">
         <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C23" s="67" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D23" s="77" t="n">
+        <v>16</v>
+      </c>
+      <c r="E23" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="F23" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="H23" s="79" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="I23" s="80" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="K23" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="L23" s="76" t="n">
+        <v>9</v>
+      </c>
+      <c r="M23" s="83" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="N23" s="75" t="inlineStr">
+        <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="65" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="B24" s="66" t="inlineStr">
+        <is>
           <t>Nederland</t>
         </is>
       </c>
-      <c r="C23" s="83" t="n">
+      <c r="C24" s="67" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D24" s="68" t="n">
+        <v>11</v>
+      </c>
+      <c r="E24" s="68" t="n">
+        <v>7</v>
+      </c>
+      <c r="F24" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="71" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I24" s="72" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="K24" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="L24" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="M24" s="73" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N24" s="66" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="74" t="inlineStr"/>
+      <c r="B25" s="75" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="C25" s="83" t="n">
         <v>0.52</v>
       </c>
-      <c r="D23" s="76" t="n">
+      <c r="D25" s="76" t="n">
         <v>12</v>
       </c>
-      <c r="E23" s="76" t="n">
+      <c r="E25" s="76" t="n">
         <v>7</v>
       </c>
-      <c r="F23" s="76" t="n">
+      <c r="F25" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="G23" s="78" t="n">
+      <c r="G25" s="78" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="79" t="inlineStr">
+      <c r="H25" s="79" t="inlineStr">
         <is>
           <t>5–1</t>
         </is>
       </c>
-      <c r="I23" s="80" t="n">
+      <c r="I25" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="J23" s="76" t="n">
+      <c r="J25" s="76" t="n">
         <v>9</v>
       </c>
-      <c r="K23" s="77" t="n">
+      <c r="K25" s="77" t="n">
         <v>9</v>
       </c>
-      <c r="L23" s="77" t="n">
+      <c r="L25" s="77" t="n">
         <v>20</v>
       </c>
-      <c r="M23" s="83" t="n">
+      <c r="M25" s="83" t="n">
         <v>0.48</v>
       </c>
-      <c r="N23" s="75" t="inlineStr">
+      <c r="N25" s="75" t="inlineStr">
         <is>
           <t>Sverige</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="81" t="inlineStr"/>
-      <c r="B24" s="66" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-      <c r="C24" s="83" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="D24" s="68" t="n">
-        <v>13</v>
-      </c>
-      <c r="E24" s="68" t="n">
-        <v>8</v>
-      </c>
-      <c r="F24" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="G24" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="H24" s="71" t="inlineStr">
-        <is>
-          <t>5–1</t>
-        </is>
-      </c>
-      <c r="I24" s="72" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="K24" s="69" t="n">
-        <v>2</v>
-      </c>
-      <c r="L24" s="69" t="n">
-        <v>5</v>
-      </c>
-      <c r="M24" s="83" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="N24" s="66" t="inlineStr">
-        <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="65" t="inlineStr">
-        <is>
-          <t>Gruppe G</t>
-        </is>
-      </c>
-      <c r="B25" s="75" t="inlineStr">
-        <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C25" s="83" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="D25" s="77" t="n">
-        <v>15</v>
-      </c>
-      <c r="E25" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="F25" s="76" t="n">
-        <v>7</v>
-      </c>
-      <c r="G25" s="78" t="n">
-        <v>5</v>
-      </c>
-      <c r="H25" s="79" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I25" s="80" t="n">
-        <v>8</v>
-      </c>
-      <c r="J25" s="76" t="n">
-        <v>2</v>
-      </c>
-      <c r="K25" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="L25" s="76" t="n">
-        <v>14</v>
-      </c>
-      <c r="M25" s="83" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="N25" s="75" t="inlineStr">
-        <is>
-          <t>Egypt</t>
         </is>
       </c>
     </row>
@@ -58478,75 +58476,75 @@
       <c r="A26" s="81" t="inlineStr"/>
       <c r="B26" s="66" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Sverige</t>
         </is>
       </c>
       <c r="C26" s="83" t="n">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="D26" s="68" t="n">
-        <v>17</v>
-      </c>
-      <c r="E26" s="69" t="n">
-        <v>4</v>
+        <v>13</v>
+      </c>
+      <c r="E26" s="68" t="n">
+        <v>8</v>
       </c>
       <c r="F26" s="69" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G26" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H26" s="71" t="inlineStr">
         <is>
-          <t>2–2</t>
+          <t>5–1</t>
         </is>
       </c>
       <c r="I26" s="72" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J26" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="K26" s="68" t="n">
-        <v>8</v>
+      <c r="K26" s="69" t="n">
+        <v>2</v>
       </c>
       <c r="L26" s="69" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M26" s="83" t="n">
-        <v>0.53</v>
+        <v>0.51</v>
       </c>
       <c r="N26" s="66" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Tunisia</t>
         </is>
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="65" t="inlineStr">
         <is>
-          <t>Gruppe H</t>
+          <t>Gruppe G</t>
         </is>
       </c>
       <c r="B27" s="75" t="inlineStr">
         <is>
-          <t>Saudi-Arabia</t>
-        </is>
-      </c>
-      <c r="C27" s="73" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D27" s="76" t="n">
-        <v>7</v>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="C27" s="83" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D27" s="77" t="n">
+        <v>15</v>
       </c>
       <c r="E27" s="76" t="n">
         <v>3</v>
       </c>
       <c r="F27" s="76" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G27" s="78" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H27" s="79" t="inlineStr">
         <is>
@@ -58554,23 +58552,23 @@
         </is>
       </c>
       <c r="I27" s="80" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J27" s="76" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K27" s="77" t="n">
-        <v>10</v>
-      </c>
-      <c r="L27" s="77" t="n">
-        <v>27</v>
-      </c>
-      <c r="M27" s="82" t="n">
-        <v>0.65</v>
+        <v>4</v>
+      </c>
+      <c r="L27" s="76" t="n">
+        <v>14</v>
+      </c>
+      <c r="M27" s="83" t="n">
+        <v>0.47</v>
       </c>
       <c r="N27" s="75" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>Egypt</t>
         </is>
       </c>
     </row>
@@ -58578,99 +58576,99 @@
       <c r="A28" s="81" t="inlineStr"/>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C28" s="82" t="n">
-        <v>0.74</v>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C28" s="83" t="n">
+        <v>0.47</v>
       </c>
       <c r="D28" s="68" t="n">
-        <v>23</v>
-      </c>
-      <c r="E28" s="68" t="n">
+        <v>17</v>
+      </c>
+      <c r="E28" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F28" s="69" t="n">
         <v>8</v>
       </c>
-      <c r="F28" s="69" t="n">
-        <v>9</v>
-      </c>
       <c r="G28" s="70" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H28" s="71" t="inlineStr">
         <is>
-          <t>0–0</t>
+          <t>2–2</t>
         </is>
       </c>
       <c r="I28" s="72" t="n">
+        <v>3</v>
+      </c>
+      <c r="J28" s="69" t="n">
         <v>2</v>
       </c>
-      <c r="J28" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" s="69" t="n">
-        <v>1</v>
+      <c r="K28" s="68" t="n">
+        <v>8</v>
       </c>
       <c r="L28" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="M28" s="73" t="n">
-        <v>0.26</v>
+        <v>13</v>
+      </c>
+      <c r="M28" s="83" t="n">
+        <v>0.53</v>
       </c>
       <c r="N28" s="66" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="65" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe H</t>
         </is>
       </c>
       <c r="B29" s="75" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C29" s="83" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D29" s="77" t="n">
-        <v>12</v>
-      </c>
-      <c r="E29" s="77" t="n">
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="C29" s="73" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D29" s="76" t="n">
+        <v>7</v>
+      </c>
+      <c r="E29" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="F29" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G29" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="79" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I29" s="80" t="n">
         <v>9</v>
       </c>
-      <c r="F29" s="76" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="78" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="79" t="inlineStr">
-        <is>
-          <t>3–1</t>
-        </is>
-      </c>
-      <c r="I29" s="80" t="n">
-        <v>1</v>
-      </c>
       <c r="J29" s="76" t="n">
-        <v>2</v>
-      </c>
-      <c r="K29" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="L29" s="76" t="n">
-        <v>6</v>
-      </c>
-      <c r="M29" s="83" t="n">
-        <v>0.46</v>
+        <v>8</v>
+      </c>
+      <c r="K29" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="L29" s="77" t="n">
+        <v>27</v>
+      </c>
+      <c r="M29" s="82" t="n">
+        <v>0.65</v>
       </c>
       <c r="N29" s="75" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Uruguay</t>
         </is>
       </c>
     </row>
@@ -58678,99 +58676,99 @@
       <c r="A30" s="81" t="inlineStr"/>
       <c r="B30" s="66" t="inlineStr">
         <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="C30" s="73" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D30" s="69" t="n">
-        <v>11</v>
-      </c>
-      <c r="E30" s="69" t="n">
-        <v>1</v>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C30" s="82" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D30" s="68" t="n">
+        <v>23</v>
+      </c>
+      <c r="E30" s="68" t="n">
+        <v>8</v>
       </c>
       <c r="F30" s="69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="G30" s="70" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="H30" s="71" t="inlineStr">
         <is>
-          <t>1–4</t>
+          <t>0–0</t>
         </is>
       </c>
       <c r="I30" s="72" t="n">
         <v>2</v>
       </c>
       <c r="J30" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="K30" s="68" t="n">
+        <v>3</v>
+      </c>
+      <c r="K30" s="69" t="n">
+        <v>1</v>
+      </c>
+      <c r="L30" s="69" t="n">
         <v>6</v>
       </c>
-      <c r="L30" s="68" t="n">
-        <v>12</v>
-      </c>
-      <c r="M30" s="67" t="n">
-        <v>0.63</v>
+      <c r="M30" s="73" t="n">
+        <v>0.26</v>
       </c>
       <c r="N30" s="66" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="65" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="B31" s="75" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Frankrike</t>
         </is>
       </c>
       <c r="C31" s="83" t="n">
-        <v>0.47</v>
+        <v>0.54</v>
       </c>
       <c r="D31" s="77" t="n">
+        <v>12</v>
+      </c>
+      <c r="E31" s="77" t="n">
         <v>9</v>
       </c>
-      <c r="E31" s="77" t="n">
-        <v>6</v>
-      </c>
       <c r="F31" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H31" s="79" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="I31" s="80" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="76" t="n">
         <v>3</v>
-      </c>
-      <c r="G31" s="78" t="n">
-        <v>0</v>
-      </c>
-      <c r="H31" s="79" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I31" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="J31" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="K31" s="76" t="n">
-        <v>0</v>
       </c>
       <c r="L31" s="76" t="n">
         <v>6</v>
       </c>
       <c r="M31" s="83" t="n">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="N31" s="75" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -58778,79 +58776,79 @@
       <c r="A32" s="81" t="inlineStr"/>
       <c r="B32" s="66" t="inlineStr">
         <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C32" s="67" t="n">
-        <v>0.62</v>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="C32" s="73" t="n">
+        <v>0.37</v>
       </c>
       <c r="D32" s="69" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E32" s="69" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F32" s="69" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G32" s="70" t="n">
         <v>2</v>
       </c>
       <c r="H32" s="71" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>1–4</t>
         </is>
       </c>
       <c r="I32" s="72" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J32" s="69" t="n">
         <v>4</v>
       </c>
       <c r="K32" s="68" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="L32" s="68" t="n">
-        <v>11</v>
-      </c>
-      <c r="M32" s="73" t="n">
-        <v>0.38</v>
+        <v>12</v>
+      </c>
+      <c r="M32" s="67" t="n">
+        <v>0.63</v>
       </c>
       <c r="N32" s="66" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Norge</t>
         </is>
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="65" t="inlineStr">
         <is>
-          <t>Gruppe K</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="B33" s="75" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C33" s="82" t="n">
-        <v>0.75</v>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C33" s="83" t="n">
+        <v>0.47</v>
       </c>
       <c r="D33" s="77" t="n">
         <v>9</v>
       </c>
       <c r="E33" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="F33" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="F33" s="76" t="n">
-        <v>4</v>
-      </c>
       <c r="G33" s="78" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H33" s="79" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I33" s="80" t="n">
@@ -58860,17 +58858,17 @@
         <v>3</v>
       </c>
       <c r="K33" s="76" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L33" s="76" t="n">
-        <v>8</v>
-      </c>
-      <c r="M33" s="73" t="n">
-        <v>0.25</v>
+        <v>6</v>
+      </c>
+      <c r="M33" s="83" t="n">
+        <v>0.53</v>
       </c>
       <c r="N33" s="75" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -58878,79 +58876,79 @@
       <c r="A34" s="81" t="inlineStr"/>
       <c r="B34" s="66" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C34" s="73" t="n">
-        <v>0.33</v>
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C34" s="67" t="n">
+        <v>0.62</v>
       </c>
       <c r="D34" s="69" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E34" s="69" t="n">
         <v>3</v>
       </c>
       <c r="F34" s="69" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G34" s="70" t="n">
         <v>2</v>
       </c>
       <c r="H34" s="71" t="inlineStr">
         <is>
-          <t>1–3</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I34" s="72" t="n">
+        <v>3</v>
+      </c>
+      <c r="J34" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="J34" s="69" t="n">
-        <v>5</v>
-      </c>
       <c r="K34" s="68" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L34" s="68" t="n">
-        <v>15</v>
-      </c>
-      <c r="M34" s="82" t="n">
-        <v>0.67</v>
+        <v>11</v>
+      </c>
+      <c r="M34" s="73" t="n">
+        <v>0.38</v>
       </c>
       <c r="N34" s="66" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Jordan</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="65" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe K</t>
         </is>
       </c>
       <c r="B35" s="75" t="inlineStr">
         <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C35" s="83" t="n">
-        <v>0.54</v>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C35" s="82" t="n">
+        <v>0.75</v>
       </c>
       <c r="D35" s="77" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E35" s="77" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="F35" s="76" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G35" s="78" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H35" s="79" t="inlineStr">
         <is>
-          <t>4–2</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I35" s="80" t="n">
@@ -58960,17 +58958,17 @@
         <v>3</v>
       </c>
       <c r="K35" s="76" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L35" s="76" t="n">
-        <v>11</v>
-      </c>
-      <c r="M35" s="83" t="n">
-        <v>0.46</v>
+        <v>8</v>
+      </c>
+      <c r="M35" s="73" t="n">
+        <v>0.25</v>
       </c>
       <c r="N35" s="75" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -58978,79 +58976,179 @@
       <c r="A36" s="81" t="inlineStr"/>
       <c r="B36" s="66" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Usbekistan</t>
         </is>
       </c>
       <c r="C36" s="73" t="n">
-        <v>0.37</v>
+        <v>0.33</v>
       </c>
       <c r="D36" s="69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E36" s="69" t="n">
         <v>3</v>
       </c>
       <c r="F36" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="H36" s="71" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I36" s="72" t="n">
         <v>4</v>
-      </c>
-      <c r="G36" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="H36" s="71" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I36" s="72" t="n">
-        <v>2</v>
       </c>
       <c r="J36" s="69" t="n">
         <v>5</v>
       </c>
       <c r="K36" s="68" t="n">
+        <v>6</v>
+      </c>
+      <c r="L36" s="68" t="n">
+        <v>15</v>
+      </c>
+      <c r="M36" s="82" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N36" s="66" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="65" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="B37" s="75" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C37" s="83" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D37" s="77" t="n">
+        <v>20</v>
+      </c>
+      <c r="E37" s="77" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="G37" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="H37" s="79" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="I37" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="J37" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" s="76" t="n">
+        <v>5</v>
+      </c>
+      <c r="L37" s="76" t="n">
+        <v>11</v>
+      </c>
+      <c r="M37" s="83" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N37" s="75" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="81" t="inlineStr"/>
+      <c r="B38" s="66" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C38" s="73" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D38" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="E38" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="L36" s="68" t="n">
+      <c r="G38" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="71" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I38" s="72" t="n">
+        <v>2</v>
+      </c>
+      <c r="J38" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="K38" s="68" t="n">
+        <v>4</v>
+      </c>
+      <c r="L38" s="68" t="n">
         <v>11</v>
       </c>
-      <c r="M36" s="67" t="n">
+      <c r="M38" s="67" t="n">
         <v>0.63</v>
       </c>
-      <c r="N36" s="66" t="inlineStr">
+      <c r="N38" s="66" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="14" customHeight="1">
-      <c r="A38" s="62" t="inlineStr">
+    <row r="40" ht="14" customHeight="1">
+      <c r="A40" s="62" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="54" t="inlineStr">
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="54" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B39" s="61" t="inlineStr">
+      <c r="B41" s="61" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C39" s="60" t="inlineStr">
+      <c r="C41" s="60" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D39" s="57" t="inlineStr">
+      <c r="D41" s="57" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E39" s="84" t="inlineStr">
+      <c r="E41" s="84" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -59058,8 +59156,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A40:N40"/>
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A38:N38"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-21 09:10 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Alder" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -809,13 +809,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -834,7 +834,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -858,12 +858,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -877,7 +877,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -890,8 +889,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -905,7 +904,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -915,7 +913,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -930,9 +928,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -57280,7 +57278,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N41"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -58521,423 +58519,419 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="65" t="inlineStr">
-        <is>
-          <t>Gruppe G</t>
-        </is>
-      </c>
+      <c r="A27" s="74" t="inlineStr"/>
       <c r="B27" s="75" t="inlineStr">
         <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C27" s="83" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="D27" s="77" t="n">
-        <v>15</v>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C27" s="73" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D27" s="76" t="n">
+        <v>3</v>
       </c>
       <c r="E27" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="G27" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H27" s="79" t="inlineStr">
+        <is>
+          <t>0–4</t>
+        </is>
+      </c>
+      <c r="I27" s="80" t="n">
         <v>3</v>
-      </c>
-      <c r="F27" s="76" t="n">
-        <v>7</v>
-      </c>
-      <c r="G27" s="78" t="n">
-        <v>5</v>
-      </c>
-      <c r="H27" s="79" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I27" s="80" t="n">
-        <v>8</v>
       </c>
       <c r="J27" s="76" t="n">
         <v>2</v>
       </c>
       <c r="K27" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="L27" s="76" t="n">
-        <v>14</v>
-      </c>
-      <c r="M27" s="83" t="n">
-        <v>0.47</v>
+        <v>5</v>
+      </c>
+      <c r="L27" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="M27" s="67" t="n">
+        <v>0.57</v>
       </c>
       <c r="N27" s="75" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Japan</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="81" t="inlineStr"/>
+      <c r="A28" s="65" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
       <c r="B28" s="66" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="C28" s="83" t="n">
-        <v>0.47</v>
+        <v>0.53</v>
       </c>
       <c r="D28" s="68" t="n">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="E28" s="69" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F28" s="69" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G28" s="70" t="n">
         <v>5</v>
       </c>
       <c r="H28" s="71" t="inlineStr">
         <is>
-          <t>2–2</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I28" s="72" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J28" s="69" t="n">
         <v>2</v>
       </c>
       <c r="K28" s="68" t="n">
+        <v>4</v>
+      </c>
+      <c r="L28" s="69" t="n">
+        <v>14</v>
+      </c>
+      <c r="M28" s="83" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="N28" s="66" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="74" t="inlineStr"/>
+      <c r="B29" s="75" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C29" s="83" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D29" s="77" t="n">
+        <v>17</v>
+      </c>
+      <c r="E29" s="76" t="n">
+        <v>4</v>
+      </c>
+      <c r="F29" s="76" t="n">
         <v>8</v>
       </c>
-      <c r="L28" s="69" t="n">
+      <c r="G29" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="H29" s="79" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I29" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="J29" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="L29" s="76" t="n">
         <v>13</v>
       </c>
-      <c r="M28" s="83" t="n">
+      <c r="M29" s="83" t="n">
         <v>0.53</v>
       </c>
-      <c r="N28" s="66" t="inlineStr">
+      <c r="N29" s="75" t="inlineStr">
         <is>
           <t>New Zealand</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="65" t="inlineStr">
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="65" t="inlineStr">
         <is>
           <t>Gruppe H</t>
         </is>
       </c>
-      <c r="B29" s="75" t="inlineStr">
+      <c r="B30" s="66" t="inlineStr">
         <is>
           <t>Saudi-Arabia</t>
         </is>
       </c>
-      <c r="C29" s="73" t="n">
+      <c r="C30" s="73" t="n">
         <v>0.35</v>
       </c>
-      <c r="D29" s="76" t="n">
+      <c r="D30" s="69" t="n">
         <v>7</v>
       </c>
-      <c r="E29" s="76" t="n">
+      <c r="E30" s="69" t="n">
         <v>3</v>
       </c>
-      <c r="F29" s="76" t="n">
+      <c r="F30" s="69" t="n">
         <v>3</v>
       </c>
-      <c r="G29" s="78" t="n">
-        <v>1</v>
-      </c>
-      <c r="H29" s="79" t="inlineStr">
+      <c r="G30" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H30" s="71" t="inlineStr">
         <is>
           <t>1–1</t>
         </is>
       </c>
-      <c r="I29" s="80" t="n">
+      <c r="I30" s="72" t="n">
         <v>9</v>
       </c>
-      <c r="J29" s="76" t="n">
+      <c r="J30" s="69" t="n">
         <v>8</v>
       </c>
-      <c r="K29" s="77" t="n">
+      <c r="K30" s="68" t="n">
         <v>10</v>
       </c>
-      <c r="L29" s="77" t="n">
+      <c r="L30" s="68" t="n">
         <v>27</v>
       </c>
-      <c r="M29" s="82" t="n">
+      <c r="M30" s="82" t="n">
         <v>0.65</v>
       </c>
-      <c r="N29" s="75" t="inlineStr">
+      <c r="N30" s="66" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="81" t="inlineStr"/>
-      <c r="B30" s="66" t="inlineStr">
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="74" t="inlineStr"/>
+      <c r="B31" s="75" t="inlineStr">
         <is>
           <t>Spania</t>
         </is>
       </c>
-      <c r="C30" s="82" t="n">
+      <c r="C31" s="82" t="n">
         <v>0.74</v>
       </c>
-      <c r="D30" s="68" t="n">
+      <c r="D31" s="77" t="n">
         <v>23</v>
       </c>
-      <c r="E30" s="68" t="n">
+      <c r="E31" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="F30" s="69" t="n">
+      <c r="F31" s="76" t="n">
         <v>9</v>
       </c>
-      <c r="G30" s="70" t="n">
+      <c r="G31" s="78" t="n">
         <v>6</v>
       </c>
-      <c r="H30" s="71" t="inlineStr">
+      <c r="H31" s="79" t="inlineStr">
         <is>
           <t>0–0</t>
         </is>
       </c>
-      <c r="I30" s="72" t="n">
+      <c r="I31" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="J30" s="69" t="n">
+      <c r="J31" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="K30" s="69" t="n">
-        <v>1</v>
-      </c>
-      <c r="L30" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="M30" s="73" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="N30" s="66" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="65" t="inlineStr">
-        <is>
-          <t>Gruppe I</t>
-        </is>
-      </c>
-      <c r="B31" s="75" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C31" s="83" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D31" s="77" t="n">
-        <v>12</v>
-      </c>
-      <c r="E31" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="F31" s="76" t="n">
-        <v>1</v>
-      </c>
-      <c r="G31" s="78" t="n">
-        <v>2</v>
-      </c>
-      <c r="H31" s="79" t="inlineStr">
-        <is>
-          <t>3–1</t>
-        </is>
-      </c>
-      <c r="I31" s="80" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" s="76" t="n">
-        <v>2</v>
-      </c>
       <c r="K31" s="76" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L31" s="76" t="n">
         <v>6</v>
       </c>
-      <c r="M31" s="83" t="n">
-        <v>0.46</v>
+      <c r="M31" s="73" t="n">
+        <v>0.26</v>
       </c>
       <c r="N31" s="75" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="81" t="inlineStr"/>
+      <c r="A32" s="65" t="inlineStr">
+        <is>
+          <t>Gruppe I</t>
+        </is>
+      </c>
       <c r="B32" s="66" t="inlineStr">
         <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="C32" s="73" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D32" s="69" t="n">
-        <v>11</v>
-      </c>
-      <c r="E32" s="69" t="n">
-        <v>1</v>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C32" s="83" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D32" s="68" t="n">
+        <v>12</v>
+      </c>
+      <c r="E32" s="68" t="n">
+        <v>9</v>
       </c>
       <c r="F32" s="69" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G32" s="70" t="n">
         <v>2</v>
       </c>
       <c r="H32" s="71" t="inlineStr">
         <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="I32" s="72" t="n">
+        <v>1</v>
+      </c>
+      <c r="J32" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="K32" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="L32" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="M32" s="83" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N32" s="66" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="74" t="inlineStr"/>
+      <c r="B33" s="75" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="C33" s="73" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D33" s="76" t="n">
+        <v>11</v>
+      </c>
+      <c r="E33" s="76" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="76" t="n">
+        <v>8</v>
+      </c>
+      <c r="G33" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" s="79" t="inlineStr">
+        <is>
           <t>1–4</t>
         </is>
       </c>
-      <c r="I32" s="72" t="n">
+      <c r="I33" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="J32" s="69" t="n">
+      <c r="J33" s="76" t="n">
         <v>4</v>
       </c>
-      <c r="K32" s="68" t="n">
+      <c r="K33" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="L32" s="68" t="n">
+      <c r="L33" s="77" t="n">
         <v>12</v>
       </c>
-      <c r="M32" s="67" t="n">
+      <c r="M33" s="67" t="n">
         <v>0.63</v>
       </c>
-      <c r="N32" s="66" t="inlineStr">
+      <c r="N33" s="75" t="inlineStr">
         <is>
           <t>Norge</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="65" t="inlineStr">
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="65" t="inlineStr">
         <is>
           <t>Gruppe J</t>
         </is>
       </c>
-      <c r="B33" s="75" t="inlineStr">
+      <c r="B34" s="66" t="inlineStr">
         <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="C33" s="83" t="n">
+      <c r="C34" s="83" t="n">
         <v>0.47</v>
       </c>
-      <c r="D33" s="77" t="n">
+      <c r="D34" s="68" t="n">
         <v>9</v>
       </c>
-      <c r="E33" s="77" t="n">
+      <c r="E34" s="68" t="n">
         <v>6</v>
       </c>
-      <c r="F33" s="76" t="n">
+      <c r="F34" s="69" t="n">
         <v>3</v>
       </c>
-      <c r="G33" s="78" t="n">
+      <c r="G34" s="70" t="n">
         <v>0</v>
       </c>
-      <c r="H33" s="79" t="inlineStr">
+      <c r="H34" s="71" t="inlineStr">
         <is>
           <t>3–0</t>
-        </is>
-      </c>
-      <c r="I33" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="J33" s="76" t="n">
-        <v>3</v>
-      </c>
-      <c r="K33" s="76" t="n">
-        <v>0</v>
-      </c>
-      <c r="L33" s="76" t="n">
-        <v>6</v>
-      </c>
-      <c r="M33" s="83" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N33" s="75" t="inlineStr">
-        <is>
-          <t>Algerie</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="81" t="inlineStr"/>
-      <c r="B34" s="66" t="inlineStr">
-        <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C34" s="67" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D34" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="E34" s="69" t="n">
-        <v>3</v>
-      </c>
-      <c r="F34" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="G34" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="H34" s="71" t="inlineStr">
-        <is>
-          <t>3–1</t>
         </is>
       </c>
       <c r="I34" s="72" t="n">
         <v>3</v>
       </c>
       <c r="J34" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" s="68" t="n">
-        <v>4</v>
-      </c>
-      <c r="L34" s="68" t="n">
-        <v>11</v>
-      </c>
-      <c r="M34" s="73" t="n">
-        <v>0.38</v>
+        <v>3</v>
+      </c>
+      <c r="K34" s="69" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="M34" s="83" t="n">
+        <v>0.53</v>
       </c>
       <c r="N34" s="66" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="65" t="inlineStr">
-        <is>
-          <t>Gruppe K</t>
-        </is>
-      </c>
+      <c r="A35" s="74" t="inlineStr"/>
       <c r="B35" s="75" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C35" s="82" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D35" s="77" t="n">
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C35" s="67" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D35" s="76" t="n">
         <v>9</v>
       </c>
-      <c r="E35" s="77" t="n">
+      <c r="E35" s="76" t="n">
         <v>3</v>
       </c>
       <c r="F35" s="76" t="n">
@@ -58948,207 +58942,259 @@
       </c>
       <c r="H35" s="79" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I35" s="80" t="n">
         <v>3</v>
       </c>
       <c r="J35" s="76" t="n">
+        <v>4</v>
+      </c>
+      <c r="K35" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="L35" s="77" t="n">
+        <v>11</v>
+      </c>
+      <c r="M35" s="73" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N35" s="75" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="65" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
+      <c r="B36" s="66" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C36" s="82" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D36" s="68" t="n">
+        <v>9</v>
+      </c>
+      <c r="E36" s="68" t="n">
         <v>3</v>
       </c>
-      <c r="K35" s="76" t="n">
-        <v>2</v>
-      </c>
-      <c r="L35" s="76" t="n">
-        <v>8</v>
-      </c>
-      <c r="M35" s="73" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N35" s="75" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="81" t="inlineStr"/>
-      <c r="B36" s="66" t="inlineStr">
-        <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C36" s="73" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D36" s="69" t="n">
-        <v>7</v>
-      </c>
-      <c r="E36" s="69" t="n">
-        <v>3</v>
-      </c>
       <c r="F36" s="69" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G36" s="70" t="n">
         <v>2</v>
       </c>
       <c r="H36" s="71" t="inlineStr">
         <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I36" s="72" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" s="69" t="n">
+        <v>3</v>
+      </c>
+      <c r="K36" s="69" t="n">
+        <v>2</v>
+      </c>
+      <c r="L36" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="M36" s="73" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N36" s="66" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="74" t="inlineStr"/>
+      <c r="B37" s="75" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C37" s="73" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D37" s="76" t="n">
+        <v>7</v>
+      </c>
+      <c r="E37" s="76" t="n">
+        <v>3</v>
+      </c>
+      <c r="F37" s="76" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H37" s="79" t="inlineStr">
+        <is>
           <t>1–3</t>
         </is>
       </c>
-      <c r="I36" s="72" t="n">
+      <c r="I37" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="J36" s="69" t="n">
+      <c r="J37" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="K36" s="68" t="n">
+      <c r="K37" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="L36" s="68" t="n">
+      <c r="L37" s="77" t="n">
         <v>15</v>
       </c>
-      <c r="M36" s="82" t="n">
+      <c r="M37" s="82" t="n">
         <v>0.67</v>
       </c>
-      <c r="N36" s="66" t="inlineStr">
+      <c r="N37" s="75" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="65" t="inlineStr">
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="65" t="inlineStr">
         <is>
           <t>Gruppe L</t>
         </is>
       </c>
-      <c r="B37" s="75" t="inlineStr">
+      <c r="B38" s="66" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="C37" s="83" t="n">
+      <c r="C38" s="83" t="n">
         <v>0.54</v>
       </c>
-      <c r="D37" s="77" t="n">
+      <c r="D38" s="68" t="n">
         <v>20</v>
       </c>
-      <c r="E37" s="77" t="n">
+      <c r="E38" s="68" t="n">
         <v>12</v>
       </c>
-      <c r="F37" s="76" t="n">
+      <c r="F38" s="69" t="n">
         <v>3</v>
       </c>
-      <c r="G37" s="78" t="n">
+      <c r="G38" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="H37" s="79" t="inlineStr">
+      <c r="H38" s="71" t="inlineStr">
         <is>
           <t>4–2</t>
         </is>
       </c>
-      <c r="I37" s="80" t="n">
+      <c r="I38" s="72" t="n">
         <v>3</v>
       </c>
-      <c r="J37" s="76" t="n">
+      <c r="J38" s="69" t="n">
         <v>3</v>
       </c>
-      <c r="K37" s="76" t="n">
+      <c r="K38" s="69" t="n">
         <v>5</v>
       </c>
-      <c r="L37" s="76" t="n">
+      <c r="L38" s="69" t="n">
         <v>11</v>
       </c>
-      <c r="M37" s="83" t="n">
+      <c r="M38" s="83" t="n">
         <v>0.46</v>
       </c>
-      <c r="N37" s="75" t="inlineStr">
+      <c r="N38" s="66" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="81" t="inlineStr"/>
-      <c r="B38" s="66" t="inlineStr">
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="74" t="inlineStr"/>
+      <c r="B39" s="75" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C38" s="73" t="n">
+      <c r="C39" s="73" t="n">
         <v>0.37</v>
       </c>
-      <c r="D38" s="69" t="n">
+      <c r="D39" s="76" t="n">
         <v>8</v>
       </c>
-      <c r="E38" s="69" t="n">
+      <c r="E39" s="76" t="n">
         <v>3</v>
       </c>
-      <c r="F38" s="69" t="n">
+      <c r="F39" s="76" t="n">
         <v>4</v>
       </c>
-      <c r="G38" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="71" t="inlineStr">
+      <c r="G39" s="78" t="n">
+        <v>1</v>
+      </c>
+      <c r="H39" s="79" t="inlineStr">
         <is>
           <t>1–0</t>
         </is>
       </c>
-      <c r="I38" s="72" t="n">
+      <c r="I39" s="80" t="n">
         <v>2</v>
       </c>
-      <c r="J38" s="69" t="n">
+      <c r="J39" s="76" t="n">
         <v>5</v>
       </c>
-      <c r="K38" s="68" t="n">
+      <c r="K39" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="L38" s="68" t="n">
+      <c r="L39" s="77" t="n">
         <v>11</v>
       </c>
-      <c r="M38" s="67" t="n">
+      <c r="M39" s="67" t="n">
         <v>0.63</v>
       </c>
-      <c r="N38" s="66" t="inlineStr">
+      <c r="N39" s="75" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="14" customHeight="1">
-      <c r="A40" s="62" t="inlineStr">
+    <row r="41" ht="14" customHeight="1">
+      <c r="A41" s="62" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="54" t="inlineStr">
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="54" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B41" s="61" t="inlineStr">
+      <c r="B42" s="61" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C41" s="60" t="inlineStr">
+      <c r="C42" s="60" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D41" s="57" t="inlineStr">
+      <c r="D42" s="57" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E41" s="84" t="inlineStr">
+      <c r="E42" s="84" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -59156,8 +59202,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A40:N40"/>
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="A41:N41"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-21 10:01 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -46609,7 +46609,7 @@
     <row r="66" ht="26" customHeight="1">
       <c r="A66" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Rene nullere</t>
+          <t>VM 2026 — Clean sheet</t>
         </is>
       </c>
     </row>
@@ -46636,7 +46636,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>Rene nullere</t>
+          <t>Clean sheet</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Fiks fane-overlay: riktige kategorier og unngå duplikater
Catch-all-kategorien viste alle 30 faner på nytt fordi filtrering ikke
ekskluderte allerede plasserte faner. Løst med Set som sporer brukte IDer.
Kategoriene er nå: Gruppespill og spillertropper / Sluttspill / Statistikk.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Alder" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -809,13 +809,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -834,7 +834,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -858,12 +858,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -877,6 +877,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -889,8 +890,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -904,6 +905,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -913,7 +915,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -928,9 +930,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-21 14:18 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="32-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Toppscorere" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Alder" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Lagstatistikk" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Scoringstidspunkt" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Heatmap" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Ballbesittelse" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -809,13 +809,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -834,7 +834,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -858,12 +858,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -877,7 +877,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -890,8 +889,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -905,7 +904,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -915,7 +913,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -930,9 +928,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -17627,7 +17625,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — 32-delsfinale</t>
+          <t>VM 2026 — 16-delsfinale</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-22 12:20 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,40 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="7" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Scorere og assists" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Alder" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -1385,13 +1385,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1410,7 +1410,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1438,8 +1438,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1465,8 +1465,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1489,7 +1489,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1504,9 +1504,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Rett dato for nattlige kamper — bruk norsk dato fra FIFA API
Dato hentes nå fra FIFA API (Date-feltet, UTC+2) i stedet for
kilde-Excel, slik at dato og klokkeslett alltid er konsistente.
26 kamper hadde feil dato fordi kampene krysser midnatt i norsk tid.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1918,7 +1918,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>11.06 04:00</t>
+          <t>12.06 04:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -2002,7 +2002,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>18.06 03:00</t>
+          <t>19.06 03:00</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -2044,7 +2044,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>24.06 03:00</t>
+          <t>25.06 03:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -2070,7 +2070,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>24.06 03:00</t>
+          <t>25.06 03:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -6012,7 +6012,7 @@
       </c>
       <c r="B3" s="108" t="inlineStr">
         <is>
-          <t>16.06 03:00</t>
+          <t>17.06 03:00</t>
         </is>
       </c>
       <c r="C3" s="109" t="inlineStr">
@@ -6126,7 +6126,7 @@
       </c>
       <c r="B6" s="111" t="inlineStr">
         <is>
-          <t>22.06 05:00</t>
+          <t>23.06 05:00</t>
         </is>
       </c>
       <c r="C6" s="112" t="inlineStr">
@@ -6134,11 +6134,7 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="D6" s="113" t="inlineStr">
-        <is>
-          <t>– – –</t>
-        </is>
-      </c>
+      <c r="D6" s="113" t="inlineStr"/>
       <c r="E6" s="112" t="inlineStr">
         <is>
           <t>Algerie</t>
@@ -6156,7 +6152,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>27.06 04:00</t>
+          <t>28.06 04:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -6182,7 +6178,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>27.06 04:00</t>
+          <t>28.06 04:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -10134,7 +10130,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>17.06 04:00</t>
+          <t>18.06 04:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -10202,7 +10198,7 @@
       </c>
       <c r="B6" s="111" t="inlineStr">
         <is>
-          <t>23.06 04:00</t>
+          <t>24.06 04:00</t>
         </is>
       </c>
       <c r="C6" s="112" t="inlineStr">
@@ -10228,7 +10224,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>27.06 01:30</t>
+          <t>28.06 01:30</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -10254,7 +10250,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>27.06 01:30</t>
+          <t>28.06 01:30</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -14224,7 +14220,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>17.06 01:00</t>
+          <t>18.06 01:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -14292,7 +14288,7 @@
       </c>
       <c r="B6" s="111" t="inlineStr">
         <is>
-          <t>23.06 01:00</t>
+          <t>24.06 01:00</t>
         </is>
       </c>
       <c r="C6" s="112" t="inlineStr">
@@ -30054,7 +30050,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>18.06 00:00</t>
+          <t>19.06 00:00</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -56060,7 +56056,7 @@
       </c>
       <c r="B3" s="108" t="inlineStr">
         <is>
-          <t>13.06 00:00</t>
+          <t>14.06 00:00</t>
         </is>
       </c>
       <c r="C3" s="109" t="inlineStr">
@@ -56102,7 +56098,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>13.06 03:00</t>
+          <t>14.06 03:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -56144,7 +56140,7 @@
       </c>
       <c r="B5" s="108" t="inlineStr">
         <is>
-          <t>19.06 00:00</t>
+          <t>20.06 00:00</t>
         </is>
       </c>
       <c r="C5" s="109" t="inlineStr">
@@ -56186,7 +56182,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>19.06 02:30</t>
+          <t>20.06 02:30</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -56228,7 +56224,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>24.06 00:00</t>
+          <t>25.06 00:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -56254,7 +56250,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>24.06 00:00</t>
+          <t>25.06 00:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -60188,7 +60184,7 @@
       </c>
       <c r="B3" s="108" t="inlineStr">
         <is>
-          <t>12.06 03:00</t>
+          <t>13.06 03:00</t>
         </is>
       </c>
       <c r="C3" s="109" t="inlineStr">
@@ -60314,7 +60310,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>19.06 05:00</t>
+          <t>20.06 05:00</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -60356,7 +60352,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>25.06 04:00</t>
+          <t>26.06 04:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -60382,7 +60378,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>25.06 04:00</t>
+          <t>26.06 04:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -64376,7 +64372,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>14.06 01:00</t>
+          <t>15.06 01:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -64460,7 +64456,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>20.06 02:00</t>
+          <t>21.06 02:00</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -68516,7 +68512,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>14.06 04:00</t>
+          <t>15.06 04:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -68642,7 +68638,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>25.06 01:00</t>
+          <t>26.06 01:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -68668,7 +68664,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>25.06 01:00</t>
+          <t>26.06 01:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -72676,7 +72672,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>15.06 03:00</t>
+          <t>16.06 03:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -72760,7 +72756,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>21.06 03:00</t>
+          <t>22.06 03:00</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -72802,7 +72798,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>26.06 05:00</t>
+          <t>27.06 05:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -72828,7 +72824,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>26.06 05:00</t>
+          <t>27.06 05:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -76814,7 +76810,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>15.06 00:00</t>
+          <t>16.06 00:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -76898,7 +76894,7 @@
       </c>
       <c r="B6" s="108" t="inlineStr">
         <is>
-          <t>21.06 00:00</t>
+          <t>22.06 00:00</t>
         </is>
       </c>
       <c r="C6" s="109" t="inlineStr">
@@ -76940,7 +76936,7 @@
       </c>
       <c r="B7" s="114" t="inlineStr">
         <is>
-          <t>26.06 02:00</t>
+          <t>27.06 02:00</t>
         </is>
       </c>
       <c r="C7" s="115" t="inlineStr">
@@ -76966,7 +76962,7 @@
       </c>
       <c r="B8" s="111" t="inlineStr">
         <is>
-          <t>26.06 02:00</t>
+          <t>27.06 02:00</t>
         </is>
       </c>
       <c r="C8" s="112" t="inlineStr">
@@ -80936,7 +80932,7 @@
       </c>
       <c r="B4" s="108" t="inlineStr">
         <is>
-          <t>16.06 00:00</t>
+          <t>17.06 00:00</t>
         </is>
       </c>
       <c r="C4" s="109" t="inlineStr">
@@ -81008,7 +81004,7 @@
       </c>
       <c r="B6" s="111" t="inlineStr">
         <is>
-          <t>22.06 02:00</t>
+          <t>23.06 02:00</t>
         </is>
       </c>
       <c r="C6" s="112" t="inlineStr">
@@ -81016,11 +81012,7 @@
           <t>Norge</t>
         </is>
       </c>
-      <c r="D6" s="113" t="inlineStr">
-        <is>
-          <t>– – –</t>
-        </is>
-      </c>
+      <c r="D6" s="113" t="inlineStr"/>
       <c r="E6" s="112" t="inlineStr">
         <is>
           <t>Senegal</t>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-22 18:28 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,40 +1,40 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="7" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Scorere og assists" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Alder" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -1385,13 +1385,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1410,7 +1410,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1438,8 +1438,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1465,8 +1465,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1489,7 +1489,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1504,9 +1504,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -46940,7 +46940,7 @@
       </c>
       <c r="F56" s="132" t="inlineStr">
         <is>
-          <t>18.06</t>
+          <t>19.06</t>
         </is>
       </c>
       <c r="G56" s="132" t="n">
@@ -46973,7 +46973,7 @@
       </c>
       <c r="F57" s="132" t="inlineStr">
         <is>
-          <t>14.06</t>
+          <t>15.06</t>
         </is>
       </c>
       <c r="G57" s="132" t="n">
@@ -47105,7 +47105,7 @@
       </c>
       <c r="F61" s="113" t="inlineStr">
         <is>
-          <t>12.06</t>
+          <t>13.06</t>
         </is>
       </c>
       <c r="G61" s="113" t="n">
@@ -47138,7 +47138,7 @@
       </c>
       <c r="F62" s="116" t="inlineStr">
         <is>
-          <t>16.06</t>
+          <t>17.06</t>
         </is>
       </c>
       <c r="G62" s="116" t="n">
@@ -49257,35 +49257,35 @@
     </row>
     <row r="138" ht="16" customHeight="1" s="98">
       <c r="A138" s="114" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B138" s="115" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Østerrike</t>
         </is>
       </c>
       <c r="C138" s="116" t="inlineStr">
         <is>
-          <t>Gruppe B</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D138" s="116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E138" s="116" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F138" s="116" t="inlineStr">
         <is>
-          <t>6,5</t>
+          <t>14,0</t>
         </is>
       </c>
       <c r="G138" s="116" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H138" s="116" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
@@ -49295,23 +49295,23 @@
       </c>
       <c r="B139" s="112" t="inlineStr">
         <is>
-          <t>Frankrike</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C139" s="113" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D139" s="113" t="n">
         <v>1</v>
       </c>
       <c r="E139" s="113" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F139" s="113" t="inlineStr">
         <is>
-          <t>11,0</t>
+          <t>13,0</t>
         </is>
       </c>
       <c r="G139" s="113" t="n">
@@ -49319,7 +49319,7 @@
       </c>
       <c r="H139" s="113" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>62%</t>
         </is>
       </c>
     </row>
@@ -49329,46 +49329,46 @@
       </c>
       <c r="B140" s="115" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
       <c r="C140" s="116" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe B</t>
         </is>
       </c>
       <c r="D140" s="116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E140" s="116" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F140" s="116" t="inlineStr">
         <is>
-          <t>11,0</t>
+          <t>6,5</t>
         </is>
       </c>
       <c r="G140" s="116" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H140" s="116" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>46%</t>
         </is>
       </c>
     </row>
     <row r="141" ht="16" customHeight="1" s="98">
       <c r="A141" s="111" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B141" s="112" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Frankrike</t>
         </is>
       </c>
       <c r="C141" s="113" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="D141" s="113" t="n">
@@ -49383,26 +49383,26 @@
         </is>
       </c>
       <c r="G141" s="113" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H141" s="113" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>73%</t>
         </is>
       </c>
     </row>
     <row r="142" ht="16" customHeight="1" s="98">
       <c r="A142" s="114" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B142" s="115" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Norge</t>
         </is>
       </c>
       <c r="C142" s="116" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="D142" s="116" t="n">
@@ -49417,26 +49417,26 @@
         </is>
       </c>
       <c r="G142" s="116" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H142" s="116" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>45%</t>
         </is>
       </c>
     </row>
     <row r="143" ht="16" customHeight="1" s="98">
       <c r="A143" s="111" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B143" s="112" t="inlineStr">
         <is>
-          <t>Irak</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="C143" s="113" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D143" s="113" t="n">
@@ -49451,21 +49451,21 @@
         </is>
       </c>
       <c r="G143" s="113" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H143" s="113" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
     <row r="144" ht="16" customHeight="1" s="98">
       <c r="A144" s="114" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B144" s="115" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C144" s="116" t="inlineStr">
@@ -49477,79 +49477,79 @@
         <v>1</v>
       </c>
       <c r="E144" s="116" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F144" s="116" t="inlineStr">
         <is>
-          <t>10,0</t>
+          <t>11,0</t>
         </is>
       </c>
       <c r="G144" s="116" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H144" s="116" t="inlineStr">
         <is>
-          <t>60%</t>
+          <t>27%</t>
         </is>
       </c>
     </row>
     <row r="145" ht="16" customHeight="1" s="98">
       <c r="A145" s="111" t="n">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B145" s="112" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>Irak</t>
         </is>
       </c>
       <c r="C145" s="113" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="D145" s="113" t="n">
         <v>1</v>
       </c>
       <c r="E145" s="113" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F145" s="113" t="inlineStr">
         <is>
-          <t>10,0</t>
+          <t>11,0</t>
         </is>
       </c>
       <c r="G145" s="113" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H145" s="113" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>9%</t>
         </is>
       </c>
     </row>
     <row r="146" ht="16" customHeight="1" s="98">
       <c r="A146" s="114" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B146" s="115" t="inlineStr">
         <is>
-          <t>Saudi-Arabia</t>
+          <t>Kroatia</t>
         </is>
       </c>
       <c r="C146" s="116" t="inlineStr">
         <is>
-          <t>Gruppe H</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D146" s="116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E146" s="116" t="n">
         <v>10</v>
       </c>
       <c r="F146" s="116" t="inlineStr">
         <is>
-          <t>5,0</t>
+          <t>10,0</t>
         </is>
       </c>
       <c r="G146" s="116" t="n">
@@ -49563,35 +49563,35 @@
     </row>
     <row r="147" ht="16" customHeight="1" s="98">
       <c r="A147" s="111" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B147" s="112" t="inlineStr">
         <is>
-          <t>Østerrike</t>
+          <t>Saudi-Arabia</t>
         </is>
       </c>
       <c r="C147" s="113" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe H</t>
         </is>
       </c>
       <c r="D147" s="113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E147" s="113" t="n">
         <v>10</v>
       </c>
       <c r="F147" s="113" t="inlineStr">
         <is>
-          <t>10,0</t>
+          <t>5,0</t>
         </is>
       </c>
       <c r="G147" s="113" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H147" s="113" t="inlineStr">
         <is>
-          <t>40%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Generer Stadionoversikt-ark første gang
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -35,6 +35,7 @@
     <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
     <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
     <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -50,7 +51,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="52">
+  <fonts count="55">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -346,8 +347,24 @@
       <color rgb="006B7A99"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000F5132"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00856404"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="001A3C6B"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="45">
+  <fills count="50">
     <fill>
       <patternFill/>
     </fill>
@@ -569,6 +586,31 @@
         <fgColor rgb="000E4D5C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00006847"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001D9E75"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C7F0DF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008B0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000F5132"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="17">
     <border>
@@ -779,7 +821,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="213">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1308,6 +1350,73 @@
     <xf numFmtId="0" fontId="28" fillId="27" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="28" fillId="27" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="26" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="30" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="30" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="45" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="30" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="29" fillId="30" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="46" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="29" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="29" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="30" fillId="29" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="29" fillId="29" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="31" fillId="47" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="40" fillId="48" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="28" fillId="49" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="34" fillId="33" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="49" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="48" fillId="46" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="52" fillId="47" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="53" fillId="33" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="54" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -49057,31 +49166,31 @@
       </c>
       <c r="B132" s="115" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="C132" s="116" t="inlineStr">
         <is>
-          <t>Gruppe H</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D132" s="116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E132" s="116" t="n">
         <v>18</v>
       </c>
       <c r="F132" s="116" t="inlineStr">
         <is>
-          <t>9,0</t>
+          <t>18,0</t>
         </is>
       </c>
       <c r="G132" s="116" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="H132" s="116" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>44%</t>
         </is>
       </c>
     </row>
@@ -49091,12 +49200,12 @@
       </c>
       <c r="B133" s="112" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
       <c r="C133" s="113" t="inlineStr">
         <is>
-          <t>Gruppe E</t>
+          <t>Gruppe H</t>
         </is>
       </c>
       <c r="D133" s="113" t="n">
@@ -49121,35 +49230,35 @@
     </row>
     <row r="134" ht="16" customHeight="1" s="98">
       <c r="A134" s="114" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B134" s="115" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C134" s="116" t="inlineStr">
         <is>
-          <t>Gruppe D</t>
+          <t>Gruppe E</t>
         </is>
       </c>
       <c r="D134" s="116" t="n">
         <v>2</v>
       </c>
       <c r="E134" s="116" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F134" s="116" t="inlineStr">
         <is>
-          <t>8,0</t>
+          <t>9,0</t>
         </is>
       </c>
       <c r="G134" s="116" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H134" s="116" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>28%</t>
         </is>
       </c>
     </row>
@@ -49159,133 +49268,133 @@
       </c>
       <c r="B135" s="112" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="C135" s="113" t="inlineStr">
         <is>
-          <t>Gruppe K</t>
+          <t>Gruppe D</t>
         </is>
       </c>
       <c r="D135" s="113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E135" s="113" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F135" s="113" t="inlineStr">
         <is>
-          <t>15,0</t>
+          <t>8,0</t>
         </is>
       </c>
       <c r="G135" s="113" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H135" s="113" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>19%</t>
         </is>
       </c>
     </row>
     <row r="136" ht="16" customHeight="1" s="98">
       <c r="A136" s="114" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B136" s="115" t="inlineStr">
         <is>
-          <t>Skottland</t>
+          <t>Østerrike</t>
         </is>
       </c>
       <c r="C136" s="116" t="inlineStr">
         <is>
-          <t>Gruppe C</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D136" s="116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E136" s="116" t="n">
         <v>15</v>
       </c>
       <c r="F136" s="116" t="inlineStr">
         <is>
-          <t>7,5</t>
+          <t>15,0</t>
         </is>
       </c>
       <c r="G136" s="116" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H136" s="116" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>33%</t>
         </is>
       </c>
     </row>
     <row r="137" ht="16" customHeight="1" s="98">
       <c r="A137" s="111" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B137" s="112" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C137" s="113" t="inlineStr">
         <is>
-          <t>Gruppe D</t>
+          <t>Gruppe K</t>
         </is>
       </c>
       <c r="D137" s="113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E137" s="113" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F137" s="113" t="inlineStr">
         <is>
-          <t>7,0</t>
+          <t>15,0</t>
         </is>
       </c>
       <c r="G137" s="113" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="H137" s="113" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>27%</t>
         </is>
       </c>
     </row>
     <row r="138" ht="16" customHeight="1" s="98">
       <c r="A138" s="114" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B138" s="115" t="inlineStr">
         <is>
-          <t>Østerrike</t>
+          <t>Skottland</t>
         </is>
       </c>
       <c r="C138" s="116" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe C</t>
         </is>
       </c>
       <c r="D138" s="116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E138" s="116" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F138" s="116" t="inlineStr">
         <is>
-          <t>14,0</t>
+          <t>7,5</t>
         </is>
       </c>
       <c r="G138" s="116" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H138" s="116" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>13%</t>
         </is>
       </c>
     </row>
@@ -49295,37 +49404,37 @@
       </c>
       <c r="B139" s="112" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C139" s="113" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe D</t>
         </is>
       </c>
       <c r="D139" s="113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E139" s="113" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F139" s="113" t="inlineStr">
         <is>
-          <t>13,0</t>
+          <t>7,0</t>
         </is>
       </c>
       <c r="G139" s="113" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H139" s="113" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>43%</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1" s="98">
       <c r="A140" s="114" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B140" s="115" t="inlineStr">
         <is>
@@ -49431,12 +49540,12 @@
       </c>
       <c r="B143" s="112" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C143" s="113" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D143" s="113" t="n">
@@ -49465,12 +49574,12 @@
       </c>
       <c r="B144" s="115" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="C144" s="116" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D144" s="116" t="n">
@@ -49485,11 +49594,11 @@
         </is>
       </c>
       <c r="G144" s="116" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H144" s="116" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
@@ -60101,6 +60210,2173 @@
     <mergeCell ref="A104:D104"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A46:D46"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet30.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" style="98" min="1" max="1"/>
+    <col width="9" customWidth="1" style="98" min="2" max="2"/>
+    <col width="20" customWidth="1" style="98" min="3" max="3"/>
+    <col width="7" customWidth="1" style="98" min="4" max="4"/>
+    <col width="20" customWidth="1" style="98" min="5" max="5"/>
+    <col width="24" customWidth="1" style="98" min="6" max="6"/>
+    <col width="24" customWidth="1" style="98" min="7" max="7"/>
+    <col width="9" customWidth="1" style="98" min="8" max="8"/>
+    <col width="12" customWidth="1" style="98" min="9" max="9"/>
+    <col width="11" customWidth="1" style="98" min="10" max="10"/>
+    <col width="9" customWidth="1" style="98" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="98">
+      <c r="A1" s="105" t="inlineStr">
+        <is>
+          <t>Tilskuere og arenaer — VM 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="98">
+      <c r="A2" s="168" t="inlineStr">
+        <is>
+          <t>Dato</t>
+        </is>
+      </c>
+      <c r="B2" s="168" t="inlineStr">
+        <is>
+          <t>Gruppe</t>
+        </is>
+      </c>
+      <c r="C2" s="107" t="inlineStr">
+        <is>
+          <t>Hjemmelag</t>
+        </is>
+      </c>
+      <c r="D2" s="168" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+      <c r="E2" s="107" t="inlineStr">
+        <is>
+          <t>Bortelag</t>
+        </is>
+      </c>
+      <c r="F2" s="107" t="inlineStr">
+        <is>
+          <t>Arena</t>
+        </is>
+      </c>
+      <c r="G2" s="107" t="inlineStr">
+        <is>
+          <t>By</t>
+        </is>
+      </c>
+      <c r="H2" s="106" t="inlineStr">
+        <is>
+          <t>Land</t>
+        </is>
+      </c>
+      <c r="I2" s="190" t="inlineStr">
+        <is>
+          <t>Tilskuere</t>
+        </is>
+      </c>
+      <c r="J2" s="190" t="inlineStr">
+        <is>
+          <t>Kapasitet</t>
+        </is>
+      </c>
+      <c r="K2" s="106" t="inlineStr">
+        <is>
+          <t>Belegg %</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="98">
+      <c r="A3" s="173" t="inlineStr">
+        <is>
+          <t>11.06</t>
+        </is>
+      </c>
+      <c r="B3" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe A</t>
+        </is>
+      </c>
+      <c r="C3" s="192" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D3" s="172" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="E3" s="193" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="F3" s="192" t="inlineStr">
+        <is>
+          <t>Estadio Azteca</t>
+        </is>
+      </c>
+      <c r="G3" s="194" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="H3" s="195" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I3" s="196" t="n">
+        <v>80824</v>
+      </c>
+      <c r="J3" s="197" t="n">
+        <v>87523</v>
+      </c>
+      <c r="K3" s="198" t="n">
+        <v>0.9234601190544199</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="98">
+      <c r="A4" s="180" t="inlineStr">
+        <is>
+          <t>12.06</t>
+        </is>
+      </c>
+      <c r="B4" s="182" t="inlineStr"/>
+      <c r="C4" s="199" t="inlineStr">
+        <is>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+      <c r="D4" s="181" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="E4" s="200" t="inlineStr">
+        <is>
+          <t>Tsjekkia</t>
+        </is>
+      </c>
+      <c r="F4" s="199" t="inlineStr">
+        <is>
+          <t>Estadio Akron</t>
+        </is>
+      </c>
+      <c r="G4" s="201" t="inlineStr">
+        <is>
+          <t>Zapopan / Guadalajara</t>
+        </is>
+      </c>
+      <c r="H4" s="195" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I4" s="202" t="n">
+        <v>44985</v>
+      </c>
+      <c r="J4" s="203" t="n">
+        <v>49850</v>
+      </c>
+      <c r="K4" s="204" t="n">
+        <v>0.902407221664995</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="98">
+      <c r="A5" s="173" t="inlineStr">
+        <is>
+          <t>12.06</t>
+        </is>
+      </c>
+      <c r="B5" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe B</t>
+        </is>
+      </c>
+      <c r="C5" s="192" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D5" s="172" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E5" s="193" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+      <c r="F5" s="192" t="inlineStr">
+        <is>
+          <t>BMO Field</t>
+        </is>
+      </c>
+      <c r="G5" s="194" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="H5" s="205" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="I5" s="196" t="n">
+        <v>43002</v>
+      </c>
+      <c r="J5" s="197" t="n">
+        <v>45736</v>
+      </c>
+      <c r="K5" s="198" t="n">
+        <v>0.9402221444813713</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="98">
+      <c r="A6" s="180" t="inlineStr">
+        <is>
+          <t>13.06</t>
+        </is>
+      </c>
+      <c r="B6" s="182" t="inlineStr"/>
+      <c r="C6" s="199" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="D6" s="181" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E6" s="200" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="F6" s="199" t="inlineStr">
+        <is>
+          <t>Levi's Stadium</t>
+        </is>
+      </c>
+      <c r="G6" s="201" t="inlineStr">
+        <is>
+          <t>Santa Clara / SF Bay Area</t>
+        </is>
+      </c>
+      <c r="H6" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I6" s="202" t="n">
+        <v>67966</v>
+      </c>
+      <c r="J6" s="203" t="n">
+        <v>68500</v>
+      </c>
+      <c r="K6" s="206" t="n">
+        <v>0.9922043795620438</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="98">
+      <c r="A7" s="173" t="inlineStr">
+        <is>
+          <t>13.06</t>
+        </is>
+      </c>
+      <c r="B7" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe D</t>
+        </is>
+      </c>
+      <c r="C7" s="192" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D7" s="172" t="inlineStr">
+        <is>
+          <t>4–1</t>
+        </is>
+      </c>
+      <c r="E7" s="193" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="F7" s="192" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="G7" s="194" t="inlineStr">
+        <is>
+          <t>Inglewood / Los Angeles</t>
+        </is>
+      </c>
+      <c r="H7" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I7" s="196" t="n">
+        <v>70492</v>
+      </c>
+      <c r="J7" s="197" t="n">
+        <v>70240</v>
+      </c>
+      <c r="K7" s="206" t="n">
+        <v>1.003587699316629</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="98">
+      <c r="A8" s="180" t="inlineStr">
+        <is>
+          <t>14.06</t>
+        </is>
+      </c>
+      <c r="B8" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe C</t>
+        </is>
+      </c>
+      <c r="C8" s="199" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D8" s="181" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E8" s="200" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="F8" s="199" t="inlineStr">
+        <is>
+          <t>MetLife Stadium</t>
+        </is>
+      </c>
+      <c r="G8" s="201" t="inlineStr">
+        <is>
+          <t>East Rutherford, NJ</t>
+        </is>
+      </c>
+      <c r="H8" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I8" s="202" t="n">
+        <v>80663</v>
+      </c>
+      <c r="J8" s="203" t="n">
+        <v>82500</v>
+      </c>
+      <c r="K8" s="206" t="n">
+        <v>0.9777333333333335</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="98">
+      <c r="A9" s="173" t="inlineStr">
+        <is>
+          <t>14.06</t>
+        </is>
+      </c>
+      <c r="B9" s="174" t="inlineStr"/>
+      <c r="C9" s="192" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="D9" s="172" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="E9" s="193" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+      <c r="F9" s="192" t="inlineStr">
+        <is>
+          <t>Gillette Stadium</t>
+        </is>
+      </c>
+      <c r="G9" s="194" t="inlineStr">
+        <is>
+          <t>Foxborough / Boston</t>
+        </is>
+      </c>
+      <c r="H9" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I9" s="196" t="n">
+        <v>64146</v>
+      </c>
+      <c r="J9" s="197" t="n">
+        <v>65878</v>
+      </c>
+      <c r="K9" s="206" t="n">
+        <v>0.9737089772002793</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="98">
+      <c r="A10" s="180" t="inlineStr">
+        <is>
+          <t>14.06</t>
+        </is>
+      </c>
+      <c r="B10" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe D</t>
+        </is>
+      </c>
+      <c r="C10" s="199" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="D10" s="181" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="E10" s="200" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="F10" s="199" t="inlineStr">
+        <is>
+          <t>BC Place</t>
+        </is>
+      </c>
+      <c r="G10" s="201" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H10" s="205" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="I10" s="202" t="n">
+        <v>52497</v>
+      </c>
+      <c r="J10" s="203" t="n">
+        <v>54500</v>
+      </c>
+      <c r="K10" s="198" t="n">
+        <v>0.9632477064220184</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="98">
+      <c r="A11" s="173" t="inlineStr">
+        <is>
+          <t>14.06</t>
+        </is>
+      </c>
+      <c r="B11" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="C11" s="192" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D11" s="172" t="inlineStr">
+        <is>
+          <t>7–1</t>
+        </is>
+      </c>
+      <c r="E11" s="193" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="F11" s="192" t="inlineStr">
+        <is>
+          <t>NRG Stadium</t>
+        </is>
+      </c>
+      <c r="G11" s="194" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H11" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I11" s="196" t="n">
+        <v>68021</v>
+      </c>
+      <c r="J11" s="197" t="n">
+        <v>72220</v>
+      </c>
+      <c r="K11" s="198" t="n">
+        <v>0.9418582110218776</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="98">
+      <c r="A12" s="180" t="inlineStr">
+        <is>
+          <t>14.06</t>
+        </is>
+      </c>
+      <c r="B12" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="C12" s="199" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D12" s="181" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="E12" s="200" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F12" s="199" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G12" s="201" t="inlineStr">
+        <is>
+          <t>Arlington / Dallas</t>
+        </is>
+      </c>
+      <c r="H12" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I12" s="202" t="n">
+        <v>69285</v>
+      </c>
+      <c r="J12" s="203" t="n">
+        <v>80000</v>
+      </c>
+      <c r="K12" s="207" t="n">
+        <v>0.8660624999999998</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="98">
+      <c r="A13" s="173" t="inlineStr">
+        <is>
+          <t>15.06</t>
+        </is>
+      </c>
+      <c r="B13" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="C13" s="192" t="inlineStr">
+        <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="D13" s="172" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="E13" s="193" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="F13" s="192" t="inlineStr">
+        <is>
+          <t>Lincoln Financial Field</t>
+        </is>
+      </c>
+      <c r="G13" s="194" t="inlineStr">
+        <is>
+          <t>Philadelphia</t>
+        </is>
+      </c>
+      <c r="H13" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I13" s="196" t="n">
+        <v>68274</v>
+      </c>
+      <c r="J13" s="197" t="n">
+        <v>69796</v>
+      </c>
+      <c r="K13" s="206" t="n">
+        <v>0.9781935927560319</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="98">
+      <c r="A14" s="180" t="inlineStr">
+        <is>
+          <t>15.06</t>
+        </is>
+      </c>
+      <c r="B14" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="C14" s="199" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+      <c r="D14" s="181" t="inlineStr">
+        <is>
+          <t>5–1</t>
+        </is>
+      </c>
+      <c r="E14" s="200" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="F14" s="199" t="inlineStr">
+        <is>
+          <t>Estadio BBVA</t>
+        </is>
+      </c>
+      <c r="G14" s="201" t="inlineStr">
+        <is>
+          <t>San Nicolás / Monterrey</t>
+        </is>
+      </c>
+      <c r="H14" s="195" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I14" s="202" t="n">
+        <v>50987</v>
+      </c>
+      <c r="J14" s="203" t="n">
+        <v>53464</v>
+      </c>
+      <c r="K14" s="198" t="n">
+        <v>0.9536697590902289</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="98">
+      <c r="A15" s="173" t="inlineStr">
+        <is>
+          <t>15.06</t>
+        </is>
+      </c>
+      <c r="B15" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
+      <c r="C15" s="192" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="D15" s="172" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E15" s="193" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F15" s="192" t="inlineStr">
+        <is>
+          <t>Lumen Field</t>
+        </is>
+      </c>
+      <c r="G15" s="194" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="H15" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I15" s="196" t="n">
+        <v>66775</v>
+      </c>
+      <c r="J15" s="197" t="n">
+        <v>68740</v>
+      </c>
+      <c r="K15" s="206" t="n">
+        <v>0.9714140238580157</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="98">
+      <c r="A16" s="180" t="inlineStr">
+        <is>
+          <t>15.06</t>
+        </is>
+      </c>
+      <c r="B16" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="C16" s="199" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D16" s="181" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="E16" s="200" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+      <c r="F16" s="199" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Stadium</t>
+        </is>
+      </c>
+      <c r="G16" s="201" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H16" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I16" s="202" t="n">
+        <v>67640</v>
+      </c>
+      <c r="J16" s="203" t="n">
+        <v>71000</v>
+      </c>
+      <c r="K16" s="198" t="n">
+        <v>0.9526760563380282</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="98">
+      <c r="A17" s="173" t="inlineStr">
+        <is>
+          <t>16.06</t>
+        </is>
+      </c>
+      <c r="B17" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
+      <c r="C17" s="192" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="D17" s="172" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="E17" s="193" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="F17" s="192" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="G17" s="194" t="inlineStr">
+        <is>
+          <t>Inglewood / Los Angeles</t>
+        </is>
+      </c>
+      <c r="H17" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I17" s="196" t="n">
+        <v>70108</v>
+      </c>
+      <c r="J17" s="197" t="n">
+        <v>70240</v>
+      </c>
+      <c r="K17" s="206" t="n">
+        <v>0.998120728929385</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="98">
+      <c r="A18" s="180" t="inlineStr">
+        <is>
+          <t>16.06</t>
+        </is>
+      </c>
+      <c r="B18" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="C18" s="199" t="inlineStr">
+        <is>
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="D18" s="181" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E18" s="200" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="F18" s="199" t="inlineStr">
+        <is>
+          <t>Hard Rock Stadium</t>
+        </is>
+      </c>
+      <c r="G18" s="201" t="inlineStr">
+        <is>
+          <t>Miami Gardens / Miami</t>
+        </is>
+      </c>
+      <c r="H18" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I18" s="202" t="n">
+        <v>62764</v>
+      </c>
+      <c r="J18" s="203" t="n">
+        <v>64767</v>
+      </c>
+      <c r="K18" s="198" t="n">
+        <v>0.9690737566970834</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="98">
+      <c r="A19" s="173" t="inlineStr">
+        <is>
+          <t>16.06</t>
+        </is>
+      </c>
+      <c r="B19" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe I</t>
+        </is>
+      </c>
+      <c r="C19" s="192" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="D19" s="172" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="E19" s="193" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="F19" s="192" t="inlineStr">
+        <is>
+          <t>MetLife Stadium</t>
+        </is>
+      </c>
+      <c r="G19" s="194" t="inlineStr">
+        <is>
+          <t>East Rutherford, NJ</t>
+        </is>
+      </c>
+      <c r="H19" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I19" s="196" t="n">
+        <v>80545</v>
+      </c>
+      <c r="J19" s="197" t="n">
+        <v>82500</v>
+      </c>
+      <c r="K19" s="206" t="n">
+        <v>0.9763030303030305</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="98">
+      <c r="A20" s="180" t="inlineStr">
+        <is>
+          <t>17.06</t>
+        </is>
+      </c>
+      <c r="B20" s="182" t="inlineStr"/>
+      <c r="C20" s="199" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="D20" s="181" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="E20" s="200" t="inlineStr">
+        <is>
+          <t>Norge</t>
+        </is>
+      </c>
+      <c r="F20" s="199" t="inlineStr">
+        <is>
+          <t>Gillette Stadium</t>
+        </is>
+      </c>
+      <c r="G20" s="201" t="inlineStr">
+        <is>
+          <t>Foxborough / Boston</t>
+        </is>
+      </c>
+      <c r="H20" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I20" s="202" t="n">
+        <v>63106</v>
+      </c>
+      <c r="J20" s="203" t="n">
+        <v>65878</v>
+      </c>
+      <c r="K20" s="198" t="n">
+        <v>0.9579222198609549</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="98">
+      <c r="A21" s="173" t="inlineStr">
+        <is>
+          <t>17.06</t>
+        </is>
+      </c>
+      <c r="B21" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe J</t>
+        </is>
+      </c>
+      <c r="C21" s="192" t="inlineStr">
+        <is>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="D21" s="172" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="E21" s="193" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+      <c r="F21" s="192" t="inlineStr">
+        <is>
+          <t>Arrowhead Stadium</t>
+        </is>
+      </c>
+      <c r="G21" s="194" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="H21" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I21" s="196" t="n">
+        <v>69045</v>
+      </c>
+      <c r="J21" s="197" t="n">
+        <v>76416</v>
+      </c>
+      <c r="K21" s="204" t="n">
+        <v>0.9035411432160804</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1" s="98">
+      <c r="A22" s="180" t="inlineStr">
+        <is>
+          <t>17.06</t>
+        </is>
+      </c>
+      <c r="B22" s="182" t="inlineStr"/>
+      <c r="C22" s="199" t="inlineStr">
+        <is>
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="D22" s="181" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="E22" s="200" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F22" s="199" t="inlineStr">
+        <is>
+          <t>Levi's Stadium</t>
+        </is>
+      </c>
+      <c r="G22" s="201" t="inlineStr">
+        <is>
+          <t>Santa Clara / SF Bay Area</t>
+        </is>
+      </c>
+      <c r="H22" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I22" s="202" t="n">
+        <v>68527</v>
+      </c>
+      <c r="J22" s="203" t="n">
+        <v>68500</v>
+      </c>
+      <c r="K22" s="206" t="n">
+        <v>1.000394160583942</v>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1" s="98">
+      <c r="A23" s="173" t="inlineStr">
+        <is>
+          <t>17.06</t>
+        </is>
+      </c>
+      <c r="B23" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
+      <c r="C23" s="192" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="D23" s="172" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E23" s="193" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+      <c r="F23" s="192" t="inlineStr">
+        <is>
+          <t>NRG Stadium</t>
+        </is>
+      </c>
+      <c r="G23" s="194" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H23" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I23" s="196" t="n">
+        <v>68777</v>
+      </c>
+      <c r="J23" s="197" t="n">
+        <v>72220</v>
+      </c>
+      <c r="K23" s="198" t="n">
+        <v>0.9523262254223206</v>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1" s="98">
+      <c r="A24" s="180" t="inlineStr">
+        <is>
+          <t>17.06</t>
+        </is>
+      </c>
+      <c r="B24" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="C24" s="199" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="D24" s="181" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="E24" s="200" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+      <c r="F24" s="199" t="inlineStr">
+        <is>
+          <t>AT&amp;T Stadium</t>
+        </is>
+      </c>
+      <c r="G24" s="201" t="inlineStr">
+        <is>
+          <t>Arlington / Dallas</t>
+        </is>
+      </c>
+      <c r="H24" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I24" s="202" t="n">
+        <v>70389</v>
+      </c>
+      <c r="J24" s="203" t="n">
+        <v>80000</v>
+      </c>
+      <c r="K24" s="204" t="n">
+        <v>0.8798625</v>
+      </c>
+    </row>
+    <row r="25" ht="18" customHeight="1" s="98">
+      <c r="A25" s="173" t="inlineStr">
+        <is>
+          <t>18.06</t>
+        </is>
+      </c>
+      <c r="B25" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe A</t>
+        </is>
+      </c>
+      <c r="C25" s="192" t="inlineStr">
+        <is>
+          <t>Tsjekkia</t>
+        </is>
+      </c>
+      <c r="D25" s="172" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E25" s="193" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="F25" s="192" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Stadium</t>
+        </is>
+      </c>
+      <c r="G25" s="194" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H25" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I25" s="196" t="n">
+        <v>67442</v>
+      </c>
+      <c r="J25" s="197" t="n">
+        <v>71000</v>
+      </c>
+      <c r="K25" s="198" t="n">
+        <v>0.9498873239436619</v>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1" s="98">
+      <c r="A26" s="180" t="inlineStr">
+        <is>
+          <t>18.06</t>
+        </is>
+      </c>
+      <c r="B26" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe B</t>
+        </is>
+      </c>
+      <c r="C26" s="199" t="inlineStr">
+        <is>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="D26" s="181" t="inlineStr">
+        <is>
+          <t>4–1</t>
+        </is>
+      </c>
+      <c r="E26" s="200" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+      <c r="F26" s="199" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="G26" s="201" t="inlineStr">
+        <is>
+          <t>Inglewood / Los Angeles</t>
+        </is>
+      </c>
+      <c r="H26" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I26" s="202" t="n">
+        <v>70026</v>
+      </c>
+      <c r="J26" s="203" t="n">
+        <v>70240</v>
+      </c>
+      <c r="K26" s="206" t="n">
+        <v>0.9969533029612756</v>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1" s="98">
+      <c r="A27" s="173" t="inlineStr">
+        <is>
+          <t>18.06</t>
+        </is>
+      </c>
+      <c r="B27" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
+      <c r="C27" s="192" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="D27" s="172" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="E27" s="193" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="F27" s="192" t="inlineStr">
+        <is>
+          <t>Estadio Azteca</t>
+        </is>
+      </c>
+      <c r="G27" s="194" t="inlineStr">
+        <is>
+          <t>Mexico City</t>
+        </is>
+      </c>
+      <c r="H27" s="195" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I27" s="196" t="n">
+        <v>80824</v>
+      </c>
+      <c r="J27" s="197" t="n">
+        <v>87523</v>
+      </c>
+      <c r="K27" s="198" t="n">
+        <v>0.9234601190544199</v>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1" s="98">
+      <c r="A28" s="180" t="inlineStr">
+        <is>
+          <t>18.06</t>
+        </is>
+      </c>
+      <c r="B28" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="C28" s="199" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="D28" s="181" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="E28" s="200" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="F28" s="199" t="inlineStr">
+        <is>
+          <t>BMO Field</t>
+        </is>
+      </c>
+      <c r="G28" s="201" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="H28" s="205" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="I28" s="202" t="n">
+        <v>42942</v>
+      </c>
+      <c r="J28" s="203" t="n">
+        <v>45736</v>
+      </c>
+      <c r="K28" s="198" t="n">
+        <v>0.9389102676228791</v>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1" s="98">
+      <c r="A29" s="173" t="inlineStr">
+        <is>
+          <t>19.06</t>
+        </is>
+      </c>
+      <c r="B29" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe A</t>
+        </is>
+      </c>
+      <c r="C29" s="192" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="D29" s="172" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="E29" s="193" t="inlineStr">
+        <is>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+      <c r="F29" s="192" t="inlineStr">
+        <is>
+          <t>Estadio Akron</t>
+        </is>
+      </c>
+      <c r="G29" s="194" t="inlineStr">
+        <is>
+          <t>Zapopan / Guadalajara</t>
+        </is>
+      </c>
+      <c r="H29" s="195" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I29" s="196" t="n">
+        <v>45522</v>
+      </c>
+      <c r="J29" s="197" t="n">
+        <v>49850</v>
+      </c>
+      <c r="K29" s="204" t="n">
+        <v>0.9131795386158476</v>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1" s="98">
+      <c r="A30" s="180" t="inlineStr">
+        <is>
+          <t>19.06</t>
+        </is>
+      </c>
+      <c r="B30" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe B</t>
+        </is>
+      </c>
+      <c r="C30" s="199" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D30" s="181" t="inlineStr">
+        <is>
+          <t>6–0</t>
+        </is>
+      </c>
+      <c r="E30" s="200" t="inlineStr">
+        <is>
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="F30" s="199" t="inlineStr">
+        <is>
+          <t>BC Place</t>
+        </is>
+      </c>
+      <c r="G30" s="201" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H30" s="205" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="I30" s="202" t="n">
+        <v>52497</v>
+      </c>
+      <c r="J30" s="203" t="n">
+        <v>54500</v>
+      </c>
+      <c r="K30" s="198" t="n">
+        <v>0.9632477064220184</v>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1" s="98">
+      <c r="A31" s="173" t="inlineStr">
+        <is>
+          <t>19.06</t>
+        </is>
+      </c>
+      <c r="B31" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe D</t>
+        </is>
+      </c>
+      <c r="C31" s="192" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D31" s="172" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="E31" s="193" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="F31" s="192" t="inlineStr">
+        <is>
+          <t>Lumen Field</t>
+        </is>
+      </c>
+      <c r="G31" s="194" t="inlineStr">
+        <is>
+          <t>Seattle</t>
+        </is>
+      </c>
+      <c r="H31" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I31" s="196" t="n">
+        <v>66925</v>
+      </c>
+      <c r="J31" s="197" t="n">
+        <v>68740</v>
+      </c>
+      <c r="K31" s="206" t="n">
+        <v>0.9735961594413733</v>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1" s="98">
+      <c r="A32" s="180" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="B32" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe C</t>
+        </is>
+      </c>
+      <c r="C32" s="199" t="inlineStr">
+        <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+      <c r="D32" s="181" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="E32" s="200" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="F32" s="199" t="inlineStr">
+        <is>
+          <t>Gillette Stadium</t>
+        </is>
+      </c>
+      <c r="G32" s="201" t="inlineStr">
+        <is>
+          <t>Foxborough / Boston</t>
+        </is>
+      </c>
+      <c r="H32" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I32" s="202" t="n">
+        <v>64146</v>
+      </c>
+      <c r="J32" s="203" t="n">
+        <v>65878</v>
+      </c>
+      <c r="K32" s="206" t="n">
+        <v>0.9737089772002793</v>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1" s="98">
+      <c r="A33" s="173" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="B33" s="174" t="inlineStr"/>
+      <c r="C33" s="192" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D33" s="172" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="E33" s="193" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="F33" s="192" t="inlineStr">
+        <is>
+          <t>Lincoln Financial Field</t>
+        </is>
+      </c>
+      <c r="G33" s="194" t="inlineStr">
+        <is>
+          <t>Philadelphia</t>
+        </is>
+      </c>
+      <c r="H33" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I33" s="196" t="n">
+        <v>68324</v>
+      </c>
+      <c r="J33" s="197" t="n">
+        <v>69796</v>
+      </c>
+      <c r="K33" s="206" t="n">
+        <v>0.9789099661871741</v>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1" s="98">
+      <c r="A34" s="180" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="B34" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe D</t>
+        </is>
+      </c>
+      <c r="C34" s="199" t="inlineStr">
+        <is>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="D34" s="181" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="E34" s="200" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="F34" s="199" t="inlineStr">
+        <is>
+          <t>Levi's Stadium</t>
+        </is>
+      </c>
+      <c r="G34" s="201" t="inlineStr">
+        <is>
+          <t>Santa Clara / SF Bay Area</t>
+        </is>
+      </c>
+      <c r="H34" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I34" s="202" t="n">
+        <v>68827</v>
+      </c>
+      <c r="J34" s="203" t="n">
+        <v>68500</v>
+      </c>
+      <c r="K34" s="206" t="n">
+        <v>1.004773722627737</v>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1" s="98">
+      <c r="A35" s="173" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="B35" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="C35" s="192" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D35" s="172" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="E35" s="193" t="inlineStr">
+        <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="F35" s="192" t="inlineStr">
+        <is>
+          <t>BMO Field</t>
+        </is>
+      </c>
+      <c r="G35" s="194" t="inlineStr">
+        <is>
+          <t>Toronto</t>
+        </is>
+      </c>
+      <c r="H35" s="205" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="I35" s="196" t="n">
+        <v>43036</v>
+      </c>
+      <c r="J35" s="197" t="n">
+        <v>45736</v>
+      </c>
+      <c r="K35" s="198" t="n">
+        <v>0.9409655413678503</v>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1" s="98">
+      <c r="A36" s="180" t="inlineStr">
+        <is>
+          <t>20.06</t>
+        </is>
+      </c>
+      <c r="B36" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="C36" s="199" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D36" s="181" t="inlineStr">
+        <is>
+          <t>5–1</t>
+        </is>
+      </c>
+      <c r="E36" s="200" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+      <c r="F36" s="199" t="inlineStr">
+        <is>
+          <t>NRG Stadium</t>
+        </is>
+      </c>
+      <c r="G36" s="201" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H36" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I36" s="202" t="n">
+        <v>68777</v>
+      </c>
+      <c r="J36" s="203" t="n">
+        <v>72220</v>
+      </c>
+      <c r="K36" s="198" t="n">
+        <v>0.9523262254223206</v>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1" s="98">
+      <c r="A37" s="173" t="inlineStr">
+        <is>
+          <t>21.06</t>
+        </is>
+      </c>
+      <c r="B37" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="C37" s="192" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="D37" s="172" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="E37" s="193" t="inlineStr">
+        <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="F37" s="192" t="inlineStr">
+        <is>
+          <t>Arrowhead Stadium</t>
+        </is>
+      </c>
+      <c r="G37" s="194" t="inlineStr">
+        <is>
+          <t>Kansas City</t>
+        </is>
+      </c>
+      <c r="H37" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I37" s="196" t="n">
+        <v>68598</v>
+      </c>
+      <c r="J37" s="197" t="n">
+        <v>76416</v>
+      </c>
+      <c r="K37" s="204" t="n">
+        <v>0.8976915829145728</v>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1" s="98">
+      <c r="A38" s="180" t="inlineStr">
+        <is>
+          <t>21.06</t>
+        </is>
+      </c>
+      <c r="B38" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="C38" s="199" t="inlineStr">
+        <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="D38" s="181" t="inlineStr">
+        <is>
+          <t>0–4</t>
+        </is>
+      </c>
+      <c r="E38" s="200" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F38" s="199" t="inlineStr">
+        <is>
+          <t>Estadio BBVA</t>
+        </is>
+      </c>
+      <c r="G38" s="201" t="inlineStr">
+        <is>
+          <t>San Nicolás / Monterrey</t>
+        </is>
+      </c>
+      <c r="H38" s="195" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I38" s="202" t="n">
+        <v>51243</v>
+      </c>
+      <c r="J38" s="203" t="n">
+        <v>53464</v>
+      </c>
+      <c r="K38" s="198" t="n">
+        <v>0.9584580278318121</v>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1" s="98">
+      <c r="A39" s="173" t="inlineStr">
+        <is>
+          <t>21.06</t>
+        </is>
+      </c>
+      <c r="B39" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
+      <c r="C39" s="192" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="D39" s="172" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="E39" s="193" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="F39" s="192" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="G39" s="194" t="inlineStr">
+        <is>
+          <t>Inglewood / Los Angeles</t>
+        </is>
+      </c>
+      <c r="H39" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I39" s="196" t="n">
+        <v>70317</v>
+      </c>
+      <c r="J39" s="197" t="n">
+        <v>70240</v>
+      </c>
+      <c r="K39" s="206" t="n">
+        <v>1.001096241457859</v>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="98">
+      <c r="A40" s="180" t="inlineStr">
+        <is>
+          <t>21.06</t>
+        </is>
+      </c>
+      <c r="B40" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="C40" s="199" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="D40" s="181" t="inlineStr">
+        <is>
+          <t>4–0</t>
+        </is>
+      </c>
+      <c r="E40" s="200" t="inlineStr">
+        <is>
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="F40" s="199" t="inlineStr">
+        <is>
+          <t>Mercedes-Benz Stadium</t>
+        </is>
+      </c>
+      <c r="G40" s="201" t="inlineStr">
+        <is>
+          <t>Atlanta</t>
+        </is>
+      </c>
+      <c r="H40" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I40" s="202" t="n">
+        <v>68239</v>
+      </c>
+      <c r="J40" s="203" t="n">
+        <v>71000</v>
+      </c>
+      <c r="K40" s="198" t="n">
+        <v>0.961112676056338</v>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="98">
+      <c r="A41" s="173" t="inlineStr">
+        <is>
+          <t>22.06</t>
+        </is>
+      </c>
+      <c r="B41" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
+      <c r="C41" s="192" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="D41" s="172" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="E41" s="193" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="F41" s="192" t="inlineStr">
+        <is>
+          <t>BC Place</t>
+        </is>
+      </c>
+      <c r="G41" s="194" t="inlineStr">
+        <is>
+          <t>Vancouver</t>
+        </is>
+      </c>
+      <c r="H41" s="205" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="I41" s="196" t="n">
+        <v>52497</v>
+      </c>
+      <c r="J41" s="197" t="n">
+        <v>54500</v>
+      </c>
+      <c r="K41" s="198" t="n">
+        <v>0.9632477064220184</v>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="98">
+      <c r="A42" s="180" t="inlineStr">
+        <is>
+          <t>22.06</t>
+        </is>
+      </c>
+      <c r="B42" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="C42" s="199" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="D42" s="181" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="E42" s="200" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+      <c r="F42" s="199" t="inlineStr">
+        <is>
+          <t>Hard Rock Stadium</t>
+        </is>
+      </c>
+      <c r="G42" s="201" t="inlineStr">
+        <is>
+          <t>Miami Gardens / Miami</t>
+        </is>
+      </c>
+      <c r="H42" s="169" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I42" s="202" t="n">
+        <v>64003</v>
+      </c>
+      <c r="J42" s="203" t="n">
+        <v>64767</v>
+      </c>
+      <c r="K42" s="206" t="n">
+        <v>0.9882038692544043</v>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1" s="98">
+      <c r="A44" s="158" t="inlineStr">
+        <is>
+          <t>Belegg:</t>
+        </is>
+      </c>
+      <c r="B44" s="208" t="inlineStr">
+        <is>
+          <t>≥97% (praktisk utsolgt)</t>
+        </is>
+      </c>
+      <c r="C44" s="209" t="inlineStr">
+        <is>
+          <t>92–96%</t>
+        </is>
+      </c>
+      <c r="D44" s="210" t="inlineStr">
+        <is>
+          <t>87–91%</t>
+        </is>
+      </c>
+      <c r="E44" s="211" t="inlineStr">
+        <is>
+          <t>&lt;87%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="14" customHeight="1" s="98">
+      <c r="A45" s="166" t="inlineStr">
+        <is>
+          <t>Kapasitetstall: offisielle arenakapasiteter (ikke FIFA-sertifisert VM-kapasitet som kan avvike noe)</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="98">
+      <c r="A47" s="212" t="inlineStr">
+        <is>
+          <t>Totalt tilskuere: 2 563 003</t>
+        </is>
+      </c>
+      <c r="C47" s="212" t="inlineStr">
+        <is>
+          <t>Snitt belegg: 95.6%</t>
+        </is>
+      </c>
+      <c r="E47" s="212" t="inlineStr">
+        <is>
+          <t>Høyest: 80 824 (Mexico – Sør-Afrika)</t>
+        </is>
+      </c>
+      <c r="H47" s="212" t="inlineStr">
+        <is>
+          <t>Lavest: 42 942 (Ghana – Panama)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A45:K45"/>
+    <mergeCell ref="A1:K1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Stadionoversikt: gruppe på alle rader, smalere Dato/Bortelag/Land-kolonner
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="7" activeTab="12" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Kort" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Scorere og assists" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Alder" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubber" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Nivå 2 og lavere" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'Klubber'!$A$2:$E$2</definedName>
@@ -1494,13 +1494,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1519,7 +1519,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1547,8 +1547,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1574,8 +1574,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1598,7 +1598,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1613,9 +1613,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -60224,14 +60224,14 @@
   <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="98" min="1" max="1"/>
+    <col width="7" customWidth="1" style="98" min="1" max="1"/>
     <col width="9" customWidth="1" style="98" min="2" max="2"/>
     <col width="20" customWidth="1" style="98" min="3" max="3"/>
     <col width="7" customWidth="1" style="98" min="4" max="4"/>
-    <col width="20" customWidth="1" style="98" min="5" max="5"/>
+    <col width="16" customWidth="1" style="98" min="5" max="5"/>
     <col width="24" customWidth="1" style="98" min="6" max="6"/>
     <col width="24" customWidth="1" style="98" min="7" max="7"/>
-    <col width="9" customWidth="1" style="98" min="8" max="8"/>
+    <col width="7" customWidth="1" style="98" min="8" max="8"/>
     <col width="12" customWidth="1" style="98" min="9" max="9"/>
     <col width="11" customWidth="1" style="98" min="10" max="10"/>
     <col width="9" customWidth="1" style="98" min="11" max="11"/>
@@ -60358,7 +60358,11 @@
           <t>12.06</t>
         </is>
       </c>
-      <c r="B4" s="182" t="inlineStr"/>
+      <c r="B4" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe A</t>
+        </is>
+      </c>
       <c r="C4" s="199" t="inlineStr">
         <is>
           <t>Sør-Korea</t>
@@ -60456,7 +60460,11 @@
           <t>13.06</t>
         </is>
       </c>
-      <c r="B6" s="182" t="inlineStr"/>
+      <c r="B6" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe B</t>
+        </is>
+      </c>
       <c r="C6" s="199" t="inlineStr">
         <is>
           <t>Qatar</t>
@@ -60605,7 +60613,11 @@
           <t>14.06</t>
         </is>
       </c>
-      <c r="B9" s="174" t="inlineStr"/>
+      <c r="B9" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe C</t>
+        </is>
+      </c>
       <c r="C9" s="192" t="inlineStr">
         <is>
           <t>Haiti</t>
@@ -61162,7 +61174,11 @@
           <t>17.06</t>
         </is>
       </c>
-      <c r="B20" s="182" t="inlineStr"/>
+      <c r="B20" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe I</t>
+        </is>
+      </c>
       <c r="C20" s="199" t="inlineStr">
         <is>
           <t>Irak</t>
@@ -61260,7 +61276,11 @@
           <t>17.06</t>
         </is>
       </c>
-      <c r="B22" s="182" t="inlineStr"/>
+      <c r="B22" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe J</t>
+        </is>
+      </c>
       <c r="C22" s="199" t="inlineStr">
         <is>
           <t>Østerrike</t>
@@ -61817,7 +61837,11 @@
           <t>20.06</t>
         </is>
       </c>
-      <c r="B33" s="174" t="inlineStr"/>
+      <c r="B33" s="191" t="inlineStr">
+        <is>
+          <t>Gruppe C</t>
+        </is>
+      </c>
       <c r="C33" s="192" t="inlineStr">
         <is>
           <t>Brasil</t>

</xml_diff>

<commit_message>
Legg til FIFA-ranking-fane og oppdater data
Ny FIFA-ranking-fane i index.html. Oppdatert wc2026_stats3.json og
Excel-kildefil med siste kampdata.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -49346,31 +49346,31 @@
       </c>
       <c r="B134" s="115" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>Frankrike</t>
         </is>
       </c>
       <c r="C134" s="116" t="inlineStr">
         <is>
-          <t>Gruppe H</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="D134" s="116" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E134" s="116" t="n">
         <v>18</v>
       </c>
       <c r="F134" s="116" t="inlineStr">
         <is>
-          <t>9,0</t>
+          <t>18,0</t>
         </is>
       </c>
       <c r="G134" s="116" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H134" s="116" t="inlineStr">
         <is>
-          <t>28%</t>
+          <t>50%</t>
         </is>
       </c>
     </row>
@@ -49380,12 +49380,12 @@
       </c>
       <c r="B135" s="112" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
       <c r="C135" s="113" t="inlineStr">
         <is>
-          <t>Gruppe E</t>
+          <t>Gruppe H</t>
         </is>
       </c>
       <c r="D135" s="113" t="n">
@@ -49410,27 +49410,27 @@
     </row>
     <row r="136" ht="16" customHeight="1" s="98">
       <c r="A136" s="114" t="n">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B136" s="115" t="inlineStr">
         <is>
-          <t>Østerrike</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="C136" s="116" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe E</t>
         </is>
       </c>
       <c r="D136" s="116" t="n">
         <v>2</v>
       </c>
       <c r="E136" s="116" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F136" s="116" t="inlineStr">
         <is>
-          <t>8,0</t>
+          <t>9,0</t>
         </is>
       </c>
       <c r="G136" s="116" t="n">
@@ -49438,22 +49438,22 @@
       </c>
       <c r="H136" s="116" t="inlineStr">
         <is>
-          <t>31%</t>
+          <t>28%</t>
         </is>
       </c>
     </row>
     <row r="137" ht="16" customHeight="1" s="98">
       <c r="A137" s="111" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B137" s="112" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Østerrike</t>
         </is>
       </c>
       <c r="C137" s="113" t="inlineStr">
         <is>
-          <t>Gruppe D</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D137" s="113" t="n">
@@ -49468,113 +49468,113 @@
         </is>
       </c>
       <c r="G137" s="113" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H137" s="113" t="inlineStr">
         <is>
-          <t>19%</t>
+          <t>31%</t>
         </is>
       </c>
     </row>
     <row r="138" ht="16" customHeight="1" s="98">
       <c r="A138" s="114" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B138" s="115" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="C138" s="116" t="inlineStr">
         <is>
-          <t>Gruppe K</t>
+          <t>Gruppe D</t>
         </is>
       </c>
       <c r="D138" s="116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E138" s="116" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F138" s="116" t="inlineStr">
         <is>
-          <t>15,0</t>
+          <t>8,0</t>
         </is>
       </c>
       <c r="G138" s="116" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H138" s="116" t="inlineStr">
         <is>
-          <t>27%</t>
+          <t>19%</t>
         </is>
       </c>
     </row>
     <row r="139" ht="16" customHeight="1" s="98">
       <c r="A139" s="111" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B139" s="112" t="inlineStr">
         <is>
-          <t>Skottland</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C139" s="113" t="inlineStr">
         <is>
-          <t>Gruppe C</t>
+          <t>Gruppe K</t>
         </is>
       </c>
       <c r="D139" s="113" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E139" s="113" t="n">
         <v>15</v>
       </c>
       <c r="F139" s="113" t="inlineStr">
         <is>
-          <t>7,5</t>
+          <t>15,0</t>
         </is>
       </c>
       <c r="G139" s="113" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H139" s="113" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>27%</t>
         </is>
       </c>
     </row>
     <row r="140" ht="16" customHeight="1" s="98">
       <c r="A140" s="114" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B140" s="115" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Skottland</t>
         </is>
       </c>
       <c r="C140" s="116" t="inlineStr">
         <is>
-          <t>Gruppe D</t>
+          <t>Gruppe C</t>
         </is>
       </c>
       <c r="D140" s="116" t="n">
         <v>2</v>
       </c>
       <c r="E140" s="116" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F140" s="116" t="inlineStr">
         <is>
-          <t>7,0</t>
+          <t>7,5</t>
         </is>
       </c>
       <c r="G140" s="116" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H140" s="116" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>13%</t>
         </is>
       </c>
     </row>
@@ -49584,23 +49584,23 @@
       </c>
       <c r="B141" s="112" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C141" s="113" t="inlineStr">
         <is>
-          <t>Gruppe B</t>
+          <t>Gruppe D</t>
         </is>
       </c>
       <c r="D141" s="113" t="n">
         <v>2</v>
       </c>
       <c r="E141" s="113" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F141" s="113" t="inlineStr">
         <is>
-          <t>6,5</t>
+          <t>7,0</t>
         </is>
       </c>
       <c r="G141" s="113" t="n">
@@ -49608,7 +49608,7 @@
       </c>
       <c r="H141" s="113" t="inlineStr">
         <is>
-          <t>46%</t>
+          <t>43%</t>
         </is>
       </c>
     </row>
@@ -49618,31 +49618,31 @@
       </c>
       <c r="B142" s="115" t="inlineStr">
         <is>
-          <t>Frankrike</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
       <c r="C142" s="116" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe B</t>
         </is>
       </c>
       <c r="D142" s="116" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E142" s="116" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F142" s="116" t="inlineStr">
         <is>
-          <t>11,0</t>
+          <t>6,5</t>
         </is>
       </c>
       <c r="G142" s="116" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="H142" s="116" t="inlineStr">
         <is>
-          <t>73%</t>
+          <t>46%</t>
         </is>
       </c>
     </row>
@@ -49652,7 +49652,7 @@
       </c>
       <c r="B143" s="112" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Irak</t>
         </is>
       </c>
       <c r="C143" s="113" t="inlineStr">
@@ -49664,34 +49664,34 @@
         <v>1</v>
       </c>
       <c r="E143" s="113" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F143" s="113" t="inlineStr">
         <is>
-          <t>11,0</t>
+          <t>13,0</t>
         </is>
       </c>
       <c r="G143" s="113" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H143" s="113" t="inlineStr">
         <is>
-          <t>45%</t>
+          <t>8%</t>
         </is>
       </c>
     </row>
     <row r="144" ht="16" customHeight="1" s="98">
       <c r="A144" s="114" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B144" s="115" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Norge</t>
         </is>
       </c>
       <c r="C144" s="116" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="D144" s="116" t="n">
@@ -49706,26 +49706,26 @@
         </is>
       </c>
       <c r="G144" s="116" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H144" s="116" t="inlineStr">
         <is>
-          <t>36%</t>
+          <t>45%</t>
         </is>
       </c>
     </row>
     <row r="145" ht="16" customHeight="1" s="98">
       <c r="A145" s="111" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B145" s="112" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C145" s="113" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="D145" s="113" t="n">
@@ -49750,16 +49750,16 @@
     </row>
     <row r="146" ht="16" customHeight="1" s="98">
       <c r="A146" s="114" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B146" s="115" t="inlineStr">
         <is>
-          <t>Irak</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="C146" s="116" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D146" s="116" t="n">
@@ -49774,11 +49774,11 @@
         </is>
       </c>
       <c r="G146" s="116" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H146" s="116" t="inlineStr">
         <is>
-          <t>9%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
@@ -54108,7 +54108,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="98" min="1" max="1"/>
@@ -55944,68 +55944,64 @@
       <c r="A39" s="178" t="inlineStr"/>
       <c r="B39" s="179" t="inlineStr">
         <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C39" s="171" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D39" s="180" t="n">
-        <v>9</v>
-      </c>
-      <c r="E39" s="180" t="n">
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C39" s="187" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D39" s="181" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" s="181" t="n">
         <v>3</v>
       </c>
       <c r="F39" s="180" t="n">
         <v>4</v>
       </c>
       <c r="G39" s="182" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H39" s="183" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I39" s="184" t="n">
         <v>3</v>
       </c>
       <c r="J39" s="180" t="n">
-        <v>4</v>
-      </c>
-      <c r="K39" s="181" t="n">
-        <v>4</v>
-      </c>
-      <c r="L39" s="181" t="n">
-        <v>11</v>
-      </c>
-      <c r="M39" s="177" t="n">
-        <v>0.38</v>
+        <v>2</v>
+      </c>
+      <c r="K39" s="180" t="n">
+        <v>1</v>
+      </c>
+      <c r="L39" s="180" t="n">
+        <v>6</v>
+      </c>
+      <c r="M39" s="187" t="n">
+        <v>0.46</v>
       </c>
       <c r="N39" s="179" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Østerrike</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1" s="98">
-      <c r="A40" s="169" t="inlineStr">
-        <is>
-          <t>Gruppe K</t>
-        </is>
-      </c>
+      <c r="A40" s="185" t="inlineStr"/>
       <c r="B40" s="170" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C40" s="186" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D40" s="172" t="n">
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C40" s="171" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D40" s="173" t="n">
         <v>9</v>
       </c>
-      <c r="E40" s="172" t="n">
+      <c r="E40" s="173" t="n">
         <v>3</v>
       </c>
       <c r="F40" s="173" t="n">
@@ -56016,207 +56012,259 @@
       </c>
       <c r="H40" s="175" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I40" s="176" t="n">
         <v>3</v>
       </c>
       <c r="J40" s="173" t="n">
+        <v>4</v>
+      </c>
+      <c r="K40" s="172" t="n">
+        <v>4</v>
+      </c>
+      <c r="L40" s="172" t="n">
+        <v>11</v>
+      </c>
+      <c r="M40" s="177" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N40" s="170" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1" s="98">
+      <c r="A41" s="169" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
+      <c r="B41" s="179" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C41" s="186" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D41" s="181" t="n">
+        <v>9</v>
+      </c>
+      <c r="E41" s="181" t="n">
         <v>3</v>
       </c>
-      <c r="K40" s="173" t="n">
-        <v>2</v>
-      </c>
-      <c r="L40" s="173" t="n">
-        <v>8</v>
-      </c>
-      <c r="M40" s="177" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N40" s="170" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="18" customHeight="1" s="98">
-      <c r="A41" s="178" t="inlineStr"/>
-      <c r="B41" s="179" t="inlineStr">
-        <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C41" s="177" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D41" s="180" t="n">
-        <v>7</v>
-      </c>
-      <c r="E41" s="180" t="n">
-        <v>3</v>
-      </c>
       <c r="F41" s="180" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G41" s="182" t="n">
         <v>2</v>
       </c>
       <c r="H41" s="183" t="inlineStr">
         <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I41" s="184" t="n">
+        <v>3</v>
+      </c>
+      <c r="J41" s="180" t="n">
+        <v>3</v>
+      </c>
+      <c r="K41" s="180" t="n">
+        <v>2</v>
+      </c>
+      <c r="L41" s="180" t="n">
+        <v>8</v>
+      </c>
+      <c r="M41" s="177" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N41" s="179" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1" s="98">
+      <c r="A42" s="185" t="inlineStr"/>
+      <c r="B42" s="170" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C42" s="177" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D42" s="173" t="n">
+        <v>7</v>
+      </c>
+      <c r="E42" s="173" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="173" t="n">
+        <v>2</v>
+      </c>
+      <c r="G42" s="174" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="175" t="inlineStr">
+        <is>
           <t>1–3</t>
         </is>
       </c>
-      <c r="I41" s="184" t="n">
+      <c r="I42" s="176" t="n">
         <v>4</v>
       </c>
-      <c r="J41" s="180" t="n">
+      <c r="J42" s="173" t="n">
         <v>5</v>
       </c>
-      <c r="K41" s="181" t="n">
+      <c r="K42" s="172" t="n">
         <v>6</v>
       </c>
-      <c r="L41" s="181" t="n">
+      <c r="L42" s="172" t="n">
         <v>15</v>
       </c>
-      <c r="M41" s="186" t="n">
+      <c r="M42" s="186" t="n">
         <v>0.67</v>
       </c>
-      <c r="N41" s="179" t="inlineStr">
+      <c r="N42" s="170" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="18" customHeight="1" s="98">
-      <c r="A42" s="169" t="inlineStr">
+    <row r="43" ht="18" customHeight="1" s="98">
+      <c r="A43" s="169" t="inlineStr">
         <is>
           <t>Gruppe L</t>
         </is>
       </c>
-      <c r="B42" s="170" t="inlineStr">
+      <c r="B43" s="179" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="C42" s="187" t="n">
+      <c r="C43" s="187" t="n">
         <v>0.54</v>
       </c>
-      <c r="D42" s="172" t="n">
+      <c r="D43" s="181" t="n">
         <v>20</v>
       </c>
-      <c r="E42" s="172" t="n">
+      <c r="E43" s="181" t="n">
         <v>12</v>
       </c>
-      <c r="F42" s="173" t="n">
+      <c r="F43" s="180" t="n">
         <v>3</v>
       </c>
-      <c r="G42" s="174" t="n">
+      <c r="G43" s="182" t="n">
         <v>5</v>
       </c>
-      <c r="H42" s="175" t="inlineStr">
+      <c r="H43" s="183" t="inlineStr">
         <is>
           <t>4–2</t>
         </is>
       </c>
-      <c r="I42" s="176" t="n">
+      <c r="I43" s="184" t="n">
         <v>3</v>
       </c>
-      <c r="J42" s="173" t="n">
+      <c r="J43" s="180" t="n">
         <v>3</v>
       </c>
-      <c r="K42" s="173" t="n">
+      <c r="K43" s="180" t="n">
         <v>5</v>
       </c>
-      <c r="L42" s="173" t="n">
+      <c r="L43" s="180" t="n">
         <v>11</v>
       </c>
-      <c r="M42" s="187" t="n">
+      <c r="M43" s="187" t="n">
         <v>0.46</v>
       </c>
-      <c r="N42" s="170" t="inlineStr">
+      <c r="N43" s="179" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="18" customHeight="1" s="98">
-      <c r="A43" s="178" t="inlineStr"/>
-      <c r="B43" s="179" t="inlineStr">
+    <row r="44" ht="18" customHeight="1" s="98">
+      <c r="A44" s="185" t="inlineStr"/>
+      <c r="B44" s="170" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C43" s="177" t="n">
+      <c r="C44" s="177" t="n">
         <v>0.37</v>
       </c>
-      <c r="D43" s="180" t="n">
+      <c r="D44" s="173" t="n">
         <v>8</v>
       </c>
-      <c r="E43" s="180" t="n">
+      <c r="E44" s="173" t="n">
         <v>3</v>
       </c>
-      <c r="F43" s="180" t="n">
+      <c r="F44" s="173" t="n">
         <v>4</v>
       </c>
-      <c r="G43" s="182" t="n">
-        <v>1</v>
-      </c>
-      <c r="H43" s="183" t="inlineStr">
+      <c r="G44" s="174" t="n">
+        <v>1</v>
+      </c>
+      <c r="H44" s="175" t="inlineStr">
         <is>
           <t>1–0</t>
         </is>
       </c>
-      <c r="I43" s="184" t="n">
+      <c r="I44" s="176" t="n">
         <v>2</v>
       </c>
-      <c r="J43" s="180" t="n">
+      <c r="J44" s="173" t="n">
         <v>5</v>
       </c>
-      <c r="K43" s="181" t="n">
+      <c r="K44" s="172" t="n">
         <v>4</v>
       </c>
-      <c r="L43" s="181" t="n">
+      <c r="L44" s="172" t="n">
         <v>11</v>
       </c>
-      <c r="M43" s="171" t="n">
+      <c r="M44" s="171" t="n">
         <v>0.63</v>
       </c>
-      <c r="N43" s="179" t="inlineStr">
+      <c r="N44" s="170" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
     </row>
-    <row r="45" ht="14" customHeight="1" s="98">
-      <c r="A45" s="166" t="inlineStr">
+    <row r="46" ht="14" customHeight="1" s="98">
+      <c r="A46" s="166" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="18" customHeight="1" s="98">
-      <c r="A46" s="158" t="inlineStr">
+    <row r="47" ht="18" customHeight="1" s="98">
+      <c r="A47" s="158" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B46" s="165" t="inlineStr">
+      <c r="B47" s="165" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C46" s="164" t="inlineStr">
+      <c r="C47" s="164" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D46" s="161" t="inlineStr">
+      <c r="D47" s="161" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E46" s="188" t="inlineStr">
+      <c r="E47" s="188" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -56224,7 +56272,7 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A45:N45"/>
+    <mergeCell ref="A46:N46"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>

</xml_diff>

<commit_message>
Oppdater ballbesittelse med runde 2-kamper (22-23. juni)
- France vs Iraq 3-0, Norway vs Senegal 3-2, Jordan vs Algeria 1-2
- Komplett statistikk (poss, skudd, corners, kort) i wc2026_stats3.json
- Regenerert docs/index.html med oppdatert Ballbesittelse-ark

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -54415,7 +54415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N47"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" style="98" min="1" max="1"/>
@@ -56151,99 +56151,95 @@
       <c r="A37" s="178" t="inlineStr"/>
       <c r="B37" s="179" t="inlineStr">
         <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C37" s="171" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D37" s="181" t="n">
+        <v>19</v>
+      </c>
+      <c r="E37" s="181" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="180" t="n">
+        <v>9</v>
+      </c>
+      <c r="G37" s="182" t="n">
+        <v>5</v>
+      </c>
+      <c r="H37" s="183" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="I37" s="184" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="180" t="n">
+        <v>3</v>
+      </c>
+      <c r="K37" s="180" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="180" t="n">
+        <v>4</v>
+      </c>
+      <c r="M37" s="177" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="N37" s="179" t="inlineStr">
+        <is>
           <t>Irak</t>
         </is>
       </c>
-      <c r="C37" s="177" t="n">
+    </row>
+    <row r="38" ht="18" customHeight="1" s="98">
+      <c r="A38" s="185" t="inlineStr"/>
+      <c r="B38" s="170" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="C38" s="177" t="n">
         <v>0.37</v>
       </c>
-      <c r="D37" s="180" t="n">
+      <c r="D38" s="173" t="n">
         <v>11</v>
       </c>
-      <c r="E37" s="180" t="n">
-        <v>1</v>
-      </c>
-      <c r="F37" s="180" t="n">
+      <c r="E38" s="173" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="173" t="n">
         <v>8</v>
       </c>
-      <c r="G37" s="182" t="n">
+      <c r="G38" s="174" t="n">
         <v>2</v>
       </c>
-      <c r="H37" s="183" t="inlineStr">
+      <c r="H38" s="175" t="inlineStr">
         <is>
           <t>1–4</t>
         </is>
       </c>
-      <c r="I37" s="184" t="n">
+      <c r="I38" s="176" t="n">
         <v>2</v>
       </c>
-      <c r="J37" s="180" t="n">
+      <c r="J38" s="173" t="n">
         <v>4</v>
       </c>
-      <c r="K37" s="181" t="n">
+      <c r="K38" s="172" t="n">
         <v>6</v>
       </c>
-      <c r="L37" s="181" t="n">
+      <c r="L38" s="172" t="n">
         <v>12</v>
       </c>
-      <c r="M37" s="171" t="n">
+      <c r="M38" s="171" t="n">
         <v>0.63</v>
       </c>
-      <c r="N37" s="179" t="inlineStr">
+      <c r="N38" s="170" t="inlineStr">
         <is>
           <t>Norge</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1" s="98">
-      <c r="A38" s="169" t="inlineStr">
-        <is>
-          <t>Gruppe J</t>
-        </is>
-      </c>
-      <c r="B38" s="170" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C38" s="187" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D38" s="172" t="n">
-        <v>9</v>
-      </c>
-      <c r="E38" s="172" t="n">
-        <v>6</v>
-      </c>
-      <c r="F38" s="173" t="n">
-        <v>3</v>
-      </c>
-      <c r="G38" s="174" t="n">
-        <v>0</v>
-      </c>
-      <c r="H38" s="175" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I38" s="176" t="n">
-        <v>3</v>
-      </c>
-      <c r="J38" s="173" t="n">
-        <v>3</v>
-      </c>
-      <c r="K38" s="173" t="n">
-        <v>0</v>
-      </c>
-      <c r="L38" s="173" t="n">
-        <v>6</v>
-      </c>
-      <c r="M38" s="187" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N38" s="170" t="inlineStr">
-        <is>
-          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -56251,114 +56247,114 @@
       <c r="A39" s="178" t="inlineStr"/>
       <c r="B39" s="179" t="inlineStr">
         <is>
+          <t>Norge</t>
+        </is>
+      </c>
+      <c r="C39" s="177" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D39" s="180" t="n">
+        <v>12</v>
+      </c>
+      <c r="E39" s="180" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" s="180" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="182" t="n">
+        <v>4</v>
+      </c>
+      <c r="H39" s="183" t="inlineStr">
+        <is>
+          <t>3–2</t>
+        </is>
+      </c>
+      <c r="I39" s="184" t="n">
+        <v>5</v>
+      </c>
+      <c r="J39" s="180" t="n">
+        <v>6</v>
+      </c>
+      <c r="K39" s="180" t="n">
+        <v>6</v>
+      </c>
+      <c r="L39" s="181" t="n">
+        <v>17</v>
+      </c>
+      <c r="M39" s="171" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="N39" s="179" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="18" customHeight="1" s="98">
+      <c r="A40" s="169" t="inlineStr">
+        <is>
+          <t>Gruppe J</t>
+        </is>
+      </c>
+      <c r="B40" s="170" t="inlineStr">
+        <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="C39" s="187" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D39" s="181" t="n">
-        <v>12</v>
-      </c>
-      <c r="E39" s="181" t="n">
+      <c r="C40" s="187" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D40" s="172" t="n">
+        <v>9</v>
+      </c>
+      <c r="E40" s="172" t="n">
+        <v>6</v>
+      </c>
+      <c r="F40" s="173" t="n">
         <v>3</v>
       </c>
-      <c r="F39" s="180" t="n">
-        <v>4</v>
-      </c>
-      <c r="G39" s="182" t="n">
-        <v>5</v>
-      </c>
-      <c r="H39" s="183" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I39" s="184" t="n">
-        <v>3</v>
-      </c>
-      <c r="J39" s="180" t="n">
-        <v>2</v>
-      </c>
-      <c r="K39" s="180" t="n">
-        <v>1</v>
-      </c>
-      <c r="L39" s="180" t="n">
-        <v>6</v>
-      </c>
-      <c r="M39" s="187" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="N39" s="179" t="inlineStr">
-        <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="18" customHeight="1" s="98">
-      <c r="A40" s="185" t="inlineStr"/>
-      <c r="B40" s="170" t="inlineStr">
-        <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C40" s="171" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D40" s="173" t="n">
-        <v>9</v>
-      </c>
-      <c r="E40" s="173" t="n">
-        <v>3</v>
-      </c>
-      <c r="F40" s="173" t="n">
-        <v>4</v>
-      </c>
       <c r="G40" s="174" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H40" s="175" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I40" s="176" t="n">
         <v>3</v>
       </c>
       <c r="J40" s="173" t="n">
-        <v>4</v>
-      </c>
-      <c r="K40" s="172" t="n">
-        <v>4</v>
-      </c>
-      <c r="L40" s="172" t="n">
-        <v>11</v>
-      </c>
-      <c r="M40" s="177" t="n">
-        <v>0.38</v>
+        <v>3</v>
+      </c>
+      <c r="K40" s="173" t="n">
+        <v>0</v>
+      </c>
+      <c r="L40" s="173" t="n">
+        <v>6</v>
+      </c>
+      <c r="M40" s="187" t="n">
+        <v>0.53</v>
       </c>
       <c r="N40" s="170" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1" s="98">
-      <c r="A41" s="169" t="inlineStr">
-        <is>
-          <t>Gruppe K</t>
-        </is>
-      </c>
+      <c r="A41" s="178" t="inlineStr"/>
       <c r="B41" s="179" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C41" s="186" t="n">
-        <v>0.75</v>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C41" s="187" t="n">
+        <v>0.54</v>
       </c>
       <c r="D41" s="181" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E41" s="181" t="n">
         <v>3</v>
@@ -56367,31 +56363,31 @@
         <v>4</v>
       </c>
       <c r="G41" s="182" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H41" s="183" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I41" s="184" t="n">
         <v>3</v>
       </c>
       <c r="J41" s="180" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K41" s="180" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L41" s="180" t="n">
-        <v>8</v>
-      </c>
-      <c r="M41" s="177" t="n">
-        <v>0.25</v>
+        <v>6</v>
+      </c>
+      <c r="M41" s="187" t="n">
+        <v>0.46</v>
       </c>
       <c r="N41" s="179" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Østerrike</t>
         </is>
       </c>
     </row>
@@ -56399,179 +56395,327 @@
       <c r="A42" s="185" t="inlineStr"/>
       <c r="B42" s="170" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C42" s="177" t="n">
-        <v>0.33</v>
+        <v>0.25</v>
       </c>
       <c r="D42" s="173" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E42" s="173" t="n">
+        <v>4</v>
+      </c>
+      <c r="F42" s="173" t="n">
+        <v>4</v>
+      </c>
+      <c r="G42" s="174" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="175" t="inlineStr">
+        <is>
+          <t>1–2</t>
+        </is>
+      </c>
+      <c r="I42" s="176" t="n">
+        <v>6</v>
+      </c>
+      <c r="J42" s="173" t="n">
         <v>3</v>
       </c>
-      <c r="F42" s="173" t="n">
+      <c r="K42" s="172" t="n">
+        <v>8</v>
+      </c>
+      <c r="L42" s="172" t="n">
+        <v>17</v>
+      </c>
+      <c r="M42" s="186" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="N42" s="170" t="inlineStr">
+        <is>
+          <t>Algerie</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="18" customHeight="1" s="98">
+      <c r="A43" s="178" t="inlineStr"/>
+      <c r="B43" s="179" t="inlineStr">
+        <is>
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C43" s="171" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D43" s="180" t="n">
+        <v>9</v>
+      </c>
+      <c r="E43" s="180" t="n">
+        <v>3</v>
+      </c>
+      <c r="F43" s="180" t="n">
+        <v>4</v>
+      </c>
+      <c r="G43" s="182" t="n">
         <v>2</v>
       </c>
-      <c r="G42" s="174" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" s="175" t="inlineStr">
-        <is>
-          <t>1–3</t>
-        </is>
-      </c>
-      <c r="I42" s="176" t="n">
-        <v>4</v>
-      </c>
-      <c r="J42" s="173" t="n">
-        <v>5</v>
-      </c>
-      <c r="K42" s="172" t="n">
-        <v>6</v>
-      </c>
-      <c r="L42" s="172" t="n">
-        <v>15</v>
-      </c>
-      <c r="M42" s="186" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="N42" s="170" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="18" customHeight="1" s="98">
-      <c r="A43" s="169" t="inlineStr">
-        <is>
-          <t>Gruppe L</t>
-        </is>
-      </c>
-      <c r="B43" s="179" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C43" s="187" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D43" s="181" t="n">
-        <v>20</v>
-      </c>
-      <c r="E43" s="181" t="n">
-        <v>12</v>
-      </c>
-      <c r="F43" s="180" t="n">
-        <v>3</v>
-      </c>
-      <c r="G43" s="182" t="n">
-        <v>5</v>
-      </c>
       <c r="H43" s="183" t="inlineStr">
         <is>
-          <t>4–2</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I43" s="184" t="n">
         <v>3</v>
       </c>
       <c r="J43" s="180" t="n">
-        <v>3</v>
-      </c>
-      <c r="K43" s="180" t="n">
-        <v>5</v>
-      </c>
-      <c r="L43" s="180" t="n">
+        <v>4</v>
+      </c>
+      <c r="K43" s="181" t="n">
+        <v>4</v>
+      </c>
+      <c r="L43" s="181" t="n">
         <v>11</v>
       </c>
-      <c r="M43" s="187" t="n">
-        <v>0.46</v>
+      <c r="M43" s="177" t="n">
+        <v>0.38</v>
       </c>
       <c r="N43" s="179" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>Jordan</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1" s="98">
-      <c r="A44" s="185" t="inlineStr"/>
+      <c r="A44" s="169" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
       <c r="B44" s="170" t="inlineStr">
         <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="C44" s="177" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D44" s="173" t="n">
-        <v>8</v>
-      </c>
-      <c r="E44" s="173" t="n">
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C44" s="186" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D44" s="172" t="n">
+        <v>9</v>
+      </c>
+      <c r="E44" s="172" t="n">
         <v>3</v>
       </c>
       <c r="F44" s="173" t="n">
         <v>4</v>
       </c>
       <c r="G44" s="174" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H44" s="175" t="inlineStr">
         <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I44" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="J44" s="173" t="n">
+        <v>3</v>
+      </c>
+      <c r="K44" s="173" t="n">
+        <v>2</v>
+      </c>
+      <c r="L44" s="173" t="n">
+        <v>8</v>
+      </c>
+      <c r="M44" s="177" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N44" s="170" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1" s="98">
+      <c r="A45" s="178" t="inlineStr"/>
+      <c r="B45" s="179" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C45" s="177" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D45" s="180" t="n">
+        <v>7</v>
+      </c>
+      <c r="E45" s="180" t="n">
+        <v>3</v>
+      </c>
+      <c r="F45" s="180" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="182" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" s="183" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I45" s="184" t="n">
+        <v>4</v>
+      </c>
+      <c r="J45" s="180" t="n">
+        <v>5</v>
+      </c>
+      <c r="K45" s="181" t="n">
+        <v>6</v>
+      </c>
+      <c r="L45" s="181" t="n">
+        <v>15</v>
+      </c>
+      <c r="M45" s="186" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N45" s="179" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1" s="98">
+      <c r="A46" s="169" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="B46" s="170" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C46" s="187" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D46" s="172" t="n">
+        <v>20</v>
+      </c>
+      <c r="E46" s="172" t="n">
+        <v>12</v>
+      </c>
+      <c r="F46" s="173" t="n">
+        <v>3</v>
+      </c>
+      <c r="G46" s="174" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" s="175" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="I46" s="176" t="n">
+        <v>3</v>
+      </c>
+      <c r="J46" s="173" t="n">
+        <v>3</v>
+      </c>
+      <c r="K46" s="173" t="n">
+        <v>5</v>
+      </c>
+      <c r="L46" s="173" t="n">
+        <v>11</v>
+      </c>
+      <c r="M46" s="187" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N46" s="170" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1" s="98">
+      <c r="A47" s="178" t="inlineStr"/>
+      <c r="B47" s="179" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C47" s="177" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D47" s="180" t="n">
+        <v>8</v>
+      </c>
+      <c r="E47" s="180" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="180" t="n">
+        <v>4</v>
+      </c>
+      <c r="G47" s="182" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="183" t="inlineStr">
+        <is>
           <t>1–0</t>
         </is>
       </c>
-      <c r="I44" s="176" t="n">
+      <c r="I47" s="184" t="n">
         <v>2</v>
       </c>
-      <c r="J44" s="173" t="n">
+      <c r="J47" s="180" t="n">
         <v>5</v>
       </c>
-      <c r="K44" s="172" t="n">
+      <c r="K47" s="181" t="n">
         <v>4</v>
       </c>
-      <c r="L44" s="172" t="n">
+      <c r="L47" s="181" t="n">
         <v>11</v>
       </c>
-      <c r="M44" s="171" t="n">
+      <c r="M47" s="171" t="n">
         <v>0.63</v>
       </c>
-      <c r="N44" s="170" t="inlineStr">
+      <c r="N47" s="179" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
     </row>
-    <row r="46" ht="14" customHeight="1" s="98">
-      <c r="A46" s="166" t="inlineStr">
+    <row r="49" ht="14" customHeight="1" s="98">
+      <c r="A49" s="166" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1" s="98">
-      <c r="A47" s="158" t="inlineStr">
+    <row r="50" ht="18" customHeight="1" s="98">
+      <c r="A50" s="158" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B47" s="165" t="inlineStr">
+      <c r="B50" s="165" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C47" s="164" t="inlineStr">
+      <c r="C50" s="164" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D47" s="161" t="inlineStr">
+      <c r="D50" s="161" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E47" s="188" t="inlineStr">
+      <c r="E50" s="188" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -56579,9 +56723,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A46:N46"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="I2:N2"/>
+    <mergeCell ref="A49:N49"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-23 21:27 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,38 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Kort" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Scorere og assists" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Alder" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Lagstatistikk" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Scoringstidspunkt" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Heatmap" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Ballbesittelse" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Stadionoversikt" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -842,13 +842,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -867,7 +867,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -891,12 +891,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -910,7 +910,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -923,8 +922,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -938,7 +937,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -948,7 +946,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -963,9 +961,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -32407,35 +32405,35 @@
     </row>
     <row r="122" ht="16" customHeight="1">
       <c r="A122" s="4" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>England</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>Gruppe F</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D122" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E122" s="14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>14,5</t>
+          <t>30,0</t>
         </is>
       </c>
       <c r="G122" s="14" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="H122" s="14" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>40%</t>
         </is>
       </c>
     </row>
@@ -32445,31 +32443,31 @@
       </c>
       <c r="B123" s="8" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Sverige</t>
         </is>
       </c>
       <c r="C123" s="15" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe F</t>
         </is>
       </c>
       <c r="D123" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E123" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F123" s="15" t="inlineStr">
         <is>
-          <t>28,0</t>
+          <t>14,5</t>
         </is>
       </c>
       <c r="G123" s="15" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H123" s="15" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>52%</t>
         </is>
       </c>
     </row>
@@ -33635,23 +33633,23 @@
       </c>
       <c r="B158" s="5" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C158" s="14" t="inlineStr">
         <is>
-          <t>Gruppe F</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D158" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E158" s="14" t="n">
         <v>8</v>
       </c>
       <c r="F158" s="14" t="inlineStr">
         <is>
-          <t>4,0</t>
+          <t>8,0</t>
         </is>
       </c>
       <c r="G158" s="14" t="n">
@@ -33665,27 +33663,27 @@
     </row>
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="7" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B159" s="8" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="C159" s="15" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe F</t>
         </is>
       </c>
       <c r="D159" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E159" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F159" s="15" t="inlineStr">
         <is>
-          <t>7,0</t>
+          <t>4,0</t>
         </is>
       </c>
       <c r="G159" s="15" t="n">
@@ -33693,7 +33691,7 @@
       </c>
       <c r="H159" s="15" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Oppdater lagstatistikk og ballbesittelse 23. juni
45 kamper inkl. dagens runde: Norge 3-2 Senegal, Jordan 1-2 Algerie,
Portugal 5-0 Usbekistan. Ballbesittelse-ark har 45 kamper, lagstatistikk
oppdatert med timeline, skudd og formasjonsdata.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -32343,65 +32343,65 @@
       </c>
       <c r="B120" s="5" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>England</t>
         </is>
       </c>
       <c r="C120" s="14" t="inlineStr">
         <is>
-          <t>Gruppe G</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D120" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E120" s="14" t="n">
         <v>33</v>
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>16,5</t>
+          <t>33,0</t>
         </is>
       </c>
       <c r="G120" s="14" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="H120" s="14" t="inlineStr">
         <is>
-          <t>30%</t>
+          <t>36%</t>
         </is>
       </c>
     </row>
     <row r="121" ht="16" customHeight="1">
       <c r="A121" s="7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B121" s="8" t="inlineStr">
         <is>
-          <t>Frankrike</t>
+          <t>Egypt</t>
         </is>
       </c>
       <c r="C121" s="15" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe G</t>
         </is>
       </c>
       <c r="D121" s="15" t="n">
         <v>2</v>
       </c>
       <c r="E121" s="15" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="F121" s="15" t="inlineStr">
         <is>
-          <t>15,0</t>
+          <t>16,5</t>
         </is>
       </c>
       <c r="G121" s="15" t="n">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="H121" s="15" t="inlineStr">
         <is>
-          <t>43%</t>
+          <t>30%</t>
         </is>
       </c>
     </row>
@@ -32411,31 +32411,31 @@
       </c>
       <c r="B122" s="5" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>Frankrike</t>
         </is>
       </c>
       <c r="C122" s="14" t="inlineStr">
         <is>
-          <t>Gruppe F</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="D122" s="14" t="n">
         <v>2</v>
       </c>
       <c r="E122" s="14" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>14,5</t>
+          <t>15,0</t>
         </is>
       </c>
       <c r="G122" s="14" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H122" s="14" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>43%</t>
         </is>
       </c>
     </row>
@@ -32445,31 +32445,31 @@
       </c>
       <c r="B123" s="8" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Sverige</t>
         </is>
       </c>
       <c r="C123" s="15" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe F</t>
         </is>
       </c>
       <c r="D123" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E123" s="15" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F123" s="15" t="inlineStr">
         <is>
-          <t>28,0</t>
+          <t>14,5</t>
         </is>
       </c>
       <c r="G123" s="15" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="H123" s="15" t="inlineStr">
         <is>
-          <t>39%</t>
+          <t>52%</t>
         </is>
       </c>
     </row>
@@ -33635,23 +33635,23 @@
       </c>
       <c r="B158" s="5" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="C158" s="14" t="inlineStr">
         <is>
-          <t>Gruppe F</t>
+          <t>Gruppe L</t>
         </is>
       </c>
       <c r="D158" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E158" s="14" t="n">
         <v>8</v>
       </c>
       <c r="F158" s="14" t="inlineStr">
         <is>
-          <t>4,0</t>
+          <t>8,0</t>
         </is>
       </c>
       <c r="G158" s="14" t="n">
@@ -33665,27 +33665,27 @@
     </row>
     <row r="159" ht="16" customHeight="1">
       <c r="A159" s="7" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B159" s="8" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="C159" s="15" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe F</t>
         </is>
       </c>
       <c r="D159" s="15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E159" s="15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F159" s="15" t="inlineStr">
         <is>
-          <t>7,0</t>
+          <t>4,0</t>
         </is>
       </c>
       <c r="G159" s="15" t="n">
@@ -33693,7 +33693,7 @@
       </c>
       <c r="H159" s="15" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>25%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gi nytt navn: 16-delsfinale -> 16-delsfinaler, 8-delsfinale -> 8-delsfinaler
Oppdaterer RUNDE_MAP, RUNDE_ORDER, RUNDE_TITLER og GAMLE_NAVN i
add_sluttspill_sheet.py slik at gamle arknavn ryddes automatisk ved neste kjøring.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -19,8 +19,8 @@
     <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
@@ -17742,7 +17742,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — 16-delsfinale</t>
+          <t>VM 2026 — 16-delsfinaler</t>
         </is>
       </c>
     </row>
@@ -18148,7 +18148,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — 8-delsfinale</t>
+          <t>VM 2026 — 8-delsfinaler</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Gi nytt navn: 16-delsfinale -> 16-delsfinaler, 8-delsfinale -> 8-delsfinaler (#61)
Oppdaterer RUNDE_MAP, RUNDE_ORDER, RUNDE_TITLER og GAMLE_NAVN i
add_sluttspill_sheet.py slik at gamle arknavn ryddes automatisk ved neste kjøring.

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -19,8 +19,8 @@
     <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinale" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinale" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
@@ -17742,7 +17742,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — 16-delsfinale</t>
+          <t>VM 2026 — 16-delsfinaler</t>
         </is>
       </c>
     </row>
@@ -18148,7 +18148,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — 8-delsfinale</t>
+          <t>VM 2026 — 8-delsfinaler</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-24 06:02 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -37689,7 +37689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N51"/>
+  <dimension ref="A1:N54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -39769,31 +39769,31 @@
       </c>
       <c r="B44" s="67" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C44" s="83" t="n">
-        <v>0.75</v>
+        <v>0.66</v>
       </c>
       <c r="D44" s="69" t="n">
+        <v>20</v>
+      </c>
+      <c r="E44" s="69" t="n">
         <v>9</v>
       </c>
-      <c r="E44" s="69" t="n">
-        <v>3</v>
-      </c>
       <c r="F44" s="70" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G44" s="71" t="n">
+        <v>6</v>
+      </c>
+      <c r="H44" s="72" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I44" s="73" t="n">
         <v>2</v>
-      </c>
-      <c r="H44" s="72" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I44" s="73" t="n">
-        <v>3</v>
       </c>
       <c r="J44" s="70" t="n">
         <v>3</v>
@@ -39802,10 +39802,10 @@
         <v>2</v>
       </c>
       <c r="L44" s="70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M44" s="74" t="n">
-        <v>0.25</v>
+        <v>0.34</v>
       </c>
       <c r="N44" s="67" t="inlineStr">
         <is>
@@ -39821,43 +39821,43 @@
         </is>
       </c>
       <c r="C45" s="83" t="n">
-        <v>0.66</v>
+        <v>0.75</v>
       </c>
       <c r="D45" s="78" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E45" s="78" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="F45" s="77" t="n">
         <v>4</v>
       </c>
       <c r="G45" s="79" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H45" s="80" t="inlineStr">
         <is>
-          <t>5–0</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I45" s="81" t="n">
         <v>3</v>
       </c>
       <c r="J45" s="77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K45" s="77" t="n">
         <v>2</v>
       </c>
       <c r="L45" s="77" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M45" s="74" t="n">
-        <v>0.34</v>
+        <v>0.25</v>
       </c>
       <c r="N45" s="76" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -39865,179 +39865,323 @@
       <c r="A46" s="82" t="inlineStr"/>
       <c r="B46" s="67" t="inlineStr">
         <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C46" s="83" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D46" s="69" t="n">
+        <v>16</v>
+      </c>
+      <c r="E46" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="F46" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G46" s="71" t="n">
+        <v>3</v>
+      </c>
+      <c r="H46" s="72" t="inlineStr">
+        <is>
+          <t>5–0</t>
+        </is>
+      </c>
+      <c r="I46" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J46" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K46" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="L46" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="M46" s="74" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="N46" s="67" t="inlineStr">
+        <is>
           <t>Usbekistan</t>
         </is>
       </c>
-      <c r="C46" s="74" t="n">
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="75" t="inlineStr"/>
+      <c r="B47" s="76" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C47" s="74" t="n">
         <v>0.33</v>
       </c>
-      <c r="D46" s="70" t="n">
+      <c r="D47" s="77" t="n">
         <v>7</v>
       </c>
-      <c r="E46" s="70" t="n">
+      <c r="E47" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="F46" s="70" t="n">
+      <c r="F47" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="G46" s="71" t="n">
+      <c r="G47" s="79" t="n">
         <v>2</v>
       </c>
-      <c r="H46" s="72" t="inlineStr">
+      <c r="H47" s="80" t="inlineStr">
         <is>
           <t>1–3</t>
         </is>
       </c>
-      <c r="I46" s="73" t="n">
+      <c r="I47" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="J46" s="70" t="n">
+      <c r="J47" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="K46" s="69" t="n">
+      <c r="K47" s="78" t="n">
         <v>6</v>
       </c>
-      <c r="L46" s="69" t="n">
+      <c r="L47" s="78" t="n">
         <v>15</v>
       </c>
-      <c r="M46" s="83" t="n">
+      <c r="M47" s="83" t="n">
         <v>0.67</v>
       </c>
-      <c r="N46" s="67" t="inlineStr">
+      <c r="N47" s="76" t="inlineStr">
         <is>
           <t>Colombia</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="66" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="66" t="inlineStr">
         <is>
           <t>Gruppe L</t>
         </is>
       </c>
-      <c r="B47" s="76" t="inlineStr">
+      <c r="B48" s="67" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="C47" s="84" t="n">
+      <c r="C48" s="84" t="n">
         <v>0.54</v>
       </c>
-      <c r="D47" s="78" t="n">
+      <c r="D48" s="69" t="n">
         <v>20</v>
       </c>
-      <c r="E47" s="78" t="n">
+      <c r="E48" s="69" t="n">
         <v>12</v>
       </c>
-      <c r="F47" s="77" t="n">
+      <c r="F48" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="G47" s="79" t="n">
+      <c r="G48" s="71" t="n">
         <v>5</v>
       </c>
-      <c r="H47" s="80" t="inlineStr">
+      <c r="H48" s="72" t="inlineStr">
         <is>
           <t>4–2</t>
         </is>
       </c>
-      <c r="I47" s="81" t="n">
+      <c r="I48" s="73" t="n">
         <v>3</v>
       </c>
-      <c r="J47" s="77" t="n">
+      <c r="J48" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="K47" s="77" t="n">
+      <c r="K48" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="L47" s="77" t="n">
+      <c r="L48" s="70" t="n">
         <v>11</v>
       </c>
-      <c r="M47" s="84" t="n">
+      <c r="M48" s="84" t="n">
         <v>0.46</v>
       </c>
-      <c r="N47" s="76" t="inlineStr">
+      <c r="N48" s="67" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="82" t="inlineStr"/>
-      <c r="B48" s="67" t="inlineStr">
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="75" t="inlineStr"/>
+      <c r="B49" s="76" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C49" s="83" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D49" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="E49" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="G49" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="H49" s="80" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I49" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J49" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K49" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L49" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="M49" s="74" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N49" s="76" t="inlineStr">
         <is>
           <t>Ghana</t>
         </is>
       </c>
-      <c r="C48" s="74" t="n">
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="82" t="inlineStr"/>
+      <c r="B50" s="67" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C50" s="74" t="n">
         <v>0.37</v>
       </c>
-      <c r="D48" s="70" t="n">
+      <c r="D50" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="E48" s="70" t="n">
+      <c r="E50" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="F48" s="70" t="n">
+      <c r="F50" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="G48" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H48" s="72" t="inlineStr">
+      <c r="G50" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H50" s="72" t="inlineStr">
         <is>
           <t>1–0</t>
         </is>
       </c>
-      <c r="I48" s="73" t="n">
+      <c r="I50" s="73" t="n">
         <v>2</v>
       </c>
-      <c r="J48" s="70" t="n">
+      <c r="J50" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="K48" s="69" t="n">
+      <c r="K50" s="69" t="n">
         <v>4</v>
       </c>
-      <c r="L48" s="69" t="n">
+      <c r="L50" s="69" t="n">
         <v>11</v>
       </c>
-      <c r="M48" s="68" t="n">
+      <c r="M50" s="68" t="n">
         <v>0.63</v>
       </c>
-      <c r="N48" s="67" t="inlineStr">
+      <c r="N50" s="67" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="14" customHeight="1">
-      <c r="A50" s="63" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="75" t="inlineStr"/>
+      <c r="B51" s="76" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C51" s="74" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D51" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E51" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F51" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="G51" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="80" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I51" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="L51" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="M51" s="68" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="N51" s="76" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="14" customHeight="1">
+      <c r="A53" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="55" t="inlineStr">
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B51" s="62" t="inlineStr">
+      <c r="B54" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C51" s="61" t="inlineStr">
+      <c r="C54" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D51" s="58" t="inlineStr">
+      <c r="D54" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E51" s="85" t="inlineStr">
+      <c r="E54" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -40045,9 +40189,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A50:N50"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="I2:N2"/>
+    <mergeCell ref="A53:N53"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-25 07:40 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -37998,7 +37998,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N54"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -38214,47 +38214,47 @@
       <c r="A6" s="82" t="inlineStr"/>
       <c r="B6" s="67" t="inlineStr">
         <is>
-          <t>Sør-Korea</t>
-        </is>
-      </c>
-      <c r="C6" s="68" t="n">
-        <v>0.62</v>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="C6" s="74" t="n">
+        <v>0.31</v>
       </c>
       <c r="D6" s="69" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E6" s="69" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F6" s="70" t="n">
         <v>5</v>
       </c>
       <c r="G6" s="71" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H6" s="72" t="inlineStr">
         <is>
-          <t>2–1</t>
+          <t>1–0</t>
         </is>
       </c>
       <c r="I6" s="73" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="70" t="n">
         <v>3</v>
       </c>
       <c r="K6" s="70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L6" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="M6" s="74" t="n">
-        <v>0.38</v>
+        <v>7</v>
+      </c>
+      <c r="M6" s="83" t="n">
+        <v>0.6899999999999999</v>
       </c>
       <c r="N6" s="67" t="inlineStr">
         <is>
-          <t>Tsjekkia</t>
+          <t>Sør-Korea</t>
         </is>
       </c>
     </row>
@@ -38262,75 +38262,71 @@
       <c r="A7" s="75" t="inlineStr"/>
       <c r="B7" s="76" t="inlineStr">
         <is>
-          <t>Tsjekkia</t>
-        </is>
-      </c>
-      <c r="C7" s="74" t="n">
-        <v>0.39</v>
-      </c>
-      <c r="D7" s="77" t="n">
-        <v>12</v>
-      </c>
-      <c r="E7" s="77" t="n">
-        <v>3</v>
+          <t>Sør-Korea</t>
+        </is>
+      </c>
+      <c r="C7" s="68" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D7" s="78" t="n">
+        <v>15</v>
+      </c>
+      <c r="E7" s="78" t="n">
+        <v>7</v>
       </c>
       <c r="F7" s="77" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G7" s="79" t="n">
         <v>3</v>
       </c>
       <c r="H7" s="80" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>2–1</t>
         </is>
       </c>
       <c r="I7" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="J7" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="78" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" s="78" t="n">
-        <v>17</v>
-      </c>
-      <c r="M7" s="68" t="n">
-        <v>0.61</v>
+      <c r="M7" s="74" t="n">
+        <v>0.38</v>
       </c>
       <c r="N7" s="76" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
+          <t>Tsjekkia</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe B</t>
-        </is>
-      </c>
+      <c r="A8" s="82" t="inlineStr"/>
       <c r="B8" s="67" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C8" s="68" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D8" s="69" t="n">
-        <v>13</v>
+          <t>Tsjekkia</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="n">
+        <v>0.39</v>
+      </c>
+      <c r="D8" s="70" t="n">
+        <v>12</v>
       </c>
       <c r="E8" s="70" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="70" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" s="71" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="H8" s="72" t="inlineStr">
         <is>
@@ -38338,23 +38334,23 @@
         </is>
       </c>
       <c r="I8" s="73" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="J8" s="70" t="n">
         <v>4</v>
       </c>
       <c r="K8" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L8" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="M8" s="74" t="n">
-        <v>0.4</v>
+        <v>5</v>
+      </c>
+      <c r="L8" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="M8" s="68" t="n">
+        <v>0.61</v>
       </c>
       <c r="N8" s="67" t="inlineStr">
         <is>
-          <t>Bosnia-Hercegovina</t>
+          <t>Sør-Afrika</t>
         </is>
       </c>
     </row>
@@ -38362,95 +38358,99 @@
       <c r="A9" s="75" t="inlineStr"/>
       <c r="B9" s="76" t="inlineStr">
         <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="C9" s="83" t="n">
-        <v>0.78</v>
+          <t>Tsjekkia</t>
+        </is>
+      </c>
+      <c r="C9" s="84" t="n">
+        <v>0.51</v>
       </c>
       <c r="D9" s="78" t="n">
-        <v>31</v>
-      </c>
-      <c r="E9" s="78" t="n">
-        <v>10</v>
+        <v>12</v>
+      </c>
+      <c r="E9" s="77" t="n">
+        <v>1</v>
       </c>
       <c r="F9" s="77" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G9" s="79" t="n">
-        <v>13</v>
+        <v>4</v>
       </c>
       <c r="H9" s="80" t="inlineStr">
         <is>
-          <t>6–0</t>
+          <t>0–3</t>
         </is>
       </c>
       <c r="I9" s="81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J9" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="77" t="n">
+        <v>11</v>
+      </c>
+      <c r="M9" s="84" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="N9" s="76" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe B</t>
+        </is>
+      </c>
+      <c r="B10" s="67" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+      <c r="C10" s="68" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D10" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="E10" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="F10" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="72" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="I10" s="73" t="n">
         <v>0</v>
       </c>
-      <c r="L9" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="M9" s="74" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="N9" s="76" t="inlineStr">
+      <c r="J10" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="K10" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L10" s="70" t="n">
+        <v>9</v>
+      </c>
+      <c r="M10" s="84" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="N10" s="67" t="inlineStr">
         <is>
           <t>Qatar</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="82" t="inlineStr"/>
-      <c r="B10" s="67" t="inlineStr">
-        <is>
-          <t>Qatar</t>
-        </is>
-      </c>
-      <c r="C10" s="74" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D10" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="E10" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="F10" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H10" s="72" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I10" s="73" t="n">
-        <v>9</v>
-      </c>
-      <c r="J10" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="K10" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="L10" s="69" t="n">
-        <v>27</v>
-      </c>
-      <c r="M10" s="83" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="N10" s="67" t="inlineStr">
-        <is>
-          <t>Sveits</t>
         </is>
       </c>
     </row>
@@ -38458,99 +38458,95 @@
       <c r="A11" s="75" t="inlineStr"/>
       <c r="B11" s="76" t="inlineStr">
         <is>
-          <t>Sveits</t>
+          <t>Canada</t>
         </is>
       </c>
       <c r="C11" s="68" t="n">
-        <v>0.62</v>
+        <v>0.6</v>
       </c>
       <c r="D11" s="78" t="n">
         <v>13</v>
       </c>
-      <c r="E11" s="78" t="n">
+      <c r="E11" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="H11" s="80" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I11" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="L11" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="F11" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="G11" s="79" t="n">
+      <c r="M11" s="74" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="N11" s="76" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="82" t="inlineStr"/>
+      <c r="B12" s="67" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="C12" s="83" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D12" s="69" t="n">
+        <v>31</v>
+      </c>
+      <c r="E12" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="F12" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="G12" s="71" t="n">
+        <v>13</v>
+      </c>
+      <c r="H12" s="72" t="inlineStr">
+        <is>
+          <t>6–0</t>
+        </is>
+      </c>
+      <c r="I12" s="73" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="H11" s="80" t="inlineStr">
-        <is>
-          <t>4–1</t>
-        </is>
-      </c>
-      <c r="I11" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="M11" s="74" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N11" s="76" t="inlineStr">
-        <is>
-          <t>Bosnia-Hercegovina</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe C</t>
-        </is>
-      </c>
-      <c r="B12" s="67" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C12" s="84" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D12" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="E12" s="69" t="n">
-        <v>5</v>
-      </c>
-      <c r="F12" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="G12" s="71" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="72" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I12" s="73" t="n">
-        <v>6</v>
-      </c>
-      <c r="J12" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="K12" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="L12" s="69" t="n">
-        <v>13</v>
-      </c>
-      <c r="M12" s="84" t="n">
-        <v>0.46</v>
+      <c r="M12" s="74" t="n">
+        <v>0.22</v>
       </c>
       <c r="N12" s="67" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Qatar</t>
         </is>
       </c>
     </row>
@@ -38558,47 +38554,47 @@
       <c r="A13" s="75" t="inlineStr"/>
       <c r="B13" s="76" t="inlineStr">
         <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C13" s="68" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="D13" s="78" t="n">
-        <v>9</v>
-      </c>
-      <c r="E13" s="78" t="n">
+          <t>Qatar</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D13" s="77" t="n">
         <v>5</v>
+      </c>
+      <c r="E13" s="77" t="n">
+        <v>3</v>
       </c>
       <c r="F13" s="77" t="n">
         <v>2</v>
       </c>
       <c r="G13" s="79" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H13" s="80" t="inlineStr">
         <is>
-          <t>3–0</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I13" s="81" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="J13" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="K13" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="M13" s="74" t="n">
-        <v>0.43</v>
+      <c r="K13" s="78" t="n">
+        <v>10</v>
+      </c>
+      <c r="L13" s="78" t="n">
+        <v>27</v>
+      </c>
+      <c r="M13" s="83" t="n">
+        <v>0.7</v>
       </c>
       <c r="N13" s="76" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Sveits</t>
         </is>
       </c>
     </row>
@@ -38606,47 +38602,47 @@
       <c r="A14" s="82" t="inlineStr"/>
       <c r="B14" s="67" t="inlineStr">
         <is>
-          <t>Haiti</t>
-        </is>
-      </c>
-      <c r="C14" s="84" t="n">
-        <v>0.5</v>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="C14" s="68" t="n">
+        <v>0.62</v>
       </c>
       <c r="D14" s="69" t="n">
         <v>13</v>
       </c>
-      <c r="E14" s="70" t="n">
+      <c r="E14" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F14" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="F14" s="70" t="n">
-        <v>7</v>
-      </c>
       <c r="G14" s="71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H14" s="72" t="inlineStr">
         <is>
-          <t>0–1</t>
+          <t>4–1</t>
         </is>
       </c>
       <c r="I14" s="73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J14" s="70" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K14" s="70" t="n">
         <v>3</v>
       </c>
       <c r="L14" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="M14" s="84" t="n">
-        <v>0.5</v>
+        <v>4</v>
+      </c>
+      <c r="M14" s="74" t="n">
+        <v>0.38</v>
       </c>
       <c r="N14" s="67" t="inlineStr">
         <is>
-          <t>Skottland</t>
+          <t>Bosnia-Hercegovina</t>
         </is>
       </c>
     </row>
@@ -38654,99 +38650,99 @@
       <c r="A15" s="75" t="inlineStr"/>
       <c r="B15" s="76" t="inlineStr">
         <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-      <c r="C15" s="74" t="n">
-        <v>0.4</v>
+          <t>Sveits</t>
+        </is>
+      </c>
+      <c r="C15" s="68" t="n">
+        <v>0.55</v>
       </c>
       <c r="D15" s="77" t="n">
         <v>6</v>
       </c>
       <c r="E15" s="77" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F15" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="80" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="I15" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="79" t="n">
+      <c r="J15" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="H15" s="80" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="I15" s="81" t="n">
-        <v>4</v>
-      </c>
-      <c r="J15" s="77" t="n">
-        <v>5</v>
-      </c>
       <c r="K15" s="78" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L15" s="78" t="n">
-        <v>12</v>
-      </c>
-      <c r="M15" s="68" t="n">
-        <v>0.6</v>
+        <v>13</v>
+      </c>
+      <c r="M15" s="84" t="n">
+        <v>0.45</v>
       </c>
       <c r="N15" s="76" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Canada</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="66" t="inlineStr">
         <is>
-          <t>Gruppe D</t>
+          <t>Gruppe C</t>
         </is>
       </c>
       <c r="B16" s="67" t="inlineStr">
         <is>
-          <t>Australia</t>
-        </is>
-      </c>
-      <c r="C16" s="74" t="n">
-        <v>0.37</v>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C16" s="84" t="n">
+        <v>0.54</v>
       </c>
       <c r="D16" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="E16" s="70" t="n">
+      <c r="E16" s="69" t="n">
+        <v>5</v>
+      </c>
+      <c r="F16" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H16" s="72" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I16" s="73" t="n">
+        <v>6</v>
+      </c>
+      <c r="J16" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="G16" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H16" s="72" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I16" s="73" t="n">
-        <v>11</v>
-      </c>
-      <c r="J16" s="70" t="n">
-        <v>10</v>
-      </c>
-      <c r="K16" s="69" t="n">
-        <v>7</v>
-      </c>
       <c r="L16" s="69" t="n">
-        <v>28</v>
-      </c>
-      <c r="M16" s="68" t="n">
-        <v>0.63</v>
+        <v>13</v>
+      </c>
+      <c r="M16" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N16" s="67" t="inlineStr">
         <is>
-          <t>Tyrkia</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
@@ -38754,27 +38750,27 @@
       <c r="A17" s="75" t="inlineStr"/>
       <c r="B17" s="76" t="inlineStr">
         <is>
-          <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="C17" s="83" t="n">
-        <v>0.78</v>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C17" s="68" t="n">
+        <v>0.57</v>
       </c>
       <c r="D17" s="78" t="n">
-        <v>33</v>
+        <v>9</v>
       </c>
       <c r="E17" s="78" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F17" s="77" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="G17" s="79" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="H17" s="80" t="inlineStr">
         <is>
-          <t>0–1</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I17" s="81" t="n">
@@ -38784,17 +38780,17 @@
         <v>2</v>
       </c>
       <c r="K17" s="77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L17" s="77" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="M17" s="74" t="n">
-        <v>0.22</v>
+        <v>0.43</v>
       </c>
       <c r="N17" s="76" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Haiti</t>
         </is>
       </c>
     </row>
@@ -38802,47 +38798,47 @@
       <c r="A18" s="82" t="inlineStr"/>
       <c r="B18" s="67" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C18" s="68" t="n">
-        <v>0.63</v>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="C18" s="84" t="n">
+        <v>0.5</v>
       </c>
       <c r="D18" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="E18" s="69" t="n">
-        <v>6</v>
+        <v>13</v>
+      </c>
+      <c r="E18" s="70" t="n">
+        <v>3</v>
       </c>
       <c r="F18" s="70" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G18" s="71" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="H18" s="72" t="inlineStr">
         <is>
-          <t>4–1</t>
+          <t>0–1</t>
         </is>
       </c>
       <c r="I18" s="73" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J18" s="70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K18" s="70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L18" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="M18" s="74" t="n">
-        <v>0.37</v>
+      <c r="M18" s="84" t="n">
+        <v>0.5</v>
       </c>
       <c r="N18" s="67" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Skottland</t>
         </is>
       </c>
     </row>
@@ -38850,99 +38846,99 @@
       <c r="A19" s="75" t="inlineStr"/>
       <c r="B19" s="76" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C19" s="68" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="D19" s="78" t="n">
-        <v>8</v>
+          <t>Skottland</t>
+        </is>
+      </c>
+      <c r="C19" s="74" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="D19" s="77" t="n">
+        <v>6</v>
       </c>
       <c r="E19" s="77" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F19" s="77" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G19" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H19" s="80" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I19" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="J19" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="H19" s="80" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I19" s="81" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="77" t="n">
+      <c r="K19" s="78" t="n">
         <v>3</v>
       </c>
-      <c r="K19" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="L19" s="77" t="n">
-        <v>5</v>
-      </c>
-      <c r="M19" s="74" t="n">
-        <v>0.37</v>
+      <c r="L19" s="78" t="n">
+        <v>12</v>
+      </c>
+      <c r="M19" s="68" t="n">
+        <v>0.6</v>
       </c>
       <c r="N19" s="76" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="66" t="inlineStr">
         <is>
-          <t>Gruppe E</t>
+          <t>Gruppe D</t>
         </is>
       </c>
       <c r="B20" s="67" t="inlineStr">
         <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C20" s="83" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D20" s="69" t="n">
-        <v>26</v>
-      </c>
-      <c r="E20" s="69" t="n">
-        <v>15</v>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C20" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D20" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E20" s="70" t="n">
+        <v>4</v>
       </c>
       <c r="F20" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H20" s="72" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I20" s="73" t="n">
+        <v>11</v>
+      </c>
+      <c r="J20" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="K20" s="69" t="n">
         <v>7</v>
       </c>
-      <c r="G20" s="71" t="n">
-        <v>4</v>
-      </c>
-      <c r="H20" s="72" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I20" s="73" t="n">
-        <v>4</v>
-      </c>
-      <c r="J20" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K20" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="L20" s="70" t="n">
-        <v>10</v>
-      </c>
-      <c r="M20" s="74" t="n">
-        <v>0.25</v>
+      <c r="L20" s="69" t="n">
+        <v>28</v>
+      </c>
+      <c r="M20" s="68" t="n">
+        <v>0.63</v>
       </c>
       <c r="N20" s="67" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Tyrkia</t>
         </is>
       </c>
     </row>
@@ -38950,47 +38946,47 @@
       <c r="A21" s="75" t="inlineStr"/>
       <c r="B21" s="76" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-      <c r="C21" s="84" t="n">
-        <v>0.49</v>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="C21" s="83" t="n">
+        <v>0.78</v>
       </c>
       <c r="D21" s="78" t="n">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="E21" s="78" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F21" s="77" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="G21" s="79" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
       <c r="H21" s="80" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>0–1</t>
         </is>
       </c>
       <c r="I21" s="81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="77" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K21" s="77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L21" s="77" t="n">
-        <v>10</v>
-      </c>
-      <c r="M21" s="84" t="n">
-        <v>0.51</v>
+        <v>6</v>
+      </c>
+      <c r="M21" s="74" t="n">
+        <v>0.22</v>
       </c>
       <c r="N21" s="76" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -38998,47 +38994,47 @@
       <c r="A22" s="82" t="inlineStr"/>
       <c r="B22" s="67" t="inlineStr">
         <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="C22" s="83" t="n">
-        <v>0.65</v>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C22" s="68" t="n">
+        <v>0.63</v>
       </c>
       <c r="D22" s="69" t="n">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E22" s="69" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="F22" s="70" t="n">
         <v>5</v>
       </c>
       <c r="G22" s="71" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="H22" s="72" t="inlineStr">
         <is>
-          <t>7–1</t>
+          <t>4–1</t>
         </is>
       </c>
       <c r="I22" s="73" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J22" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K22" s="70" t="n">
         <v>2</v>
       </c>
       <c r="L22" s="70" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="M22" s="74" t="n">
-        <v>0.35</v>
+        <v>0.37</v>
       </c>
       <c r="N22" s="67" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -39046,99 +39042,99 @@
       <c r="A23" s="75" t="inlineStr"/>
       <c r="B23" s="76" t="inlineStr">
         <is>
-          <t>Tyskland</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="C23" s="68" t="n">
-        <v>0.55</v>
+        <v>0.63</v>
       </c>
       <c r="D23" s="78" t="n">
-        <v>16</v>
-      </c>
-      <c r="E23" s="78" t="n">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="E23" s="77" t="n">
+        <v>2</v>
       </c>
       <c r="F23" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="79" t="n">
         <v>5</v>
       </c>
-      <c r="G23" s="79" t="n">
-        <v>4</v>
-      </c>
       <c r="H23" s="80" t="inlineStr">
         <is>
-          <t>2–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I23" s="81" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J23" s="77" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" s="77" t="n">
         <v>2</v>
       </c>
       <c r="L23" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="M23" s="84" t="n">
-        <v>0.45</v>
+        <v>5</v>
+      </c>
+      <c r="M23" s="74" t="n">
+        <v>0.37</v>
       </c>
       <c r="N23" s="76" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
+          <t>Australia</t>
         </is>
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="66" t="inlineStr">
         <is>
-          <t>Gruppe F</t>
+          <t>Gruppe E</t>
         </is>
       </c>
       <c r="B24" s="67" t="inlineStr">
         <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="C24" s="68" t="n">
-        <v>0.6</v>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="C24" s="83" t="n">
+        <v>0.75</v>
       </c>
       <c r="D24" s="69" t="n">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c r="E24" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="F24" s="70" t="n">
         <v>7</v>
       </c>
-      <c r="F24" s="70" t="n">
+      <c r="G24" s="71" t="n">
         <v>4</v>
       </c>
-      <c r="G24" s="71" t="n">
-        <v>0</v>
-      </c>
       <c r="H24" s="72" t="inlineStr">
         <is>
-          <t>2–2</t>
+          <t>0–0</t>
         </is>
       </c>
       <c r="I24" s="73" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J24" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K24" s="70" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L24" s="70" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="M24" s="74" t="n">
-        <v>0.4</v>
+        <v>0.25</v>
       </c>
       <c r="N24" s="67" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -39146,47 +39142,47 @@
       <c r="A25" s="75" t="inlineStr"/>
       <c r="B25" s="76" t="inlineStr">
         <is>
-          <t>Nederland</t>
+          <t>Elfenbenskysten</t>
         </is>
       </c>
       <c r="C25" s="84" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="D25" s="77" t="n">
-        <v>12</v>
-      </c>
-      <c r="E25" s="77" t="n">
-        <v>7</v>
+        <v>0.49</v>
+      </c>
+      <c r="D25" s="78" t="n">
+        <v>16</v>
+      </c>
+      <c r="E25" s="78" t="n">
+        <v>4</v>
       </c>
       <c r="F25" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G25" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="G25" s="79" t="n">
-        <v>2</v>
-      </c>
       <c r="H25" s="80" t="inlineStr">
         <is>
-          <t>5–1</t>
+          <t>1–0</t>
         </is>
       </c>
       <c r="I25" s="81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J25" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="K25" s="78" t="n">
-        <v>9</v>
-      </c>
-      <c r="L25" s="78" t="n">
-        <v>20</v>
+        <v>8</v>
+      </c>
+      <c r="K25" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L25" s="77" t="n">
+        <v>10</v>
       </c>
       <c r="M25" s="84" t="n">
-        <v>0.48</v>
+        <v>0.51</v>
       </c>
       <c r="N25" s="76" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>Ecuador</t>
         </is>
       </c>
     </row>
@@ -39194,47 +39190,47 @@
       <c r="A26" s="82" t="inlineStr"/>
       <c r="B26" s="67" t="inlineStr">
         <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-      <c r="C26" s="84" t="n">
-        <v>0.49</v>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C26" s="83" t="n">
+        <v>0.65</v>
       </c>
       <c r="D26" s="69" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="E26" s="69" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F26" s="70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G26" s="71" t="n">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c r="H26" s="72" t="inlineStr">
         <is>
-          <t>5–1</t>
+          <t>7–1</t>
         </is>
       </c>
       <c r="I26" s="73" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J26" s="70" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K26" s="70" t="n">
         <v>2</v>
       </c>
       <c r="L26" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="M26" s="84" t="n">
-        <v>0.51</v>
+        <v>7</v>
+      </c>
+      <c r="M26" s="74" t="n">
+        <v>0.35</v>
       </c>
       <c r="N26" s="67" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -39242,99 +39238,99 @@
       <c r="A27" s="75" t="inlineStr"/>
       <c r="B27" s="76" t="inlineStr">
         <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-      <c r="C27" s="74" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="D27" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="E27" s="77" t="n">
-        <v>1</v>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C27" s="68" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D27" s="78" t="n">
+        <v>16</v>
+      </c>
+      <c r="E27" s="78" t="n">
+        <v>7</v>
       </c>
       <c r="F27" s="77" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G27" s="79" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H27" s="80" t="inlineStr">
         <is>
-          <t>0–4</t>
+          <t>2–1</t>
         </is>
       </c>
       <c r="I27" s="81" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J27" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="K27" s="78" t="n">
-        <v>5</v>
-      </c>
-      <c r="L27" s="78" t="n">
-        <v>10</v>
-      </c>
-      <c r="M27" s="68" t="n">
-        <v>0.57</v>
+      <c r="K27" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L27" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="M27" s="84" t="n">
+        <v>0.45</v>
       </c>
       <c r="N27" s="76" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Elfenbenskysten</t>
         </is>
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="66" t="inlineStr">
         <is>
-          <t>Gruppe G</t>
+          <t>Gruppe F</t>
         </is>
       </c>
       <c r="B28" s="67" t="inlineStr">
         <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C28" s="84" t="n">
-        <v>0.53</v>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="C28" s="68" t="n">
+        <v>0.6</v>
       </c>
       <c r="D28" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="E28" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="E28" s="69" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G28" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="72" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I28" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K28" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="F28" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="G28" s="71" t="n">
-        <v>5</v>
-      </c>
-      <c r="H28" s="72" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I28" s="73" t="n">
+      <c r="L28" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="J28" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K28" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L28" s="70" t="n">
-        <v>14</v>
-      </c>
-      <c r="M28" s="84" t="n">
-        <v>0.47</v>
+      <c r="M28" s="74" t="n">
+        <v>0.4</v>
       </c>
       <c r="N28" s="67" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Japan</t>
         </is>
       </c>
     </row>
@@ -39342,47 +39338,47 @@
       <c r="A29" s="75" t="inlineStr"/>
       <c r="B29" s="76" t="inlineStr">
         <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C29" s="83" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="D29" s="78" t="n">
-        <v>22</v>
-      </c>
-      <c r="E29" s="78" t="n">
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="C29" s="84" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="D29" s="77" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" s="77" t="n">
         <v>7</v>
       </c>
       <c r="F29" s="77" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G29" s="79" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H29" s="80" t="inlineStr">
         <is>
-          <t>0–0</t>
+          <t>5–1</t>
         </is>
       </c>
       <c r="I29" s="81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J29" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K29" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="L29" s="77" t="n">
-        <v>7</v>
-      </c>
-      <c r="M29" s="74" t="n">
-        <v>0.32</v>
+        <v>9</v>
+      </c>
+      <c r="K29" s="78" t="n">
+        <v>9</v>
+      </c>
+      <c r="L29" s="78" t="n">
+        <v>20</v>
+      </c>
+      <c r="M29" s="84" t="n">
+        <v>0.48</v>
       </c>
       <c r="N29" s="76" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Sverige</t>
         </is>
       </c>
     </row>
@@ -39390,47 +39386,47 @@
       <c r="A30" s="82" t="inlineStr"/>
       <c r="B30" s="67" t="inlineStr">
         <is>
-          <t>Iran</t>
+          <t>Sverige</t>
         </is>
       </c>
       <c r="C30" s="84" t="n">
-        <v>0.47</v>
+        <v>0.49</v>
       </c>
       <c r="D30" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="E30" s="70" t="n">
-        <v>4</v>
+        <v>13</v>
+      </c>
+      <c r="E30" s="69" t="n">
+        <v>8</v>
       </c>
       <c r="F30" s="70" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="G30" s="71" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H30" s="72" t="inlineStr">
         <is>
-          <t>2–2</t>
+          <t>5–1</t>
         </is>
       </c>
       <c r="I30" s="73" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J30" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="K30" s="69" t="n">
-        <v>8</v>
+      <c r="K30" s="70" t="n">
+        <v>2</v>
       </c>
       <c r="L30" s="70" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="M30" s="84" t="n">
-        <v>0.53</v>
+        <v>0.51</v>
       </c>
       <c r="N30" s="67" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Tunisia</t>
         </is>
       </c>
     </row>
@@ -39438,75 +39434,75 @@
       <c r="A31" s="75" t="inlineStr"/>
       <c r="B31" s="76" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="C31" s="74" t="n">
-        <v>0.44</v>
+        <v>0.43</v>
       </c>
       <c r="D31" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E31" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G31" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H31" s="80" t="inlineStr">
+        <is>
+          <t>0–4</t>
+        </is>
+      </c>
+      <c r="I31" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J31" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K31" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="L31" s="78" t="n">
         <v>10</v>
       </c>
-      <c r="E31" s="77" t="n">
-        <v>5</v>
-      </c>
-      <c r="F31" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="G31" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H31" s="80" t="inlineStr">
-        <is>
-          <t>1–3</t>
-        </is>
-      </c>
-      <c r="I31" s="81" t="n">
-        <v>6</v>
-      </c>
-      <c r="J31" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="K31" s="78" t="n">
-        <v>7</v>
-      </c>
-      <c r="L31" s="78" t="n">
-        <v>19</v>
-      </c>
       <c r="M31" s="68" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.57</v>
       </c>
       <c r="N31" s="76" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Japan</t>
         </is>
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="66" t="inlineStr">
         <is>
-          <t>Gruppe H</t>
+          <t>Gruppe G</t>
         </is>
       </c>
       <c r="B32" s="67" t="inlineStr">
         <is>
-          <t>Saudi-Arabia</t>
-        </is>
-      </c>
-      <c r="C32" s="74" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D32" s="70" t="n">
-        <v>7</v>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="C32" s="84" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D32" s="69" t="n">
+        <v>15</v>
       </c>
       <c r="E32" s="70" t="n">
         <v>3</v>
       </c>
       <c r="F32" s="70" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G32" s="71" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H32" s="72" t="inlineStr">
         <is>
@@ -39514,23 +39510,23 @@
         </is>
       </c>
       <c r="I32" s="73" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="J32" s="70" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="K32" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="L32" s="69" t="n">
-        <v>27</v>
-      </c>
-      <c r="M32" s="83" t="n">
-        <v>0.65</v>
+        <v>4</v>
+      </c>
+      <c r="L32" s="70" t="n">
+        <v>14</v>
+      </c>
+      <c r="M32" s="84" t="n">
+        <v>0.47</v>
       </c>
       <c r="N32" s="67" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>Egypt</t>
         </is>
       </c>
     </row>
@@ -39538,20 +39534,20 @@
       <c r="A33" s="75" t="inlineStr"/>
       <c r="B33" s="76" t="inlineStr">
         <is>
-          <t>Spania</t>
+          <t>Belgia</t>
         </is>
       </c>
       <c r="C33" s="83" t="n">
-        <v>0.74</v>
+        <v>0.68</v>
       </c>
       <c r="D33" s="78" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E33" s="78" t="n">
+        <v>7</v>
+      </c>
+      <c r="F33" s="77" t="n">
         <v>8</v>
-      </c>
-      <c r="F33" s="77" t="n">
-        <v>9</v>
       </c>
       <c r="G33" s="79" t="n">
         <v>6</v>
@@ -39562,23 +39558,23 @@
         </is>
       </c>
       <c r="I33" s="81" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J33" s="77" t="n">
         <v>3</v>
       </c>
       <c r="K33" s="77" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="L33" s="77" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M33" s="74" t="n">
-        <v>0.26</v>
+        <v>0.32</v>
       </c>
       <c r="N33" s="76" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>Iran</t>
         </is>
       </c>
     </row>
@@ -39586,47 +39582,47 @@
       <c r="A34" s="82" t="inlineStr"/>
       <c r="B34" s="67" t="inlineStr">
         <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C34" s="83" t="n">
-        <v>0.65</v>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C34" s="84" t="n">
+        <v>0.47</v>
       </c>
       <c r="D34" s="69" t="n">
-        <v>21</v>
-      </c>
-      <c r="E34" s="69" t="n">
-        <v>9</v>
+        <v>17</v>
+      </c>
+      <c r="E34" s="70" t="n">
+        <v>4</v>
       </c>
       <c r="F34" s="70" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="G34" s="71" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H34" s="72" t="inlineStr">
         <is>
-          <t>4–0</t>
+          <t>2–2</t>
         </is>
       </c>
       <c r="I34" s="73" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J34" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="K34" s="70" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="K34" s="69" t="n">
+        <v>8</v>
       </c>
       <c r="L34" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="M34" s="74" t="n">
-        <v>0.35</v>
+        <v>13</v>
+      </c>
+      <c r="M34" s="84" t="n">
+        <v>0.53</v>
       </c>
       <c r="N34" s="67" t="inlineStr">
         <is>
-          <t>Saudi-Arabia</t>
+          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -39634,99 +39630,99 @@
       <c r="A35" s="75" t="inlineStr"/>
       <c r="B35" s="76" t="inlineStr">
         <is>
-          <t>Uruguay</t>
-        </is>
-      </c>
-      <c r="C35" s="83" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D35" s="78" t="n">
-        <v>16</v>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C35" s="74" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="D35" s="77" t="n">
+        <v>10</v>
       </c>
       <c r="E35" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="F35" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="F35" s="77" t="n">
+      <c r="G35" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H35" s="80" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I35" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="K35" s="78" t="n">
         <v>7</v>
       </c>
-      <c r="G35" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H35" s="80" t="inlineStr">
-        <is>
-          <t>2–2</t>
-        </is>
-      </c>
-      <c r="I35" s="81" t="n">
-        <v>4</v>
-      </c>
-      <c r="J35" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K35" s="78" t="n">
-        <v>4</v>
-      </c>
-      <c r="L35" s="77" t="n">
-        <v>11</v>
-      </c>
-      <c r="M35" s="74" t="n">
-        <v>0.34</v>
+      <c r="L35" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="M35" s="68" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="N35" s="76" t="inlineStr">
         <is>
-          <t>Kapp Verde</t>
+          <t>Egypt</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
       <c r="A36" s="66" t="inlineStr">
         <is>
-          <t>Gruppe I</t>
+          <t>Gruppe H</t>
         </is>
       </c>
       <c r="B36" s="67" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C36" s="84" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D36" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="E36" s="69" t="n">
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="C36" s="74" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D36" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="E36" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F36" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G36" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H36" s="72" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I36" s="73" t="n">
         <v>9</v>
       </c>
-      <c r="F36" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="71" t="n">
-        <v>2</v>
-      </c>
-      <c r="H36" s="72" t="inlineStr">
-        <is>
-          <t>3–1</t>
-        </is>
-      </c>
-      <c r="I36" s="73" t="n">
-        <v>1</v>
-      </c>
       <c r="J36" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K36" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="L36" s="70" t="n">
-        <v>6</v>
-      </c>
-      <c r="M36" s="84" t="n">
-        <v>0.46</v>
+        <v>8</v>
+      </c>
+      <c r="K36" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="L36" s="69" t="n">
+        <v>27</v>
+      </c>
+      <c r="M36" s="83" t="n">
+        <v>0.65</v>
       </c>
       <c r="N36" s="67" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Uruguay</t>
         </is>
       </c>
     </row>
@@ -39734,47 +39730,47 @@
       <c r="A37" s="75" t="inlineStr"/>
       <c r="B37" s="76" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C37" s="68" t="n">
-        <v>0.5600000000000001</v>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C37" s="83" t="n">
+        <v>0.74</v>
       </c>
       <c r="D37" s="78" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="E37" s="78" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F37" s="77" t="n">
         <v>9</v>
       </c>
       <c r="G37" s="79" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H37" s="80" t="inlineStr">
         <is>
-          <t>3–0</t>
+          <t>0–0</t>
         </is>
       </c>
       <c r="I37" s="81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J37" s="77" t="n">
         <v>3</v>
       </c>
       <c r="K37" s="77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L37" s="77" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="M37" s="74" t="n">
-        <v>0.44</v>
+        <v>0.26</v>
       </c>
       <c r="N37" s="76" t="inlineStr">
         <is>
-          <t>Irak</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
@@ -39782,47 +39778,47 @@
       <c r="A38" s="82" t="inlineStr"/>
       <c r="B38" s="67" t="inlineStr">
         <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="C38" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D38" s="70" t="n">
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C38" s="83" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D38" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="E38" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="F38" s="70" t="n">
         <v>11</v>
       </c>
-      <c r="E38" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="F38" s="70" t="n">
-        <v>8</v>
-      </c>
       <c r="G38" s="71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H38" s="72" t="inlineStr">
         <is>
-          <t>1–4</t>
+          <t>4–0</t>
         </is>
       </c>
       <c r="I38" s="73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J38" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="K38" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="L38" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="M38" s="68" t="n">
-        <v>0.63</v>
+        <v>1</v>
+      </c>
+      <c r="K38" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L38" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="M38" s="74" t="n">
+        <v>0.35</v>
       </c>
       <c r="N38" s="67" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Saudi-Arabia</t>
         </is>
       </c>
     </row>
@@ -39830,99 +39826,99 @@
       <c r="A39" s="75" t="inlineStr"/>
       <c r="B39" s="76" t="inlineStr">
         <is>
-          <t>Norge</t>
-        </is>
-      </c>
-      <c r="C39" s="74" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="D39" s="77" t="n">
-        <v>12</v>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="C39" s="83" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D39" s="78" t="n">
+        <v>16</v>
       </c>
       <c r="E39" s="77" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F39" s="77" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G39" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="H39" s="80" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I39" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="H39" s="80" t="inlineStr">
-        <is>
-          <t>3–2</t>
-        </is>
-      </c>
-      <c r="I39" s="81" t="n">
-        <v>5</v>
-      </c>
       <c r="J39" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="K39" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="L39" s="78" t="n">
-        <v>17</v>
-      </c>
-      <c r="M39" s="68" t="n">
-        <v>0.57</v>
+        <v>3</v>
+      </c>
+      <c r="K39" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="L39" s="77" t="n">
+        <v>11</v>
+      </c>
+      <c r="M39" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N39" s="76" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="66" t="inlineStr">
         <is>
-          <t>Gruppe J</t>
+          <t>Gruppe I</t>
         </is>
       </c>
       <c r="B40" s="67" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>Frankrike</t>
         </is>
       </c>
       <c r="C40" s="84" t="n">
-        <v>0.47</v>
+        <v>0.54</v>
       </c>
       <c r="D40" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="E40" s="69" t="n">
         <v>9</v>
       </c>
-      <c r="E40" s="69" t="n">
-        <v>6</v>
-      </c>
       <c r="F40" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H40" s="72" t="inlineStr">
+        <is>
+          <t>3–1</t>
+        </is>
+      </c>
+      <c r="I40" s="73" t="n">
+        <v>1</v>
+      </c>
+      <c r="J40" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K40" s="70" t="n">
         <v>3</v>
-      </c>
-      <c r="G40" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H40" s="72" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I40" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J40" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="K40" s="70" t="n">
-        <v>0</v>
       </c>
       <c r="L40" s="70" t="n">
         <v>6</v>
       </c>
       <c r="M40" s="84" t="n">
-        <v>0.53</v>
+        <v>0.46</v>
       </c>
       <c r="N40" s="67" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -39930,47 +39926,47 @@
       <c r="A41" s="75" t="inlineStr"/>
       <c r="B41" s="76" t="inlineStr">
         <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C41" s="84" t="n">
-        <v>0.54</v>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C41" s="68" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="D41" s="78" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="E41" s="78" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F41" s="77" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="G41" s="79" t="n">
         <v>5</v>
       </c>
       <c r="H41" s="80" t="inlineStr">
         <is>
-          <t>2–0</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I41" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="J41" s="77" t="n">
-        <v>2</v>
-      </c>
       <c r="K41" s="77" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L41" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="M41" s="84" t="n">
-        <v>0.46</v>
+        <v>4</v>
+      </c>
+      <c r="M41" s="74" t="n">
+        <v>0.44</v>
       </c>
       <c r="N41" s="76" t="inlineStr">
         <is>
-          <t>Østerrike</t>
+          <t>Irak</t>
         </is>
       </c>
     </row>
@@ -39978,47 +39974,47 @@
       <c r="A42" s="82" t="inlineStr"/>
       <c r="B42" s="67" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Irak</t>
         </is>
       </c>
       <c r="C42" s="74" t="n">
-        <v>0.25</v>
+        <v>0.37</v>
       </c>
       <c r="D42" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="E42" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="E42" s="70" t="n">
+      <c r="G42" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="72" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="I42" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J42" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="F42" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="G42" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="72" t="inlineStr">
-        <is>
-          <t>1–2</t>
-        </is>
-      </c>
-      <c r="I42" s="73" t="n">
+      <c r="K42" s="69" t="n">
         <v>6</v>
       </c>
-      <c r="J42" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="K42" s="69" t="n">
-        <v>8</v>
-      </c>
       <c r="L42" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="M42" s="83" t="n">
-        <v>0.75</v>
+        <v>12</v>
+      </c>
+      <c r="M42" s="68" t="n">
+        <v>0.63</v>
       </c>
       <c r="N42" s="67" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Norge</t>
         </is>
       </c>
     </row>
@@ -40026,99 +40022,99 @@
       <c r="A43" s="75" t="inlineStr"/>
       <c r="B43" s="76" t="inlineStr">
         <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C43" s="68" t="n">
-        <v>0.62</v>
+          <t>Norge</t>
+        </is>
+      </c>
+      <c r="C43" s="74" t="n">
+        <v>0.43</v>
       </c>
       <c r="D43" s="77" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E43" s="77" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F43" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G43" s="79" t="n">
         <v>4</v>
       </c>
-      <c r="G43" s="79" t="n">
-        <v>2</v>
-      </c>
       <c r="H43" s="80" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>3–2</t>
         </is>
       </c>
       <c r="I43" s="81" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J43" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="K43" s="78" t="n">
-        <v>4</v>
+        <v>6</v>
+      </c>
+      <c r="K43" s="77" t="n">
+        <v>6</v>
       </c>
       <c r="L43" s="78" t="n">
-        <v>11</v>
-      </c>
-      <c r="M43" s="74" t="n">
-        <v>0.38</v>
+        <v>17</v>
+      </c>
+      <c r="M43" s="68" t="n">
+        <v>0.57</v>
       </c>
       <c r="N43" s="76" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="66" t="inlineStr">
         <is>
-          <t>Gruppe K</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="B44" s="67" t="inlineStr">
         <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="C44" s="83" t="n">
-        <v>0.66</v>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C44" s="84" t="n">
+        <v>0.47</v>
       </c>
       <c r="D44" s="69" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E44" s="69" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F44" s="70" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G44" s="71" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H44" s="72" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I44" s="73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J44" s="70" t="n">
         <v>3</v>
       </c>
       <c r="K44" s="70" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L44" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="M44" s="74" t="n">
-        <v>0.34</v>
+        <v>6</v>
+      </c>
+      <c r="M44" s="84" t="n">
+        <v>0.53</v>
       </c>
       <c r="N44" s="67" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -40126,14 +40122,14 @@
       <c r="A45" s="75" t="inlineStr"/>
       <c r="B45" s="76" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C45" s="83" t="n">
-        <v>0.75</v>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C45" s="84" t="n">
+        <v>0.54</v>
       </c>
       <c r="D45" s="78" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E45" s="78" t="n">
         <v>3</v>
@@ -40142,31 +40138,31 @@
         <v>4</v>
       </c>
       <c r="G45" s="79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H45" s="80" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I45" s="81" t="n">
         <v>3</v>
       </c>
       <c r="J45" s="77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K45" s="77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L45" s="77" t="n">
-        <v>8</v>
-      </c>
-      <c r="M45" s="74" t="n">
-        <v>0.25</v>
+        <v>6</v>
+      </c>
+      <c r="M45" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N45" s="76" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Østerrike</t>
         </is>
       </c>
     </row>
@@ -40174,47 +40170,47 @@
       <c r="A46" s="82" t="inlineStr"/>
       <c r="B46" s="67" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C46" s="83" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D46" s="69" t="n">
-        <v>16</v>
-      </c>
-      <c r="E46" s="69" t="n">
-        <v>9</v>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C46" s="74" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D46" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E46" s="70" t="n">
+        <v>4</v>
       </c>
       <c r="F46" s="70" t="n">
         <v>4</v>
       </c>
       <c r="G46" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="72" t="inlineStr">
+        <is>
+          <t>1–2</t>
+        </is>
+      </c>
+      <c r="I46" s="73" t="n">
+        <v>6</v>
+      </c>
+      <c r="J46" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="H46" s="72" t="inlineStr">
-        <is>
-          <t>5–0</t>
-        </is>
-      </c>
-      <c r="I46" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J46" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K46" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L46" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="M46" s="74" t="n">
-        <v>0.34</v>
+      <c r="K46" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="L46" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="M46" s="83" t="n">
+        <v>0.75</v>
       </c>
       <c r="N46" s="67" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -40222,99 +40218,99 @@
       <c r="A47" s="75" t="inlineStr"/>
       <c r="B47" s="76" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C47" s="74" t="n">
-        <v>0.33</v>
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C47" s="68" t="n">
+        <v>0.62</v>
       </c>
       <c r="D47" s="77" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E47" s="77" t="n">
         <v>3</v>
       </c>
       <c r="F47" s="77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G47" s="79" t="n">
         <v>2</v>
       </c>
       <c r="H47" s="80" t="inlineStr">
         <is>
-          <t>1–3</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I47" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J47" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="J47" s="77" t="n">
-        <v>5</v>
-      </c>
       <c r="K47" s="78" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L47" s="78" t="n">
-        <v>15</v>
-      </c>
-      <c r="M47" s="83" t="n">
-        <v>0.67</v>
+        <v>11</v>
+      </c>
+      <c r="M47" s="74" t="n">
+        <v>0.38</v>
       </c>
       <c r="N47" s="76" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Jordan</t>
         </is>
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="66" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe K</t>
         </is>
       </c>
       <c r="B48" s="67" t="inlineStr">
         <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C48" s="84" t="n">
-        <v>0.54</v>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C48" s="83" t="n">
+        <v>0.66</v>
       </c>
       <c r="D48" s="69" t="n">
         <v>20</v>
       </c>
       <c r="E48" s="69" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F48" s="70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G48" s="71" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H48" s="72" t="inlineStr">
         <is>
-          <t>4–2</t>
+          <t>1–0</t>
         </is>
       </c>
       <c r="I48" s="73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J48" s="70" t="n">
         <v>3</v>
       </c>
       <c r="K48" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L48" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="M48" s="84" t="n">
-        <v>0.46</v>
+        <v>7</v>
+      </c>
+      <c r="M48" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N48" s="67" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -40322,47 +40318,47 @@
       <c r="A49" s="75" t="inlineStr"/>
       <c r="B49" s="76" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C49" s="83" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="D49" s="78" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E49" s="78" t="n">
+        <v>3</v>
+      </c>
+      <c r="F49" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="F49" s="77" t="n">
+      <c r="G49" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H49" s="80" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I49" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J49" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K49" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L49" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="G49" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H49" s="80" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I49" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J49" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K49" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L49" s="77" t="n">
-        <v>2</v>
-      </c>
       <c r="M49" s="74" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="N49" s="76" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -40370,47 +40366,47 @@
       <c r="A50" s="82" t="inlineStr"/>
       <c r="B50" s="67" t="inlineStr">
         <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="C50" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D50" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="E50" s="70" t="n">
-        <v>3</v>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C50" s="83" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D50" s="69" t="n">
+        <v>16</v>
+      </c>
+      <c r="E50" s="69" t="n">
+        <v>9</v>
       </c>
       <c r="F50" s="70" t="n">
         <v>4</v>
       </c>
       <c r="G50" s="71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H50" s="72" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>5–0</t>
         </is>
       </c>
       <c r="I50" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J50" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="J50" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="K50" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L50" s="69" t="n">
-        <v>11</v>
-      </c>
-      <c r="M50" s="68" t="n">
-        <v>0.63</v>
+      <c r="K50" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="L50" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="M50" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N50" s="67" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Usbekistan</t>
         </is>
       </c>
     </row>
@@ -40418,79 +40414,275 @@
       <c r="A51" s="75" t="inlineStr"/>
       <c r="B51" s="76" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Usbekistan</t>
         </is>
       </c>
       <c r="C51" s="74" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="D51" s="78" t="n">
-        <v>8</v>
+        <v>0.33</v>
+      </c>
+      <c r="D51" s="77" t="n">
+        <v>7</v>
       </c>
       <c r="E51" s="77" t="n">
         <v>3</v>
       </c>
       <c r="F51" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G51" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H51" s="80" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I51" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="G51" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H51" s="80" t="inlineStr">
+      <c r="J51" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="K51" s="78" t="n">
+        <v>6</v>
+      </c>
+      <c r="L51" s="78" t="n">
+        <v>15</v>
+      </c>
+      <c r="M51" s="83" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N51" s="76" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="B52" s="67" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C52" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D52" s="69" t="n">
+        <v>20</v>
+      </c>
+      <c r="E52" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="F52" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G52" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H52" s="72" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="I52" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J52" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K52" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="L52" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="M52" s="84" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N52" s="67" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="75" t="inlineStr"/>
+      <c r="B53" s="76" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C53" s="83" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D53" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="E53" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="F53" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="G53" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="H53" s="80" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I53" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K53" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L53" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="M53" s="74" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N53" s="76" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="82" t="inlineStr"/>
+      <c r="B54" s="67" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C54" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D54" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E54" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F54" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G54" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H54" s="72" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I54" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K54" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="L54" s="69" t="n">
+        <v>11</v>
+      </c>
+      <c r="M54" s="68" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N54" s="67" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="75" t="inlineStr"/>
+      <c r="B55" s="76" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C55" s="74" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D55" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E55" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F55" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="G55" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H55" s="80" t="inlineStr">
         <is>
           <t>0–1</t>
         </is>
       </c>
-      <c r="I51" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J51" s="77" t="n">
+      <c r="I55" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J55" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="K51" s="77" t="n">
+      <c r="K55" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="L51" s="77" t="n">
+      <c r="L55" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="M51" s="68" t="n">
+      <c r="M55" s="68" t="n">
         <v>0.58</v>
       </c>
-      <c r="N51" s="76" t="inlineStr">
+      <c r="N55" s="76" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="53" ht="14" customHeight="1">
-      <c r="A53" s="63" t="inlineStr">
+    <row r="57" ht="14" customHeight="1">
+      <c r="A57" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="55" t="inlineStr">
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B54" s="62" t="inlineStr">
+      <c r="B58" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C54" s="61" t="inlineStr">
+      <c r="C58" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D54" s="58" t="inlineStr">
+      <c r="D58" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E54" s="85" t="inlineStr">
+      <c r="E58" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -40499,8 +40691,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
+    <mergeCell ref="A57:N57"/>
     <mergeCell ref="I2:N2"/>
-    <mergeCell ref="A53:N53"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-25 08:48 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -48051,7 +48051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N58"/>
+  <dimension ref="A1:N60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -48899,99 +48899,95 @@
       <c r="A19" s="75" t="inlineStr"/>
       <c r="B19" s="76" t="inlineStr">
         <is>
-          <t>Skottland</t>
-        </is>
-      </c>
-      <c r="C19" s="74" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="D19" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="E19" s="77" t="n">
-        <v>0</v>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="C19" s="83" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D19" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="E19" s="78" t="n">
+        <v>12</v>
       </c>
       <c r="F19" s="77" t="n">
         <v>3</v>
       </c>
       <c r="G19" s="79" t="n">
+        <v>4</v>
+      </c>
+      <c r="H19" s="80" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="I19" s="81" t="n">
         <v>3</v>
       </c>
-      <c r="H19" s="80" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="I19" s="81" t="n">
-        <v>4</v>
-      </c>
       <c r="J19" s="77" t="n">
-        <v>5</v>
-      </c>
-      <c r="K19" s="78" t="n">
-        <v>3</v>
-      </c>
-      <c r="L19" s="78" t="n">
-        <v>12</v>
-      </c>
-      <c r="M19" s="68" t="n">
-        <v>0.6</v>
+        <v>2</v>
+      </c>
+      <c r="K19" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L19" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="M19" s="74" t="n">
+        <v>0.31</v>
       </c>
       <c r="N19" s="76" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Haiti</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe D</t>
-        </is>
-      </c>
+      <c r="A20" s="82" t="inlineStr"/>
       <c r="B20" s="67" t="inlineStr">
         <is>
-          <t>Australia</t>
+          <t>Skottland</t>
         </is>
       </c>
       <c r="C20" s="74" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="D20" s="70" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E20" s="70" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F20" s="70" t="n">
         <v>3</v>
       </c>
       <c r="G20" s="71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H20" s="72" t="inlineStr">
         <is>
-          <t>2–0</t>
+          <t>0–1</t>
         </is>
       </c>
       <c r="I20" s="73" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="J20" s="70" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="K20" s="69" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="L20" s="69" t="n">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="M20" s="68" t="n">
-        <v>0.63</v>
+        <v>0.6</v>
       </c>
       <c r="N20" s="67" t="inlineStr">
         <is>
-          <t>Tyrkia</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
@@ -48999,95 +48995,99 @@
       <c r="A21" s="75" t="inlineStr"/>
       <c r="B21" s="76" t="inlineStr">
         <is>
+          <t>Skottland</t>
+        </is>
+      </c>
+      <c r="C21" s="84" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="D21" s="77" t="n">
+        <v>11</v>
+      </c>
+      <c r="E21" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" s="79" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" s="80" t="inlineStr">
+        <is>
+          <t>0–3</t>
+        </is>
+      </c>
+      <c r="I21" s="81" t="n">
+        <v>7</v>
+      </c>
+      <c r="J21" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="K21" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="L21" s="78" t="n">
+        <v>21</v>
+      </c>
+      <c r="M21" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="N21" s="76" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe D</t>
+        </is>
+      </c>
+      <c r="B22" s="67" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="C22" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D22" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E22" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="F22" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G22" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" s="72" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I22" s="73" t="n">
+        <v>11</v>
+      </c>
+      <c r="J22" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="K22" s="69" t="n">
+        <v>7</v>
+      </c>
+      <c r="L22" s="69" t="n">
+        <v>28</v>
+      </c>
+      <c r="M22" s="68" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N22" s="67" t="inlineStr">
+        <is>
           <t>Tyrkia</t>
-        </is>
-      </c>
-      <c r="C21" s="83" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="D21" s="78" t="n">
-        <v>33</v>
-      </c>
-      <c r="E21" s="78" t="n">
-        <v>6</v>
-      </c>
-      <c r="F21" s="77" t="n">
-        <v>15</v>
-      </c>
-      <c r="G21" s="79" t="n">
-        <v>12</v>
-      </c>
-      <c r="H21" s="80" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="I21" s="81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J21" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="L21" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="M21" s="74" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="N21" s="76" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="82" t="inlineStr"/>
-      <c r="B22" s="67" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C22" s="68" t="n">
-        <v>0.63</v>
-      </c>
-      <c r="D22" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="E22" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="G22" s="71" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" s="72" t="inlineStr">
-        <is>
-          <t>4–1</t>
-        </is>
-      </c>
-      <c r="I22" s="73" t="n">
-        <v>4</v>
-      </c>
-      <c r="J22" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K22" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L22" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="M22" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="N22" s="67" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -49095,79 +49095,75 @@
       <c r="A23" s="75" t="inlineStr"/>
       <c r="B23" s="76" t="inlineStr">
         <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="C23" s="68" t="n">
-        <v>0.63</v>
+          <t>Tyrkia</t>
+        </is>
+      </c>
+      <c r="C23" s="83" t="n">
+        <v>0.78</v>
       </c>
       <c r="D23" s="78" t="n">
-        <v>8</v>
-      </c>
-      <c r="E23" s="77" t="n">
+        <v>33</v>
+      </c>
+      <c r="E23" s="78" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" s="77" t="n">
+        <v>15</v>
+      </c>
+      <c r="G23" s="79" t="n">
+        <v>12</v>
+      </c>
+      <c r="H23" s="80" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I23" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="F23" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="79" t="n">
-        <v>5</v>
-      </c>
-      <c r="H23" s="80" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I23" s="81" t="n">
-        <v>0</v>
-      </c>
       <c r="J23" s="77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" s="77" t="n">
         <v>2</v>
       </c>
       <c r="L23" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="M23" s="74" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N23" s="76" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="82" t="inlineStr"/>
+      <c r="B24" s="67" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C24" s="68" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="D24" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="E24" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="F24" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="M23" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="N23" s="76" t="inlineStr">
-        <is>
-          <t>Australia</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe E</t>
-        </is>
-      </c>
-      <c r="B24" s="67" t="inlineStr">
-        <is>
-          <t>Ecuador</t>
-        </is>
-      </c>
-      <c r="C24" s="83" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D24" s="69" t="n">
-        <v>26</v>
-      </c>
-      <c r="E24" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="F24" s="70" t="n">
-        <v>7</v>
-      </c>
       <c r="G24" s="71" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="H24" s="72" t="inlineStr">
         <is>
-          <t>0–0</t>
+          <t>4–1</t>
         </is>
       </c>
       <c r="I24" s="73" t="n">
@@ -49177,17 +49173,17 @@
         <v>2</v>
       </c>
       <c r="K24" s="70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="L24" s="70" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="M24" s="74" t="n">
-        <v>0.25</v>
+        <v>0.37</v>
       </c>
       <c r="N24" s="67" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -49195,91 +49191,95 @@
       <c r="A25" s="75" t="inlineStr"/>
       <c r="B25" s="76" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-      <c r="C25" s="84" t="n">
-        <v>0.49</v>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C25" s="68" t="n">
+        <v>0.63</v>
       </c>
       <c r="D25" s="78" t="n">
-        <v>16</v>
-      </c>
-      <c r="E25" s="78" t="n">
-        <v>4</v>
+        <v>8</v>
+      </c>
+      <c r="E25" s="77" t="n">
+        <v>2</v>
       </c>
       <c r="F25" s="77" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="G25" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="H25" s="80" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I25" s="81" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="H25" s="80" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I25" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" s="77" t="n">
-        <v>8</v>
-      </c>
       <c r="K25" s="77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L25" s="77" t="n">
-        <v>10</v>
-      </c>
-      <c r="M25" s="84" t="n">
-        <v>0.51</v>
+        <v>5</v>
+      </c>
+      <c r="M25" s="74" t="n">
+        <v>0.37</v>
       </c>
       <c r="N25" s="76" t="inlineStr">
         <is>
+          <t>Australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe E</t>
+        </is>
+      </c>
+      <c r="B26" s="67" t="inlineStr">
+        <is>
           <t>Ecuador</t>
         </is>
       </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="82" t="inlineStr"/>
-      <c r="B26" s="67" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
       <c r="C26" s="83" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="D26" s="69" t="n">
         <v>26</v>
       </c>
       <c r="E26" s="69" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="F26" s="70" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="G26" s="71" t="n">
+        <v>4</v>
+      </c>
+      <c r="H26" s="72" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I26" s="73" t="n">
+        <v>4</v>
+      </c>
+      <c r="J26" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K26" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="L26" s="70" t="n">
         <v>10</v>
       </c>
-      <c r="H26" s="72" t="inlineStr">
-        <is>
-          <t>7–1</t>
-        </is>
-      </c>
-      <c r="I26" s="73" t="n">
-        <v>0</v>
-      </c>
-      <c r="J26" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="K26" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L26" s="70" t="n">
-        <v>7</v>
-      </c>
       <c r="M26" s="74" t="n">
-        <v>0.35</v>
+        <v>0.25</v>
       </c>
       <c r="N26" s="67" t="inlineStr">
         <is>
@@ -49291,79 +49291,75 @@
       <c r="A27" s="75" t="inlineStr"/>
       <c r="B27" s="76" t="inlineStr">
         <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="C27" s="68" t="n">
-        <v>0.55</v>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="C27" s="84" t="n">
+        <v>0.49</v>
       </c>
       <c r="D27" s="78" t="n">
         <v>16</v>
       </c>
       <c r="E27" s="78" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F27" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G27" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H27" s="80" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I27" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="K27" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L27" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="M27" s="84" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="N27" s="76" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="82" t="inlineStr"/>
+      <c r="B28" s="67" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C28" s="83" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D28" s="69" t="n">
+        <v>26</v>
+      </c>
+      <c r="E28" s="69" t="n">
+        <v>11</v>
+      </c>
+      <c r="F28" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="G27" s="79" t="n">
-        <v>4</v>
-      </c>
-      <c r="H27" s="80" t="inlineStr">
-        <is>
-          <t>2–1</t>
-        </is>
-      </c>
-      <c r="I27" s="81" t="n">
-        <v>5</v>
-      </c>
-      <c r="J27" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="K27" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="L27" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="M27" s="84" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="N27" s="76" t="inlineStr">
-        <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe F</t>
-        </is>
-      </c>
-      <c r="B28" s="67" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="C28" s="68" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="D28" s="69" t="n">
-        <v>11</v>
-      </c>
-      <c r="E28" s="69" t="n">
-        <v>7</v>
-      </c>
-      <c r="F28" s="70" t="n">
-        <v>4</v>
-      </c>
       <c r="G28" s="71" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="H28" s="72" t="inlineStr">
         <is>
-          <t>2–2</t>
+          <t>7–1</t>
         </is>
       </c>
       <c r="I28" s="73" t="n">
@@ -49373,17 +49369,17 @@
         <v>5</v>
       </c>
       <c r="K28" s="70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L28" s="70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M28" s="74" t="n">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="N28" s="67" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
@@ -49391,95 +49387,99 @@
       <c r="A29" s="75" t="inlineStr"/>
       <c r="B29" s="76" t="inlineStr">
         <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C29" s="68" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D29" s="78" t="n">
+        <v>16</v>
+      </c>
+      <c r="E29" s="78" t="n">
+        <v>7</v>
+      </c>
+      <c r="F29" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" s="79" t="n">
+        <v>4</v>
+      </c>
+      <c r="H29" s="80" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="I29" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="J29" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K29" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L29" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="M29" s="84" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="N29" s="76" t="inlineStr">
+        <is>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe F</t>
+        </is>
+      </c>
+      <c r="B30" s="67" t="inlineStr">
+        <is>
           <t>Nederland</t>
         </is>
       </c>
-      <c r="C29" s="84" t="n">
-        <v>0.52</v>
-      </c>
-      <c r="D29" s="77" t="n">
-        <v>12</v>
-      </c>
-      <c r="E29" s="77" t="n">
+      <c r="C30" s="68" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D30" s="69" t="n">
+        <v>11</v>
+      </c>
+      <c r="E30" s="69" t="n">
         <v>7</v>
       </c>
-      <c r="F29" s="77" t="n">
+      <c r="F30" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G30" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="72" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I30" s="73" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K30" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="G29" s="79" t="n">
-        <v>2</v>
-      </c>
-      <c r="H29" s="80" t="inlineStr">
-        <is>
-          <t>5–1</t>
-        </is>
-      </c>
-      <c r="I29" s="81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J29" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="K29" s="78" t="n">
-        <v>9</v>
-      </c>
-      <c r="L29" s="78" t="n">
-        <v>20</v>
-      </c>
-      <c r="M29" s="84" t="n">
-        <v>0.48</v>
-      </c>
-      <c r="N29" s="76" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="82" t="inlineStr"/>
-      <c r="B30" s="67" t="inlineStr">
-        <is>
-          <t>Sverige</t>
-        </is>
-      </c>
-      <c r="C30" s="84" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="D30" s="69" t="n">
-        <v>13</v>
-      </c>
-      <c r="E30" s="69" t="n">
+      <c r="L30" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="F30" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="G30" s="71" t="n">
-        <v>2</v>
-      </c>
-      <c r="H30" s="72" t="inlineStr">
-        <is>
-          <t>5–1</t>
-        </is>
-      </c>
-      <c r="I30" s="73" t="n">
-        <v>1</v>
-      </c>
-      <c r="J30" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K30" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L30" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="M30" s="84" t="n">
-        <v>0.51</v>
+      <c r="M30" s="74" t="n">
+        <v>0.4</v>
       </c>
       <c r="N30" s="67" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Japan</t>
         </is>
       </c>
     </row>
@@ -49487,99 +49487,95 @@
       <c r="A31" s="75" t="inlineStr"/>
       <c r="B31" s="76" t="inlineStr">
         <is>
-          <t>Tunisia</t>
-        </is>
-      </c>
-      <c r="C31" s="74" t="n">
-        <v>0.43</v>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="C31" s="84" t="n">
+        <v>0.52</v>
       </c>
       <c r="D31" s="77" t="n">
+        <v>12</v>
+      </c>
+      <c r="E31" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="F31" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="E31" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="F31" s="77" t="n">
-        <v>1</v>
-      </c>
       <c r="G31" s="79" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H31" s="80" t="inlineStr">
         <is>
-          <t>0–4</t>
+          <t>5–1</t>
         </is>
       </c>
       <c r="I31" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="J31" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="K31" s="78" t="n">
+        <v>9</v>
+      </c>
+      <c r="L31" s="78" t="n">
+        <v>20</v>
+      </c>
+      <c r="M31" s="84" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="N31" s="76" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="82" t="inlineStr"/>
+      <c r="B32" s="67" t="inlineStr">
+        <is>
+          <t>Sverige</t>
+        </is>
+      </c>
+      <c r="C32" s="84" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="D32" s="69" t="n">
+        <v>13</v>
+      </c>
+      <c r="E32" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F32" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="J31" s="77" t="n">
+      <c r="G32" s="71" t="n">
         <v>2</v>
       </c>
-      <c r="K31" s="78" t="n">
-        <v>5</v>
-      </c>
-      <c r="L31" s="78" t="n">
-        <v>10</v>
-      </c>
-      <c r="M31" s="68" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="N31" s="76" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe G</t>
-        </is>
-      </c>
-      <c r="B32" s="67" t="inlineStr">
-        <is>
-          <t>Belgia</t>
-        </is>
-      </c>
-      <c r="C32" s="84" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="D32" s="69" t="n">
-        <v>15</v>
-      </c>
-      <c r="E32" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="F32" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="G32" s="71" t="n">
-        <v>5</v>
-      </c>
       <c r="H32" s="72" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>5–1</t>
         </is>
       </c>
       <c r="I32" s="73" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="J32" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="K32" s="69" t="n">
-        <v>4</v>
+      <c r="K32" s="70" t="n">
+        <v>2</v>
       </c>
       <c r="L32" s="70" t="n">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="M32" s="84" t="n">
-        <v>0.47</v>
+        <v>0.51</v>
       </c>
       <c r="N32" s="67" t="inlineStr">
         <is>
-          <t>Egypt</t>
+          <t>Tunisia</t>
         </is>
       </c>
     </row>
@@ -49587,95 +49583,99 @@
       <c r="A33" s="75" t="inlineStr"/>
       <c r="B33" s="76" t="inlineStr">
         <is>
+          <t>Tunisia</t>
+        </is>
+      </c>
+      <c r="C33" s="74" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D33" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E33" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H33" s="80" t="inlineStr">
+        <is>
+          <t>0–4</t>
+        </is>
+      </c>
+      <c r="I33" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J33" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K33" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="L33" s="78" t="n">
+        <v>10</v>
+      </c>
+      <c r="M33" s="68" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="N33" s="76" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe G</t>
+        </is>
+      </c>
+      <c r="B34" s="67" t="inlineStr">
+        <is>
           <t>Belgia</t>
         </is>
       </c>
-      <c r="C33" s="83" t="n">
-        <v>0.68</v>
-      </c>
-      <c r="D33" s="78" t="n">
-        <v>22</v>
-      </c>
-      <c r="E33" s="78" t="n">
+      <c r="C34" s="84" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="D34" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="E34" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F34" s="70" t="n">
         <v>7</v>
-      </c>
-      <c r="F33" s="77" t="n">
-        <v>8</v>
-      </c>
-      <c r="G33" s="79" t="n">
-        <v>6</v>
-      </c>
-      <c r="H33" s="80" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I33" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K33" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="L33" s="77" t="n">
-        <v>7</v>
-      </c>
-      <c r="M33" s="74" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="N33" s="76" t="inlineStr">
-        <is>
-          <t>Iran</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="82" t="inlineStr"/>
-      <c r="B34" s="67" t="inlineStr">
-        <is>
-          <t>Iran</t>
-        </is>
-      </c>
-      <c r="C34" s="84" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D34" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="E34" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="F34" s="70" t="n">
-        <v>8</v>
       </c>
       <c r="G34" s="71" t="n">
         <v>5</v>
       </c>
       <c r="H34" s="72" t="inlineStr">
         <is>
-          <t>2–2</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I34" s="73" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="J34" s="70" t="n">
         <v>2</v>
       </c>
       <c r="K34" s="69" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="L34" s="70" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="M34" s="84" t="n">
-        <v>0.53</v>
+        <v>0.47</v>
       </c>
       <c r="N34" s="67" t="inlineStr">
         <is>
-          <t>New Zealand</t>
+          <t>Egypt</t>
         </is>
       </c>
     </row>
@@ -49683,99 +49683,95 @@
       <c r="A35" s="75" t="inlineStr"/>
       <c r="B35" s="76" t="inlineStr">
         <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="C35" s="83" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="D35" s="78" t="n">
+        <v>22</v>
+      </c>
+      <c r="E35" s="78" t="n">
+        <v>7</v>
+      </c>
+      <c r="F35" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="G35" s="79" t="n">
+        <v>6</v>
+      </c>
+      <c r="H35" s="80" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I35" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K35" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="L35" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="M35" s="74" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="N35" s="76" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="82" t="inlineStr"/>
+      <c r="B36" s="67" t="inlineStr">
+        <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C36" s="84" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D36" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="E36" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="F36" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="G36" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H36" s="72" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I36" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J36" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="K36" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="L36" s="70" t="n">
+        <v>13</v>
+      </c>
+      <c r="M36" s="84" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N36" s="67" t="inlineStr">
+        <is>
           <t>New Zealand</t>
-        </is>
-      </c>
-      <c r="C35" s="74" t="n">
-        <v>0.44</v>
-      </c>
-      <c r="D35" s="77" t="n">
-        <v>10</v>
-      </c>
-      <c r="E35" s="77" t="n">
-        <v>5</v>
-      </c>
-      <c r="F35" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="G35" s="79" t="n">
-        <v>3</v>
-      </c>
-      <c r="H35" s="80" t="inlineStr">
-        <is>
-          <t>1–3</t>
-        </is>
-      </c>
-      <c r="I35" s="81" t="n">
-        <v>6</v>
-      </c>
-      <c r="J35" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="K35" s="78" t="n">
-        <v>7</v>
-      </c>
-      <c r="L35" s="78" t="n">
-        <v>19</v>
-      </c>
-      <c r="M35" s="68" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="N35" s="76" t="inlineStr">
-        <is>
-          <t>Egypt</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe H</t>
-        </is>
-      </c>
-      <c r="B36" s="67" t="inlineStr">
-        <is>
-          <t>Saudi-Arabia</t>
-        </is>
-      </c>
-      <c r="C36" s="74" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D36" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="E36" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="F36" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="G36" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H36" s="72" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I36" s="73" t="n">
-        <v>9</v>
-      </c>
-      <c r="J36" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="K36" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="L36" s="69" t="n">
-        <v>27</v>
-      </c>
-      <c r="M36" s="83" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="N36" s="67" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
         </is>
       </c>
     </row>
@@ -49783,95 +49779,99 @@
       <c r="A37" s="75" t="inlineStr"/>
       <c r="B37" s="76" t="inlineStr">
         <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C37" s="83" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="D37" s="78" t="n">
-        <v>23</v>
-      </c>
-      <c r="E37" s="78" t="n">
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C37" s="74" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="D37" s="77" t="n">
+        <v>10</v>
+      </c>
+      <c r="E37" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="F37" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" s="79" t="n">
+        <v>3</v>
+      </c>
+      <c r="H37" s="80" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I37" s="81" t="n">
+        <v>6</v>
+      </c>
+      <c r="J37" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="K37" s="78" t="n">
+        <v>7</v>
+      </c>
+      <c r="L37" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="M37" s="68" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="N37" s="76" t="inlineStr">
+        <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="B38" s="67" t="inlineStr">
+        <is>
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="C38" s="74" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D38" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="E38" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F38" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G38" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="72" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I38" s="73" t="n">
+        <v>9</v>
+      </c>
+      <c r="J38" s="70" t="n">
         <v>8</v>
       </c>
-      <c r="F37" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="G37" s="79" t="n">
-        <v>6</v>
-      </c>
-      <c r="H37" s="80" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I37" s="81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J37" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K37" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L37" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="M37" s="74" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="N37" s="76" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="82" t="inlineStr"/>
-      <c r="B38" s="67" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C38" s="83" t="n">
+      <c r="K38" s="69" t="n">
+        <v>10</v>
+      </c>
+      <c r="L38" s="69" t="n">
+        <v>27</v>
+      </c>
+      <c r="M38" s="83" t="n">
         <v>0.65</v>
       </c>
-      <c r="D38" s="69" t="n">
-        <v>21</v>
-      </c>
-      <c r="E38" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="F38" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="G38" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H38" s="72" t="inlineStr">
-        <is>
-          <t>4–0</t>
-        </is>
-      </c>
-      <c r="I38" s="73" t="n">
-        <v>1</v>
-      </c>
-      <c r="J38" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="K38" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="L38" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="M38" s="74" t="n">
-        <v>0.35</v>
-      </c>
       <c r="N38" s="67" t="inlineStr">
         <is>
-          <t>Saudi-Arabia</t>
+          <t>Uruguay</t>
         </is>
       </c>
     </row>
@@ -49879,43 +49879,43 @@
       <c r="A39" s="75" t="inlineStr"/>
       <c r="B39" s="76" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>Spania</t>
         </is>
       </c>
       <c r="C39" s="83" t="n">
-        <v>0.66</v>
+        <v>0.74</v>
       </c>
       <c r="D39" s="78" t="n">
-        <v>16</v>
-      </c>
-      <c r="E39" s="77" t="n">
+        <v>23</v>
+      </c>
+      <c r="E39" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="F39" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G39" s="79" t="n">
+        <v>6</v>
+      </c>
+      <c r="H39" s="80" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I39" s="81" t="n">
         <v>2</v>
-      </c>
-      <c r="F39" s="77" t="n">
-        <v>7</v>
-      </c>
-      <c r="G39" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H39" s="80" t="inlineStr">
-        <is>
-          <t>2–2</t>
-        </is>
-      </c>
-      <c r="I39" s="81" t="n">
-        <v>4</v>
       </c>
       <c r="J39" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="K39" s="78" t="n">
-        <v>4</v>
+      <c r="K39" s="77" t="n">
+        <v>1</v>
       </c>
       <c r="L39" s="77" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="M39" s="74" t="n">
-        <v>0.34</v>
+        <v>0.26</v>
       </c>
       <c r="N39" s="76" t="inlineStr">
         <is>
@@ -49924,54 +49924,50 @@
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe I</t>
-        </is>
-      </c>
+      <c r="A40" s="82" t="inlineStr"/>
       <c r="B40" s="67" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C40" s="84" t="n">
-        <v>0.54</v>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C40" s="83" t="n">
+        <v>0.65</v>
       </c>
       <c r="D40" s="69" t="n">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E40" s="69" t="n">
         <v>9</v>
       </c>
       <c r="F40" s="70" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="G40" s="71" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40" s="72" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>4–0</t>
         </is>
       </c>
       <c r="I40" s="73" t="n">
         <v>1</v>
       </c>
       <c r="J40" s="70" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K40" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="L40" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="L40" s="70" t="n">
-        <v>6</v>
-      </c>
-      <c r="M40" s="84" t="n">
-        <v>0.46</v>
+      <c r="M40" s="74" t="n">
+        <v>0.35</v>
       </c>
       <c r="N40" s="67" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Saudi-Arabia</t>
         </is>
       </c>
     </row>
@@ -49979,95 +49975,99 @@
       <c r="A41" s="75" t="inlineStr"/>
       <c r="B41" s="76" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C41" s="68" t="n">
-        <v>0.5600000000000001</v>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="C41" s="83" t="n">
+        <v>0.66</v>
       </c>
       <c r="D41" s="78" t="n">
-        <v>19</v>
-      </c>
-      <c r="E41" s="78" t="n">
-        <v>5</v>
+        <v>16</v>
+      </c>
+      <c r="E41" s="77" t="n">
+        <v>2</v>
       </c>
       <c r="F41" s="77" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="G41" s="79" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H41" s="80" t="inlineStr">
         <is>
-          <t>3–0</t>
+          <t>2–2</t>
         </is>
       </c>
       <c r="I41" s="81" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J41" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="K41" s="77" t="n">
-        <v>0</v>
+      <c r="K41" s="78" t="n">
+        <v>4</v>
       </c>
       <c r="L41" s="77" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="M41" s="74" t="n">
-        <v>0.44</v>
+        <v>0.34</v>
       </c>
       <c r="N41" s="76" t="inlineStr">
         <is>
-          <t>Irak</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="82" t="inlineStr"/>
+      <c r="A42" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe I</t>
+        </is>
+      </c>
       <c r="B42" s="67" t="inlineStr">
         <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="C42" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D42" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="E42" s="70" t="n">
-        <v>1</v>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C42" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D42" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="E42" s="69" t="n">
+        <v>9</v>
       </c>
       <c r="F42" s="70" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G42" s="71" t="n">
         <v>2</v>
       </c>
       <c r="H42" s="72" t="inlineStr">
         <is>
-          <t>1–4</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I42" s="73" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="J42" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="K42" s="69" t="n">
+      <c r="K42" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L42" s="70" t="n">
         <v>6</v>
       </c>
-      <c r="L42" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="M42" s="68" t="n">
-        <v>0.63</v>
+      <c r="M42" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N42" s="67" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -50075,99 +50075,95 @@
       <c r="A43" s="75" t="inlineStr"/>
       <c r="B43" s="76" t="inlineStr">
         <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C43" s="68" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="D43" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="E43" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="F43" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G43" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" s="80" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="I43" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J43" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K43" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L43" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="M43" s="74" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="N43" s="76" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="82" t="inlineStr"/>
+      <c r="B44" s="67" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="C44" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D44" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="E44" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F44" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="G44" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H44" s="72" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="I44" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J44" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="K44" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="L44" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="M44" s="68" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N44" s="67" t="inlineStr">
+        <is>
           <t>Norge</t>
-        </is>
-      </c>
-      <c r="C43" s="74" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="D43" s="77" t="n">
-        <v>12</v>
-      </c>
-      <c r="E43" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="F43" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="G43" s="79" t="n">
-        <v>4</v>
-      </c>
-      <c r="H43" s="80" t="inlineStr">
-        <is>
-          <t>3–2</t>
-        </is>
-      </c>
-      <c r="I43" s="81" t="n">
-        <v>5</v>
-      </c>
-      <c r="J43" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="K43" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="L43" s="78" t="n">
-        <v>17</v>
-      </c>
-      <c r="M43" s="68" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="N43" s="76" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe J</t>
-        </is>
-      </c>
-      <c r="B44" s="67" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C44" s="84" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D44" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="E44" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="F44" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="G44" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H44" s="72" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I44" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J44" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="K44" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="L44" s="70" t="n">
-        <v>6</v>
-      </c>
-      <c r="M44" s="84" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N44" s="67" t="inlineStr">
-        <is>
-          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -50175,91 +50171,95 @@
       <c r="A45" s="75" t="inlineStr"/>
       <c r="B45" s="76" t="inlineStr">
         <is>
+          <t>Norge</t>
+        </is>
+      </c>
+      <c r="C45" s="74" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D45" s="77" t="n">
+        <v>12</v>
+      </c>
+      <c r="E45" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="F45" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G45" s="79" t="n">
+        <v>4</v>
+      </c>
+      <c r="H45" s="80" t="inlineStr">
+        <is>
+          <t>3–2</t>
+        </is>
+      </c>
+      <c r="I45" s="81" t="n">
+        <v>5</v>
+      </c>
+      <c r="J45" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="K45" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="L45" s="78" t="n">
+        <v>17</v>
+      </c>
+      <c r="M45" s="68" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="N45" s="76" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe J</t>
+        </is>
+      </c>
+      <c r="B46" s="67" t="inlineStr">
+        <is>
           <t>Argentina</t>
         </is>
       </c>
-      <c r="C45" s="84" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D45" s="78" t="n">
-        <v>12</v>
-      </c>
-      <c r="E45" s="78" t="n">
+      <c r="C46" s="84" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D46" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="E46" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="F46" s="70" t="n">
         <v>3</v>
-      </c>
-      <c r="F45" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="G45" s="79" t="n">
-        <v>5</v>
-      </c>
-      <c r="H45" s="80" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I45" s="81" t="n">
-        <v>3</v>
-      </c>
-      <c r="J45" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="K45" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L45" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="M45" s="84" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="N45" s="76" t="inlineStr">
-        <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="82" t="inlineStr"/>
-      <c r="B46" s="67" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-      <c r="C46" s="74" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="D46" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="E46" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="F46" s="70" t="n">
-        <v>4</v>
       </c>
       <c r="G46" s="71" t="n">
         <v>0</v>
       </c>
       <c r="H46" s="72" t="inlineStr">
         <is>
-          <t>1–2</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I46" s="73" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="J46" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="K46" s="69" t="n">
-        <v>8</v>
-      </c>
-      <c r="L46" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="M46" s="83" t="n">
-        <v>0.75</v>
+      <c r="K46" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="L46" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="M46" s="84" t="n">
+        <v>0.53</v>
       </c>
       <c r="N46" s="67" t="inlineStr">
         <is>
@@ -50271,99 +50271,95 @@
       <c r="A47" s="75" t="inlineStr"/>
       <c r="B47" s="76" t="inlineStr">
         <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C47" s="68" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D47" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="E47" s="77" t="n">
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C47" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D47" s="78" t="n">
+        <v>12</v>
+      </c>
+      <c r="E47" s="78" t="n">
         <v>3</v>
       </c>
       <c r="F47" s="77" t="n">
         <v>4</v>
       </c>
       <c r="G47" s="79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H47" s="80" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I47" s="81" t="n">
         <v>3</v>
       </c>
       <c r="J47" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K47" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L47" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="M47" s="84" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N47" s="76" t="inlineStr">
+        <is>
+          <t>Østerrike</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="82" t="inlineStr"/>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C48" s="74" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D48" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E48" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="K47" s="78" t="n">
+      <c r="F48" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="L47" s="78" t="n">
-        <v>11</v>
-      </c>
-      <c r="M47" s="74" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="N47" s="76" t="inlineStr">
-        <is>
-          <t>Jordan</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe K</t>
-        </is>
-      </c>
-      <c r="B48" s="67" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="C48" s="83" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D48" s="69" t="n">
-        <v>20</v>
-      </c>
-      <c r="E48" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="F48" s="70" t="n">
-        <v>5</v>
-      </c>
       <c r="G48" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="72" t="inlineStr">
+        <is>
+          <t>1–2</t>
+        </is>
+      </c>
+      <c r="I48" s="73" t="n">
         <v>6</v>
-      </c>
-      <c r="H48" s="72" t="inlineStr">
-        <is>
-          <t>1–0</t>
-        </is>
-      </c>
-      <c r="I48" s="73" t="n">
-        <v>2</v>
       </c>
       <c r="J48" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="K48" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L48" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="M48" s="74" t="n">
-        <v>0.34</v>
+      <c r="K48" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="L48" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="M48" s="83" t="n">
+        <v>0.75</v>
       </c>
       <c r="N48" s="67" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -50371,16 +50367,16 @@
       <c r="A49" s="75" t="inlineStr"/>
       <c r="B49" s="76" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C49" s="83" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D49" s="78" t="n">
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C49" s="68" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D49" s="77" t="n">
         <v>9</v>
       </c>
-      <c r="E49" s="78" t="n">
+      <c r="E49" s="77" t="n">
         <v>3</v>
       </c>
       <c r="F49" s="77" t="n">
@@ -50391,62 +50387,66 @@
       </c>
       <c r="H49" s="80" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I49" s="81" t="n">
         <v>3</v>
       </c>
       <c r="J49" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K49" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="L49" s="77" t="n">
-        <v>8</v>
+        <v>4</v>
+      </c>
+      <c r="K49" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="L49" s="78" t="n">
+        <v>11</v>
       </c>
       <c r="M49" s="74" t="n">
-        <v>0.25</v>
+        <v>0.38</v>
       </c>
       <c r="N49" s="76" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Jordan</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="82" t="inlineStr"/>
+      <c r="A50" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe K</t>
+        </is>
+      </c>
       <c r="B50" s="67" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="C50" s="83" t="n">
         <v>0.66</v>
       </c>
       <c r="D50" s="69" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E50" s="69" t="n">
         <v>9</v>
       </c>
       <c r="F50" s="70" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G50" s="71" t="n">
+        <v>6</v>
+      </c>
+      <c r="H50" s="72" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I50" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J50" s="70" t="n">
         <v>3</v>
-      </c>
-      <c r="H50" s="72" t="inlineStr">
-        <is>
-          <t>5–0</t>
-        </is>
-      </c>
-      <c r="I50" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J50" s="70" t="n">
-        <v>2</v>
       </c>
       <c r="K50" s="70" t="n">
         <v>2</v>
@@ -50459,7 +50459,7 @@
       </c>
       <c r="N50" s="67" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -50467,99 +50467,95 @@
       <c r="A51" s="75" t="inlineStr"/>
       <c r="B51" s="76" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C51" s="74" t="n">
-        <v>0.33</v>
-      </c>
-      <c r="D51" s="77" t="n">
-        <v>7</v>
-      </c>
-      <c r="E51" s="77" t="n">
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C51" s="83" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D51" s="78" t="n">
+        <v>9</v>
+      </c>
+      <c r="E51" s="78" t="n">
         <v>3</v>
       </c>
       <c r="F51" s="77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G51" s="79" t="n">
         <v>2</v>
       </c>
       <c r="H51" s="80" t="inlineStr">
         <is>
-          <t>1–3</t>
+          <t>1–1</t>
         </is>
       </c>
       <c r="I51" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J51" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L51" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="M51" s="74" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="N51" s="76" t="inlineStr">
+        <is>
+          <t>DR Kongo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="82" t="inlineStr"/>
+      <c r="B52" s="67" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C52" s="83" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D52" s="69" t="n">
+        <v>16</v>
+      </c>
+      <c r="E52" s="69" t="n">
+        <v>9</v>
+      </c>
+      <c r="F52" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="J51" s="77" t="n">
-        <v>5</v>
-      </c>
-      <c r="K51" s="78" t="n">
-        <v>6</v>
-      </c>
-      <c r="L51" s="78" t="n">
-        <v>15</v>
-      </c>
-      <c r="M51" s="83" t="n">
-        <v>0.67</v>
-      </c>
-      <c r="N51" s="76" t="inlineStr">
-        <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe L</t>
-        </is>
-      </c>
-      <c r="B52" s="67" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C52" s="84" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D52" s="69" t="n">
-        <v>20</v>
-      </c>
-      <c r="E52" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="F52" s="70" t="n">
+      <c r="G52" s="71" t="n">
         <v>3</v>
       </c>
-      <c r="G52" s="71" t="n">
-        <v>5</v>
-      </c>
       <c r="H52" s="72" t="inlineStr">
         <is>
-          <t>4–2</t>
+          <t>5–0</t>
         </is>
       </c>
       <c r="I52" s="73" t="n">
         <v>3</v>
       </c>
       <c r="J52" s="70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K52" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L52" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="M52" s="84" t="n">
-        <v>0.46</v>
+        <v>7</v>
+      </c>
+      <c r="M52" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N52" s="67" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>Usbekistan</t>
         </is>
       </c>
     </row>
@@ -50567,95 +50563,99 @@
       <c r="A53" s="75" t="inlineStr"/>
       <c r="B53" s="76" t="inlineStr">
         <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="C53" s="74" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="D53" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="E53" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F53" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G53" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H53" s="80" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I53" s="81" t="n">
+        <v>4</v>
+      </c>
+      <c r="J53" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="K53" s="78" t="n">
+        <v>6</v>
+      </c>
+      <c r="L53" s="78" t="n">
+        <v>15</v>
+      </c>
+      <c r="M53" s="83" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N53" s="76" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="B54" s="67" t="inlineStr">
+        <is>
           <t>England</t>
         </is>
       </c>
-      <c r="C53" s="83" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="D53" s="78" t="n">
-        <v>19</v>
-      </c>
-      <c r="E53" s="78" t="n">
-        <v>4</v>
-      </c>
-      <c r="F53" s="77" t="n">
-        <v>8</v>
-      </c>
-      <c r="G53" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H53" s="80" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I53" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J53" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L53" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="M53" s="74" t="n">
-        <v>0.22</v>
-      </c>
-      <c r="N53" s="76" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="82" t="inlineStr"/>
-      <c r="B54" s="67" t="inlineStr">
-        <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="C54" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D54" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="E54" s="70" t="n">
+      <c r="C54" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D54" s="69" t="n">
+        <v>20</v>
+      </c>
+      <c r="E54" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="F54" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="F54" s="70" t="n">
-        <v>4</v>
-      </c>
       <c r="G54" s="71" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H54" s="72" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>4–2</t>
         </is>
       </c>
       <c r="I54" s="73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J54" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K54" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="K54" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L54" s="69" t="n">
+      <c r="L54" s="70" t="n">
         <v>11</v>
       </c>
-      <c r="M54" s="68" t="n">
-        <v>0.63</v>
+      <c r="M54" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N54" s="67" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Kroatia</t>
         </is>
       </c>
     </row>
@@ -50663,79 +50663,175 @@
       <c r="A55" s="75" t="inlineStr"/>
       <c r="B55" s="76" t="inlineStr">
         <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C55" s="83" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D55" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="E55" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="F55" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="G55" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="H55" s="80" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I55" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J55" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K55" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L55" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="M55" s="74" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N55" s="76" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="82" t="inlineStr"/>
+      <c r="B56" s="67" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C56" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D56" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E56" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G56" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H56" s="72" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I56" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J56" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K56" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="L56" s="69" t="n">
+        <v>11</v>
+      </c>
+      <c r="M56" s="68" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N56" s="67" t="inlineStr">
+        <is>
           <t>Panama</t>
         </is>
       </c>
-      <c r="C55" s="74" t="n">
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="75" t="inlineStr"/>
+      <c r="B57" s="76" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C57" s="74" t="n">
         <v>0.42</v>
       </c>
-      <c r="D55" s="78" t="n">
+      <c r="D57" s="78" t="n">
         <v>8</v>
       </c>
-      <c r="E55" s="77" t="n">
+      <c r="E57" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="F55" s="77" t="n">
+      <c r="F57" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="G55" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H55" s="80" t="inlineStr">
+      <c r="G57" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" s="80" t="inlineStr">
         <is>
           <t>0–1</t>
         </is>
       </c>
-      <c r="I55" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J55" s="77" t="n">
+      <c r="I57" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J57" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="K55" s="77" t="n">
+      <c r="K57" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="L55" s="77" t="n">
+      <c r="L57" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="M55" s="68" t="n">
+      <c r="M57" s="68" t="n">
         <v>0.58</v>
       </c>
-      <c r="N55" s="76" t="inlineStr">
+      <c r="N57" s="76" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="14" customHeight="1">
-      <c r="A57" s="63" t="inlineStr">
+    <row r="59" ht="14" customHeight="1">
+      <c r="A59" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="55" t="inlineStr">
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B58" s="62" t="inlineStr">
+      <c r="B60" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C58" s="61" t="inlineStr">
+      <c r="C60" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D58" s="58" t="inlineStr">
+      <c r="D60" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E58" s="85" t="inlineStr">
+      <c r="E60" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -50743,8 +50839,8 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A59:N59"/>
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A57:N57"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-26 09:44 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -17953,7 +17953,11 @@
       </c>
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr"/>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>Joao Pinheiro</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Flytt P-kolonnen til mellom Lag og K i gruppe-tabellene (A-L)
Ny kolonnerekke: Lag, P, K, V, U, T, MF, MM, MD

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1644,42 +1644,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -1689,31 +1689,31 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>3</v>
+      <c r="B12" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -1722,12 +1722,12 @@
           <t>Sør-Afrika</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
@@ -1735,18 +1735,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -1755,31 +1755,31 @@
           <t>Sør-Korea</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -1788,33 +1788,34 @@
           <t>Tsjekkia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -5798,42 +5799,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -5843,31 +5844,31 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>2</v>
+      <c r="B12" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -5876,31 +5877,31 @@
           <t>Østerrike</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" s="18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -5909,31 +5910,31 @@
           <t>Algerie</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -5942,33 +5943,34 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -9922,42 +9924,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -9967,31 +9969,31 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>2</v>
+      <c r="B12" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -10000,31 +10002,31 @@
           <t>Portugal</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="G13" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -10033,15 +10035,15 @@
           <t>DR Kongo</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="E14" s="4" t="n">
         <v>1</v>
       </c>
@@ -10049,15 +10051,15 @@
         <v>1</v>
       </c>
       <c r="G14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -10066,33 +10068,34 @@
           <t>Usbekistan</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -14062,42 +14065,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -14107,31 +14110,31 @@
           <t>England</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -14140,31 +14143,31 @@
           <t>Ghana</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="G13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -14173,31 +14176,31 @@
           <t>Kroatia</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -14206,33 +14209,34 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -21554,42 +21558,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -21599,31 +21603,31 @@
           <t>Sveits</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -21632,12 +21636,12 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
@@ -21645,18 +21649,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -21665,12 +21669,12 @@
           <t>Bosnia-Hercegovina</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -21678,18 +21682,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -21698,33 +21702,34 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -55289,42 +55294,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -55334,31 +55339,31 @@
           <t>Brasil</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -55367,31 +55372,31 @@
           <t>Marokko</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="D13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -55400,31 +55405,31 @@
           <t>Skottland</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -55433,33 +55438,34 @@
           <t>Haiti</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -59473,42 +59479,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -59518,31 +59524,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -59551,12 +59557,12 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
@@ -59564,18 +59570,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -59584,12 +59590,12 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -59597,18 +59603,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -59617,33 +59623,34 @@
           <t>Tyrkia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -63671,42 +63678,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -63716,31 +63723,31 @@
           <t>Tyskland</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -63749,31 +63756,31 @@
           <t>Elfenbenskysten</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="D13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -63782,12 +63789,12 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -63795,18 +63802,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -63815,33 +63822,34 @@
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -67861,42 +67869,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -67906,31 +67914,31 @@
           <t>Nederland</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -67939,31 +67947,31 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -67972,12 +67980,12 @@
           <t>Sverige</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -67985,18 +67993,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -68005,33 +68013,34 @@
           <t>Tunisia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -72039,42 +72048,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -72084,31 +72093,31 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -72117,31 +72126,31 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>2</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -72150,31 +72159,31 @@
           <t>Belgia</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -72183,33 +72192,34 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -76177,42 +76187,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -76222,31 +76232,31 @@
           <t>Spania</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -76255,31 +76265,31 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>3</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -76288,31 +76298,31 @@
           <t>Kapp Verde</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -76321,15 +76331,15 @@
           <t>Saudi-Arabia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
       </c>
@@ -76337,17 +76347,18 @@
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -80299,42 +80310,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -80344,31 +80355,31 @@
           <t>Frankrike</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>2</v>
+      <c r="B12" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -80377,31 +80388,31 @@
           <t>Norge</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
-        <v>2</v>
+      <c r="B13" s="19" t="n">
+        <v>6</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -80410,31 +80421,31 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -80443,33 +80454,34 @@
           <t>Irak</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Flytt P-kolonnen til mellom Lag og K i gruppe-tabellene (A-L) (#79)
Ny kolonnerekke: Lag, P, K, V, U, T, MF, MM, MD

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1644,42 +1644,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -1689,31 +1689,31 @@
           <t>Mexico</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>3</v>
+      <c r="B12" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -1722,12 +1722,12 @@
           <t>Sør-Afrika</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
@@ -1735,18 +1735,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -1755,31 +1755,31 @@
           <t>Sør-Korea</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="E14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -1788,33 +1788,34 @@
           <t>Tsjekkia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -5798,42 +5799,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -5843,31 +5844,31 @@
           <t>Argentina</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>2</v>
+      <c r="B12" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -5876,31 +5877,31 @@
           <t>Østerrike</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" s="18" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -5909,31 +5910,31 @@
           <t>Algerie</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -5942,33 +5943,34 @@
           <t>Jordan</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -9922,42 +9924,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -9967,31 +9969,31 @@
           <t>Colombia</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>2</v>
+      <c r="B12" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -10000,31 +10002,31 @@
           <t>Portugal</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="G13" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -10033,15 +10035,15 @@
           <t>DR Kongo</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="E14" s="4" t="n">
         <v>1</v>
       </c>
@@ -10049,15 +10051,15 @@
         <v>1</v>
       </c>
       <c r="G14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -10066,33 +10068,34 @@
           <t>Usbekistan</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-7</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -14062,42 +14065,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -14107,31 +14110,31 @@
           <t>England</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -14140,31 +14143,31 @@
           <t>Ghana</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="G13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="H13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -14173,31 +14176,31 @@
           <t>Kroatia</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -14206,33 +14209,34 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -21558,42 +21562,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -21603,31 +21607,31 @@
           <t>Sveits</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -21636,12 +21640,12 @@
           <t>Canada</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
@@ -21649,18 +21653,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -21669,12 +21673,12 @@
           <t>Bosnia-Hercegovina</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -21682,18 +21686,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>5</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -21702,33 +21706,34 @@
           <t>Qatar</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -55293,42 +55298,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -55338,31 +55343,31 @@
           <t>Brasil</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -55371,31 +55376,31 @@
           <t>Marokko</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>7</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="D13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="E13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+3</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -55404,31 +55409,31 @@
           <t>Skottland</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -55437,33 +55442,34 @@
           <t>Haiti</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -59477,42 +59483,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -59522,31 +59528,31 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>8</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -59555,12 +59561,12 @@
           <t>Australia</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>4</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
         <v>1</v>
       </c>
@@ -59568,18 +59574,18 @@
         <v>1</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -59588,12 +59594,12 @@
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -59601,18 +59607,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -59621,33 +59627,34 @@
           <t>Tyrkia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
         <v>3</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>3</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -63675,42 +63682,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -63720,31 +63727,31 @@
           <t>Tyskland</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
+      <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="F12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -63753,31 +63760,31 @@
           <t>Elfenbenskysten</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="D13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -63786,12 +63793,12 @@
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -63799,18 +63806,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -63819,33 +63826,34 @@
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-8</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -67865,42 +67873,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -67910,31 +67918,31 @@
           <t>Nederland</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+6</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -67943,31 +67951,31 @@
           <t>Japan</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -67976,12 +67984,12 @@
           <t>Sverige</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="D14" s="4" t="n">
         <v>1</v>
       </c>
@@ -67989,18 +67997,18 @@
         <v>1</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -68009,33 +68017,34 @@
           <t>Tunisia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-10</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -72043,42 +72052,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -72088,31 +72097,31 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -72121,31 +72130,31 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>2</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -72154,31 +72163,31 @@
           <t>Belgia</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="G14" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -72187,33 +72196,34 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="F15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-2</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -76181,42 +76191,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -76226,31 +76236,31 @@
           <t>Spania</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
         <v>1</v>
       </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -76259,31 +76269,31 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>2</v>
       </c>
       <c r="C13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>3</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -76292,31 +76302,31 @@
           <t>Kapp Verde</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>2</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>2</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -76325,15 +76335,15 @@
           <t>Saudi-Arabia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
         <v>1</v>
       </c>
@@ -76341,17 +76351,18 @@
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -80303,42 +80314,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -80348,31 +80359,31 @@
           <t>Frankrike</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>2</v>
+      <c r="B12" s="13" t="n">
+        <v>6</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>2</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="H12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -80381,31 +80392,31 @@
           <t>Norge</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
-        <v>2</v>
+      <c r="B13" s="19" t="n">
+        <v>6</v>
       </c>
       <c r="C13" s="18" t="n">
         <v>2</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F13" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -80414,31 +80425,31 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="C14" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-3</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -80447,33 +80458,34 @@
           <t>Irak</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>2</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
       </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
-      </c>
-    </row>
+    </row>
+    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-26 15:41 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1815,7 +1815,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -5970,7 +5969,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -10095,7 +10093,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -14236,7 +14233,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -21733,7 +21729,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -55469,7 +55464,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -59654,7 +59648,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -63853,7 +63846,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -68044,7 +68036,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -72223,7 +72214,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -76362,7 +76352,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>
@@ -80485,7 +80474,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="24" customHeight="1">
       <c r="A17" s="10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-26 15:54 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Scorere og assists" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-27 07:06 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -43481,7 +43481,7 @@
       </c>
       <c r="D108" s="24" t="inlineStr">
         <is>
-          <t>MAHMOUD ABUNADA</t>
+          <t>Mahmoud Abunada</t>
         </is>
       </c>
       <c r="E108" s="24" t="inlineStr">
@@ -43511,7 +43511,7 @@
       </c>
       <c r="D109" s="24" t="inlineStr">
         <is>
-          <t>MOHAMED MANAI</t>
+          <t>Mohamed Manai</t>
         </is>
       </c>
       <c r="E109" s="24" t="inlineStr">
@@ -43541,7 +43541,7 @@
       </c>
       <c r="D110" s="29" t="inlineStr">
         <is>
-          <t>Cameron BURGESS</t>
+          <t>Cameron Burgess</t>
         </is>
       </c>
       <c r="E110" s="29" t="inlineStr">
@@ -43571,7 +43571,7 @@
       </c>
       <c r="D111" s="32" t="inlineStr">
         <is>
-          <t>MOHAMED HANY</t>
+          <t>Mohamed Hany</t>
         </is>
       </c>
       <c r="E111" s="32" t="inlineStr">
@@ -43601,7 +43601,7 @@
       </c>
       <c r="D112" s="5" t="inlineStr">
         <is>
-          <t>AYMEN HUSSEIN</t>
+          <t>Aymen Hussein</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
@@ -43631,7 +43631,7 @@
       </c>
       <c r="D113" s="8" t="inlineStr">
         <is>
-          <t>YAZAN ALARAB</t>
+          <t>Yazan Alarab</t>
         </is>
       </c>
       <c r="E113" s="8" t="inlineStr">
@@ -43661,7 +43661,7 @@
       </c>
       <c r="D114" s="5" t="inlineStr">
         <is>
-          <t>Yassine BOUNOU</t>
+          <t>Yassine Bounou</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
@@ -43691,7 +43691,7 @@
       </c>
       <c r="D115" s="8" t="inlineStr">
         <is>
-          <t>Damian BOBADILLA</t>
+          <t>Damian Bobadilla</t>
         </is>
       </c>
       <c r="E115" s="8" t="inlineStr">
@@ -43721,7 +43721,7 @@
       </c>
       <c r="D116" s="5" t="inlineStr">
         <is>
-          <t>HASSAN ALTAMBAKTI</t>
+          <t>Hassan Altambakti</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
@@ -43751,7 +43751,7 @@
       </c>
       <c r="D117" s="8" t="inlineStr">
         <is>
-          <t>Miro MUHEIM</t>
+          <t>Miro Muheim</t>
         </is>
       </c>
       <c r="E117" s="8" t="inlineStr">
@@ -43781,7 +43781,7 @@
       </c>
       <c r="D118" s="5" t="inlineStr">
         <is>
-          <t>Ellyes SKHIRI</t>
+          <t>Ellyes Skhiri</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
@@ -43811,7 +43811,7 @@
       </c>
       <c r="D119" s="8" t="inlineStr">
         <is>
-          <t>Abduvohid NEMATOV</t>
+          <t>Abduvohid Nematov</t>
         </is>
       </c>
       <c r="E119" s="8" t="inlineStr">
@@ -55686,11 +55686,15 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="I59" s="92" t="n"/>
+      <c r="I59" s="92" t="n">
+        <v>70492</v>
+      </c>
       <c r="J59" s="93" t="n">
         <v>70240</v>
       </c>
-      <c r="K59" s="82" t="n"/>
+      <c r="K59" s="102" t="n">
+        <v>1.003587699316629</v>
+      </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="77" t="inlineStr">
@@ -56188,12 +56192,12 @@
     <row r="73" ht="18" customHeight="1">
       <c r="A73" s="108" t="inlineStr">
         <is>
-          <t>Totalt tilskuere: 4 152 659</t>
+          <t>Totalt tilskuere: 4 223 151</t>
         </is>
       </c>
       <c r="C73" s="108" t="inlineStr">
         <is>
-          <t>Snitt belegg: 95.5%</t>
+          <t>Snitt belegg: 95.6%</t>
         </is>
       </c>
       <c r="E73" s="108" t="inlineStr">

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-27 07:23 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -49522,7 +49522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N68"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -51490,47 +51490,47 @@
       <c r="A42" s="82" t="inlineStr"/>
       <c r="B42" s="67" t="inlineStr">
         <is>
+          <t>Egypt</t>
+        </is>
+      </c>
+      <c r="C42" s="68" t="n">
+        <v>0.62</v>
+      </c>
+      <c r="D42" s="69" t="n">
+        <v>14</v>
+      </c>
+      <c r="E42" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F42" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" s="71" t="n">
+        <v>6</v>
+      </c>
+      <c r="H42" s="72" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I42" s="73" t="n">
+        <v>5</v>
+      </c>
+      <c r="J42" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="K42" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L42" s="70" t="n">
+        <v>12</v>
+      </c>
+      <c r="M42" s="74" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="N42" s="67" t="inlineStr">
+        <is>
           <t>Iran</t>
-        </is>
-      </c>
-      <c r="C42" s="84" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D42" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="E42" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="F42" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="G42" s="71" t="n">
-        <v>5</v>
-      </c>
-      <c r="H42" s="72" t="inlineStr">
-        <is>
-          <t>2–2</t>
-        </is>
-      </c>
-      <c r="I42" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J42" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K42" s="69" t="n">
-        <v>8</v>
-      </c>
-      <c r="L42" s="70" t="n">
-        <v>13</v>
-      </c>
-      <c r="M42" s="84" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="N42" s="67" t="inlineStr">
-        <is>
-          <t>New Zealand</t>
         </is>
       </c>
     </row>
@@ -51538,99 +51538,95 @@
       <c r="A43" s="75" t="inlineStr"/>
       <c r="B43" s="76" t="inlineStr">
         <is>
+          <t>Iran</t>
+        </is>
+      </c>
+      <c r="C43" s="84" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="D43" s="78" t="n">
+        <v>17</v>
+      </c>
+      <c r="E43" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F43" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="G43" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="H43" s="80" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I43" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J43" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K43" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="L43" s="77" t="n">
+        <v>13</v>
+      </c>
+      <c r="M43" s="84" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="N43" s="76" t="inlineStr">
+        <is>
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="C43" s="74" t="n">
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="82" t="inlineStr"/>
+      <c r="B44" s="67" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C44" s="74" t="n">
         <v>0.44</v>
       </c>
-      <c r="D43" s="77" t="n">
+      <c r="D44" s="70" t="n">
         <v>10</v>
       </c>
-      <c r="E43" s="77" t="n">
+      <c r="E44" s="70" t="n">
         <v>5</v>
       </c>
-      <c r="F43" s="77" t="n">
+      <c r="F44" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="G43" s="79" t="n">
+      <c r="G44" s="71" t="n">
         <v>3</v>
       </c>
-      <c r="H43" s="80" t="inlineStr">
+      <c r="H44" s="72" t="inlineStr">
         <is>
           <t>1–3</t>
         </is>
       </c>
-      <c r="I43" s="81" t="n">
+      <c r="I44" s="73" t="n">
         <v>6</v>
       </c>
-      <c r="J43" s="77" t="n">
+      <c r="J44" s="70" t="n">
         <v>6</v>
       </c>
-      <c r="K43" s="78" t="n">
+      <c r="K44" s="69" t="n">
         <v>7</v>
       </c>
-      <c r="L43" s="78" t="n">
+      <c r="L44" s="69" t="n">
         <v>19</v>
       </c>
-      <c r="M43" s="68" t="n">
+      <c r="M44" s="68" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="N43" s="76" t="inlineStr">
+      <c r="N44" s="67" t="inlineStr">
         <is>
           <t>Egypt</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe H</t>
-        </is>
-      </c>
-      <c r="B44" s="67" t="inlineStr">
-        <is>
-          <t>Saudi-Arabia</t>
-        </is>
-      </c>
-      <c r="C44" s="74" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="D44" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="E44" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="F44" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="G44" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H44" s="72" t="inlineStr">
-        <is>
-          <t>1–1</t>
-        </is>
-      </c>
-      <c r="I44" s="73" t="n">
-        <v>9</v>
-      </c>
-      <c r="J44" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="K44" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="L44" s="69" t="n">
-        <v>27</v>
-      </c>
-      <c r="M44" s="83" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="N44" s="67" t="inlineStr">
-        <is>
-          <t>Uruguay</t>
         </is>
       </c>
     </row>
@@ -51638,91 +51634,95 @@
       <c r="A45" s="75" t="inlineStr"/>
       <c r="B45" s="76" t="inlineStr">
         <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C45" s="83" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="D45" s="78" t="n">
-        <v>23</v>
-      </c>
-      <c r="E45" s="78" t="n">
-        <v>8</v>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="C45" s="84" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D45" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="E45" s="77" t="n">
+        <v>2</v>
       </c>
       <c r="F45" s="77" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="G45" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H45" s="80" t="inlineStr">
+        <is>
+          <t>1–5</t>
+        </is>
+      </c>
+      <c r="I45" s="81" t="n">
+        <v>12</v>
+      </c>
+      <c r="J45" s="77" t="n">
+        <v>11</v>
+      </c>
+      <c r="K45" s="78" t="n">
+        <v>10</v>
+      </c>
+      <c r="L45" s="78" t="n">
+        <v>33</v>
+      </c>
+      <c r="M45" s="68" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="N45" s="76" t="inlineStr">
+        <is>
+          <t>Belgia</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe H</t>
+        </is>
+      </c>
+      <c r="B46" s="67" t="inlineStr">
+        <is>
+          <t>Kapp Verde</t>
+        </is>
+      </c>
+      <c r="C46" s="84" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="D46" s="69" t="n">
+        <v>15</v>
+      </c>
+      <c r="E46" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="G46" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H46" s="72" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I46" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J46" s="70" t="n">
+        <v>0</v>
+      </c>
+      <c r="K46" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L46" s="70" t="n">
         <v>6</v>
       </c>
-      <c r="H45" s="80" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I45" s="81" t="n">
-        <v>2</v>
-      </c>
-      <c r="J45" s="77" t="n">
-        <v>3</v>
-      </c>
-      <c r="K45" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L45" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="M45" s="74" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="N45" s="76" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="18" customHeight="1">
-      <c r="A46" s="82" t="inlineStr"/>
-      <c r="B46" s="67" t="inlineStr">
-        <is>
-          <t>Spania</t>
-        </is>
-      </c>
-      <c r="C46" s="83" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="D46" s="69" t="n">
-        <v>21</v>
-      </c>
-      <c r="E46" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="F46" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="G46" s="71" t="n">
-        <v>1</v>
-      </c>
-      <c r="H46" s="72" t="inlineStr">
-        <is>
-          <t>4–0</t>
-        </is>
-      </c>
-      <c r="I46" s="73" t="n">
-        <v>1</v>
-      </c>
-      <c r="J46" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="K46" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="L46" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="M46" s="74" t="n">
-        <v>0.35</v>
+      <c r="M46" s="84" t="n">
+        <v>0.49</v>
       </c>
       <c r="N46" s="67" t="inlineStr">
         <is>
@@ -51734,99 +51734,95 @@
       <c r="A47" s="75" t="inlineStr"/>
       <c r="B47" s="76" t="inlineStr">
         <is>
+          <t>Saudi-Arabia</t>
+        </is>
+      </c>
+      <c r="C47" s="74" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D47" s="77" t="n">
+        <v>7</v>
+      </c>
+      <c r="E47" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F47" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="G47" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H47" s="80" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I47" s="81" t="n">
+        <v>9</v>
+      </c>
+      <c r="J47" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="K47" s="78" t="n">
+        <v>10</v>
+      </c>
+      <c r="L47" s="78" t="n">
+        <v>27</v>
+      </c>
+      <c r="M47" s="83" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="N47" s="76" t="inlineStr">
+        <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="C47" s="83" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D47" s="78" t="n">
-        <v>16</v>
-      </c>
-      <c r="E47" s="77" t="n">
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="82" t="inlineStr"/>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C48" s="83" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="D48" s="69" t="n">
+        <v>23</v>
+      </c>
+      <c r="E48" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="F48" s="70" t="n">
+        <v>9</v>
+      </c>
+      <c r="G48" s="71" t="n">
+        <v>6</v>
+      </c>
+      <c r="H48" s="72" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I48" s="73" t="n">
         <v>2</v>
       </c>
-      <c r="F47" s="77" t="n">
-        <v>7</v>
-      </c>
-      <c r="G47" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H47" s="80" t="inlineStr">
-        <is>
-          <t>2–2</t>
-        </is>
-      </c>
-      <c r="I47" s="81" t="n">
-        <v>4</v>
-      </c>
-      <c r="J47" s="77" t="n">
+      <c r="J48" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="K47" s="78" t="n">
-        <v>4</v>
-      </c>
-      <c r="L47" s="77" t="n">
-        <v>11</v>
-      </c>
-      <c r="M47" s="74" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="N47" s="76" t="inlineStr">
-        <is>
-          <t>Kapp Verde</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe I</t>
-        </is>
-      </c>
-      <c r="B48" s="67" t="inlineStr">
-        <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C48" s="84" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D48" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="E48" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="F48" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="71" t="n">
-        <v>2</v>
-      </c>
-      <c r="H48" s="72" t="inlineStr">
-        <is>
-          <t>3–1</t>
-        </is>
-      </c>
-      <c r="I48" s="73" t="n">
-        <v>1</v>
-      </c>
-      <c r="J48" s="70" t="n">
-        <v>2</v>
-      </c>
       <c r="K48" s="70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L48" s="70" t="n">
         <v>6</v>
       </c>
-      <c r="M48" s="84" t="n">
-        <v>0.46</v>
+      <c r="M48" s="74" t="n">
+        <v>0.26</v>
       </c>
       <c r="N48" s="67" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
@@ -51834,47 +51830,47 @@
       <c r="A49" s="75" t="inlineStr"/>
       <c r="B49" s="76" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C49" s="68" t="n">
-        <v>0.5600000000000001</v>
+          <t>Spania</t>
+        </is>
+      </c>
+      <c r="C49" s="83" t="n">
+        <v>0.65</v>
       </c>
       <c r="D49" s="78" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E49" s="78" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="F49" s="77" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G49" s="79" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="H49" s="80" t="inlineStr">
         <is>
-          <t>3–0</t>
+          <t>4–0</t>
         </is>
       </c>
       <c r="I49" s="81" t="n">
         <v>1</v>
       </c>
       <c r="J49" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L49" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="K49" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="L49" s="77" t="n">
-        <v>4</v>
-      </c>
       <c r="M49" s="74" t="n">
-        <v>0.44</v>
+        <v>0.35</v>
       </c>
       <c r="N49" s="76" t="inlineStr">
         <is>
-          <t>Irak</t>
+          <t>Saudi-Arabia</t>
         </is>
       </c>
     </row>
@@ -51882,47 +51878,47 @@
       <c r="A50" s="82" t="inlineStr"/>
       <c r="B50" s="67" t="inlineStr">
         <is>
-          <t>Irak</t>
-        </is>
-      </c>
-      <c r="C50" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D50" s="70" t="n">
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="C50" s="83" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D50" s="69" t="n">
+        <v>16</v>
+      </c>
+      <c r="E50" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F50" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="G50" s="71" t="n">
+        <v>7</v>
+      </c>
+      <c r="H50" s="72" t="inlineStr">
+        <is>
+          <t>2–2</t>
+        </is>
+      </c>
+      <c r="I50" s="73" t="n">
+        <v>4</v>
+      </c>
+      <c r="J50" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K50" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="L50" s="70" t="n">
         <v>11</v>
       </c>
-      <c r="E50" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="F50" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="G50" s="71" t="n">
-        <v>2</v>
-      </c>
-      <c r="H50" s="72" t="inlineStr">
-        <is>
-          <t>1–4</t>
-        </is>
-      </c>
-      <c r="I50" s="73" t="n">
-        <v>2</v>
-      </c>
-      <c r="J50" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="K50" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="L50" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="M50" s="68" t="n">
-        <v>0.63</v>
+      <c r="M50" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N50" s="67" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Kapp Verde</t>
         </is>
       </c>
     </row>
@@ -51930,95 +51926,99 @@
       <c r="A51" s="75" t="inlineStr"/>
       <c r="B51" s="76" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="C51" s="74" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="D51" s="77" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D51" s="78" t="n">
+        <v>6</v>
+      </c>
+      <c r="E51" s="78" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="G51" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H51" s="80" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I51" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J51" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K51" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L51" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="M51" s="83" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="N51" s="76" t="inlineStr">
+        <is>
+          <t>Spania</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe I</t>
+        </is>
+      </c>
+      <c r="B52" s="67" t="inlineStr">
+        <is>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C52" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D52" s="69" t="n">
         <v>12</v>
       </c>
-      <c r="E51" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="F51" s="77" t="n">
-        <v>2</v>
-      </c>
-      <c r="G51" s="79" t="n">
-        <v>4</v>
-      </c>
-      <c r="H51" s="80" t="inlineStr">
-        <is>
-          <t>3–2</t>
-        </is>
-      </c>
-      <c r="I51" s="81" t="n">
-        <v>5</v>
-      </c>
-      <c r="J51" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="K51" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="L51" s="78" t="n">
-        <v>17</v>
-      </c>
-      <c r="M51" s="68" t="n">
-        <v>0.57</v>
-      </c>
-      <c r="N51" s="76" t="inlineStr">
-        <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="82" t="inlineStr"/>
-      <c r="B52" s="67" t="inlineStr">
-        <is>
-          <t>Norge</t>
-        </is>
-      </c>
-      <c r="C52" s="74" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="D52" s="70" t="n">
-        <v>10</v>
-      </c>
-      <c r="E52" s="70" t="n">
-        <v>5</v>
+      <c r="E52" s="69" t="n">
+        <v>9</v>
       </c>
       <c r="F52" s="70" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G52" s="71" t="n">
         <v>2</v>
       </c>
       <c r="H52" s="72" t="inlineStr">
         <is>
-          <t>1–4</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I52" s="73" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J52" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="K52" s="69" t="n">
-        <v>10</v>
-      </c>
-      <c r="L52" s="69" t="n">
-        <v>19</v>
-      </c>
-      <c r="M52" s="68" t="n">
-        <v>0.57</v>
+        <v>2</v>
+      </c>
+      <c r="K52" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L52" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="M52" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N52" s="67" t="inlineStr">
         <is>
-          <t>Frankrike</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -52026,99 +52026,95 @@
       <c r="A53" s="75" t="inlineStr"/>
       <c r="B53" s="76" t="inlineStr">
         <is>
-          <t>Senegal</t>
-        </is>
-      </c>
-      <c r="C53" s="83" t="n">
-        <v>0.6899999999999999</v>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C53" s="68" t="n">
+        <v>0.5600000000000001</v>
       </c>
       <c r="D53" s="78" t="n">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="E53" s="78" t="n">
+        <v>5</v>
+      </c>
+      <c r="F53" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G53" s="79" t="n">
+        <v>5</v>
+      </c>
+      <c r="H53" s="80" t="inlineStr">
+        <is>
+          <t>3–0</t>
+        </is>
+      </c>
+      <c r="I53" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J53" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K53" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="M53" s="74" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="N53" s="76" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="82" t="inlineStr"/>
+      <c r="B54" s="67" t="inlineStr">
+        <is>
+          <t>Irak</t>
+        </is>
+      </c>
+      <c r="C54" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D54" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="E54" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="G54" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H54" s="72" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="I54" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J54" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="K54" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="L54" s="69" t="n">
         <v>12</v>
       </c>
-      <c r="F53" s="77" t="n">
-        <v>11</v>
-      </c>
-      <c r="G53" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H53" s="80" t="inlineStr">
-        <is>
-          <t>5–0</t>
-        </is>
-      </c>
-      <c r="I53" s="81" t="n">
-        <v>5</v>
-      </c>
-      <c r="J53" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K53" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L53" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="M53" s="74" t="n">
-        <v>0.31</v>
-      </c>
-      <c r="N53" s="76" t="inlineStr">
-        <is>
-          <t>Irak</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="66" t="inlineStr">
-        <is>
-          <t>Gruppe J</t>
-        </is>
-      </c>
-      <c r="B54" s="67" t="inlineStr">
-        <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C54" s="84" t="n">
-        <v>0.47</v>
-      </c>
-      <c r="D54" s="69" t="n">
-        <v>9</v>
-      </c>
-      <c r="E54" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="F54" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="G54" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="72" t="inlineStr">
-        <is>
-          <t>3–0</t>
-        </is>
-      </c>
-      <c r="I54" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J54" s="70" t="n">
-        <v>3</v>
-      </c>
-      <c r="K54" s="70" t="n">
-        <v>0</v>
-      </c>
-      <c r="L54" s="70" t="n">
-        <v>6</v>
-      </c>
-      <c r="M54" s="84" t="n">
-        <v>0.53</v>
+      <c r="M54" s="68" t="n">
+        <v>0.63</v>
       </c>
       <c r="N54" s="67" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Norge</t>
         </is>
       </c>
     </row>
@@ -52126,47 +52122,47 @@
       <c r="A55" s="75" t="inlineStr"/>
       <c r="B55" s="76" t="inlineStr">
         <is>
-          <t>Argentina</t>
-        </is>
-      </c>
-      <c r="C55" s="84" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="D55" s="78" t="n">
+          <t>Norge</t>
+        </is>
+      </c>
+      <c r="C55" s="74" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D55" s="77" t="n">
         <v>12</v>
       </c>
-      <c r="E55" s="78" t="n">
-        <v>3</v>
+      <c r="E55" s="77" t="n">
+        <v>6</v>
       </c>
       <c r="F55" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G55" s="79" t="n">
         <v>4</v>
       </c>
-      <c r="G55" s="79" t="n">
+      <c r="H55" s="80" t="inlineStr">
+        <is>
+          <t>3–2</t>
+        </is>
+      </c>
+      <c r="I55" s="81" t="n">
         <v>5</v>
       </c>
-      <c r="H55" s="80" t="inlineStr">
-        <is>
-          <t>2–0</t>
-        </is>
-      </c>
-      <c r="I55" s="81" t="n">
-        <v>3</v>
-      </c>
       <c r="J55" s="77" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K55" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L55" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="M55" s="84" t="n">
-        <v>0.46</v>
+      <c r="L55" s="78" t="n">
+        <v>17</v>
+      </c>
+      <c r="M55" s="68" t="n">
+        <v>0.57</v>
       </c>
       <c r="N55" s="76" t="inlineStr">
         <is>
-          <t>Østerrike</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -52174,47 +52170,47 @@
       <c r="A56" s="82" t="inlineStr"/>
       <c r="B56" s="67" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Norge</t>
         </is>
       </c>
       <c r="C56" s="74" t="n">
-        <v>0.25</v>
+        <v>0.43</v>
       </c>
       <c r="D56" s="70" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E56" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="F56" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G56" s="71" t="n">
+        <v>2</v>
+      </c>
+      <c r="H56" s="72" t="inlineStr">
+        <is>
+          <t>1–4</t>
+        </is>
+      </c>
+      <c r="I56" s="73" t="n">
         <v>4</v>
       </c>
-      <c r="F56" s="70" t="n">
-        <v>4</v>
-      </c>
-      <c r="G56" s="71" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="72" t="inlineStr">
-        <is>
-          <t>1–2</t>
-        </is>
-      </c>
-      <c r="I56" s="73" t="n">
-        <v>6</v>
-      </c>
       <c r="J56" s="70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K56" s="69" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="L56" s="69" t="n">
-        <v>17</v>
-      </c>
-      <c r="M56" s="83" t="n">
-        <v>0.75</v>
+        <v>19</v>
+      </c>
+      <c r="M56" s="68" t="n">
+        <v>0.57</v>
       </c>
       <c r="N56" s="67" t="inlineStr">
         <is>
-          <t>Algerie</t>
+          <t>Frankrike</t>
         </is>
       </c>
     </row>
@@ -52222,99 +52218,99 @@
       <c r="A57" s="75" t="inlineStr"/>
       <c r="B57" s="76" t="inlineStr">
         <is>
-          <t>Østerrike</t>
-        </is>
-      </c>
-      <c r="C57" s="68" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="D57" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="E57" s="77" t="n">
-        <v>3</v>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="C57" s="83" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D57" s="78" t="n">
+        <v>30</v>
+      </c>
+      <c r="E57" s="78" t="n">
+        <v>12</v>
       </c>
       <c r="F57" s="77" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="G57" s="79" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="H57" s="80" t="inlineStr">
         <is>
-          <t>3–1</t>
+          <t>5–0</t>
         </is>
       </c>
       <c r="I57" s="81" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J57" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="K57" s="78" t="n">
-        <v>4</v>
-      </c>
-      <c r="L57" s="78" t="n">
-        <v>11</v>
+        <v>0</v>
+      </c>
+      <c r="K57" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L57" s="77" t="n">
+        <v>6</v>
       </c>
       <c r="M57" s="74" t="n">
-        <v>0.38</v>
+        <v>0.31</v>
       </c>
       <c r="N57" s="76" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Irak</t>
         </is>
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="66" t="inlineStr">
         <is>
-          <t>Gruppe K</t>
+          <t>Gruppe J</t>
         </is>
       </c>
       <c r="B58" s="67" t="inlineStr">
         <is>
-          <t>Colombia</t>
-        </is>
-      </c>
-      <c r="C58" s="83" t="n">
-        <v>0.66</v>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C58" s="84" t="n">
+        <v>0.47</v>
       </c>
       <c r="D58" s="69" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E58" s="69" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="F58" s="70" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G58" s="71" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="H58" s="72" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I58" s="73" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J58" s="70" t="n">
         <v>3</v>
       </c>
       <c r="K58" s="70" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L58" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="M58" s="74" t="n">
-        <v>0.34</v>
+        <v>6</v>
+      </c>
+      <c r="M58" s="84" t="n">
+        <v>0.53</v>
       </c>
       <c r="N58" s="67" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -52322,14 +52318,14 @@
       <c r="A59" s="75" t="inlineStr"/>
       <c r="B59" s="76" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C59" s="83" t="n">
-        <v>0.75</v>
+          <t>Argentina</t>
+        </is>
+      </c>
+      <c r="C59" s="84" t="n">
+        <v>0.54</v>
       </c>
       <c r="D59" s="78" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E59" s="78" t="n">
         <v>3</v>
@@ -52338,31 +52334,31 @@
         <v>4</v>
       </c>
       <c r="G59" s="79" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H59" s="80" t="inlineStr">
         <is>
-          <t>1–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I59" s="81" t="n">
         <v>3</v>
       </c>
       <c r="J59" s="77" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" s="77" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L59" s="77" t="n">
-        <v>8</v>
-      </c>
-      <c r="M59" s="74" t="n">
-        <v>0.25</v>
+        <v>6</v>
+      </c>
+      <c r="M59" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N59" s="76" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Østerrike</t>
         </is>
       </c>
     </row>
@@ -52370,47 +52366,47 @@
       <c r="A60" s="82" t="inlineStr"/>
       <c r="B60" s="67" t="inlineStr">
         <is>
-          <t>Portugal</t>
-        </is>
-      </c>
-      <c r="C60" s="83" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="D60" s="69" t="n">
-        <v>16</v>
-      </c>
-      <c r="E60" s="69" t="n">
-        <v>9</v>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="C60" s="74" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D60" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E60" s="70" t="n">
+        <v>4</v>
       </c>
       <c r="F60" s="70" t="n">
         <v>4</v>
       </c>
       <c r="G60" s="71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" s="72" t="inlineStr">
+        <is>
+          <t>1–2</t>
+        </is>
+      </c>
+      <c r="I60" s="73" t="n">
+        <v>6</v>
+      </c>
+      <c r="J60" s="70" t="n">
         <v>3</v>
       </c>
-      <c r="H60" s="72" t="inlineStr">
-        <is>
-          <t>5–0</t>
-        </is>
-      </c>
-      <c r="I60" s="73" t="n">
-        <v>3</v>
-      </c>
-      <c r="J60" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="K60" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L60" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="M60" s="74" t="n">
-        <v>0.34</v>
+      <c r="K60" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="L60" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="M60" s="83" t="n">
+        <v>0.75</v>
       </c>
       <c r="N60" s="67" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
+          <t>Algerie</t>
         </is>
       </c>
     </row>
@@ -52418,99 +52414,99 @@
       <c r="A61" s="75" t="inlineStr"/>
       <c r="B61" s="76" t="inlineStr">
         <is>
-          <t>Usbekistan</t>
-        </is>
-      </c>
-      <c r="C61" s="74" t="n">
-        <v>0.33</v>
+          <t>Østerrike</t>
+        </is>
+      </c>
+      <c r="C61" s="68" t="n">
+        <v>0.62</v>
       </c>
       <c r="D61" s="77" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E61" s="77" t="n">
         <v>3</v>
       </c>
       <c r="F61" s="77" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G61" s="79" t="n">
         <v>2</v>
       </c>
       <c r="H61" s="80" t="inlineStr">
         <is>
-          <t>1–3</t>
+          <t>3–1</t>
         </is>
       </c>
       <c r="I61" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J61" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="J61" s="77" t="n">
-        <v>5</v>
-      </c>
       <c r="K61" s="78" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="L61" s="78" t="n">
-        <v>15</v>
-      </c>
-      <c r="M61" s="83" t="n">
-        <v>0.67</v>
+        <v>11</v>
+      </c>
+      <c r="M61" s="74" t="n">
+        <v>0.38</v>
       </c>
       <c r="N61" s="76" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Jordan</t>
         </is>
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="66" t="inlineStr">
         <is>
-          <t>Gruppe L</t>
+          <t>Gruppe K</t>
         </is>
       </c>
       <c r="B62" s="67" t="inlineStr">
         <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="C62" s="84" t="n">
-        <v>0.54</v>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="C62" s="83" t="n">
+        <v>0.66</v>
       </c>
       <c r="D62" s="69" t="n">
         <v>20</v>
       </c>
       <c r="E62" s="69" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F62" s="70" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G62" s="71" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H62" s="72" t="inlineStr">
         <is>
-          <t>4–2</t>
+          <t>1–0</t>
         </is>
       </c>
       <c r="I62" s="73" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J62" s="70" t="n">
         <v>3</v>
       </c>
       <c r="K62" s="70" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="L62" s="70" t="n">
-        <v>11</v>
-      </c>
-      <c r="M62" s="84" t="n">
-        <v>0.46</v>
+        <v>7</v>
+      </c>
+      <c r="M62" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N62" s="67" t="inlineStr">
         <is>
-          <t>Kroatia</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -52518,47 +52514,47 @@
       <c r="A63" s="75" t="inlineStr"/>
       <c r="B63" s="76" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="C63" s="83" t="n">
-        <v>0.78</v>
+        <v>0.75</v>
       </c>
       <c r="D63" s="78" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="E63" s="78" t="n">
+        <v>3</v>
+      </c>
+      <c r="F63" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="F63" s="77" t="n">
+      <c r="G63" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H63" s="80" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="I63" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J63" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="K63" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="L63" s="77" t="n">
         <v>8</v>
       </c>
-      <c r="G63" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="H63" s="80" t="inlineStr">
-        <is>
-          <t>0–0</t>
-        </is>
-      </c>
-      <c r="I63" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J63" s="77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" s="77" t="n">
-        <v>1</v>
-      </c>
-      <c r="L63" s="77" t="n">
-        <v>2</v>
-      </c>
       <c r="M63" s="74" t="n">
-        <v>0.22</v>
+        <v>0.25</v>
       </c>
       <c r="N63" s="76" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -52566,47 +52562,47 @@
       <c r="A64" s="82" t="inlineStr"/>
       <c r="B64" s="67" t="inlineStr">
         <is>
-          <t>Ghana</t>
-        </is>
-      </c>
-      <c r="C64" s="74" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="D64" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="E64" s="70" t="n">
-        <v>3</v>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="C64" s="83" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="D64" s="69" t="n">
+        <v>16</v>
+      </c>
+      <c r="E64" s="69" t="n">
+        <v>9</v>
       </c>
       <c r="F64" s="70" t="n">
         <v>4</v>
       </c>
       <c r="G64" s="71" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H64" s="72" t="inlineStr">
         <is>
-          <t>1–0</t>
+          <t>5–0</t>
         </is>
       </c>
       <c r="I64" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J64" s="70" t="n">
         <v>2</v>
       </c>
-      <c r="J64" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="K64" s="69" t="n">
-        <v>4</v>
-      </c>
-      <c r="L64" s="69" t="n">
-        <v>11</v>
-      </c>
-      <c r="M64" s="68" t="n">
-        <v>0.63</v>
+      <c r="K64" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="L64" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="M64" s="74" t="n">
+        <v>0.34</v>
       </c>
       <c r="N64" s="67" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Usbekistan</t>
         </is>
       </c>
     </row>
@@ -52614,79 +52610,275 @@
       <c r="A65" s="75" t="inlineStr"/>
       <c r="B65" s="76" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Usbekistan</t>
         </is>
       </c>
       <c r="C65" s="74" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="D65" s="78" t="n">
-        <v>8</v>
+        <v>0.33</v>
+      </c>
+      <c r="D65" s="77" t="n">
+        <v>7</v>
       </c>
       <c r="E65" s="77" t="n">
         <v>3</v>
       </c>
       <c r="F65" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G65" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H65" s="80" t="inlineStr">
+        <is>
+          <t>1–3</t>
+        </is>
+      </c>
+      <c r="I65" s="81" t="n">
         <v>4</v>
       </c>
-      <c r="G65" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H65" s="80" t="inlineStr">
+      <c r="J65" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="K65" s="78" t="n">
+        <v>6</v>
+      </c>
+      <c r="L65" s="78" t="n">
+        <v>15</v>
+      </c>
+      <c r="M65" s="83" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="N65" s="76" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="18" customHeight="1">
+      <c r="A66" s="66" t="inlineStr">
+        <is>
+          <t>Gruppe L</t>
+        </is>
+      </c>
+      <c r="B66" s="67" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C66" s="84" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="D66" s="69" t="n">
+        <v>20</v>
+      </c>
+      <c r="E66" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="F66" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G66" s="71" t="n">
+        <v>5</v>
+      </c>
+      <c r="H66" s="72" t="inlineStr">
+        <is>
+          <t>4–2</t>
+        </is>
+      </c>
+      <c r="I66" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J66" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="K66" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="L66" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="M66" s="84" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="N66" s="67" t="inlineStr">
+        <is>
+          <t>Kroatia</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="18" customHeight="1">
+      <c r="A67" s="75" t="inlineStr"/>
+      <c r="B67" s="76" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C67" s="83" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="D67" s="78" t="n">
+        <v>19</v>
+      </c>
+      <c r="E67" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="F67" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="G67" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="H67" s="80" t="inlineStr">
+        <is>
+          <t>0–0</t>
+        </is>
+      </c>
+      <c r="I67" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J67" s="77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K67" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L67" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="M67" s="74" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="N67" s="76" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="18" customHeight="1">
+      <c r="A68" s="82" t="inlineStr"/>
+      <c r="B68" s="67" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+      <c r="C68" s="74" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="D68" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="E68" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="F68" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="G68" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H68" s="72" t="inlineStr">
+        <is>
+          <t>1–0</t>
+        </is>
+      </c>
+      <c r="I68" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J68" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="K68" s="69" t="n">
+        <v>4</v>
+      </c>
+      <c r="L68" s="69" t="n">
+        <v>11</v>
+      </c>
+      <c r="M68" s="68" t="n">
+        <v>0.63</v>
+      </c>
+      <c r="N68" s="67" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="75" t="inlineStr"/>
+      <c r="B69" s="76" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C69" s="74" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D69" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F69" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="G69" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" s="80" t="inlineStr">
         <is>
           <t>0–1</t>
         </is>
       </c>
-      <c r="I65" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J65" s="77" t="n">
+      <c r="I69" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J69" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="K65" s="77" t="n">
+      <c r="K69" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="L65" s="77" t="n">
+      <c r="L69" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="M65" s="68" t="n">
+      <c r="M69" s="68" t="n">
         <v>0.58</v>
       </c>
-      <c r="N65" s="76" t="inlineStr">
+      <c r="N69" s="76" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="14" customHeight="1">
-      <c r="A67" s="63" t="inlineStr">
+    <row r="71" ht="14" customHeight="1">
+      <c r="A71" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="55" t="inlineStr">
+    <row r="72" ht="18" customHeight="1">
+      <c r="A72" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B68" s="62" t="inlineStr">
+      <c r="B72" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C68" s="61" t="inlineStr">
+      <c r="C72" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D68" s="58" t="inlineStr">
+      <c r="D72" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E68" s="85" t="inlineStr">
+      <c r="E72" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -52695,7 +52887,7 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A67:N67"/>
+    <mergeCell ref="A71:N71"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Legg til stadionnavn i alle sluttspill-runder
8-delsfinaler, kvartfinaler, semifinaler, bronsefinale og finale
har nå stadionnavn fra FIFA API i Excel-arket.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -17881,7 +17881,7 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -17900,7 +17900,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -17937,7 +17937,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>28.06</t>
+          <t>28.06 21:00</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -17952,17 +17952,21 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Joao Pinheiro</t>
+          <t>João Pedro Silva Pinheiro</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>29.06</t>
+          <t>29.06 19:00</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -17977,13 +17981,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Houston Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>29.06</t>
+          <t>29.06 22:30</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -17998,13 +18006,17 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Boston Stadium</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>29.06</t>
+          <t>30.06 03:00</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -18019,13 +18031,17 @@
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Monterrey Stadium</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>30.06 19:00</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -18040,13 +18056,17 @@
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>30.06 23:00</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -18061,13 +18081,17 @@
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>01.07 03:00</t>
         </is>
       </c>
       <c r="B9" s="21" t="inlineStr">
@@ -18082,13 +18106,17 @@
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Mexico City Stadium</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>01.07</t>
+          <t>01.07 18:00</t>
         </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
@@ -18103,13 +18131,17 @@
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
       <c r="G10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>01.07</t>
+          <t>01.07 22:00</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
@@ -18124,13 +18156,17 @@
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Seattle Stadium</t>
+        </is>
+      </c>
       <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>01.07</t>
+          <t>02.07 02:00</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -18145,13 +18181,17 @@
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>San Francisco Bay Area Stadium</t>
+        </is>
+      </c>
       <c r="G12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>02.07</t>
+          <t>02.07 21:00</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
@@ -18166,13 +18206,17 @@
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>02.07</t>
+          <t>03.07 01:00</t>
         </is>
       </c>
       <c r="B14" s="22" t="inlineStr">
@@ -18187,13 +18231,17 @@
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="8" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Toronto Stadium</t>
+        </is>
+      </c>
       <c r="G14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>02.07</t>
+          <t>03.07 05:00</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
@@ -18208,13 +18256,17 @@
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>BC Place Vancouver</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>03.07</t>
+          <t>03.07 20:00</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -18229,13 +18281,17 @@
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>03.07</t>
+          <t>04.07 00:00</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -18250,13 +18306,17 @@
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
       <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>03.07</t>
+          <t>04.07 03:30</t>
         </is>
       </c>
       <c r="B18" s="22" t="inlineStr">
@@ -18271,7 +18331,11 @@
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
       <c r="G18" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18291,7 +18355,7 @@
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18310,7 +18374,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18347,7 +18411,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>04.07</t>
+          <t>04.07 19:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18362,13 +18426,17 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Houston Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>04.07</t>
+          <t>04.07 23:00</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
@@ -18383,13 +18451,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Philadelphia Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>05.07</t>
+          <t>05.07 22:00</t>
         </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
@@ -18404,13 +18476,17 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>05.07</t>
+          <t>06.07 02:00</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
@@ -18425,13 +18501,17 @@
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Mexico City Stadium</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>06.07</t>
+          <t>06.07 21:00</t>
         </is>
       </c>
       <c r="B7" s="21" t="inlineStr">
@@ -18446,13 +18526,17 @@
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>06.07</t>
+          <t>07.07 02:00</t>
         </is>
       </c>
       <c r="B8" s="22" t="inlineStr">
@@ -18467,13 +18551,17 @@
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Seattle Stadium</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>07.07</t>
+          <t>07.07 18:00</t>
         </is>
       </c>
       <c r="B9" s="21" t="inlineStr">
@@ -18488,13 +18576,17 @@
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>07.07</t>
+          <t>07.07 22:00</t>
         </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
@@ -18509,7 +18601,11 @@
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>BC Place Vancouver</t>
+        </is>
+      </c>
       <c r="G10" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18529,7 +18625,7 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18548,7 +18644,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18585,7 +18681,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>09.07</t>
+          <t>09.07 22:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18600,13 +18696,17 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Boston Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>10.07</t>
+          <t>10.07 21:00</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
@@ -18621,13 +18721,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>11.07</t>
+          <t>11.07 23:00</t>
         </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
@@ -18642,13 +18746,17 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>11.07</t>
+          <t>12.07 03:00</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
@@ -18663,7 +18771,11 @@
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18683,7 +18795,7 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18702,7 +18814,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18739,7 +18851,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>14.07</t>
+          <t>14.07 21:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18754,13 +18866,17 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>15.07</t>
+          <t>15.07 21:00</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
@@ -18775,7 +18891,11 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18795,7 +18915,7 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18814,7 +18934,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18851,7 +18971,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>18.07</t>
+          <t>18.07 23:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18866,7 +18986,11 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18886,7 +19010,7 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18905,7 +19029,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18942,7 +19066,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>19.07</t>
+          <t>19.07 21:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18957,7 +19081,11 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Legg til stadionnavn i alle sluttspill-runder (#92)
8-delsfinaler, kvartfinaler, semifinaler, bronsefinale og finale
har nå stadionnavn fra FIFA API i Excel-arket.

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -17881,7 +17881,7 @@
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -17900,7 +17900,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -17937,7 +17937,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>28.06</t>
+          <t>28.06 21:00</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -17952,17 +17952,21 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Joao Pinheiro</t>
+          <t>João Pedro Silva Pinheiro</t>
         </is>
       </c>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>29.06</t>
+          <t>29.06 19:00</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -17977,13 +17981,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Houston Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>29.06</t>
+          <t>29.06 22:30</t>
         </is>
       </c>
       <c r="B5" s="5" t="inlineStr">
@@ -17998,13 +18006,17 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Boston Stadium</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>29.06</t>
+          <t>30.06 03:00</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
@@ -18019,13 +18031,17 @@
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Monterrey Stadium</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>30.06 19:00</t>
         </is>
       </c>
       <c r="B7" s="5" t="inlineStr">
@@ -18040,13 +18056,17 @@
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>30.06 23:00</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
@@ -18061,13 +18081,17 @@
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>30.06</t>
+          <t>01.07 03:00</t>
         </is>
       </c>
       <c r="B9" s="21" t="inlineStr">
@@ -18082,13 +18106,17 @@
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Mexico City Stadium</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>01.07</t>
+          <t>01.07 18:00</t>
         </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
@@ -18103,13 +18131,17 @@
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
       <c r="G10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="17" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>01.07</t>
+          <t>01.07 22:00</t>
         </is>
       </c>
       <c r="B11" s="21" t="inlineStr">
@@ -18124,13 +18156,17 @@
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr"/>
-      <c r="F11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Seattle Stadium</t>
+        </is>
+      </c>
       <c r="G11" s="5" t="inlineStr"/>
     </row>
     <row r="12" ht="17" customHeight="1">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>01.07</t>
+          <t>02.07 02:00</t>
         </is>
       </c>
       <c r="B12" s="8" t="inlineStr">
@@ -18145,13 +18181,17 @@
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr"/>
-      <c r="F12" s="8" t="inlineStr"/>
+      <c r="F12" s="8" t="inlineStr">
+        <is>
+          <t>San Francisco Bay Area Stadium</t>
+        </is>
+      </c>
       <c r="G12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="17" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>02.07</t>
+          <t>02.07 21:00</t>
         </is>
       </c>
       <c r="B13" s="21" t="inlineStr">
@@ -18166,13 +18206,17 @@
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr"/>
     </row>
     <row r="14" ht="17" customHeight="1">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>02.07</t>
+          <t>03.07 01:00</t>
         </is>
       </c>
       <c r="B14" s="22" t="inlineStr">
@@ -18187,13 +18231,17 @@
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr"/>
-      <c r="F14" s="8" t="inlineStr"/>
+      <c r="F14" s="8" t="inlineStr">
+        <is>
+          <t>Toronto Stadium</t>
+        </is>
+      </c>
       <c r="G14" s="8" t="inlineStr"/>
     </row>
     <row r="15" ht="17" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>02.07</t>
+          <t>03.07 05:00</t>
         </is>
       </c>
       <c r="B15" s="21" t="inlineStr">
@@ -18208,13 +18256,17 @@
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>BC Place Vancouver</t>
+        </is>
+      </c>
       <c r="G15" s="5" t="inlineStr"/>
     </row>
     <row r="16" ht="17" customHeight="1">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>03.07</t>
+          <t>03.07 20:00</t>
         </is>
       </c>
       <c r="B16" s="8" t="inlineStr">
@@ -18229,13 +18281,17 @@
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr"/>
+      <c r="F16" s="8" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="17" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>03.07</t>
+          <t>04.07 00:00</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
@@ -18250,13 +18306,17 @@
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
-      <c r="F17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
       <c r="G17" s="5" t="inlineStr"/>
     </row>
     <row r="18" ht="17" customHeight="1">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>03.07</t>
+          <t>04.07 03:30</t>
         </is>
       </c>
       <c r="B18" s="22" t="inlineStr">
@@ -18271,7 +18331,11 @@
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr"/>
+      <c r="F18" s="8" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
       <c r="G18" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18291,7 +18355,7 @@
   <dimension ref="A1:G10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18310,7 +18374,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18347,7 +18411,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>04.07</t>
+          <t>04.07 19:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18362,13 +18426,17 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Houston Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>04.07</t>
+          <t>04.07 23:00</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
@@ -18383,13 +18451,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Philadelphia Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>05.07</t>
+          <t>05.07 22:00</t>
         </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
@@ -18404,13 +18476,17 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>05.07</t>
+          <t>06.07 02:00</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
@@ -18425,13 +18501,17 @@
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Mexico City Stadium</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="17" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>06.07</t>
+          <t>06.07 21:00</t>
         </is>
       </c>
       <c r="B7" s="21" t="inlineStr">
@@ -18446,13 +18526,17 @@
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G7" s="5" t="inlineStr"/>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>06.07</t>
+          <t>07.07 02:00</t>
         </is>
       </c>
       <c r="B8" s="22" t="inlineStr">
@@ -18467,13 +18551,17 @@
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr"/>
-      <c r="F8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>Seattle Stadium</t>
+        </is>
+      </c>
       <c r="G8" s="8" t="inlineStr"/>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>07.07</t>
+          <t>07.07 18:00</t>
         </is>
       </c>
       <c r="B9" s="21" t="inlineStr">
@@ -18488,13 +18576,17 @@
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>07.07</t>
+          <t>07.07 22:00</t>
         </is>
       </c>
       <c r="B10" s="22" t="inlineStr">
@@ -18509,7 +18601,11 @@
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr"/>
-      <c r="F10" s="8" t="inlineStr"/>
+      <c r="F10" s="8" t="inlineStr">
+        <is>
+          <t>BC Place Vancouver</t>
+        </is>
+      </c>
       <c r="G10" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18529,7 +18625,7 @@
   <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18548,7 +18644,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18585,7 +18681,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>09.07</t>
+          <t>09.07 22:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18600,13 +18696,17 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Boston Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>10.07</t>
+          <t>10.07 21:00</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
@@ -18621,13 +18721,17 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Los Angeles Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="17" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>11.07</t>
+          <t>11.07 23:00</t>
         </is>
       </c>
       <c r="B5" s="21" t="inlineStr">
@@ -18642,13 +18746,17 @@
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr"/>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
       <c r="G5" s="5" t="inlineStr"/>
     </row>
     <row r="6" ht="17" customHeight="1">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>11.07</t>
+          <t>12.07 03:00</t>
         </is>
       </c>
       <c r="B6" s="22" t="inlineStr">
@@ -18663,7 +18771,11 @@
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr"/>
-      <c r="F6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Kansas City Stadium</t>
+        </is>
+      </c>
       <c r="G6" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18683,7 +18795,7 @@
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18702,7 +18814,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18739,7 +18851,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>14.07</t>
+          <t>14.07 21:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18754,13 +18866,17 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Dallas Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
     <row r="4" ht="17" customHeight="1">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>15.07</t>
+          <t>15.07 21:00</t>
         </is>
       </c>
       <c r="B4" s="22" t="inlineStr">
@@ -18775,7 +18891,11 @@
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr"/>
-      <c r="F4" s="8" t="inlineStr"/>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Atlanta Stadium</t>
+        </is>
+      </c>
       <c r="G4" s="8" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18795,7 +18915,7 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18814,7 +18934,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18851,7 +18971,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>18.07</t>
+          <t>18.07 23:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18866,7 +18986,11 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
@@ -18886,7 +19010,7 @@
   <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
@@ -18905,7 +19029,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -18942,7 +19066,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>19.07</t>
+          <t>19.07 21:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -18957,7 +19081,11 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
       <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fiks P-kolonne til posisjon B i gruppe G, H og I
Tabellheader hadde P som siste kolonne i stedet for kolonne B.
Retter tab_cols og vals i add_kamper_sheets.py, og regenererer
alle 12 gruppeark med --full.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1572,7 +1572,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Yael Falcon Perez</t>
+          <t>Yael Falcón Pérez</t>
         </is>
       </c>
     </row>
@@ -9714,7 +9714,7 @@
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Abdulrahman Aljassim</t>
+          <t>Abdulrahman Al Jassim</t>
         </is>
       </c>
     </row>
@@ -13854,7 +13854,7 @@
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Clement Turpin</t>
+          <t>Clément Turpin</t>
         </is>
       </c>
     </row>
@@ -14000,7 +14000,11 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>– – –</t>
+        </is>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>England</t>
@@ -14026,7 +14030,11 @@
           <t>Kroatia</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr"/>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>– – –</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Ghana</t>
@@ -60992,7 +61000,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>70 492</t>
+        </is>
+      </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Los Angeles Stadium</t>
@@ -61042,7 +61054,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Clement Turpin</t>
+          <t>Clément Turpin</t>
         </is>
       </c>
     </row>
@@ -65072,7 +65084,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Francois Letexier</t>
+          <t>François Letexier</t>
         </is>
       </c>
     </row>
@@ -65114,7 +65126,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Juan Gabriel Benitez</t>
+          <t>Juan Gabriel Benítez</t>
         </is>
       </c>
     </row>
@@ -69270,7 +69282,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Yael Falcon Perez</t>
+          <t>Yael Falcón Pérez</t>
         </is>
       </c>
     </row>
@@ -69394,7 +69406,11 @@
           <t>Kansas City Stadium</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr"/>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Katia Garcia</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
@@ -69432,7 +69448,11 @@
           <t>Dallas Stadium</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr"/>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Ivan Barton</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n"/>
@@ -73514,7 +73534,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Dario Herrera</t>
+          <t>Darío Herrera</t>
         </is>
       </c>
     </row>
@@ -73670,42 +73690,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -73715,31 +73735,31 @@
           <t>Belgia</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -73748,31 +73768,31 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -73781,31 +73801,31 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -73814,31 +73834,31 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -77756,7 +77776,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>Espen Eskas</t>
+          <t>Espen Eskås</t>
         </is>
       </c>
     </row>
@@ -77840,7 +77860,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Francois Letexier</t>
+          <t>François Letexier</t>
         </is>
       </c>
     </row>
@@ -77870,42 +77890,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -77915,31 +77935,31 @@
           <t>Spania</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -77948,31 +77968,31 @@
           <t>Kapp Verde</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>2</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -77981,31 +78001,31 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -78014,31 +78034,31 @@
           <t>Saudi-Arabia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="E15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="F15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -82044,42 +82064,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -82089,31 +82109,31 @@
           <t>Frankrike</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>3</v>
+      <c r="B12" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+8</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -82122,31 +82142,31 @@
           <t>Norge</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="D13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -82155,31 +82175,31 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -82188,31 +82208,31 @@
           <t>Irak</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Fiks P-kolonne til posisjon B i gruppe G, H og I (#93)
Tabellheader hadde P som siste kolonne i stedet for kolonne B.
Retter tab_cols og vals i add_kamper_sheets.py, og regenererer
alle 12 gruppeark med --full.

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1572,7 +1572,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Yael Falcon Perez</t>
+          <t>Yael Falcón Pérez</t>
         </is>
       </c>
     </row>
@@ -9714,7 +9714,7 @@
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Abdulrahman Aljassim</t>
+          <t>Abdulrahman Al Jassim</t>
         </is>
       </c>
     </row>
@@ -13854,7 +13854,7 @@
       </c>
       <c r="H3" s="12" t="inlineStr">
         <is>
-          <t>Clement Turpin</t>
+          <t>Clément Turpin</t>
         </is>
       </c>
     </row>
@@ -14000,7 +14000,11 @@
           <t>Panama</t>
         </is>
       </c>
-      <c r="D7" s="14" t="inlineStr"/>
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>– – –</t>
+        </is>
+      </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
           <t>England</t>
@@ -14026,7 +14030,11 @@
           <t>Kroatia</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr"/>
+      <c r="D8" s="15" t="inlineStr">
+        <is>
+          <t>– – –</t>
+        </is>
+      </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
           <t>Ghana</t>
@@ -60992,7 +61000,11 @@
           <t>USA</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr"/>
+      <c r="F7" s="11" t="inlineStr">
+        <is>
+          <t>70 492</t>
+        </is>
+      </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
           <t>Los Angeles Stadium</t>
@@ -61042,7 +61054,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Clement Turpin</t>
+          <t>Clément Turpin</t>
         </is>
       </c>
     </row>
@@ -65072,7 +65084,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Francois Letexier</t>
+          <t>François Letexier</t>
         </is>
       </c>
     </row>
@@ -65114,7 +65126,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Juan Gabriel Benitez</t>
+          <t>Juan Gabriel Benítez</t>
         </is>
       </c>
     </row>
@@ -69270,7 +69282,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>Yael Falcon Perez</t>
+          <t>Yael Falcón Pérez</t>
         </is>
       </c>
     </row>
@@ -69394,7 +69406,11 @@
           <t>Kansas City Stadium</t>
         </is>
       </c>
-      <c r="H7" s="12" t="inlineStr"/>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>Katia Garcia</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="11" t="inlineStr">
@@ -69432,7 +69448,11 @@
           <t>Dallas Stadium</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr"/>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Ivan Barton</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="16" t="n"/>
@@ -73514,7 +73534,7 @@
       </c>
       <c r="H5" s="12" t="inlineStr">
         <is>
-          <t>Dario Herrera</t>
+          <t>Darío Herrera</t>
         </is>
       </c>
     </row>
@@ -73670,42 +73690,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -73715,31 +73735,31 @@
           <t>Belgia</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="D12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+4</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -73748,31 +73768,31 @@
           <t>Egypt</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>5</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="D13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="G13" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -73781,31 +73801,31 @@
           <t>Iran</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>0</v>
-      </c>
-      <c r="F14" s="4" t="n">
-        <v>3</v>
       </c>
       <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -73814,31 +73834,31 @@
           <t>New Zealand</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="E15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="G15" s="7" t="n">
         <v>4</v>
       </c>
-      <c r="G15" s="7" t="n">
+      <c r="H15" s="7" t="n">
         <v>10</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-6</t>
         </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -77756,7 +77776,7 @@
       </c>
       <c r="H6" s="12" t="inlineStr">
         <is>
-          <t>Espen Eskas</t>
+          <t>Espen Eskås</t>
         </is>
       </c>
     </row>
@@ -77840,7 +77860,7 @@
       </c>
       <c r="H8" s="12" t="inlineStr">
         <is>
-          <t>Francois Letexier</t>
+          <t>François Letexier</t>
         </is>
       </c>
     </row>
@@ -77870,42 +77890,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -77915,31 +77935,31 @@
           <t>Spania</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
+      <c r="B12" s="13" t="n">
+        <v>7</v>
+      </c>
+      <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="C12" s="11" t="n">
+      <c r="D12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="D12" s="11" t="n">
-        <v>1</v>
-      </c>
       <c r="E12" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="G12" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+5</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>7</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -77948,31 +77968,31 @@
           <t>Kapp Verde</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>3</v>
       </c>
       <c r="C13" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="D13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="F13" s="18" t="n">
         <v>0</v>
-      </c>
-      <c r="F13" s="18" t="n">
-        <v>2</v>
       </c>
       <c r="G13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="H13" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>0</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -77981,31 +78001,31 @@
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="C14" s="4" t="n">
+      <c r="D14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="E14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="4" t="n">
-        <v>1</v>
-      </c>
       <c r="F14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" s="4" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>4</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>-1</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -78014,31 +78034,31 @@
           <t>Saudi-Arabia</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="7" t="n">
+      <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="E15" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="F15" s="7" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>5</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-4</t>
         </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">
@@ -82044,42 +82064,42 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
           <t>K</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>U</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>T</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>MF</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>MM</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>MD</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>P</t>
         </is>
       </c>
     </row>
@@ -82089,31 +82109,31 @@
           <t>Frankrike</t>
         </is>
       </c>
-      <c r="B12" s="11" t="n">
-        <v>3</v>
+      <c r="B12" s="13" t="n">
+        <v>9</v>
       </c>
       <c r="C12" s="11" t="n">
         <v>3</v>
       </c>
       <c r="D12" s="11" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="H12" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="H12" s="11" t="inlineStr">
+      <c r="I12" s="11" t="inlineStr">
         <is>
           <t>+8</t>
         </is>
-      </c>
-      <c r="I12" s="13" t="n">
-        <v>9</v>
       </c>
     </row>
     <row r="13" ht="17" customHeight="1">
@@ -82122,31 +82142,31 @@
           <t>Norge</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
+        <v>6</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="D13" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="E13" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="18" t="n">
-        <v>1</v>
-      </c>
       <c r="F13" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="H13" s="18" t="n">
         <v>7</v>
       </c>
-      <c r="H13" s="18" t="inlineStr">
+      <c r="I13" s="18" t="inlineStr">
         <is>
           <t>+1</t>
         </is>
-      </c>
-      <c r="I13" s="19" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="14" ht="17" customHeight="1">
@@ -82155,31 +82175,31 @@
           <t>Senegal</t>
         </is>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="6" t="n">
         <v>3</v>
       </c>
       <c r="C14" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="F14" s="4" t="n">
         <v>2</v>
       </c>
-      <c r="F14" s="4" t="n">
+      <c r="G14" s="4" t="n">
         <v>8</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="H14" s="4" t="n">
         <v>6</v>
       </c>
-      <c r="H14" s="4" t="inlineStr">
+      <c r="I14" s="4" t="inlineStr">
         <is>
           <t>+2</t>
         </is>
-      </c>
-      <c r="I14" s="6" t="n">
-        <v>3</v>
       </c>
     </row>
     <row r="15" ht="17" customHeight="1">
@@ -82188,31 +82208,31 @@
           <t>Irak</t>
         </is>
       </c>
-      <c r="B15" s="7" t="n">
+      <c r="B15" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="7" t="n">
         <v>3</v>
-      </c>
-      <c r="C15" s="7" t="n">
-        <v>0</v>
       </c>
       <c r="D15" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="F15" s="7" t="n">
-        <v>1</v>
-      </c>
       <c r="G15" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="I15" s="7" t="inlineStr">
         <is>
           <t>-11</t>
         </is>
-      </c>
-      <c r="I15" s="9" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="17" ht="24" customHeight="1">

</xml_diff>

<commit_message>
Vis ekstraomganger og straffespark i sluttspill-ark
Henter ResultType, HomeTeamPenaltyScore og AwayTeamPenaltyScore fra
FIFA API. Resultat-kolonnen viser naa ekstraomganger og straffespark.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -17891,7 +17891,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18365,7 +18365,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18635,7 +18635,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18805,7 +18805,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18925,7 +18925,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -19020,7 +19020,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>

</xml_diff>

<commit_message>
Vis ekstraomganger og straffespark i sluttspill-ark (#95)
Henter ResultType, HomeTeamPenaltyScore og AwayTeamPenaltyScore fra
FIFA API. Resultat-kolonnen viser naa ekstraomganger og straffespark.

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,41 +1,41 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Aldersfordeling" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Spillere etter klubbland" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Klubbdominans" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Kort" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Scorere og assists" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Alder" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Lagstatistikk" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Scoringstidspunkt" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Heatmap" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Ballbesittelse" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Stadionoversikt" sheetId="29" state="visible" r:id="rId29"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -883,13 +883,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -908,7 +908,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -936,8 +936,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -963,8 +963,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,7 +987,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1002,9 +1002,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -17891,7 +17891,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18365,7 +18365,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18635,7 +18635,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18805,7 +18805,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -18925,7 +18925,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>
@@ -19020,7 +19020,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="24" customWidth="1" min="6" max="6"/>

</xml_diff>

<commit_message>
Skill mellom kampstraffer og straffesparkkonkurranse
Cacher Period, HomePenaltyGoals og AwayPenaltyGoals fra FIFA timeline API.
Shooter-identifikasjon: Period >= 9 = straffesparkkonkurranse (FIFA standard).
Seksjon 3 har naa tre tabeller:
  - Straffespark per lag (ordinaer tid + ekstraomganger)
  - Kampstraffer per spiller
  - Straffesparkkonkurranse per spiller (dukker opp naar forste shootout er spilt)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -50829,7 +50829,7 @@
     <row r="95" ht="26" customHeight="1">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Straffespark per lag</t>
+          <t>VM 2026 — Straffespark per lag (ordinær tid + ekstraomganger)</t>
         </is>
       </c>
     </row>
@@ -51060,7 +51060,7 @@
     <row r="106" ht="26" customHeight="1">
       <c r="A106" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Straffespark per spiller</t>
+          <t>VM 2026 — Kampstraffer per spiller (ordinær tid + ekstraomganger)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-28 07:05 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -48592,7 +48592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N76"/>
+  <dimension ref="A1:N78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -52068,79 +52068,175 @@
       <c r="A73" s="75" t="inlineStr"/>
       <c r="B73" s="76" t="inlineStr">
         <is>
-          <t>Panama</t>
-        </is>
-      </c>
-      <c r="C73" s="74" t="n">
-        <v>0.42</v>
+          <t>Kroatia</t>
+        </is>
+      </c>
+      <c r="C73" s="84" t="n">
+        <v>0.53</v>
       </c>
       <c r="D73" s="78" t="n">
         <v>8</v>
       </c>
-      <c r="E73" s="77" t="n">
+      <c r="E73" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="F73" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="G73" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H73" s="80" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="I73" s="81" t="n">
+        <v>2</v>
+      </c>
+      <c r="J73" s="77" t="n">
         <v>3</v>
       </c>
-      <c r="F73" s="77" t="n">
-        <v>4</v>
-      </c>
-      <c r="G73" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="H73" s="80" t="inlineStr">
-        <is>
-          <t>0–1</t>
-        </is>
-      </c>
-      <c r="I73" s="81" t="n">
-        <v>1</v>
-      </c>
-      <c r="J73" s="77" t="n">
-        <v>2</v>
-      </c>
       <c r="K73" s="77" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="L73" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="M73" s="68" t="n">
+      <c r="M73" s="84" t="n">
+        <v>0.47</v>
+      </c>
+      <c r="N73" s="76" t="inlineStr">
+        <is>
+          <t>Ghana</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="18" customHeight="1">
+      <c r="A74" s="82" t="inlineStr"/>
+      <c r="B74" s="67" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C74" s="74" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="D74" s="70" t="n">
+        <v>9</v>
+      </c>
+      <c r="E74" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F74" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="G74" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H74" s="72" t="inlineStr">
+        <is>
+          <t>0–2</t>
+        </is>
+      </c>
+      <c r="I74" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J74" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="K74" s="69" t="n">
+        <v>8</v>
+      </c>
+      <c r="L74" s="69" t="n">
+        <v>17</v>
+      </c>
+      <c r="M74" s="83" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="N74" s="67" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="75" t="inlineStr"/>
+      <c r="B75" s="76" t="inlineStr">
+        <is>
+          <t>Panama</t>
+        </is>
+      </c>
+      <c r="C75" s="74" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="D75" s="78" t="n">
+        <v>8</v>
+      </c>
+      <c r="E75" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="F75" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="G75" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" s="80" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I75" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J75" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="K75" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="L75" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="M75" s="68" t="n">
         <v>0.58</v>
       </c>
-      <c r="N73" s="76" t="inlineStr">
+      <c r="N75" s="76" t="inlineStr">
         <is>
           <t>Kroatia</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="14" customHeight="1">
-      <c r="A75" s="63" t="inlineStr">
+    <row r="77" ht="14" customHeight="1">
+      <c r="A77" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="55" t="inlineStr">
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B76" s="62" t="inlineStr">
+      <c r="B78" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C76" s="61" t="inlineStr">
+      <c r="C78" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D76" s="58" t="inlineStr">
+      <c r="D78" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E76" s="85" t="inlineStr">
+      <c r="E78" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -52149,8 +52245,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A75:N75"/>
     <mergeCell ref="I2:N2"/>
+    <mergeCell ref="A77:N77"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-29 11:18 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -908,13 +908,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -933,7 +933,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -957,12 +957,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -976,7 +976,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -989,8 +988,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1004,7 +1003,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1014,7 +1012,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1029,9 +1027,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -18065,6 +18063,173 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Sluttspill — Scorere og assists   1 mål · 0 assists</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Lag</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Kamper</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mål</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Assist</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Stephen Eustaquio</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="25" t="n"/>
+    </row>
+    <row r="4" ht="8" customHeight="1">
+      <c r="A4" s="122" t="n"/>
+      <c r="B4" s="122" t="n"/>
+      <c r="C4" s="122" t="n"/>
+      <c r="D4" s="122" t="n"/>
+      <c r="E4" s="122" t="n"/>
+      <c r="F4" s="122" t="n"/>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>Sluttspill — Kort   2 gule · 0 røde</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Lag</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Gule</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Røde</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Nathan Saliba</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D7" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="125" t="n"/>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Niko Sigur</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D8" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="127" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A1:F1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -18276,7 +18441,11 @@
           <t>Dallas Stadium</t>
         </is>
       </c>
-      <c r="G7" s="5" t="inlineStr"/>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>Jesús Valenzuela Sáez</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="17" customHeight="1">
       <c r="A8" s="7" t="inlineStr">
@@ -18301,7 +18470,11 @@
           <t>New York/New Jersey Stadium</t>
         </is>
       </c>
-      <c r="G8" s="8" t="inlineStr"/>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Danny Desmond Makkelie</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="17" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
@@ -18326,7 +18499,11 @@
           <t>Mexico City Stadium</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr"/>
+      <c r="G9" s="5" t="inlineStr">
+        <is>
+          <t>Slavko Vincic</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="17" customHeight="1">
       <c r="A10" s="7" t="inlineStr">
@@ -18561,7 +18738,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18831,7 +19008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19001,7 +19178,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19112,101 +19289,6 @@
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>VM 2026 — Bronsefinale</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Dato og kl.slett</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Hjemmelag</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Resultat</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Bortelag</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Tilskuere</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Stadion</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Dommer</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>18.07 23:00</t>
-        </is>
-      </c>
-      <c r="B3" s="21" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr"/>
-      <c r="D3" s="21" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Miami Stadium</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -19237,7 +19319,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Finale</t>
+          <t>VM 2026 — Bronsefinale</t>
         </is>
       </c>
     </row>
@@ -19281,7 +19363,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>19.07 21:00</t>
+          <t>18.07 23:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -19298,7 +19380,7 @@
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>New York/New Jersey Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -19317,162 +19399,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Sluttspill — Scorere og assists   1 mål · 0 assists</t>
+          <t>VM 2026 — Finale</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Lag</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Kamper</t>
+          <t>Hjemmelag</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Bortelag</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Mål</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Assist</t>
+          <t>Tilskuere</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Stadion</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Dommer</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Stephen Eustaquio</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="25" t="n"/>
-    </row>
-    <row r="4" ht="8" customHeight="1">
-      <c r="A4" s="122" t="n"/>
-      <c r="B4" s="122" t="n"/>
-      <c r="C4" s="122" t="n"/>
-      <c r="D4" s="122" t="n"/>
-      <c r="E4" s="122" t="n"/>
-      <c r="F4" s="122" t="n"/>
-    </row>
-    <row r="5" ht="28" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
-        <is>
-          <t>Sluttspill — Kort   2 gule · 0 røde</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Lag</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Gule</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Røde</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Nathan Saliba</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D7" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="125" t="n"/>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Niko Sigur</t>
-        </is>
-      </c>
-      <c r="C8" s="8" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D8" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="127" t="n"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>19.07 21:00</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr"/>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A5:E5"/>
-    <mergeCell ref="A1:F1"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Oppdater kampdata: sluttspill-spillere med riktig navn
Gabriel Magalhães vises nå korrekt i assist-kolonne (var 430601).
Excel regenerert etter fix i add_sluttspill_spillere_sheet.py (#112).

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -908,13 +908,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -933,7 +933,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -957,12 +957,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -976,6 +976,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -988,8 +989,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1003,6 +1004,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1012,7 +1014,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1027,9 +1029,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -18295,7 +18297,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>430601</t>
+          <t>Bruno Guimaraes</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -18317,12 +18319,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Bruno Guimaraes</t>
+          <t>Chemsdine Talbi</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Marokko</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
@@ -18339,12 +18341,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Chemsdine Talbi</t>
+          <t>Crysencio Summerville</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Nederland</t>
         </is>
       </c>
       <c r="D13" s="14" t="n">
@@ -18361,12 +18363,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Crysencio Summerville</t>
+          <t>Florian Wirtz</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Nederland</t>
+          <t>Tyskland</t>
         </is>
       </c>
       <c r="D14" s="15" t="n">
@@ -18383,12 +18385,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Florian Wirtz</t>
+          <t>Gabriel Magalhães</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Tyskland</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">

</xml_diff>

<commit_message>
Oppdater kampdata: sluttspill-spillere med riktig navn (#113)
Gabriel Magalhães vises nå korrekt i assist-kolonne (var 430601).
Excel regenerert etter fix i add_sluttspill_spillere_sheet.py (#112).

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -908,13 +908,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -933,7 +933,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -957,12 +957,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="l"/>
+        <axPos val="b"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -976,6 +976,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -988,8 +989,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1003,6 +1004,7 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
+        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1012,7 +1014,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1027,9 +1029,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -18295,7 +18297,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>430601</t>
+          <t>Bruno Guimaraes</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -18317,12 +18319,12 @@
       </c>
       <c r="B12" s="8" t="inlineStr">
         <is>
-          <t>Bruno Guimaraes</t>
+          <t>Chemsdine Talbi</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Brasil</t>
+          <t>Marokko</t>
         </is>
       </c>
       <c r="D12" s="15" t="n">
@@ -18339,12 +18341,12 @@
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Chemsdine Talbi</t>
+          <t>Crysencio Summerville</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Nederland</t>
         </is>
       </c>
       <c r="D13" s="14" t="n">
@@ -18361,12 +18363,12 @@
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>Crysencio Summerville</t>
+          <t>Florian Wirtz</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Nederland</t>
+          <t>Tyskland</t>
         </is>
       </c>
       <c r="D14" s="15" t="n">
@@ -18383,12 +18385,12 @@
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>Florian Wirtz</t>
+          <t>Gabriel Magalhães</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Tyskland</t>
+          <t>Brasil</t>
         </is>
       </c>
       <c r="D15" s="14" t="n">

</xml_diff>

<commit_message>
Stadionoversikt: inkluder sluttspill-kamper (#115)
* Fiks: vis straffesparkresultat i sluttspill-ark (#113)

FIFA API returnerer result_type=2 (e.o.) også for kamper som ble avgjort
på straffespark. Sjekk nå pen_h/pen_a direkte istedet for result_type==3,
slik at f.eks. Tyskland–Paraguay vises som "1 – 1  (e.str. 3–4)".

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

* Stadionoversikt: inkluder sluttspill-kamper

add_stadion_sheet.py leste kun kamper_resultater.json (gruppespill).
Nå leses også sluttspill_cache.json slik at 16-delsfinaler og videre
vises i Stadionoversikt-arket etterhvert som de spilles.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>

---------

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -19,13 +19,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="19" state="visible" r:id="rId19"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
@@ -18065,630 +18065,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>Sluttspill — Scorere og assists   8 mål · 6 assists</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Lag</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Kamper</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Mål</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Assist</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Casemiro</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="25" t="n"/>
-    </row>
-    <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>Cody Gakpo</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="25" t="n"/>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Gabriel Martinelli</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="25" t="n"/>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>Issa Diop</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="25" t="n"/>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Julio Enciso</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="25" t="n"/>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>Kai Havertz</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="25" t="n"/>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>Kaishu Sano</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="25" t="n"/>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>Stephen Eustaquio</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="25" t="n"/>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Bruno Guimaraes</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Chemsdine Talbi</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Crysencio Summerville</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Florian Wirtz</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Gabriel Magalhães</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Matias Galarza</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="122" t="n"/>
-      <c r="B17" s="122" t="n"/>
-      <c r="C17" s="122" t="n"/>
-      <c r="D17" s="122" t="n"/>
-      <c r="E17" s="122" t="n"/>
-      <c r="F17" s="122" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>Sluttspill — Kort   11 gule · 0 røde</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Lag</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Gule</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Røde</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Andres Cubas</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D20" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="125" t="n"/>
-    </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Casemiro</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D21" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="127" t="n"/>
-    </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Daichi Kamada</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D22" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="125" t="n"/>
-    </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Danilo</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D23" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="127" t="n"/>
-    </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Gustavo Alfaro</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D24" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="125" t="n"/>
-    </row>
-    <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Issa Diop</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D25" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="127" t="n"/>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Julian Nagelsmann</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D26" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="125" t="n"/>
-    </row>
-    <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Junnosuke Suzuki</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D27" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="127" t="n"/>
-    </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Kaishu Sano</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D28" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="125" t="n"/>
-    </row>
-    <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Nathan Saliba</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D29" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="127" t="n"/>
-    </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Niko Sigur</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D30" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="125" t="n"/>
-    </row>
-  </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A18:E18"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -18832,7 +18208,7 @@
       </c>
       <c r="C5" s="13" t="inlineStr">
         <is>
-          <t>1 – 1  (e.o.)</t>
+          <t>1 – 1  (e.str. 3–4)</t>
         </is>
       </c>
       <c r="D5" s="12" t="inlineStr">
@@ -18869,7 +18245,7 @@
       </c>
       <c r="C6" s="13" t="inlineStr">
         <is>
-          <t>1 – 1  (e.o.)</t>
+          <t>1 – 1  (e.str. 2–3)</t>
         </is>
       </c>
       <c r="D6" s="12" t="inlineStr">
@@ -19245,7 +18621,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19515,7 +18891,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19685,7 +19061,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19796,6 +19172,101 @@
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>VM 2026 — Bronsefinale</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Dato og kl.slett</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Hjemmelag</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Bortelag</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Tilskuere</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Stadion</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Dommer</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>18.07 23:00</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr"/>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>Miami Stadium</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -19826,7 +19297,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Bronsefinale</t>
+          <t>VM 2026 — Finale</t>
         </is>
       </c>
     </row>
@@ -19870,7 +19341,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>18.07 23:00</t>
+          <t>19.07 21:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -19887,7 +19358,7 @@
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Miami Stadium</t>
+          <t>New York/New Jersey Stadium</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -19906,90 +19377,619 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Finale</t>
+          <t>Sluttspill — Scorere og assists   8 mål · 6 assists</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Dato og kl.slett</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Hjemmelag</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Resultat</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Bortelag</t>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Lag</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Kamper</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Tilskuere</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Stadion</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Dommer</t>
+          <t>Mål</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Assist</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>19.07 21:00</t>
-        </is>
-      </c>
-      <c r="B3" s="21" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr"/>
-      <c r="D3" s="21" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>New York/New Jersey Stadium</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
+      <c r="A3" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Casemiro</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="25" t="n"/>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Cody Gakpo</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="25" t="n"/>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Gabriel Martinelli</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="25" t="n"/>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Issa Diop</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="25" t="n"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Julio Enciso</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="25" t="n"/>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Kai Havertz</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="25" t="n"/>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Kaishu Sano</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="25" t="n"/>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Stephen Eustaquio</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="25" t="n"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Bruno Guimaraes</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Chemsdine Talbi</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Crysencio Summerville</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Florian Wirtz</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Gabriel Magalhães</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Matias Galarza</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1">
+      <c r="A17" s="122" t="n"/>
+      <c r="B17" s="122" t="n"/>
+      <c r="C17" s="122" t="n"/>
+      <c r="D17" s="122" t="n"/>
+      <c r="E17" s="122" t="n"/>
+      <c r="F17" s="122" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Sluttspill — Kort   11 gule · 0 røde</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Lag</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Gule</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Røde</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Andres Cubas</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D20" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="125" t="n"/>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Casemiro</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D21" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="127" t="n"/>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Daichi Kamada</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D22" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="125" t="n"/>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Danilo</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D23" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="127" t="n"/>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo Alfaro</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D24" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="125" t="n"/>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Issa Diop</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="D25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="127" t="n"/>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Julian Nagelsmann</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D26" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="125" t="n"/>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Junnosuke Suzuki</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D27" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="127" t="n"/>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Kaishu Sano</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D28" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="125" t="n"/>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Nathan Saliba</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D29" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="127" t="n"/>
+    </row>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Niko Sigur</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D30" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="125" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:E18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -59107,7 +59107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K79"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -62859,57 +62859,261 @@
         <v>0.961112676056338</v>
       </c>
     </row>
+    <row r="75" ht="18" customHeight="1">
+      <c r="A75" s="70" t="inlineStr">
+        <is>
+          <t>28.06</t>
+        </is>
+      </c>
+      <c r="B75" s="87" t="inlineStr">
+        <is>
+          <t>16-delsfinaler</t>
+        </is>
+      </c>
+      <c r="C75" s="88" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="D75" s="69" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="E75" s="89" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="F75" s="88" t="inlineStr">
+        <is>
+          <t>SoFi Stadium</t>
+        </is>
+      </c>
+      <c r="G75" s="90" t="inlineStr">
+        <is>
+          <t>Inglewood / Los Angeles</t>
+        </is>
+      </c>
+      <c r="H75" s="66" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I75" s="92" t="n">
+        <v>69237</v>
+      </c>
+      <c r="J75" s="93" t="n">
+        <v>70240</v>
+      </c>
+      <c r="K75" s="102" t="n">
+        <v>0.9857203872437359</v>
+      </c>
+    </row>
     <row r="76" ht="18" customHeight="1">
-      <c r="A76" s="55" t="inlineStr">
+      <c r="A76" s="77" t="inlineStr">
+        <is>
+          <t>29.06</t>
+        </is>
+      </c>
+      <c r="B76" s="87" t="inlineStr">
+        <is>
+          <t>16-delsfinaler</t>
+        </is>
+      </c>
+      <c r="C76" s="95" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D76" s="78" t="inlineStr">
+        <is>
+          <t>2–1</t>
+        </is>
+      </c>
+      <c r="E76" s="96" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="F76" s="95" t="inlineStr">
+        <is>
+          <t>NRG Stadium</t>
+        </is>
+      </c>
+      <c r="G76" s="97" t="inlineStr">
+        <is>
+          <t>Houston</t>
+        </is>
+      </c>
+      <c r="H76" s="66" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I76" s="98" t="n">
+        <v>68777</v>
+      </c>
+      <c r="J76" s="99" t="n">
+        <v>72220</v>
+      </c>
+      <c r="K76" s="94" t="n">
+        <v>0.9523262254223206</v>
+      </c>
+    </row>
+    <row r="77" ht="18" customHeight="1">
+      <c r="A77" s="70" t="inlineStr">
+        <is>
+          <t>29.06</t>
+        </is>
+      </c>
+      <c r="B77" s="87" t="inlineStr">
+        <is>
+          <t>16-delsfinaler</t>
+        </is>
+      </c>
+      <c r="C77" s="88" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D77" s="69" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E77" s="89" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="F77" s="88" t="inlineStr">
+        <is>
+          <t>Gillette Stadium</t>
+        </is>
+      </c>
+      <c r="G77" s="90" t="inlineStr">
+        <is>
+          <t>Foxborough / Boston</t>
+        </is>
+      </c>
+      <c r="H77" s="66" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I77" s="92" t="n">
+        <v>63945</v>
+      </c>
+      <c r="J77" s="93" t="n">
+        <v>65878</v>
+      </c>
+      <c r="K77" s="102" t="n">
+        <v>0.9706578827529675</v>
+      </c>
+    </row>
+    <row r="78" ht="18" customHeight="1">
+      <c r="A78" s="77" t="inlineStr">
+        <is>
+          <t>30.06</t>
+        </is>
+      </c>
+      <c r="B78" s="87" t="inlineStr">
+        <is>
+          <t>16-delsfinaler</t>
+        </is>
+      </c>
+      <c r="C78" s="95" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D78" s="78" t="inlineStr">
+        <is>
+          <t>1–1</t>
+        </is>
+      </c>
+      <c r="E78" s="96" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="F78" s="95" t="inlineStr">
+        <is>
+          <t>Estadio BBVA</t>
+        </is>
+      </c>
+      <c r="G78" s="97" t="inlineStr">
+        <is>
+          <t>San Nicolás / Monterrey</t>
+        </is>
+      </c>
+      <c r="H78" s="91" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="I78" s="98" t="n">
+        <v>51243</v>
+      </c>
+      <c r="J78" s="99" t="n">
+        <v>53464</v>
+      </c>
+      <c r="K78" s="94" t="n">
+        <v>0.9584580278318121</v>
+      </c>
+    </row>
+    <row r="80" ht="18" customHeight="1">
+      <c r="A80" s="55" t="inlineStr">
         <is>
           <t>Belegg:</t>
         </is>
       </c>
-      <c r="B76" s="104" t="inlineStr">
+      <c r="B80" s="104" t="inlineStr">
         <is>
           <t>≥97% (praktisk utsolgt)</t>
         </is>
       </c>
-      <c r="C76" s="105" t="inlineStr">
+      <c r="C80" s="105" t="inlineStr">
         <is>
           <t>92–96%</t>
         </is>
       </c>
-      <c r="D76" s="106" t="inlineStr">
+      <c r="D80" s="106" t="inlineStr">
         <is>
           <t>87–91%</t>
         </is>
       </c>
-      <c r="E76" s="107" t="inlineStr">
+      <c r="E80" s="107" t="inlineStr">
         <is>
           <t>&lt;87%</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="14" customHeight="1">
-      <c r="A77" s="63" t="inlineStr">
+    <row r="81" ht="14" customHeight="1">
+      <c r="A81" s="63" t="inlineStr">
         <is>
           <t>Kapasitetstall: offisielle arenakapasiteter (ikke FIFA-sertifisert VM-kapasitet som kan avvike noe)</t>
         </is>
       </c>
     </row>
-    <row r="79" ht="18" customHeight="1">
-      <c r="A79" s="108" t="inlineStr">
-        <is>
-          <t>Totalt tilskuere: 4 644 549</t>
-        </is>
-      </c>
-      <c r="C79" s="108" t="inlineStr">
-        <is>
-          <t>Snitt belegg: 95.5%</t>
-        </is>
-      </c>
-      <c r="E79" s="108" t="inlineStr">
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="108" t="inlineStr">
+        <is>
+          <t>Totalt tilskuere: 4 897 751</t>
+        </is>
+      </c>
+      <c r="C83" s="108" t="inlineStr">
+        <is>
+          <t>Snitt belegg: 95.6%</t>
+        </is>
+      </c>
+      <c r="E83" s="108" t="inlineStr">
         <is>
           <t>Høyest: 80 824 (Mexico – Sør-Afrika)</t>
         </is>
       </c>
-      <c r="H79" s="108" t="inlineStr">
+      <c r="H83" s="108" t="inlineStr">
         <is>
           <t>Lavest: 42 942 (Ghana – Panama)</t>
         </is>
@@ -62917,8 +63121,8 @@
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A77:K77"/>
     <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A81:K81"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-30 06:57 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -908,13 +908,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -933,7 +933,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -957,12 +957,12 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
-        <axPos val="b"/>
+        <axPos val="l"/>
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -976,7 +976,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
-        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
@@ -989,8 +988,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1004,7 +1003,6 @@
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
-        <crosses val="autoZero"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
@@ -1014,7 +1012,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1029,9 +1027,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -18065,6 +18063,630 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>Sluttspill — Scorere og assists   8 mål · 6 assists</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Lag</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Kamper</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Mål</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Assist</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="17" customHeight="1">
+      <c r="A3" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>Casemiro</t>
+        </is>
+      </c>
+      <c r="C3" s="24" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" s="25" t="n"/>
+    </row>
+    <row r="4" ht="17" customHeight="1">
+      <c r="A4" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Cody Gakpo</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="25" t="n"/>
+    </row>
+    <row r="5" ht="17" customHeight="1">
+      <c r="A5" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Gabriel Martinelli</t>
+        </is>
+      </c>
+      <c r="C5" s="24" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D5" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="25" t="n"/>
+    </row>
+    <row r="6" ht="17" customHeight="1">
+      <c r="A6" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Issa Diop</t>
+        </is>
+      </c>
+      <c r="C6" s="24" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="25" t="n"/>
+    </row>
+    <row r="7" ht="17" customHeight="1">
+      <c r="A7" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B7" s="24" t="inlineStr">
+        <is>
+          <t>Julio Enciso</t>
+        </is>
+      </c>
+      <c r="C7" s="24" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="25" t="n"/>
+    </row>
+    <row r="8" ht="17" customHeight="1">
+      <c r="A8" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>Kai Havertz</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" s="25" t="n"/>
+    </row>
+    <row r="9" ht="17" customHeight="1">
+      <c r="A9" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>Kaishu Sano</t>
+        </is>
+      </c>
+      <c r="C9" s="24" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="25" t="n"/>
+    </row>
+    <row r="10" ht="17" customHeight="1">
+      <c r="A10" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Stephen Eustaquio</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="25" t="n"/>
+    </row>
+    <row r="11" ht="17" customHeight="1">
+      <c r="A11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Bruno Guimaraes</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="14" t="n"/>
+      <c r="F11" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" ht="17" customHeight="1">
+      <c r="A12" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="8" t="inlineStr">
+        <is>
+          <t>Chemsdine Talbi</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="17" customHeight="1">
+      <c r="A13" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Crysencio Summerville</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="17" customHeight="1">
+      <c r="A14" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B14" s="8" t="inlineStr">
+        <is>
+          <t>Florian Wirtz</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D14" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" ht="17" customHeight="1">
+      <c r="A15" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Gabriel Magalhães</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D15" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="14" t="n"/>
+      <c r="F15" s="14" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" ht="17" customHeight="1">
+      <c r="A16" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Matias Galarza</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D16" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" ht="8" customHeight="1">
+      <c r="A17" s="122" t="n"/>
+      <c r="B17" s="122" t="n"/>
+      <c r="C17" s="122" t="n"/>
+      <c r="D17" s="122" t="n"/>
+      <c r="E17" s="122" t="n"/>
+      <c r="F17" s="122" t="n"/>
+    </row>
+    <row r="18" ht="28" customHeight="1">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Sluttspill — Kort   11 gule · 0 røde</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Spiller</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Lag</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Gule</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Røde</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="17" customHeight="1">
+      <c r="A20" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Andres Cubas</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D20" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="125" t="n"/>
+    </row>
+    <row r="21" ht="17" customHeight="1">
+      <c r="A21" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B21" s="8" t="inlineStr">
+        <is>
+          <t>Casemiro</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D21" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="127" t="n"/>
+    </row>
+    <row r="22" ht="17" customHeight="1">
+      <c r="A22" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Daichi Kamada</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D22" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="125" t="n"/>
+    </row>
+    <row r="23" ht="17" customHeight="1">
+      <c r="A23" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t>Danilo</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="D23" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="127" t="n"/>
+    </row>
+    <row r="24" ht="17" customHeight="1">
+      <c r="A24" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>Gustavo Alfaro</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D24" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="125" t="n"/>
+    </row>
+    <row r="25" ht="17" customHeight="1">
+      <c r="A25" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B25" s="8" t="inlineStr">
+        <is>
+          <t>Issa Diop</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+      <c r="D25" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="127" t="n"/>
+    </row>
+    <row r="26" ht="17" customHeight="1">
+      <c r="A26" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Julian Nagelsmann</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="D26" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="125" t="n"/>
+    </row>
+    <row r="27" ht="17" customHeight="1">
+      <c r="A27" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>Junnosuke Suzuki</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D27" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="127" t="n"/>
+    </row>
+    <row r="28" ht="17" customHeight="1">
+      <c r="A28" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>Kaishu Sano</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D28" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="125" t="n"/>
+    </row>
+    <row r="29" ht="17" customHeight="1">
+      <c r="A29" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>Nathan Saliba</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D29" s="126" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="127" t="n"/>
+    </row>
+    <row r="30" ht="17" customHeight="1">
+      <c r="A30" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>Niko Sigur</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="D30" s="124" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="125" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A18:E18"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -18621,7 +19243,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -18891,7 +19513,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19061,7 +19683,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -19172,101 +19794,6 @@
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr"/>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:G3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
-        <is>
-          <t>VM 2026 — Bronsefinale</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Dato og kl.slett</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Hjemmelag</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Resultat</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Bortelag</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Tilskuere</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Stadion</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Dommer</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>18.07 23:00</t>
-        </is>
-      </c>
-      <c r="B3" s="21" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="inlineStr"/>
-      <c r="D3" s="21" t="inlineStr">
-        <is>
-          <t>TBA</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>Miami Stadium</t>
-        </is>
-      </c>
-      <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -19297,7 +19824,7 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>VM 2026 — Finale</t>
+          <t>VM 2026 — Bronsefinale</t>
         </is>
       </c>
     </row>
@@ -19341,7 +19868,7 @@
     <row r="3" ht="17" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>19.07 21:00</t>
+          <t>18.07 23:00</t>
         </is>
       </c>
       <c r="B3" s="21" t="inlineStr">
@@ -19358,7 +19885,7 @@
       <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>New York/New Jersey Stadium</t>
+          <t>Miami Stadium</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr"/>
@@ -19377,619 +19904,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="10" t="inlineStr">
         <is>
-          <t>Sluttspill — Scorere og assists   8 mål · 6 assists</t>
+          <t>VM 2026 — Finale</t>
         </is>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>#</t>
+          <t>Dato og kl.slett</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Lag</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Kamper</t>
+          <t>Hjemmelag</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Resultat</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Bortelag</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Mål</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Assist</t>
+          <t>Tilskuere</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Stadion</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Dommer</t>
         </is>
       </c>
     </row>
     <row r="3" ht="17" customHeight="1">
-      <c r="A3" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B3" s="24" t="inlineStr">
-        <is>
-          <t>Casemiro</t>
-        </is>
-      </c>
-      <c r="C3" s="24" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F3" s="25" t="n"/>
-    </row>
-    <row r="4" ht="17" customHeight="1">
-      <c r="A4" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="24" t="inlineStr">
-        <is>
-          <t>Cody Gakpo</t>
-        </is>
-      </c>
-      <c r="C4" s="24" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E4" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F4" s="25" t="n"/>
-    </row>
-    <row r="5" ht="17" customHeight="1">
-      <c r="A5" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="24" t="inlineStr">
-        <is>
-          <t>Gabriel Martinelli</t>
-        </is>
-      </c>
-      <c r="C5" s="24" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D5" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E5" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="25" t="n"/>
-    </row>
-    <row r="6" ht="17" customHeight="1">
-      <c r="A6" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="24" t="inlineStr">
-        <is>
-          <t>Issa Diop</t>
-        </is>
-      </c>
-      <c r="C6" s="24" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D6" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E6" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="25" t="n"/>
-    </row>
-    <row r="7" ht="17" customHeight="1">
-      <c r="A7" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B7" s="24" t="inlineStr">
-        <is>
-          <t>Julio Enciso</t>
-        </is>
-      </c>
-      <c r="C7" s="24" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D7" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="25" t="n"/>
-    </row>
-    <row r="8" ht="17" customHeight="1">
-      <c r="A8" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B8" s="24" t="inlineStr">
-        <is>
-          <t>Kai Havertz</t>
-        </is>
-      </c>
-      <c r="C8" s="24" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F8" s="25" t="n"/>
-    </row>
-    <row r="9" ht="17" customHeight="1">
-      <c r="A9" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B9" s="24" t="inlineStr">
-        <is>
-          <t>Kaishu Sano</t>
-        </is>
-      </c>
-      <c r="C9" s="24" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D9" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E9" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="25" t="n"/>
-    </row>
-    <row r="10" ht="17" customHeight="1">
-      <c r="A10" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="B10" s="24" t="inlineStr">
-        <is>
-          <t>Stephen Eustaquio</t>
-        </is>
-      </c>
-      <c r="C10" s="24" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D10" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="E10" s="25" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="25" t="n"/>
-    </row>
-    <row r="11" ht="17" customHeight="1">
-      <c r="A11" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Bruno Guimaraes</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D11" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E11" s="14" t="n"/>
-      <c r="F11" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" ht="17" customHeight="1">
-      <c r="A12" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
-        <is>
-          <t>Chemsdine Talbi</t>
-        </is>
-      </c>
-      <c r="C12" s="8" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E12" s="15" t="n"/>
-      <c r="F12" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" ht="17" customHeight="1">
-      <c r="A13" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Crysencio Summerville</t>
-        </is>
-      </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="D13" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" ht="17" customHeight="1">
-      <c r="A14" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Florian Wirtz</t>
-        </is>
-      </c>
-      <c r="C14" s="8" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D14" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="15" t="n"/>
-      <c r="F14" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" ht="17" customHeight="1">
-      <c r="A15" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Gabriel Magalhães</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D15" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="E15" s="14" t="n"/>
-      <c r="F15" s="14" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" ht="17" customHeight="1">
-      <c r="A16" s="7" t="n">
-        <v>9</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
-        <is>
-          <t>Matias Galarza</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D16" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="15" t="n"/>
-      <c r="F16" s="15" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" ht="8" customHeight="1">
-      <c r="A17" s="122" t="n"/>
-      <c r="B17" s="122" t="n"/>
-      <c r="C17" s="122" t="n"/>
-      <c r="D17" s="122" t="n"/>
-      <c r="E17" s="122" t="n"/>
-      <c r="F17" s="122" t="n"/>
-    </row>
-    <row r="18" ht="28" customHeight="1">
-      <c r="A18" s="10" t="inlineStr">
-        <is>
-          <t>Sluttspill — Kort   11 gule · 0 røde</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="inlineStr">
-        <is>
-          <t>Spiller</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr">
-        <is>
-          <t>Lag</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Gule</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Røde</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="17" customHeight="1">
-      <c r="A20" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>Andres Cubas</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D20" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="125" t="n"/>
-    </row>
-    <row r="21" ht="17" customHeight="1">
-      <c r="A21" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>Casemiro</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D21" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="127" t="n"/>
-    </row>
-    <row r="22" ht="17" customHeight="1">
-      <c r="A22" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Daichi Kamada</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D22" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E22" s="125" t="n"/>
-    </row>
-    <row r="23" ht="17" customHeight="1">
-      <c r="A23" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>Danilo</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="inlineStr">
-        <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="D23" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="127" t="n"/>
-    </row>
-    <row r="24" ht="17" customHeight="1">
-      <c r="A24" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>Gustavo Alfaro</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
-        </is>
-      </c>
-      <c r="D24" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="125" t="n"/>
-    </row>
-    <row r="25" ht="17" customHeight="1">
-      <c r="A25" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>Issa Diop</t>
-        </is>
-      </c>
-      <c r="C25" s="8" t="inlineStr">
-        <is>
-          <t>Marokko</t>
-        </is>
-      </c>
-      <c r="D25" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="127" t="n"/>
-    </row>
-    <row r="26" ht="17" customHeight="1">
-      <c r="A26" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B26" s="5" t="inlineStr">
-        <is>
-          <t>Julian Nagelsmann</t>
-        </is>
-      </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="D26" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="125" t="n"/>
-    </row>
-    <row r="27" ht="17" customHeight="1">
-      <c r="A27" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B27" s="8" t="inlineStr">
-        <is>
-          <t>Junnosuke Suzuki</t>
-        </is>
-      </c>
-      <c r="C27" s="8" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D27" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E27" s="127" t="n"/>
-    </row>
-    <row r="28" ht="17" customHeight="1">
-      <c r="A28" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B28" s="5" t="inlineStr">
-        <is>
-          <t>Kaishu Sano</t>
-        </is>
-      </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>Japan</t>
-        </is>
-      </c>
-      <c r="D28" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E28" s="125" t="n"/>
-    </row>
-    <row r="29" ht="17" customHeight="1">
-      <c r="A29" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>Nathan Saliba</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D29" s="126" t="n">
-        <v>1</v>
-      </c>
-      <c r="E29" s="127" t="n"/>
-    </row>
-    <row r="30" ht="17" customHeight="1">
-      <c r="A30" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>Niko Sigur</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>Canada</t>
-        </is>
-      </c>
-      <c r="D30" s="124" t="n">
-        <v>1</v>
-      </c>
-      <c r="E30" s="125" t="n"/>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>19.07 21:00</t>
+        </is>
+      </c>
+      <c r="B3" s="21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="inlineStr"/>
+      <c r="D3" s="21" t="inlineStr">
+        <is>
+          <t>TBA</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr">
+        <is>
+          <t>New York/New Jersey Stadium</t>
+        </is>
+      </c>
+      <c r="G3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A18:E18"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -51104,7 +51102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N81"/>
+  <dimension ref="A1:N82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -54824,79 +54822,127 @@
       <c r="A78" s="82" t="inlineStr"/>
       <c r="B78" s="67" t="inlineStr">
         <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="C78" s="68" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="D78" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="E78" s="70" t="n">
+        <v>2</v>
+      </c>
+      <c r="F78" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="G78" s="71" t="n">
+        <v>1</v>
+      </c>
+      <c r="H78" s="72" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I78" s="73" t="n">
+        <v>1</v>
+      </c>
+      <c r="J78" s="70" t="n">
+        <v>6</v>
+      </c>
+      <c r="K78" s="69" t="n">
+        <v>7</v>
+      </c>
+      <c r="L78" s="69" t="n">
+        <v>14</v>
+      </c>
+      <c r="M78" s="74" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N78" s="67" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="18" customHeight="1">
+      <c r="A79" s="75" t="inlineStr"/>
+      <c r="B79" s="76" t="inlineStr">
+        <is>
           <t>Tyskland</t>
         </is>
       </c>
-      <c r="C78" s="83" t="n">
+      <c r="C79" s="83" t="n">
         <v>0.75</v>
       </c>
-      <c r="D78" s="69" t="n">
+      <c r="D79" s="78" t="n">
         <v>21</v>
       </c>
-      <c r="E78" s="69" t="n">
+      <c r="E79" s="78" t="n">
         <v>7</v>
       </c>
-      <c r="F78" s="70" t="n">
+      <c r="F79" s="77" t="n">
         <v>5</v>
       </c>
-      <c r="G78" s="71" t="n">
+      <c r="G79" s="79" t="n">
         <v>9</v>
       </c>
-      <c r="H78" s="72" t="inlineStr">
+      <c r="H79" s="80" t="inlineStr">
         <is>
           <t>1–1 (pens)</t>
         </is>
       </c>
-      <c r="I78" s="73" t="n">
+      <c r="I79" s="81" t="n">
         <v>2</v>
       </c>
-      <c r="J78" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="K78" s="70" t="n">
+      <c r="J79" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="K79" s="77" t="n">
         <v>4</v>
       </c>
-      <c r="L78" s="70" t="n">
+      <c r="L79" s="77" t="n">
         <v>7</v>
       </c>
-      <c r="M78" s="74" t="n">
+      <c r="M79" s="74" t="n">
         <v>0.25</v>
       </c>
-      <c r="N78" s="67" t="inlineStr">
+      <c r="N79" s="76" t="inlineStr">
         <is>
           <t>Paraguay</t>
         </is>
       </c>
     </row>
-    <row r="80" ht="14" customHeight="1">
-      <c r="A80" s="63" t="inlineStr">
+    <row r="81" ht="14" customHeight="1">
+      <c r="A81" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="81" ht="18" customHeight="1">
-      <c r="A81" s="55" t="inlineStr">
+    <row r="82" ht="18" customHeight="1">
+      <c r="A82" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B81" s="62" t="inlineStr">
+      <c r="B82" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C81" s="61" t="inlineStr">
+      <c r="C82" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D81" s="58" t="inlineStr">
+      <c r="D82" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E81" s="85" t="inlineStr">
+      <c r="E82" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -54905,7 +54951,7 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A80:N80"/>
+    <mergeCell ref="A81:N81"/>
     <mergeCell ref="I2:N2"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-30 08:04 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -20796,7 +20796,9 @@
           <t>MF</t>
         </is>
       </c>
-      <c r="F25" s="6" t="n"/>
+      <c r="F25" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="G25" s="6" t="n"/>
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
@@ -21320,7 +21322,9 @@
       </c>
       <c r="F41" s="6" t="n"/>
       <c r="G41" s="6" t="n"/>
-      <c r="H41" s="4" t="n"/>
+      <c r="H41" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="14" t="n">
         <v>16</v>
@@ -21392,7 +21396,9 @@
       <c r="G43" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H43" s="4" t="n"/>
+      <c r="H43" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I43" s="4" t="n"/>
       <c r="J43" s="14" t="n">
         <v>145</v>
@@ -55631,7 +55637,9 @@
         </is>
       </c>
       <c r="F21" s="6" t="n"/>
-      <c r="G21" s="6" t="n"/>
+      <c r="G21" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="14" t="n">
@@ -55694,10 +55702,12 @@
           <t>MF</t>
         </is>
       </c>
-      <c r="F23" s="6" t="n"/>
+      <c r="F23" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="G23" s="6" t="n"/>
       <c r="H23" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="14" t="n">
@@ -55798,7 +55808,7 @@
       </c>
       <c r="F26" s="9" t="n"/>
       <c r="G26" s="9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
@@ -56254,7 +56264,9 @@
           <t>FW</t>
         </is>
       </c>
-      <c r="F40" s="9" t="n"/>
+      <c r="F40" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G40" s="9" t="n"/>
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="7" t="n"/>
@@ -56679,7 +56691,9 @@
         </is>
       </c>
       <c r="F54" s="6" t="n"/>
-      <c r="G54" s="6" t="n"/>
+      <c r="G54" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
       <c r="J54" s="14" t="n">
@@ -56910,10 +56924,12 @@
           <t>DF</t>
         </is>
       </c>
-      <c r="F61" s="9" t="n"/>
+      <c r="F61" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G61" s="9" t="n"/>
       <c r="H61" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="15" t="n">
@@ -65135,7 +65151,9 @@
       </c>
       <c r="F61" s="9" t="n"/>
       <c r="G61" s="9" t="n"/>
-      <c r="H61" s="7" t="n"/>
+      <c r="H61" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="15" t="n">
         <v>313</v>
@@ -65295,7 +65313,9 @@
           <t>FW</t>
         </is>
       </c>
-      <c r="F66" s="6" t="n"/>
+      <c r="F66" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="G66" s="6" t="n">
         <v>2</v>
       </c>
@@ -65428,9 +65448,11 @@
       <c r="F70" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="G70" s="6" t="n"/>
+      <c r="G70" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H70" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I70" s="4" t="n"/>
       <c r="J70" s="14" t="n">
@@ -68176,10 +68198,12 @@
         </is>
       </c>
       <c r="F25" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G25" s="6" t="n"/>
-      <c r="H25" s="4" t="n"/>
+      <c r="H25" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="14" t="n">
         <v>255</v>
@@ -68277,7 +68301,9 @@
         <v>1</v>
       </c>
       <c r="G28" s="9" t="n"/>
-      <c r="H28" s="7" t="n"/>
+      <c r="H28" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="15" t="n">
         <v>236</v>
@@ -68503,7 +68529,7 @@
       </c>
       <c r="F35" s="6" t="n"/>
       <c r="G35" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
@@ -72510,7 +72536,7 @@
         </is>
       </c>
       <c r="F29" s="6" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G29" s="6" t="n">
         <v>1</v>
@@ -72941,7 +72967,7 @@
         <v>2</v>
       </c>
       <c r="G42" s="9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H42" s="7" t="n">
         <v>1</v>
@@ -73571,7 +73597,9 @@
         <v>2</v>
       </c>
       <c r="G62" s="6" t="n"/>
-      <c r="H62" s="4" t="n"/>
+      <c r="H62" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I62" s="4" t="n"/>
       <c r="J62" s="14" t="n">
         <v>278</v>
@@ -73863,11 +73891,15 @@
           <t>DF</t>
         </is>
       </c>
-      <c r="F71" s="9" t="n"/>
+      <c r="F71" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="G71" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="H71" s="7" t="n"/>
+      <c r="H71" s="7" t="n">
+        <v>1</v>
+      </c>
       <c r="I71" s="7" t="n"/>
       <c r="J71" s="15" t="n">
         <v>199</v>
@@ -73899,7 +73931,9 @@
       </c>
       <c r="F72" s="6" t="n"/>
       <c r="G72" s="6" t="n"/>
-      <c r="H72" s="4" t="n"/>
+      <c r="H72" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="I72" s="4" t="n"/>
       <c r="J72" s="14" t="n">
         <v>23</v>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-30 08:25 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -2851,7 +2851,7 @@
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="14" t="n">
-        <v>302</v>
+        <v>402</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
@@ -2951,7 +2951,7 @@
       </c>
       <c r="I51" s="7" t="n"/>
       <c r="J51" s="15" t="n">
-        <v>202</v>
+        <v>301</v>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
@@ -2985,7 +2985,7 @@
       </c>
       <c r="I52" s="4" t="n"/>
       <c r="J52" s="14" t="n">
-        <v>242</v>
+        <v>293</v>
       </c>
     </row>
     <row r="53" ht="16" customHeight="1">
@@ -3019,7 +3019,7 @@
       </c>
       <c r="I53" s="7" t="n"/>
       <c r="J53" s="15" t="n">
-        <v>281</v>
+        <v>381</v>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
@@ -3051,7 +3051,7 @@
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
       <c r="J54" s="14" t="n">
-        <v>187</v>
+        <v>287</v>
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
@@ -3085,7 +3085,7 @@
       <c r="H55" s="7" t="n"/>
       <c r="I55" s="7" t="n"/>
       <c r="J55" s="15" t="n">
-        <v>34</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
@@ -3149,7 +3149,7 @@
       <c r="H57" s="7" t="n"/>
       <c r="I57" s="7" t="n"/>
       <c r="J57" s="15" t="n">
-        <v>135</v>
+        <v>184</v>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
@@ -3217,7 +3217,7 @@
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
       <c r="J59" s="15" t="n">
-        <v>166</v>
+        <v>255</v>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
@@ -3251,7 +3251,7 @@
         <v>1</v>
       </c>
       <c r="J60" s="14" t="n">
-        <v>152</v>
+        <v>252</v>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
@@ -3283,7 +3283,7 @@
       <c r="H61" s="7" t="n"/>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="15" t="n">
-        <v>302</v>
+        <v>402</v>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
@@ -3315,7 +3315,7 @@
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
       <c r="J62" s="14" t="n">
-        <v>171</v>
+        <v>182</v>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
@@ -3379,7 +3379,7 @@
       <c r="H64" s="4" t="n"/>
       <c r="I64" s="4" t="n"/>
       <c r="J64" s="14" t="n">
-        <v>152</v>
+        <v>241</v>
       </c>
     </row>
     <row r="65" ht="16" customHeight="1">
@@ -3477,7 +3477,7 @@
       <c r="H67" s="7" t="n"/>
       <c r="I67" s="7" t="n"/>
       <c r="J67" s="15" t="n">
-        <v>302</v>
+        <v>402</v>
       </c>
     </row>
     <row r="68" ht="16" customHeight="1">
@@ -3509,7 +3509,7 @@
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
       <c r="J68" s="14" t="n">
-        <v>302</v>
+        <v>402</v>
       </c>
     </row>
     <row r="69" ht="16" customHeight="1">
@@ -18273,7 +18273,7 @@
       </c>
       <c r="B10" s="24" t="inlineStr">
         <is>
-          <t>Stephen Eustaquio</t>
+          <t>Stephen Eustáquio</t>
         </is>
       </c>
       <c r="C10" s="24" t="inlineStr">
@@ -18295,7 +18295,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Bruno Guimaraes</t>
+          <t>Bruno Guimarães</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -18405,7 +18405,7 @@
       </c>
       <c r="B16" s="8" t="inlineStr">
         <is>
-          <t>Matias Galarza</t>
+          <t>Matías Galarza</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
@@ -18469,7 +18469,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Andres Cubas</t>
+          <t>Andrés Cubas</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -20639,7 +20639,7 @@
       </c>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="15" t="n">
-        <v>306</v>
+        <v>405</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
@@ -20705,7 +20705,7 @@
       </c>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="15" t="n">
-        <v>277</v>
+        <v>315</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -20803,7 +20803,7 @@
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="14" t="n">
-        <v>239</v>
+        <v>338</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
@@ -20905,7 +20905,7 @@
       <c r="H28" s="7" t="n"/>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="15" t="n">
-        <v>270</v>
+        <v>370</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -20939,7 +20939,7 @@
       </c>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="14" t="n">
-        <v>103</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -20971,7 +20971,7 @@
       <c r="H30" s="7" t="n"/>
       <c r="I30" s="7" t="n"/>
       <c r="J30" s="15" t="n">
-        <v>147</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" ht="16" customHeight="1">
@@ -21005,7 +21005,7 @@
       </c>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="14" t="n">
-        <v>251</v>
+        <v>351</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -21037,7 +21037,7 @@
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="7" t="n"/>
       <c r="J32" s="15" t="n">
-        <v>78</v>
+        <v>104</v>
       </c>
     </row>
     <row r="33" ht="16" customHeight="1">
@@ -21069,7 +21069,7 @@
       <c r="H33" s="4" t="n"/>
       <c r="I33" s="4" t="n"/>
       <c r="J33" s="14" t="n">
-        <v>54</v>
+        <v>115</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
@@ -21101,7 +21101,7 @@
       <c r="H34" s="7" t="n"/>
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="15" t="n">
-        <v>306</v>
+        <v>405</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -21133,7 +21133,7 @@
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="14" t="n">
-        <v>231</v>
+        <v>309</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
@@ -21196,8 +21196,8 @@
       <c r="G37" s="6" t="n"/>
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
-      <c r="J37" s="36" t="n">
-        <v>0</v>
+      <c r="J37" s="14" t="n">
+        <v>22</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
@@ -21293,7 +21293,7 @@
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="15" t="n">
-        <v>292</v>
+        <v>391</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
@@ -21327,7 +21327,7 @@
       </c>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="14" t="n">
-        <v>16</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
@@ -21363,7 +21363,7 @@
       <c r="H42" s="7" t="n"/>
       <c r="I42" s="7" t="n"/>
       <c r="J42" s="15" t="n">
-        <v>57</v>
+        <v>84</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
@@ -21401,7 +21401,7 @@
       </c>
       <c r="I43" s="4" t="n"/>
       <c r="J43" s="14" t="n">
-        <v>145</v>
+        <v>206</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
@@ -45974,7 +45974,7 @@
       </c>
       <c r="C150" s="5" t="inlineStr">
         <is>
-          <t>Yazan Alarab</t>
+          <t>Yazan Al-Arab</t>
         </is>
       </c>
       <c r="D150" s="5" t="inlineStr">
@@ -46024,7 +46024,7 @@
       </c>
       <c r="C152" s="5" t="inlineStr">
         <is>
-          <t>Damian Bobadilla</t>
+          <t>Damián Bobadilla</t>
         </is>
       </c>
       <c r="D152" s="5" t="inlineStr">
@@ -46049,7 +46049,7 @@
       </c>
       <c r="C153" s="8" t="inlineStr">
         <is>
-          <t>Hassan Altambakti</t>
+          <t>Hassan Al-Tambakti</t>
         </is>
       </c>
       <c r="D153" s="8" t="inlineStr">
@@ -55577,7 +55577,7 @@
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="14" t="n">
-        <v>308</v>
+        <v>413</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
@@ -55643,7 +55643,7 @@
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="14" t="n">
-        <v>308</v>
+        <v>413</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -55675,7 +55675,7 @@
       <c r="H22" s="7" t="n"/>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="15" t="n">
-        <v>308</v>
+        <v>413</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -55711,7 +55711,7 @@
       </c>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="14" t="n">
-        <v>221</v>
+        <v>317</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -55779,7 +55779,7 @@
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="14" t="n">
-        <v>293</v>
+        <v>398</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
@@ -55813,7 +55813,7 @@
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="15" t="n">
-        <v>273</v>
+        <v>374</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -55847,7 +55847,7 @@
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
       <c r="J27" s="14" t="n">
-        <v>191</v>
+        <v>260</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
@@ -55975,7 +55975,7 @@
       <c r="H31" s="4" t="n"/>
       <c r="I31" s="4" t="n"/>
       <c r="J31" s="14" t="n">
-        <v>259</v>
+        <v>364</v>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
@@ -56073,7 +56073,7 @@
       </c>
       <c r="I34" s="7" t="n"/>
       <c r="J34" s="15" t="n">
-        <v>293</v>
+        <v>397</v>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
@@ -56107,7 +56107,7 @@
       </c>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="14" t="n">
-        <v>86</v>
+        <v>95</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
@@ -56139,7 +56139,7 @@
       <c r="H36" s="7" t="n"/>
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="15" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -56171,7 +56171,7 @@
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
       <c r="J37" s="14" t="n">
-        <v>46</v>
+        <v>102</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
@@ -56205,7 +56205,7 @@
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="15" t="n">
-        <v>206</v>
+        <v>255</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
@@ -56271,7 +56271,7 @@
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="15" t="n">
-        <v>63</v>
+        <v>98</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
@@ -56403,7 +56403,7 @@
       <c r="H44" s="7" t="n"/>
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="15" t="n">
-        <v>149</v>
+        <v>254</v>
       </c>
     </row>
     <row r="46" ht="24" customHeight="1">
@@ -56499,7 +56499,7 @@
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="14" t="n">
-        <v>308</v>
+        <v>443</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
@@ -56535,7 +56535,7 @@
       <c r="H49" s="7" t="n"/>
       <c r="I49" s="7" t="n"/>
       <c r="J49" s="15" t="n">
-        <v>308</v>
+        <v>443</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
@@ -56567,7 +56567,7 @@
       <c r="H50" s="4" t="n"/>
       <c r="I50" s="4" t="n"/>
       <c r="J50" s="14" t="n">
-        <v>200</v>
+        <v>335</v>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
@@ -56663,7 +56663,7 @@
       <c r="H53" s="7" t="n"/>
       <c r="I53" s="7" t="n"/>
       <c r="J53" s="15" t="n">
-        <v>205</v>
+        <v>290</v>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
@@ -56697,7 +56697,7 @@
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
       <c r="J54" s="14" t="n">
-        <v>48</v>
+        <v>91</v>
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
@@ -56729,7 +56729,7 @@
       <c r="H55" s="7" t="n"/>
       <c r="I55" s="7" t="n"/>
       <c r="J55" s="15" t="n">
-        <v>191</v>
+        <v>283</v>
       </c>
     </row>
     <row r="56" ht="16" customHeight="1">
@@ -56765,7 +56765,7 @@
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
       <c r="J56" s="14" t="n">
-        <v>53</v>
+        <v>96</v>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
@@ -56799,7 +56799,7 @@
       <c r="H57" s="7" t="n"/>
       <c r="I57" s="7" t="n"/>
       <c r="J57" s="15" t="n">
-        <v>232</v>
+        <v>316</v>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
@@ -56833,7 +56833,7 @@
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
       <c r="J58" s="14" t="n">
-        <v>255</v>
+        <v>390</v>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
@@ -56864,8 +56864,8 @@
       <c r="G59" s="9" t="n"/>
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
-      <c r="J59" s="35" t="n">
-        <v>0</v>
+      <c r="J59" s="15" t="n">
+        <v>38</v>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
@@ -56933,7 +56933,7 @@
       </c>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="15" t="n">
-        <v>205</v>
+        <v>340</v>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
@@ -56965,7 +56965,7 @@
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
       <c r="J62" s="14" t="n">
-        <v>58</v>
+        <v>108</v>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
@@ -57063,7 +57063,7 @@
       <c r="H65" s="7" t="n"/>
       <c r="I65" s="7" t="n"/>
       <c r="J65" s="15" t="n">
-        <v>308</v>
+        <v>390</v>
       </c>
     </row>
     <row r="66" ht="16" customHeight="1">
@@ -57193,7 +57193,7 @@
       <c r="H69" s="7" t="n"/>
       <c r="I69" s="7" t="n"/>
       <c r="J69" s="15" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
@@ -57225,7 +57225,7 @@
       <c r="H70" s="4" t="n"/>
       <c r="I70" s="4" t="n"/>
       <c r="J70" s="14" t="n">
-        <v>274</v>
+        <v>367</v>
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
@@ -57257,7 +57257,7 @@
       <c r="H71" s="7" t="n"/>
       <c r="I71" s="7" t="n"/>
       <c r="J71" s="15" t="n">
-        <v>293</v>
+        <v>428</v>
       </c>
     </row>
     <row r="72" ht="16" customHeight="1">
@@ -57321,7 +57321,7 @@
       <c r="H73" s="7" t="n"/>
       <c r="I73" s="7" t="n"/>
       <c r="J73" s="15" t="n">
-        <v>108</v>
+        <v>162</v>
       </c>
     </row>
     <row r="75" ht="24" customHeight="1">
@@ -64758,7 +64758,7 @@
       <c r="H49" s="7" t="n"/>
       <c r="I49" s="7" t="n"/>
       <c r="J49" s="15" t="n">
-        <v>153</v>
+        <v>190</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
@@ -64824,7 +64824,7 @@
       </c>
       <c r="I51" s="7" t="n"/>
       <c r="J51" s="15" t="n">
-        <v>276</v>
+        <v>384</v>
       </c>
     </row>
     <row r="52" ht="16" customHeight="1">
@@ -64890,7 +64890,7 @@
       </c>
       <c r="I53" s="7" t="n"/>
       <c r="J53" s="15" t="n">
-        <v>216</v>
+        <v>352</v>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
@@ -64988,7 +64988,7 @@
       <c r="H56" s="4" t="n"/>
       <c r="I56" s="4" t="n"/>
       <c r="J56" s="14" t="n">
-        <v>66</v>
+        <v>95</v>
       </c>
     </row>
     <row r="57" ht="16" customHeight="1">
@@ -65024,7 +65024,7 @@
         <v>1</v>
       </c>
       <c r="J57" s="15" t="n">
-        <v>131</v>
+        <v>231</v>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
@@ -65058,7 +65058,7 @@
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
       <c r="J58" s="14" t="n">
-        <v>103</v>
+        <v>178</v>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
@@ -65090,7 +65090,7 @@
       <c r="H59" s="7" t="n"/>
       <c r="I59" s="7" t="n"/>
       <c r="J59" s="15" t="n">
-        <v>313</v>
+        <v>451</v>
       </c>
     </row>
     <row r="60" ht="16" customHeight="1">
@@ -65122,7 +65122,7 @@
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
       <c r="J60" s="14" t="n">
-        <v>18</v>
+        <v>156</v>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
@@ -65156,7 +65156,7 @@
       </c>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="15" t="n">
-        <v>313</v>
+        <v>451</v>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
@@ -65188,7 +65188,7 @@
       <c r="H62" s="4" t="n"/>
       <c r="I62" s="4" t="n"/>
       <c r="J62" s="14" t="n">
-        <v>313</v>
+        <v>451</v>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
@@ -65220,7 +65220,7 @@
       <c r="H63" s="7" t="n"/>
       <c r="I63" s="7" t="n"/>
       <c r="J63" s="15" t="n">
-        <v>107</v>
+        <v>216</v>
       </c>
     </row>
     <row r="64" ht="16" customHeight="1">
@@ -65322,7 +65322,7 @@
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
       <c r="J66" s="14" t="n">
-        <v>305</v>
+        <v>367</v>
       </c>
     </row>
     <row r="67" ht="16" customHeight="1">
@@ -65353,8 +65353,8 @@
       <c r="G67" s="9" t="n"/>
       <c r="H67" s="7" t="n"/>
       <c r="I67" s="7" t="n"/>
-      <c r="J67" s="35" t="n">
-        <v>0</v>
+      <c r="J67" s="15" t="n">
+        <v>28</v>
       </c>
     </row>
     <row r="68" ht="16" customHeight="1">
@@ -65386,7 +65386,7 @@
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
       <c r="J68" s="14" t="n">
-        <v>81</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69" ht="16" customHeight="1">
@@ -65456,7 +65456,7 @@
       </c>
       <c r="I70" s="4" t="n"/>
       <c r="J70" s="14" t="n">
-        <v>199</v>
+        <v>336</v>
       </c>
     </row>
     <row r="71" ht="16" customHeight="1">
@@ -65487,8 +65487,8 @@
       <c r="G71" s="9" t="n"/>
       <c r="H71" s="7" t="n"/>
       <c r="I71" s="7" t="n"/>
-      <c r="J71" s="35" t="n">
-        <v>0</v>
+      <c r="J71" s="15" t="n">
+        <v>77</v>
       </c>
     </row>
     <row r="72" ht="16" customHeight="1">
@@ -68006,7 +68006,7 @@
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="14" t="n">
-        <v>305</v>
+        <v>442</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
@@ -68038,7 +68038,7 @@
       <c r="H20" s="7" t="n"/>
       <c r="I20" s="7" t="n"/>
       <c r="J20" s="15" t="n">
-        <v>176</v>
+        <v>300</v>
       </c>
     </row>
     <row r="21" ht="16" customHeight="1">
@@ -68070,7 +68070,7 @@
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
       <c r="J21" s="14" t="n">
-        <v>12</v>
+        <v>66</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -68102,7 +68102,7 @@
       <c r="H22" s="7" t="n"/>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="15" t="n">
-        <v>282</v>
+        <v>419</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -68136,7 +68136,7 @@
       </c>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="14" t="n">
-        <v>216</v>
+        <v>300</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -68170,7 +68170,7 @@
       <c r="H24" s="7" t="n"/>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="15" t="n">
-        <v>255</v>
+        <v>392</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -68206,7 +68206,7 @@
       </c>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="14" t="n">
-        <v>255</v>
+        <v>392</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
@@ -68238,7 +68238,7 @@
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="15" t="n">
-        <v>35</v>
+        <v>122</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -68306,7 +68306,7 @@
       </c>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="15" t="n">
-        <v>236</v>
+        <v>305</v>
       </c>
     </row>
     <row r="29" ht="16" customHeight="1">
@@ -68337,8 +68337,8 @@
       <c r="G29" s="6" t="n"/>
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
-      <c r="J29" s="36" t="n">
-        <v>0</v>
+      <c r="J29" s="14" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -68534,7 +68534,7 @@
       <c r="H35" s="4" t="n"/>
       <c r="I35" s="4" t="n"/>
       <c r="J35" s="14" t="n">
-        <v>281</v>
+        <v>405</v>
       </c>
     </row>
     <row r="36" ht="16" customHeight="1">
@@ -68570,7 +68570,7 @@
       <c r="H36" s="7" t="n"/>
       <c r="I36" s="7" t="n"/>
       <c r="J36" s="15" t="n">
-        <v>181</v>
+        <v>319</v>
       </c>
     </row>
     <row r="37" ht="16" customHeight="1">
@@ -68604,7 +68604,7 @@
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
       <c r="J37" s="14" t="n">
-        <v>268</v>
+        <v>360</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
@@ -68638,7 +68638,7 @@
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="15" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
@@ -68738,7 +68738,7 @@
       <c r="H41" s="4" t="n"/>
       <c r="I41" s="4" t="n"/>
       <c r="J41" s="14" t="n">
-        <v>249</v>
+        <v>299</v>
       </c>
     </row>
     <row r="42" ht="16" customHeight="1">
@@ -68770,7 +68770,7 @@
       <c r="H42" s="7" t="n"/>
       <c r="I42" s="7" t="n"/>
       <c r="J42" s="15" t="n">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
@@ -68838,7 +68838,7 @@
       <c r="H44" s="7" t="n"/>
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="15" t="n">
-        <v>106</v>
+        <v>174</v>
       </c>
     </row>
     <row r="46" ht="24" customHeight="1">
@@ -72208,7 +72208,7 @@
       <c r="H19" s="4" t="n"/>
       <c r="I19" s="4" t="n"/>
       <c r="J19" s="14" t="n">
-        <v>297</v>
+        <v>432</v>
       </c>
     </row>
     <row r="20" ht="16" customHeight="1">
@@ -72271,8 +72271,8 @@
       <c r="G21" s="6" t="n"/>
       <c r="H21" s="4" t="n"/>
       <c r="I21" s="4" t="n"/>
-      <c r="J21" s="36" t="n">
-        <v>0</v>
+      <c r="J21" s="14" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="22" ht="16" customHeight="1">
@@ -72308,7 +72308,7 @@
       <c r="H22" s="7" t="n"/>
       <c r="I22" s="7" t="n"/>
       <c r="J22" s="15" t="n">
-        <v>297</v>
+        <v>432</v>
       </c>
     </row>
     <row r="23" ht="16" customHeight="1">
@@ -72340,7 +72340,7 @@
       <c r="H23" s="4" t="n"/>
       <c r="I23" s="4" t="n"/>
       <c r="J23" s="14" t="n">
-        <v>113</v>
+        <v>189</v>
       </c>
     </row>
     <row r="24" ht="16" customHeight="1">
@@ -72374,7 +72374,7 @@
       <c r="H24" s="7" t="n"/>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="15" t="n">
-        <v>297</v>
+        <v>432</v>
       </c>
     </row>
     <row r="25" ht="16" customHeight="1">
@@ -72406,7 +72406,7 @@
       <c r="H25" s="4" t="n"/>
       <c r="I25" s="4" t="n"/>
       <c r="J25" s="14" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
@@ -72440,7 +72440,7 @@
       <c r="H26" s="7" t="n"/>
       <c r="I26" s="7" t="n"/>
       <c r="J26" s="15" t="n">
-        <v>282</v>
+        <v>374</v>
       </c>
     </row>
     <row r="27" ht="16" customHeight="1">
@@ -72471,8 +72471,8 @@
       <c r="G27" s="6" t="n"/>
       <c r="H27" s="4" t="n"/>
       <c r="I27" s="4" t="n"/>
-      <c r="J27" s="36" t="n">
-        <v>0</v>
+      <c r="J27" s="14" t="n">
+        <v>58</v>
       </c>
     </row>
     <row r="28" ht="16" customHeight="1">
@@ -72544,7 +72544,7 @@
       <c r="H29" s="4" t="n"/>
       <c r="I29" s="4" t="n"/>
       <c r="J29" s="14" t="n">
-        <v>268</v>
+        <v>394</v>
       </c>
     </row>
     <row r="30" ht="16" customHeight="1">
@@ -72676,7 +72676,7 @@
       </c>
       <c r="I33" s="4" t="n"/>
       <c r="J33" s="14" t="n">
-        <v>199</v>
+        <v>291</v>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
@@ -72806,7 +72806,7 @@
       <c r="H37" s="4" t="n"/>
       <c r="I37" s="4" t="n"/>
       <c r="J37" s="14" t="n">
-        <v>168</v>
+        <v>245</v>
       </c>
     </row>
     <row r="38" ht="16" customHeight="1">
@@ -72838,7 +72838,7 @@
       <c r="H38" s="7" t="n"/>
       <c r="I38" s="7" t="n"/>
       <c r="J38" s="15" t="n">
-        <v>86</v>
+        <v>145</v>
       </c>
     </row>
     <row r="39" ht="16" customHeight="1">
@@ -72870,7 +72870,7 @@
       <c r="H39" s="4" t="n"/>
       <c r="I39" s="4" t="n"/>
       <c r="J39" s="14" t="n">
-        <v>236</v>
+        <v>360</v>
       </c>
     </row>
     <row r="40" ht="16" customHeight="1">
@@ -72904,7 +72904,7 @@
       <c r="H40" s="7" t="n"/>
       <c r="I40" s="7" t="n"/>
       <c r="J40" s="15" t="n">
-        <v>297</v>
+        <v>432</v>
       </c>
     </row>
     <row r="41" ht="16" customHeight="1">
@@ -72974,7 +72974,7 @@
       </c>
       <c r="I42" s="7" t="n"/>
       <c r="J42" s="15" t="n">
-        <v>147</v>
+        <v>282</v>
       </c>
     </row>
     <row r="43" ht="16" customHeight="1">
@@ -73005,8 +73005,8 @@
       <c r="G43" s="6" t="n"/>
       <c r="H43" s="4" t="n"/>
       <c r="I43" s="4" t="n"/>
-      <c r="J43" s="36" t="n">
-        <v>0</v>
+      <c r="J43" s="14" t="n">
+        <v>43</v>
       </c>
     </row>
     <row r="44" ht="16" customHeight="1">
@@ -73038,7 +73038,7 @@
       <c r="H44" s="7" t="n"/>
       <c r="I44" s="7" t="n"/>
       <c r="J44" s="15" t="n">
-        <v>25</v>
+        <v>68</v>
       </c>
     </row>
     <row r="46" ht="24" customHeight="1">
@@ -73134,7 +73134,7 @@
       <c r="H48" s="4" t="n"/>
       <c r="I48" s="4" t="n"/>
       <c r="J48" s="14" t="n">
-        <v>301</v>
+        <v>405</v>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
@@ -73166,7 +73166,7 @@
       <c r="H49" s="7" t="n"/>
       <c r="I49" s="7" t="n"/>
       <c r="J49" s="15" t="n">
-        <v>146</v>
+        <v>181</v>
       </c>
     </row>
     <row r="50" ht="16" customHeight="1">
@@ -73200,7 +73200,7 @@
       </c>
       <c r="I50" s="4" t="n"/>
       <c r="J50" s="14" t="n">
-        <v>162</v>
+        <v>267</v>
       </c>
     </row>
     <row r="51" ht="16" customHeight="1">
@@ -73297,8 +73297,8 @@
       <c r="G53" s="9" t="n"/>
       <c r="H53" s="7" t="n"/>
       <c r="I53" s="7" t="n"/>
-      <c r="J53" s="35" t="n">
-        <v>0</v>
+      <c r="J53" s="15" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="54" ht="16" customHeight="1">
@@ -73330,7 +73330,7 @@
       <c r="H54" s="4" t="n"/>
       <c r="I54" s="4" t="n"/>
       <c r="J54" s="14" t="n">
-        <v>202</v>
+        <v>225</v>
       </c>
     </row>
     <row r="55" ht="16" customHeight="1">
@@ -73430,7 +73430,7 @@
       <c r="H57" s="7" t="n"/>
       <c r="I57" s="7" t="n"/>
       <c r="J57" s="15" t="n">
-        <v>225</v>
+        <v>295</v>
       </c>
     </row>
     <row r="58" ht="16" customHeight="1">
@@ -73464,7 +73464,7 @@
       <c r="H58" s="4" t="n"/>
       <c r="I58" s="4" t="n"/>
       <c r="J58" s="14" t="n">
-        <v>170</v>
+        <v>271</v>
       </c>
     </row>
     <row r="59" ht="16" customHeight="1">
@@ -73532,7 +73532,7 @@
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
       <c r="J60" s="14" t="n">
-        <v>260</v>
+        <v>330</v>
       </c>
     </row>
     <row r="61" ht="16" customHeight="1">
@@ -73566,7 +73566,7 @@
       <c r="H61" s="7" t="n"/>
       <c r="I61" s="7" t="n"/>
       <c r="J61" s="15" t="n">
-        <v>161</v>
+        <v>242</v>
       </c>
     </row>
     <row r="62" ht="16" customHeight="1">
@@ -73602,7 +73602,7 @@
       </c>
       <c r="I62" s="4" t="n"/>
       <c r="J62" s="14" t="n">
-        <v>278</v>
+        <v>359</v>
       </c>
     </row>
     <row r="63" ht="16" customHeight="1">
@@ -73702,7 +73702,7 @@
       <c r="H65" s="7" t="n"/>
       <c r="I65" s="7" t="n"/>
       <c r="J65" s="15" t="n">
-        <v>245</v>
+        <v>349</v>
       </c>
     </row>
     <row r="66" ht="16" customHeight="1">
@@ -73736,7 +73736,7 @@
       <c r="H66" s="4" t="n"/>
       <c r="I66" s="4" t="n"/>
       <c r="J66" s="14" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="67" ht="16" customHeight="1">
@@ -73800,7 +73800,7 @@
       <c r="H68" s="4" t="n"/>
       <c r="I68" s="4" t="n"/>
       <c r="J68" s="14" t="n">
-        <v>301</v>
+        <v>405</v>
       </c>
     </row>
     <row r="69" ht="16" customHeight="1">
@@ -73832,7 +73832,7 @@
       <c r="H69" s="7" t="n"/>
       <c r="I69" s="7" t="n"/>
       <c r="J69" s="15" t="n">
-        <v>103</v>
+        <v>208</v>
       </c>
     </row>
     <row r="70" ht="16" customHeight="1">
@@ -73902,7 +73902,7 @@
       </c>
       <c r="I71" s="7" t="n"/>
       <c r="J71" s="15" t="n">
-        <v>199</v>
+        <v>303</v>
       </c>
     </row>
     <row r="72" ht="16" customHeight="1">
@@ -73936,7 +73936,7 @@
       </c>
       <c r="I72" s="4" t="n"/>
       <c r="J72" s="14" t="n">
-        <v>23</v>
+        <v>58</v>
       </c>
     </row>
     <row r="73" ht="16" customHeight="1">

</xml_diff>

<commit_message>
Auto-oppdatering 2026-06-30 08:43 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -9148,8 +9148,12 @@
           <t>FW</t>
         </is>
       </c>
-      <c r="F115" s="9" t="n"/>
-      <c r="G115" s="9" t="n"/>
+      <c r="F115" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G115" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="H115" s="7" t="n"/>
       <c r="I115" s="7" t="n"/>
       <c r="J115" s="15" t="n">
@@ -9567,7 +9571,9 @@
         </is>
       </c>
       <c r="F128" s="6" t="n"/>
-      <c r="G128" s="6" t="n"/>
+      <c r="G128" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H128" s="4" t="n"/>
       <c r="I128" s="4" t="n"/>
       <c r="J128" s="14" t="n">
@@ -11601,7 +11607,9 @@
         </is>
       </c>
       <c r="F60" s="6" t="n"/>
-      <c r="G60" s="6" t="n"/>
+      <c r="G60" s="6" t="n">
+        <v>1</v>
+      </c>
       <c r="H60" s="4" t="n"/>
       <c r="I60" s="4" t="n"/>
       <c r="J60" s="14" t="n">
@@ -13657,7 +13665,9 @@
         </is>
       </c>
       <c r="F125" s="9" t="n"/>
-      <c r="G125" s="9" t="n"/>
+      <c r="G125" s="9" t="n">
+        <v>1</v>
+      </c>
       <c r="H125" s="7" t="n"/>
       <c r="I125" s="7" t="n"/>
       <c r="J125" s="15" t="n">

</xml_diff>

<commit_message>
Regenerer Ballbesittelse-ark med Belgia-Senegal og England-DR Kongo stats
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -911,13 +911,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -936,7 +936,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -964,8 +964,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -991,8 +991,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1015,7 +1015,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1030,9 +1030,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -51614,7 +51614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N85"/>
+  <dimension ref="A1:N87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55238,47 +55238,47 @@
       </c>
       <c r="B76" s="67" t="inlineStr">
         <is>
-          <t>Brasil</t>
-        </is>
-      </c>
-      <c r="C76" s="68" t="n">
-        <v>0.6</v>
+          <t>Belgia</t>
+        </is>
+      </c>
+      <c r="C76" s="84" t="n">
+        <v>0.53</v>
       </c>
       <c r="D76" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="E76" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="F76" s="70" t="n">
+        <v>10</v>
+      </c>
+      <c r="G76" s="71" t="n">
+        <v>6</v>
+      </c>
+      <c r="H76" s="72" t="inlineStr">
+        <is>
+          <t>3–2 (aet)</t>
+        </is>
+      </c>
+      <c r="I76" s="73" t="n">
+        <v>3</v>
+      </c>
+      <c r="J76" s="70" t="n">
+        <v>11</v>
+      </c>
+      <c r="K76" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="L76" s="70" t="n">
         <v>20</v>
       </c>
-      <c r="E76" s="69" t="n">
-        <v>7</v>
-      </c>
-      <c r="F76" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="G76" s="71" t="n">
-        <v>8</v>
-      </c>
-      <c r="H76" s="72" t="inlineStr">
-        <is>
-          <t>2–1</t>
-        </is>
-      </c>
-      <c r="I76" s="73" t="n">
-        <v>2</v>
-      </c>
-      <c r="J76" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="K76" s="70" t="n">
-        <v>2</v>
-      </c>
-      <c r="L76" s="70" t="n">
-        <v>5</v>
-      </c>
-      <c r="M76" s="74" t="n">
-        <v>0.4</v>
+      <c r="M76" s="84" t="n">
+        <v>0.47</v>
       </c>
       <c r="N76" s="67" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Senegal</t>
         </is>
       </c>
     </row>
@@ -55286,47 +55286,47 @@
       <c r="A77" s="75" t="inlineStr"/>
       <c r="B77" s="76" t="inlineStr">
         <is>
-          <t>Elfenbenskysten</t>
-        </is>
-      </c>
-      <c r="C77" s="84" t="n">
-        <v>0.52</v>
+          <t>Brasil</t>
+        </is>
+      </c>
+      <c r="C77" s="68" t="n">
+        <v>0.6</v>
       </c>
       <c r="D77" s="78" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="E77" s="78" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F77" s="77" t="n">
         <v>5</v>
       </c>
       <c r="G77" s="79" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="H77" s="80" t="inlineStr">
         <is>
-          <t>1–2</t>
+          <t>2–1</t>
         </is>
       </c>
       <c r="I77" s="81" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J77" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="K77" s="77" t="n">
         <v>2</v>
       </c>
-      <c r="K77" s="77" t="n">
-        <v>3</v>
-      </c>
       <c r="L77" s="77" t="n">
-        <v>9</v>
-      </c>
-      <c r="M77" s="84" t="n">
-        <v>0.48</v>
+        <v>5</v>
+      </c>
+      <c r="M77" s="74" t="n">
+        <v>0.4</v>
       </c>
       <c r="N77" s="76" t="inlineStr">
         <is>
-          <t>Norge</t>
+          <t>Japan</t>
         </is>
       </c>
     </row>
@@ -55334,47 +55334,47 @@
       <c r="A78" s="82" t="inlineStr"/>
       <c r="B78" s="67" t="inlineStr">
         <is>
-          <t>Frankrike</t>
-        </is>
-      </c>
-      <c r="C78" s="68" t="n">
-        <v>0.61</v>
+          <t>Elfenbenskysten</t>
+        </is>
+      </c>
+      <c r="C78" s="84" t="n">
+        <v>0.52</v>
       </c>
       <c r="D78" s="69" t="n">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E78" s="69" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="F78" s="70" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="G78" s="71" t="n">
         <v>4</v>
       </c>
       <c r="H78" s="72" t="inlineStr">
         <is>
-          <t>3–0</t>
+          <t>1–2</t>
         </is>
       </c>
       <c r="I78" s="73" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J78" s="70" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K78" s="70" t="n">
         <v>3</v>
       </c>
       <c r="L78" s="70" t="n">
-        <v>8</v>
-      </c>
-      <c r="M78" s="74" t="n">
-        <v>0.39</v>
+        <v>9</v>
+      </c>
+      <c r="M78" s="84" t="n">
+        <v>0.48</v>
       </c>
       <c r="N78" s="67" t="inlineStr">
         <is>
-          <t>Sverige</t>
+          <t>Norge</t>
         </is>
       </c>
     </row>
@@ -55382,47 +55382,47 @@
       <c r="A79" s="75" t="inlineStr"/>
       <c r="B79" s="76" t="inlineStr">
         <is>
-          <t>Mexico</t>
-        </is>
-      </c>
-      <c r="C79" s="74" t="n">
-        <v>0.43</v>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="C79" s="84" t="n">
+        <v>0.54</v>
       </c>
       <c r="D79" s="78" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E79" s="78" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F79" s="77" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="G79" s="79" t="n">
         <v>3</v>
       </c>
       <c r="H79" s="80" t="inlineStr">
         <is>
-          <t>2–0</t>
+          <t>2–1</t>
         </is>
       </c>
       <c r="I79" s="81" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J79" s="77" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="K79" s="77" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L79" s="77" t="n">
-        <v>8</v>
-      </c>
-      <c r="M79" s="68" t="n">
-        <v>0.57</v>
+        <v>7</v>
+      </c>
+      <c r="M79" s="84" t="n">
+        <v>0.46</v>
       </c>
       <c r="N79" s="76" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>DR Kongo</t>
         </is>
       </c>
     </row>
@@ -55430,47 +55430,47 @@
       <c r="A80" s="82" t="inlineStr"/>
       <c r="B80" s="67" t="inlineStr">
         <is>
-          <t>Nederland</t>
-        </is>
-      </c>
-      <c r="C80" s="74" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D80" s="70" t="n">
-        <v>7</v>
-      </c>
-      <c r="E80" s="70" t="n">
-        <v>3</v>
+          <t>Frankrike</t>
+        </is>
+      </c>
+      <c r="C80" s="68" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="D80" s="69" t="n">
+        <v>25</v>
+      </c>
+      <c r="E80" s="69" t="n">
+        <v>13</v>
       </c>
       <c r="F80" s="70" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G80" s="71" t="n">
         <v>4</v>
       </c>
       <c r="H80" s="72" t="inlineStr">
         <is>
-          <t>1–1 (pens)</t>
+          <t>3–0</t>
         </is>
       </c>
       <c r="I80" s="73" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J80" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="K80" s="69" t="n">
-        <v>6</v>
-      </c>
-      <c r="L80" s="69" t="n">
-        <v>12</v>
-      </c>
-      <c r="M80" s="83" t="n">
-        <v>0.7</v>
+      <c r="K80" s="70" t="n">
+        <v>3</v>
+      </c>
+      <c r="L80" s="70" t="n">
+        <v>8</v>
+      </c>
+      <c r="M80" s="74" t="n">
+        <v>0.39</v>
       </c>
       <c r="N80" s="67" t="inlineStr">
         <is>
-          <t>Marokko</t>
+          <t>Sverige</t>
         </is>
       </c>
     </row>
@@ -55478,27 +55478,27 @@
       <c r="A81" s="75" t="inlineStr"/>
       <c r="B81" s="76" t="inlineStr">
         <is>
-          <t>Sør-Afrika</t>
-        </is>
-      </c>
-      <c r="C81" s="68" t="n">
-        <v>0.58</v>
-      </c>
-      <c r="D81" s="77" t="n">
-        <v>6</v>
-      </c>
-      <c r="E81" s="77" t="n">
-        <v>2</v>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C81" s="74" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="D81" s="78" t="n">
+        <v>15</v>
+      </c>
+      <c r="E81" s="78" t="n">
+        <v>3</v>
       </c>
       <c r="F81" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="G81" s="79" t="n">
         <v>3</v>
       </c>
-      <c r="G81" s="79" t="n">
-        <v>1</v>
-      </c>
       <c r="H81" s="80" t="inlineStr">
         <is>
-          <t>0–1</t>
+          <t>2–0</t>
         </is>
       </c>
       <c r="I81" s="81" t="n">
@@ -55507,18 +55507,18 @@
       <c r="J81" s="77" t="n">
         <v>6</v>
       </c>
-      <c r="K81" s="78" t="n">
-        <v>7</v>
-      </c>
-      <c r="L81" s="78" t="n">
-        <v>14</v>
-      </c>
-      <c r="M81" s="74" t="n">
-        <v>0.42</v>
+      <c r="K81" s="77" t="n">
+        <v>1</v>
+      </c>
+      <c r="L81" s="77" t="n">
+        <v>8</v>
+      </c>
+      <c r="M81" s="68" t="n">
+        <v>0.57</v>
       </c>
       <c r="N81" s="76" t="inlineStr">
         <is>
-          <t>Canada</t>
+          <t>Ecuador</t>
         </is>
       </c>
     </row>
@@ -55526,23 +55526,23 @@
       <c r="A82" s="82" t="inlineStr"/>
       <c r="B82" s="67" t="inlineStr">
         <is>
-          <t>Tyskland</t>
-        </is>
-      </c>
-      <c r="C82" s="83" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="D82" s="69" t="n">
-        <v>21</v>
-      </c>
-      <c r="E82" s="69" t="n">
+          <t>Nederland</t>
+        </is>
+      </c>
+      <c r="C82" s="74" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D82" s="70" t="n">
         <v>7</v>
       </c>
+      <c r="E82" s="70" t="n">
+        <v>3</v>
+      </c>
       <c r="F82" s="70" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G82" s="71" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="H82" s="72" t="inlineStr">
         <is>
@@ -55553,52 +55553,148 @@
         <v>2</v>
       </c>
       <c r="J82" s="70" t="n">
-        <v>1</v>
-      </c>
-      <c r="K82" s="70" t="n">
         <v>4</v>
       </c>
-      <c r="L82" s="70" t="n">
+      <c r="K82" s="69" t="n">
+        <v>6</v>
+      </c>
+      <c r="L82" s="69" t="n">
+        <v>12</v>
+      </c>
+      <c r="M82" s="83" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="N82" s="67" t="inlineStr">
+        <is>
+          <t>Marokko</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="18" customHeight="1">
+      <c r="A83" s="75" t="inlineStr"/>
+      <c r="B83" s="76" t="inlineStr">
+        <is>
+          <t>Sør-Afrika</t>
+        </is>
+      </c>
+      <c r="C83" s="68" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="D83" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="E83" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" s="77" t="n">
+        <v>3</v>
+      </c>
+      <c r="G83" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="H83" s="80" t="inlineStr">
+        <is>
+          <t>0–1</t>
+        </is>
+      </c>
+      <c r="I83" s="81" t="n">
+        <v>1</v>
+      </c>
+      <c r="J83" s="77" t="n">
+        <v>6</v>
+      </c>
+      <c r="K83" s="78" t="n">
         <v>7</v>
       </c>
-      <c r="M82" s="74" t="n">
+      <c r="L83" s="78" t="n">
+        <v>14</v>
+      </c>
+      <c r="M83" s="74" t="n">
+        <v>0.42</v>
+      </c>
+      <c r="N83" s="76" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="82" t="inlineStr"/>
+      <c r="B84" s="67" t="inlineStr">
+        <is>
+          <t>Tyskland</t>
+        </is>
+      </c>
+      <c r="C84" s="83" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="D84" s="69" t="n">
+        <v>21</v>
+      </c>
+      <c r="E84" s="69" t="n">
+        <v>7</v>
+      </c>
+      <c r="F84" s="70" t="n">
+        <v>5</v>
+      </c>
+      <c r="G84" s="71" t="n">
+        <v>9</v>
+      </c>
+      <c r="H84" s="72" t="inlineStr">
+        <is>
+          <t>1–1 (pens)</t>
+        </is>
+      </c>
+      <c r="I84" s="73" t="n">
+        <v>2</v>
+      </c>
+      <c r="J84" s="70" t="n">
+        <v>1</v>
+      </c>
+      <c r="K84" s="70" t="n">
+        <v>4</v>
+      </c>
+      <c r="L84" s="70" t="n">
+        <v>7</v>
+      </c>
+      <c r="M84" s="74" t="n">
         <v>0.25</v>
       </c>
-      <c r="N82" s="67" t="inlineStr">
+      <c r="N84" s="67" t="inlineStr">
         <is>
           <t>Paraguay</t>
         </is>
       </c>
     </row>
-    <row r="84" ht="14" customHeight="1">
-      <c r="A84" s="63" t="inlineStr">
+    <row r="86" ht="14" customHeight="1">
+      <c r="A86" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="85" ht="18" customHeight="1">
-      <c r="A85" s="55" t="inlineStr">
+    <row r="87" ht="18" customHeight="1">
+      <c r="A87" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B85" s="62" t="inlineStr">
+      <c r="B87" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C85" s="61" t="inlineStr">
+      <c r="C87" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D85" s="58" t="inlineStr">
+      <c r="D87" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E85" s="85" t="inlineStr">
+      <c r="E87" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -55607,8 +55703,8 @@
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="B2:G2"/>
-    <mergeCell ref="A84:N84"/>
     <mergeCell ref="I2:N2"/>
+    <mergeCell ref="A86:N86"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Regenerer Ballbesittelse-ark med USA-Bosnia-Hercegovina stats
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -51614,7 +51614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -55666,35 +55666,83 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="14" customHeight="1">
-      <c r="A86" s="63" t="inlineStr">
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="75" t="inlineStr"/>
+      <c r="B85" s="76" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C85" s="84" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D85" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="G85" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H85" s="80" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I85" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="L85" s="78" t="n">
+        <v>11</v>
+      </c>
+      <c r="M85" s="84" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="N85" s="76" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="14" customHeight="1">
+      <c r="A87" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="55" t="inlineStr">
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B87" s="62" t="inlineStr">
+      <c r="B88" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C87" s="61" t="inlineStr">
+      <c r="C88" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D87" s="58" t="inlineStr">
+      <c r="D88" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E87" s="85" t="inlineStr">
+      <c r="E88" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -55702,9 +55750,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A87:N87"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="I2:N2"/>
-    <mergeCell ref="A86:N86"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Regenerer Ballbesittelse-ark på nyeste main med USA-Bosnia-Hercegovina stats
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -914,13 +914,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -939,7 +939,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -967,8 +967,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -994,8 +994,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1018,7 +1018,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1033,9 +1033,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -52323,7 +52323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -56375,35 +56375,83 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="14" customHeight="1">
-      <c r="A86" s="63" t="inlineStr">
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="75" t="inlineStr"/>
+      <c r="B85" s="76" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C85" s="84" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D85" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="G85" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H85" s="80" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I85" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="L85" s="78" t="n">
+        <v>11</v>
+      </c>
+      <c r="M85" s="84" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="N85" s="76" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="14" customHeight="1">
+      <c r="A87" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="55" t="inlineStr">
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B87" s="62" t="inlineStr">
+      <c r="B88" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C87" s="61" t="inlineStr">
+      <c r="C88" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D87" s="58" t="inlineStr">
+      <c r="D88" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E87" s="85" t="inlineStr">
+      <c r="E88" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -56411,9 +56459,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A87:N87"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="I2:N2"/>
-    <mergeCell ref="A86:N86"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Oppdater kampstatistikk for USA-Bosnia-Hercegovina (#139)
* Oppdater kampstatistikk for USA-Bosnia-Hercegovina

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Regenerer Ballbesittelse-ark med USA-Bosnia-Hercegovina stats

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

* Regenerer Ballbesittelse-ark på nyeste main med USA-Bosnia-Hercegovina stats

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>

---------

Co-authored-by: cathrinei <cathrine@gnist.as>
Co-authored-by: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -914,13 +914,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -939,7 +939,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -967,8 +967,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -994,8 +994,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1018,7 +1018,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1033,9 +1033,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -52323,7 +52323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -56375,35 +56375,83 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="14" customHeight="1">
-      <c r="A86" s="63" t="inlineStr">
+    <row r="85" ht="18" customHeight="1">
+      <c r="A85" s="75" t="inlineStr"/>
+      <c r="B85" s="76" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="C85" s="84" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D85" s="77" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" s="77" t="n">
+        <v>2</v>
+      </c>
+      <c r="F85" s="77" t="n">
+        <v>5</v>
+      </c>
+      <c r="G85" s="79" t="n">
+        <v>2</v>
+      </c>
+      <c r="H85" s="80" t="inlineStr">
+        <is>
+          <t>2–0</t>
+        </is>
+      </c>
+      <c r="I85" s="81" t="n">
+        <v>3</v>
+      </c>
+      <c r="J85" s="77" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" s="78" t="n">
+        <v>4</v>
+      </c>
+      <c r="L85" s="78" t="n">
+        <v>11</v>
+      </c>
+      <c r="M85" s="84" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="N85" s="76" t="inlineStr">
+        <is>
+          <t>Bosnia-Hercegovina</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="14" customHeight="1">
+      <c r="A87" s="63" t="inlineStr">
         <is>
           <t>Treff = skudd på mål  |  Bom = utenfor  |  Blk. = blokkert  |  Grønn bold = flest skudd/treff</t>
         </is>
       </c>
     </row>
-    <row r="87" ht="18" customHeight="1">
-      <c r="A87" s="55" t="inlineStr">
+    <row r="88" ht="18" customHeight="1">
+      <c r="A88" s="55" t="inlineStr">
         <is>
           <t>Besittelse:</t>
         </is>
       </c>
-      <c r="B87" s="62" t="inlineStr">
+      <c r="B88" s="62" t="inlineStr">
         <is>
           <t>≥65% (dominerende)</t>
         </is>
       </c>
-      <c r="C87" s="61" t="inlineStr">
+      <c r="C88" s="61" t="inlineStr">
         <is>
           <t>55–64%</t>
         </is>
       </c>
-      <c r="D87" s="58" t="inlineStr">
+      <c r="D88" s="58" t="inlineStr">
         <is>
           <t>45–54% (jevnt)</t>
         </is>
       </c>
-      <c r="E87" s="85" t="inlineStr">
+      <c r="E88" s="85" t="inlineStr">
         <is>
           <t>≤44%</t>
         </is>
@@ -56411,9 +56459,9 @@
     </row>
   </sheetData>
   <mergeCells count="4">
+    <mergeCell ref="A87:N87"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="I2:N2"/>
-    <mergeCell ref="A86:N86"/>
     <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto-oppdatering 2026-07-02 15:41 UTC
</commit_message>
<xml_diff>
--- a/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
+++ b/VM2026_avansert_gruppetabeller_og_sluttspill.xlsx
@@ -1,42 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finale" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alder" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kort" sheetId="24" state="visible" r:id="rId24"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
+    <sheet name="Gruppe A" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Gruppe B" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Gruppe C" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Gruppe D" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Gruppe E" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Gruppe F" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Gruppe G" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Gruppe H" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Gruppe I" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Gruppe J" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Gruppe K" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Gruppe L" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sluttspill – spillere" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="16-delsfinaler" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="8-delsfinaler" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Kvartfinaler" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Semifinaler" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Bronsefinale" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Finale" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="Aldersfordeling" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="Spillere etter klubbland" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="Klubbdominans" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="Alder" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet name="Kort" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet name="Scorere og assists" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet name="Lagstatistikk" sheetId="26" state="visible" r:id="rId26"/>
+    <sheet name="Scoringstidspunkt" sheetId="27" state="visible" r:id="rId27"/>
+    <sheet name="Heatmap" sheetId="28" state="visible" r:id="rId28"/>
+    <sheet name="Ballbesittelse" sheetId="29" state="visible" r:id="rId29"/>
+    <sheet name="Stadionoversikt" sheetId="30" state="visible" r:id="rId30"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'Spillere etter klubbland'!$A$2:$I$2</definedName>
@@ -914,13 +914,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -939,7 +939,7 @@
           <idx val="0"/>
           <order val="0"/>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -967,8 +967,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -994,8 +994,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1018,7 +1018,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>4</col>
@@ -1033,9 +1033,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>